<commit_message>
prognoza biciklista (osvezavanje): 2026-10-14 11:41
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -564,7 +564,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -614,7 +614,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -664,7 +664,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -714,7 +714,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -814,7 +814,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -964,7 +964,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,17 +10514,17 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="E202" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F202" t="n">
-        <v>7.2</v>
+        <v>6.5</v>
       </c>
       <c r="G202" t="n">
         <v>60</v>
@@ -10564,23 +10564,23 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="E203" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F203" t="n">
-        <v>9.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="G203" t="n">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="H203" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I203" t="n">
         <v>0</v>
@@ -10664,11 +10664,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>11</v>
+        <v>10.8</v>
       </c>
       <c r="E205" t="n">
         <v>55</v>
@@ -10677,10 +10677,10 @@
         <v>6.5</v>
       </c>
       <c r="G205" t="n">
-        <v>490</v>
+        <v>475</v>
       </c>
       <c r="H205" t="n">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="I205" t="n">
         <v>0</v>
@@ -10714,20 +10714,20 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>13.7</v>
+        <v>13.4</v>
       </c>
       <c r="E206" t="n">
         <v>44</v>
       </c>
       <c r="F206" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
       <c r="G206" t="n">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="H206" t="n">
         <v>0</v>
@@ -10764,20 +10764,20 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
       <c r="E207" t="n">
         <v>38</v>
       </c>
       <c r="F207" t="n">
-        <v>11.5</v>
+        <v>12.2</v>
       </c>
       <c r="G207" t="n">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="H207" t="n">
         <v>0</v>
@@ -10814,11 +10814,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="E208" t="n">
         <v>34</v>
@@ -10864,17 +10864,17 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="E209" t="n">
         <v>31</v>
       </c>
       <c r="F209" t="n">
-        <v>13</v>
+        <v>13.7</v>
       </c>
       <c r="G209" t="n">
         <v>479</v>
@@ -10914,11 +10914,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>17.1</v>
+        <v>16.9</v>
       </c>
       <c r="E210" t="n">
         <v>29</v>
@@ -10927,7 +10927,7 @@
         <v>13.7</v>
       </c>
       <c r="G210" t="n">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H210" t="n">
         <v>0</v>
@@ -10964,23 +10964,23 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>16.7</v>
+        <v>16.5</v>
       </c>
       <c r="E211" t="n">
         <v>29</v>
       </c>
       <c r="F211" t="n">
-        <v>12.6</v>
+        <v>11.5</v>
       </c>
       <c r="G211" t="n">
         <v>193</v>
       </c>
       <c r="H211" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="I211" t="n">
         <v>0</v>
@@ -11014,20 +11014,20 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>14.8</v>
+        <v>14.4</v>
       </c>
       <c r="E212" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F212" t="n">
-        <v>9</v>
+        <v>6.8</v>
       </c>
       <c r="G212" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="H212" t="n">
         <v>0</v>
@@ -11064,17 +11064,17 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="E213" t="n">
         <v>39</v>
       </c>
       <c r="F213" t="n">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="G213" t="n">
         <v>0</v>
@@ -11114,17 +11114,17 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>10</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E214" t="n">
         <v>45</v>
       </c>
       <c r="F214" t="n">
-        <v>7.9</v>
+        <v>9</v>
       </c>
       <c r="G214" t="n">
         <v>0</v>
@@ -11164,17 +11164,17 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>9.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="E215" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F215" t="n">
-        <v>11.9</v>
+        <v>8.6</v>
       </c>
       <c r="G215" t="n">
         <v>0</v>
@@ -11214,17 +11214,17 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="E216" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F216" t="n">
-        <v>6.5</v>
+        <v>10.4</v>
       </c>
       <c r="G216" t="n">
         <v>0</v>
@@ -11264,17 +11264,17 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="E217" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F217" t="n">
-        <v>8.6</v>
+        <v>9.4</v>
       </c>
       <c r="G217" t="n">
         <v>0</v>
@@ -11314,17 +11314,17 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="E218" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F218" t="n">
-        <v>9.699999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="G218" t="n">
         <v>0</v>
@@ -11364,17 +11364,17 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>10.8</v>
+        <v>10.5</v>
       </c>
       <c r="E219" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F219" t="n">
-        <v>9.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="G219" t="n">
         <v>0</v>
@@ -11414,17 +11414,17 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="E220" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F220" t="n">
-        <v>11.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G220" t="n">
         <v>0</v>
@@ -11464,17 +11464,17 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="E221" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="F221" t="n">
-        <v>9.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G221" t="n">
         <v>0</v>
@@ -11514,23 +11514,23 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>8.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E222" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="F222" t="n">
-        <v>10.4</v>
+        <v>11.5</v>
       </c>
       <c r="G222" t="n">
         <v>0</v>
       </c>
       <c r="H222" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="I222" t="n">
         <v>0</v>
@@ -11564,23 +11564,23 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="E223" t="n">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="F223" t="n">
-        <v>10.4</v>
+        <v>10.8</v>
       </c>
       <c r="G223" t="n">
         <v>0</v>
       </c>
       <c r="H223" t="n">
-        <v>100</v>
+        <v>42</v>
       </c>
       <c r="I223" t="n">
         <v>0</v>
@@ -11614,23 +11614,23 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D224" t="n">
         <v>6.5</v>
       </c>
       <c r="E224" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="F224" t="n">
-        <v>7.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G224" t="n">
         <v>0</v>
       </c>
       <c r="H224" t="n">
-        <v>100</v>
+        <v>23</v>
       </c>
       <c r="I224" t="n">
         <v>0</v>
@@ -11664,23 +11664,23 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>5.9</v>
+        <v>5.6</v>
       </c>
       <c r="E225" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F225" t="n">
-        <v>8.300000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="G225" t="n">
         <v>0</v>
       </c>
       <c r="H225" t="n">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I225" t="n">
         <v>0</v>
@@ -11714,23 +11714,23 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="E226" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F226" t="n">
-        <v>10.8</v>
+        <v>10.1</v>
       </c>
       <c r="G226" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="H226" t="n">
-        <v>19</v>
+        <v>99</v>
       </c>
       <c r="I226" t="n">
         <v>0</v>
@@ -11764,23 +11764,23 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>8.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="E227" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F227" t="n">
-        <v>11.5</v>
+        <v>10.4</v>
       </c>
       <c r="G227" t="n">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="H227" t="n">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="I227" t="n">
         <v>0</v>
@@ -11814,23 +11814,23 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>11</v>
+        <v>10.8</v>
       </c>
       <c r="E228" t="n">
         <v>76</v>
       </c>
       <c r="F228" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="G228" t="n">
-        <v>349</v>
+        <v>336</v>
       </c>
       <c r="H228" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="I228" t="n">
         <v>0</v>
@@ -11864,23 +11864,23 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>13.7</v>
+        <v>13.5</v>
       </c>
       <c r="E229" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F229" t="n">
-        <v>9</v>
+        <v>10.1</v>
       </c>
       <c r="G229" t="n">
-        <v>470</v>
+        <v>449</v>
       </c>
       <c r="H229" t="n">
-        <v>97</v>
+        <v>54</v>
       </c>
       <c r="I229" t="n">
         <v>0</v>
@@ -11914,23 +11914,23 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
       <c r="E230" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F230" t="n">
         <v>10.4</v>
       </c>
       <c r="G230" t="n">
-        <v>464</v>
+        <v>491</v>
       </c>
       <c r="H230" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="I230" t="n">
         <v>0</v>
@@ -11964,23 +11964,23 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
       <c r="E231" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F231" t="n">
-        <v>11.2</v>
+        <v>10.8</v>
       </c>
       <c r="G231" t="n">
-        <v>419</v>
+        <v>490</v>
       </c>
       <c r="H231" t="n">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
@@ -12014,23 +12014,23 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>17.9</v>
+        <v>18.1</v>
       </c>
       <c r="E232" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F232" t="n">
-        <v>11.9</v>
+        <v>10.8</v>
       </c>
       <c r="G232" t="n">
-        <v>445</v>
+        <v>424</v>
       </c>
       <c r="H232" t="n">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
@@ -12064,23 +12064,23 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="E233" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F233" t="n">
-        <v>13</v>
+        <v>11.5</v>
       </c>
       <c r="G233" t="n">
-        <v>420</v>
+        <v>367</v>
       </c>
       <c r="H233" t="n">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="I233" t="n">
         <v>0</v>
@@ -12114,23 +12114,23 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D234" t="n">
         <v>18.6</v>
       </c>
       <c r="E234" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F234" t="n">
-        <v>15.5</v>
+        <v>12.6</v>
       </c>
       <c r="G234" t="n">
-        <v>337</v>
+        <v>272</v>
       </c>
       <c r="H234" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="I234" t="n">
         <v>0</v>
@@ -12164,23 +12164,23 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>17.8</v>
+        <v>18.2</v>
       </c>
       <c r="E235" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F235" t="n">
-        <v>15.5</v>
+        <v>13.3</v>
       </c>
       <c r="G235" t="n">
-        <v>184</v>
+        <v>149</v>
       </c>
       <c r="H235" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
@@ -12214,23 +12214,23 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>16.6</v>
+        <v>16.8</v>
       </c>
       <c r="E236" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F236" t="n">
-        <v>15.5</v>
+        <v>11.9</v>
       </c>
       <c r="G236" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H236" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -12264,23 +12264,23 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>15.1</v>
+        <v>14.7</v>
       </c>
       <c r="E237" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>13</v>
+        <v>10.8</v>
       </c>
       <c r="G237" t="n">
         <v>0</v>
       </c>
       <c r="H237" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
@@ -12314,17 +12314,17 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>13.9</v>
+        <v>12.7</v>
       </c>
       <c r="E238" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F238" t="n">
-        <v>12.2</v>
+        <v>11.2</v>
       </c>
       <c r="G238" t="n">
         <v>0</v>
@@ -12364,17 +12364,17 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>12.1</v>
+        <v>11.2</v>
       </c>
       <c r="E239" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F239" t="n">
-        <v>10.8</v>
+        <v>11.2</v>
       </c>
       <c r="G239" t="n">
         <v>0</v>
@@ -12414,17 +12414,17 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>10.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E240" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F240" t="n">
-        <v>8.6</v>
+        <v>11.2</v>
       </c>
       <c r="G240" t="n">
         <v>0</v>
@@ -12464,17 +12464,17 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>8.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E241" t="n">
         <v>58</v>
       </c>
       <c r="F241" t="n">
-        <v>6.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G241" t="n">
         <v>0</v>
@@ -12514,17 +12514,17 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="E242" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F242" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -12564,17 +12564,17 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="E243" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F243" t="n">
-        <v>7.2</v>
+        <v>4.7</v>
       </c>
       <c r="G243" t="n">
         <v>0</v>
@@ -12614,17 +12614,17 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>6.6</v>
+        <v>6.1</v>
       </c>
       <c r="E244" t="n">
         <v>71</v>
       </c>
       <c r="F244" t="n">
-        <v>9.699999999999999</v>
+        <v>2.2</v>
       </c>
       <c r="G244" t="n">
         <v>0</v>
@@ -12664,17 +12664,17 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="E245" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F245" t="n">
-        <v>8.6</v>
+        <v>2.9</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -12714,17 +12714,17 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="E246" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F246" t="n">
-        <v>1.8</v>
+        <v>5.4</v>
       </c>
       <c r="G246" t="n">
         <v>0</v>
@@ -12764,17 +12764,17 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="E247" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F247" t="n">
-        <v>2.5</v>
+        <v>6.1</v>
       </c>
       <c r="G247" t="n">
         <v>0</v>
@@ -12814,17 +12814,17 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="E248" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F248" t="n">
-        <v>5.4</v>
+        <v>5</v>
       </c>
       <c r="G248" t="n">
         <v>0</v>
@@ -12864,17 +12864,17 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>4.1</v>
+        <v>3.8</v>
       </c>
       <c r="E249" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F249" t="n">
-        <v>5.8</v>
+        <v>9</v>
       </c>
       <c r="G249" t="n">
         <v>0</v>
@@ -12914,20 +12914,20 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="E250" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F250" t="n">
-        <v>7.9</v>
+        <v>5.4</v>
       </c>
       <c r="G250" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H250" t="n">
         <v>0</v>
@@ -12964,23 +12964,23 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="E251" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F251" t="n">
-        <v>4.7</v>
+        <v>2.9</v>
       </c>
       <c r="G251" t="n">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="H251" t="n">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="I251" t="n">
         <v>0</v>
@@ -13014,20 +13014,20 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E252" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F252" t="n">
-        <v>4.3</v>
+        <v>3.6</v>
       </c>
       <c r="G252" t="n">
-        <v>117</v>
+        <v>191</v>
       </c>
       <c r="H252" t="n">
         <v>100</v>
@@ -13064,23 +13064,23 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>11.7</v>
+        <v>10.2</v>
       </c>
       <c r="E253" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="F253" t="n">
-        <v>10.4</v>
+        <v>3.6</v>
       </c>
       <c r="G253" t="n">
-        <v>329</v>
+        <v>122</v>
       </c>
       <c r="H253" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="I253" t="n">
         <v>0</v>
@@ -13114,23 +13114,23 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>13.9</v>
+        <v>13.6</v>
       </c>
       <c r="E254" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F254" t="n">
-        <v>8.300000000000001</v>
+        <v>6.8</v>
       </c>
       <c r="G254" t="n">
-        <v>550</v>
+        <v>534</v>
       </c>
       <c r="H254" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I254" t="n">
         <v>0</v>
@@ -13164,23 +13164,23 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="E255" t="n">
         <v>43</v>
       </c>
       <c r="F255" t="n">
-        <v>11.2</v>
+        <v>14</v>
       </c>
       <c r="G255" t="n">
-        <v>574</v>
+        <v>524</v>
       </c>
       <c r="H255" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13214,26 +13214,26 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>15.6</v>
+        <v>15.7</v>
       </c>
       <c r="E256" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F256" t="n">
-        <v>14.3</v>
+        <v>14</v>
       </c>
       <c r="G256" t="n">
-        <v>400.3</v>
+        <v>377</v>
       </c>
       <c r="H256" t="n">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="I256" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="J256" t="n">
         <v>0</v>
@@ -13264,23 +13264,23 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>15.5</v>
+        <v>15.8</v>
       </c>
       <c r="E257" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F257" t="n">
-        <v>15.5</v>
+        <v>16.2</v>
       </c>
       <c r="G257" t="n">
-        <v>396.5</v>
+        <v>299</v>
       </c>
       <c r="H257" t="n">
-        <v>34</v>
+        <v>88</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -13314,23 +13314,23 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>15</v>
+        <v>15.7</v>
       </c>
       <c r="E258" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="F258" t="n">
-        <v>17.5</v>
+        <v>16.6</v>
       </c>
       <c r="G258" t="n">
-        <v>289.5</v>
+        <v>247</v>
       </c>
       <c r="H258" t="n">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -13364,23 +13364,23 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>13.7</v>
+        <v>14.8</v>
       </c>
       <c r="E259" t="n">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="F259" t="n">
-        <v>12.8</v>
+        <v>15.4</v>
       </c>
       <c r="G259" t="n">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="H259" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="I259" t="n">
         <v>0</v>
@@ -13414,23 +13414,23 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>11.7</v>
+        <v>13</v>
       </c>
       <c r="E260" t="n">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="F260" t="n">
-        <v>8.5</v>
+        <v>10.4</v>
       </c>
       <c r="G260" t="n">
-        <v>34</v>
+        <v>28.5</v>
       </c>
       <c r="H260" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="I260" t="n">
         <v>0</v>
@@ -13464,23 +13464,23 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="E261" t="n">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="F261" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
       </c>
       <c r="H261" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I261" t="n">
         <v>0</v>
@@ -13514,7 +13514,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -13614,7 +13614,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-14T08:51:17Z</t>
+          <t>2026-10-14T09:39:03Z</t>
         </is>
       </c>
       <c r="D265" t="n">

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-14 13:03
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -564,7 +564,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -614,7 +614,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -664,7 +664,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -714,7 +714,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -814,7 +814,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -964,7 +964,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -10764,7 +10764,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D207" t="n">
@@ -10814,7 +10814,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D208" t="n">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -10914,7 +10914,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -10964,7 +10964,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -11064,7 +11064,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -11164,7 +11164,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D216" t="n">
@@ -11264,7 +11264,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D217" t="n">
@@ -11314,7 +11314,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D218" t="n">
@@ -11364,7 +11364,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D219" t="n">
@@ -11414,7 +11414,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D220" t="n">
@@ -11464,7 +11464,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -11514,7 +11514,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -11564,7 +11564,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D225" t="n">
@@ -11714,7 +11714,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -11764,7 +11764,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D228" t="n">
@@ -11864,7 +11864,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D229" t="n">
@@ -11914,7 +11914,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D230" t="n">
@@ -11964,7 +11964,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D231" t="n">
@@ -12014,7 +12014,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D232" t="n">
@@ -12064,7 +12064,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D233" t="n">
@@ -12114,7 +12114,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -12164,7 +12164,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -12214,7 +12214,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -12264,7 +12264,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -12314,7 +12314,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -12364,7 +12364,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -12414,7 +12414,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -12514,7 +12514,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -12564,7 +12564,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -12664,7 +12664,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -12714,7 +12714,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -12814,7 +12814,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -12864,7 +12864,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -12914,7 +12914,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -12964,7 +12964,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -13014,7 +13014,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -13064,7 +13064,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D253" t="n">
@@ -13114,7 +13114,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -13164,7 +13164,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -13214,7 +13214,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -13314,7 +13314,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -13364,7 +13364,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -13414,7 +13414,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -13464,7 +13464,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D261" t="n">
@@ -13514,7 +13514,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -13614,7 +13614,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-14T09:39:03Z</t>
+          <t>2026-10-14T11:03:18Z</t>
         </is>
       </c>
       <c r="D265" t="n">

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-14 19:04
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N265"/>
+  <dimension ref="A1:N267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -614,7 +614,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -664,7 +664,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -714,7 +714,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -814,7 +814,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -964,7 +964,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10539,7 +10539,7 @@
         <v>0</v>
       </c>
       <c r="K202" t="n">
-        <v>0.336</v>
+        <v>0.342</v>
       </c>
       <c r="L202" t="n">
         <v>3</v>
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -10589,7 +10589,7 @@
         <v>0</v>
       </c>
       <c r="K203" t="n">
-        <v>0.335</v>
+        <v>0.341</v>
       </c>
       <c r="L203" t="n">
         <v>3</v>
@@ -11064,17 +11064,17 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="E213" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F213" t="n">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
       <c r="G213" t="n">
         <v>0</v>
@@ -11089,7 +11089,7 @@
         <v>0</v>
       </c>
       <c r="K213" t="n">
-        <v>0.316</v>
+        <v>0.322</v>
       </c>
       <c r="L213" t="n">
         <v>3</v>
@@ -11114,17 +11114,17 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D214" t="n">
         <v>9.800000000000001</v>
       </c>
       <c r="E214" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F214" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G214" t="n">
         <v>0</v>
@@ -11139,7 +11139,7 @@
         <v>0</v>
       </c>
       <c r="K214" t="n">
-        <v>0.316</v>
+        <v>0.321</v>
       </c>
       <c r="L214" t="n">
         <v>3</v>
@@ -11164,17 +11164,17 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E215" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F215" t="n">
-        <v>8.6</v>
+        <v>5</v>
       </c>
       <c r="G215" t="n">
         <v>0</v>
@@ -11189,7 +11189,7 @@
         <v>0</v>
       </c>
       <c r="K215" t="n">
-        <v>0.315</v>
+        <v>0.32</v>
       </c>
       <c r="L215" t="n">
         <v>3</v>
@@ -11214,17 +11214,17 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>9.5</v>
+        <v>10.1</v>
       </c>
       <c r="E216" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F216" t="n">
-        <v>10.4</v>
+        <v>12.2</v>
       </c>
       <c r="G216" t="n">
         <v>0</v>
@@ -11239,7 +11239,7 @@
         <v>0</v>
       </c>
       <c r="K216" t="n">
-        <v>0.315</v>
+        <v>0.32</v>
       </c>
       <c r="L216" t="n">
         <v>3</v>
@@ -11264,17 +11264,17 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>10.1</v>
+        <v>10.6</v>
       </c>
       <c r="E217" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F217" t="n">
-        <v>9.4</v>
+        <v>7.6</v>
       </c>
       <c r="G217" t="n">
         <v>0</v>
@@ -11289,7 +11289,7 @@
         <v>0</v>
       </c>
       <c r="K217" t="n">
-        <v>0.314</v>
+        <v>0.319</v>
       </c>
       <c r="L217" t="n">
         <v>3</v>
@@ -11314,17 +11314,17 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>10.4</v>
+        <v>10.9</v>
       </c>
       <c r="E218" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F218" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G218" t="n">
         <v>0</v>
@@ -11339,7 +11339,7 @@
         <v>0</v>
       </c>
       <c r="K218" t="n">
-        <v>0.314</v>
+        <v>0.319</v>
       </c>
       <c r="L218" t="n">
         <v>4</v>
@@ -11364,7 +11364,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D219" t="n">
@@ -11374,13 +11374,13 @@
         <v>48</v>
       </c>
       <c r="F219" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G219" t="n">
         <v>0</v>
       </c>
       <c r="H219" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="I219" t="n">
         <v>0</v>
@@ -11389,7 +11389,7 @@
         <v>0</v>
       </c>
       <c r="K219" t="n">
-        <v>0.313</v>
+        <v>0.318</v>
       </c>
       <c r="L219" t="n">
         <v>4</v>
@@ -11414,17 +11414,17 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="E220" t="n">
         <v>51</v>
       </c>
       <c r="F220" t="n">
-        <v>9.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="G220" t="n">
         <v>0</v>
@@ -11439,7 +11439,7 @@
         <v>0</v>
       </c>
       <c r="K220" t="n">
-        <v>0.313</v>
+        <v>0.318</v>
       </c>
       <c r="L220" t="n">
         <v>4</v>
@@ -11464,23 +11464,23 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E221" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F221" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="G221" t="n">
         <v>0</v>
       </c>
       <c r="H221" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="I221" t="n">
         <v>0</v>
@@ -11489,7 +11489,7 @@
         <v>0</v>
       </c>
       <c r="K221" t="n">
-        <v>0.313</v>
+        <v>0.317</v>
       </c>
       <c r="L221" t="n">
         <v>4</v>
@@ -11514,23 +11514,23 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>9.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="E222" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F222" t="n">
-        <v>11.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G222" t="n">
         <v>0</v>
       </c>
       <c r="H222" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="I222" t="n">
         <v>0</v>
@@ -11539,7 +11539,7 @@
         <v>0</v>
       </c>
       <c r="K222" t="n">
-        <v>0.313</v>
+        <v>0.317</v>
       </c>
       <c r="L222" t="n">
         <v>4</v>
@@ -11564,24 +11564,24 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="E223" t="n">
+        <v>74</v>
+      </c>
+      <c r="F223" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="G223" t="n">
+        <v>0</v>
+      </c>
+      <c r="H223" t="n">
         <v>75</v>
       </c>
-      <c r="F223" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="G223" t="n">
-        <v>0</v>
-      </c>
-      <c r="H223" t="n">
-        <v>42</v>
-      </c>
       <c r="I223" t="n">
         <v>0</v>
       </c>
@@ -11589,7 +11589,7 @@
         <v>0</v>
       </c>
       <c r="K223" t="n">
-        <v>0.312</v>
+        <v>0.317</v>
       </c>
       <c r="L223" t="n">
         <v>4</v>
@@ -11614,7 +11614,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -11624,13 +11624,13 @@
         <v>85</v>
       </c>
       <c r="F224" t="n">
-        <v>9.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G224" t="n">
         <v>0</v>
       </c>
       <c r="H224" t="n">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="I224" t="n">
         <v>0</v>
@@ -11639,7 +11639,7 @@
         <v>0</v>
       </c>
       <c r="K224" t="n">
-        <v>0.312</v>
+        <v>0.316</v>
       </c>
       <c r="L224" t="n">
         <v>4</v>
@@ -11664,7 +11664,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D225" t="n">
@@ -11680,7 +11680,7 @@
         <v>0</v>
       </c>
       <c r="H225" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="I225" t="n">
         <v>0</v>
@@ -11689,7 +11689,7 @@
         <v>0</v>
       </c>
       <c r="K225" t="n">
-        <v>0.312</v>
+        <v>0.316</v>
       </c>
       <c r="L225" t="n">
         <v>4</v>
@@ -11714,11 +11714,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="E226" t="n">
         <v>93</v>
@@ -11727,10 +11727,10 @@
         <v>10.1</v>
       </c>
       <c r="G226" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H226" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I226" t="n">
         <v>0</v>
@@ -11739,7 +11739,7 @@
         <v>0</v>
       </c>
       <c r="K226" t="n">
-        <v>0.312</v>
+        <v>0.316</v>
       </c>
       <c r="L226" t="n">
         <v>4</v>
@@ -11764,11 +11764,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>8.1</v>
+        <v>8.4</v>
       </c>
       <c r="E227" t="n">
         <v>85</v>
@@ -11777,10 +11777,10 @@
         <v>10.4</v>
       </c>
       <c r="G227" t="n">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H227" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I227" t="n">
         <v>0</v>
@@ -11789,7 +11789,7 @@
         <v>0</v>
       </c>
       <c r="K227" t="n">
-        <v>0.311</v>
+        <v>0.315</v>
       </c>
       <c r="L227" t="n">
         <v>4</v>
@@ -11814,23 +11814,23 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>10.8</v>
+        <v>11.2</v>
       </c>
       <c r="E228" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F228" t="n">
         <v>10.4</v>
       </c>
       <c r="G228" t="n">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="H228" t="n">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="I228" t="n">
         <v>0</v>
@@ -11839,7 +11839,7 @@
         <v>0</v>
       </c>
       <c r="K228" t="n">
-        <v>0.31</v>
+        <v>0.314</v>
       </c>
       <c r="L228" t="n">
         <v>4</v>
@@ -11864,23 +11864,23 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>13.5</v>
+        <v>14</v>
       </c>
       <c r="E229" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F229" t="n">
-        <v>10.1</v>
+        <v>10.4</v>
       </c>
       <c r="G229" t="n">
-        <v>449</v>
+        <v>474</v>
       </c>
       <c r="H229" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="I229" t="n">
         <v>0</v>
@@ -11889,7 +11889,7 @@
         <v>0</v>
       </c>
       <c r="K229" t="n">
-        <v>0.309</v>
+        <v>0.313</v>
       </c>
       <c r="L229" t="n">
         <v>4</v>
@@ -11914,23 +11914,23 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>15.8</v>
+        <v>16.6</v>
       </c>
       <c r="E230" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F230" t="n">
-        <v>10.4</v>
+        <v>11.5</v>
       </c>
       <c r="G230" t="n">
-        <v>491</v>
+        <v>553</v>
       </c>
       <c r="H230" t="n">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="I230" t="n">
         <v>0</v>
@@ -11939,7 +11939,7 @@
         <v>0</v>
       </c>
       <c r="K230" t="n">
-        <v>0.307</v>
+        <v>0.311</v>
       </c>
       <c r="L230" t="n">
         <v>4</v>
@@ -11964,23 +11964,23 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>17.4</v>
+        <v>18.1</v>
       </c>
       <c r="E231" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>10.8</v>
+        <v>13.3</v>
       </c>
       <c r="G231" t="n">
-        <v>490</v>
+        <v>552</v>
       </c>
       <c r="H231" t="n">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
@@ -11989,7 +11989,7 @@
         <v>0</v>
       </c>
       <c r="K231" t="n">
-        <v>0.304</v>
+        <v>0.309</v>
       </c>
       <c r="L231" t="n">
         <v>4</v>
@@ -12014,23 +12014,23 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>18.1</v>
+        <v>18.8</v>
       </c>
       <c r="E232" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="F232" t="n">
-        <v>10.8</v>
+        <v>13.3</v>
       </c>
       <c r="G232" t="n">
-        <v>424</v>
+        <v>497</v>
       </c>
       <c r="H232" t="n">
-        <v>82</v>
+        <v>52</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
@@ -12039,7 +12039,7 @@
         <v>0</v>
       </c>
       <c r="K232" t="n">
-        <v>0.302</v>
+        <v>0.307</v>
       </c>
       <c r="L232" t="n">
         <v>4</v>
@@ -12064,23 +12064,23 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>18.6</v>
+        <v>19.1</v>
       </c>
       <c r="E233" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F233" t="n">
-        <v>11.5</v>
+        <v>13</v>
       </c>
       <c r="G233" t="n">
-        <v>367</v>
+        <v>395</v>
       </c>
       <c r="H233" t="n">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="I233" t="n">
         <v>0</v>
@@ -12089,7 +12089,7 @@
         <v>0</v>
       </c>
       <c r="K233" t="n">
-        <v>0.3</v>
+        <v>0.305</v>
       </c>
       <c r="L233" t="n">
         <v>4</v>
@@ -12114,23 +12114,23 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>18.6</v>
+        <v>19</v>
       </c>
       <c r="E234" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F234" t="n">
-        <v>12.6</v>
+        <v>13.3</v>
       </c>
       <c r="G234" t="n">
-        <v>272</v>
+        <v>314</v>
       </c>
       <c r="H234" t="n">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="I234" t="n">
         <v>0</v>
@@ -12139,7 +12139,7 @@
         <v>0</v>
       </c>
       <c r="K234" t="n">
-        <v>0.298</v>
+        <v>0.303</v>
       </c>
       <c r="L234" t="n">
         <v>4</v>
@@ -12164,23 +12164,23 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="E235" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F235" t="n">
-        <v>13.3</v>
+        <v>15.8</v>
       </c>
       <c r="G235" t="n">
-        <v>149</v>
+        <v>183</v>
       </c>
       <c r="H235" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
@@ -12189,7 +12189,7 @@
         <v>0</v>
       </c>
       <c r="K235" t="n">
-        <v>0.297</v>
+        <v>0.302</v>
       </c>
       <c r="L235" t="n">
         <v>4</v>
@@ -12214,7 +12214,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -12224,13 +12224,13 @@
         <v>36</v>
       </c>
       <c r="F236" t="n">
-        <v>11.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G236" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H236" t="n">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -12239,7 +12239,7 @@
         <v>0</v>
       </c>
       <c r="K236" t="n">
-        <v>0.296</v>
+        <v>0.301</v>
       </c>
       <c r="L236" t="n">
         <v>4</v>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>14.7</v>
+        <v>14.9</v>
       </c>
       <c r="E237" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F237" t="n">
-        <v>10.8</v>
+        <v>11.9</v>
       </c>
       <c r="G237" t="n">
         <v>0</v>
@@ -12289,7 +12289,7 @@
         <v>0</v>
       </c>
       <c r="K237" t="n">
-        <v>0.296</v>
+        <v>0.301</v>
       </c>
       <c r="L237" t="n">
         <v>4</v>
@@ -12314,17 +12314,17 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>12.7</v>
+        <v>12.9</v>
       </c>
       <c r="E238" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>11.2</v>
+        <v>11.9</v>
       </c>
       <c r="G238" t="n">
         <v>0</v>
@@ -12339,7 +12339,7 @@
         <v>0</v>
       </c>
       <c r="K238" t="n">
-        <v>0.296</v>
+        <v>0.3</v>
       </c>
       <c r="L238" t="n">
         <v>4</v>
@@ -12364,17 +12364,17 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="E239" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F239" t="n">
-        <v>11.2</v>
+        <v>11.9</v>
       </c>
       <c r="G239" t="n">
         <v>0</v>
@@ -12389,7 +12389,7 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>0.296</v>
+        <v>0.3</v>
       </c>
       <c r="L239" t="n">
         <v>4</v>
@@ -12414,17 +12414,17 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E240" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F240" t="n">
-        <v>11.2</v>
+        <v>7.6</v>
       </c>
       <c r="G240" t="n">
         <v>0</v>
@@ -12439,7 +12439,7 @@
         <v>0</v>
       </c>
       <c r="K240" t="n">
-        <v>0.295</v>
+        <v>0.3</v>
       </c>
       <c r="L240" t="n">
         <v>4</v>
@@ -12464,17 +12464,17 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>8.699999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E241" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F241" t="n">
-        <v>9.699999999999999</v>
+        <v>4.3</v>
       </c>
       <c r="G241" t="n">
         <v>0</v>
@@ -12489,7 +12489,7 @@
         <v>0</v>
       </c>
       <c r="K241" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L241" t="n">
         <v>4</v>
@@ -12514,17 +12514,17 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="E242" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F242" t="n">
-        <v>6.8</v>
+        <v>2.9</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -12539,7 +12539,7 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L242" t="n">
         <v>5</v>
@@ -12564,11 +12564,11 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="E243" t="n">
         <v>67</v>
@@ -12589,7 +12589,7 @@
         <v>0</v>
       </c>
       <c r="K243" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L243" t="n">
         <v>5</v>
@@ -12614,17 +12614,17 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="E244" t="n">
         <v>71</v>
       </c>
       <c r="F244" t="n">
-        <v>2.2</v>
+        <v>6.1</v>
       </c>
       <c r="G244" t="n">
         <v>0</v>
@@ -12639,7 +12639,7 @@
         <v>0</v>
       </c>
       <c r="K244" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L244" t="n">
         <v>5</v>
@@ -12664,17 +12664,17 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="E245" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F245" t="n">
-        <v>2.9</v>
+        <v>6.1</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -12689,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L245" t="n">
         <v>5</v>
@@ -12714,17 +12714,17 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="E246" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F246" t="n">
-        <v>5.4</v>
+        <v>6.5</v>
       </c>
       <c r="G246" t="n">
         <v>0</v>
@@ -12739,7 +12739,7 @@
         <v>0</v>
       </c>
       <c r="K246" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L246" t="n">
         <v>5</v>
@@ -12764,17 +12764,17 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
       <c r="E247" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F247" t="n">
-        <v>6.1</v>
+        <v>7.9</v>
       </c>
       <c r="G247" t="n">
         <v>0</v>
@@ -12789,7 +12789,7 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L247" t="n">
         <v>5</v>
@@ -12814,17 +12814,17 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="E248" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F248" t="n">
-        <v>5</v>
+        <v>2.9</v>
       </c>
       <c r="G248" t="n">
         <v>0</v>
@@ -12839,7 +12839,7 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L248" t="n">
         <v>5</v>
@@ -12864,17 +12864,17 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D249" t="n">
         <v>3.8</v>
       </c>
       <c r="E249" t="n">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="F249" t="n">
-        <v>9</v>
+        <v>3.6</v>
       </c>
       <c r="G249" t="n">
         <v>0</v>
@@ -12889,7 +12889,7 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L249" t="n">
         <v>5</v>
@@ -12914,20 +12914,20 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="E250" t="n">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="F250" t="n">
-        <v>5.4</v>
+        <v>4.7</v>
       </c>
       <c r="G250" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H250" t="n">
         <v>0</v>
@@ -12939,7 +12939,7 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L250" t="n">
         <v>5</v>
@@ -12964,23 +12964,23 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="E251" t="n">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="F251" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="G251" t="n">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H251" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I251" t="n">
         <v>0</v>
@@ -12989,7 +12989,7 @@
         <v>0</v>
       </c>
       <c r="K251" t="n">
-        <v>0.295</v>
+        <v>0.299</v>
       </c>
       <c r="L251" t="n">
         <v>5</v>
@@ -13014,23 +13014,23 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>9.300000000000001</v>
+        <v>11.1</v>
       </c>
       <c r="E252" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="F252" t="n">
-        <v>3.6</v>
+        <v>5</v>
       </c>
       <c r="G252" t="n">
-        <v>191</v>
+        <v>353</v>
       </c>
       <c r="H252" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I252" t="n">
         <v>0</v>
@@ -13039,7 +13039,7 @@
         <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>0.294</v>
+        <v>0.298</v>
       </c>
       <c r="L252" t="n">
         <v>5</v>
@@ -13064,23 +13064,23 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>10.2</v>
+        <v>13.7</v>
       </c>
       <c r="E253" t="n">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="F253" t="n">
-        <v>3.6</v>
+        <v>7.2</v>
       </c>
       <c r="G253" t="n">
-        <v>122</v>
+        <v>475</v>
       </c>
       <c r="H253" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="I253" t="n">
         <v>0</v>
@@ -13089,7 +13089,7 @@
         <v>0</v>
       </c>
       <c r="K253" t="n">
-        <v>0.293</v>
+        <v>0.297</v>
       </c>
       <c r="L253" t="n">
         <v>5</v>
@@ -13114,23 +13114,23 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>13.6</v>
+        <v>14.6</v>
       </c>
       <c r="E254" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F254" t="n">
-        <v>6.8</v>
+        <v>14.8</v>
       </c>
       <c r="G254" t="n">
-        <v>534</v>
+        <v>420</v>
       </c>
       <c r="H254" t="n">
-        <v>3</v>
+        <v>69</v>
       </c>
       <c r="I254" t="n">
         <v>0</v>
@@ -13139,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="K254" t="n">
-        <v>0.291</v>
+        <v>0.295</v>
       </c>
       <c r="L254" t="n">
         <v>5</v>
@@ -13164,23 +13164,23 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>15.6</v>
+        <v>14.5</v>
       </c>
       <c r="E255" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="F255" t="n">
-        <v>14</v>
+        <v>10.8</v>
       </c>
       <c r="G255" t="n">
-        <v>524</v>
+        <v>405</v>
       </c>
       <c r="H255" t="n">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13189,7 +13189,7 @@
         <v>0</v>
       </c>
       <c r="K255" t="n">
-        <v>0.29</v>
+        <v>0.294</v>
       </c>
       <c r="L255" t="n">
         <v>5</v>
@@ -13214,11 +13214,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="E256" t="n">
         <v>41</v>
@@ -13227,10 +13227,10 @@
         <v>14</v>
       </c>
       <c r="G256" t="n">
-        <v>377</v>
+        <v>537</v>
       </c>
       <c r="H256" t="n">
-        <v>78</v>
+        <v>4</v>
       </c>
       <c r="I256" t="n">
         <v>0</v>
@@ -13239,7 +13239,7 @@
         <v>0</v>
       </c>
       <c r="K256" t="n">
-        <v>0.288</v>
+        <v>0.292</v>
       </c>
       <c r="L256" t="n">
         <v>5</v>
@@ -13264,11 +13264,11 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>15.8</v>
+        <v>16</v>
       </c>
       <c r="E257" t="n">
         <v>39</v>
@@ -13277,10 +13277,10 @@
         <v>16.2</v>
       </c>
       <c r="G257" t="n">
-        <v>299</v>
+        <v>360</v>
       </c>
       <c r="H257" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -13289,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="K257" t="n">
-        <v>0.287</v>
+        <v>0.29</v>
       </c>
       <c r="L257" t="n">
         <v>5</v>
@@ -13314,20 +13314,20 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>15.7</v>
+        <v>16</v>
       </c>
       <c r="E258" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F258" t="n">
-        <v>16.6</v>
+        <v>17.6</v>
       </c>
       <c r="G258" t="n">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="H258" t="n">
         <v>74</v>
@@ -13339,7 +13339,7 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
-        <v>0.285</v>
+        <v>0.289</v>
       </c>
       <c r="L258" t="n">
         <v>5</v>
@@ -13364,23 +13364,23 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>14.8</v>
+        <v>15.3</v>
       </c>
       <c r="E259" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>15.4</v>
+        <v>16.6</v>
       </c>
       <c r="G259" t="n">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="H259" t="n">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="I259" t="n">
         <v>0</v>
@@ -13389,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>0.284</v>
+        <v>0.288</v>
       </c>
       <c r="L259" t="n">
         <v>5</v>
@@ -13414,23 +13414,23 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>13</v>
+        <v>13.7</v>
       </c>
       <c r="E260" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F260" t="n">
         <v>10.4</v>
       </c>
       <c r="G260" t="n">
-        <v>28.5</v>
+        <v>35</v>
       </c>
       <c r="H260" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="I260" t="n">
         <v>0</v>
@@ -13439,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>0.284</v>
+        <v>0.287</v>
       </c>
       <c r="L260" t="n">
         <v>5</v>
@@ -13464,23 +13464,23 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>10.5</v>
+        <v>11.4</v>
       </c>
       <c r="E261" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="F261" t="n">
-        <v>6.4</v>
+        <v>5.8</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
       </c>
       <c r="H261" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I261" t="n">
         <v>0</v>
@@ -13489,7 +13489,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>0.284</v>
+        <v>0.287</v>
       </c>
       <c r="L261" t="n">
         <v>5</v>
@@ -13514,23 +13514,23 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D262" t="n">
         <v>9.4</v>
       </c>
       <c r="E262" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="F262" t="n">
-        <v>4.8</v>
+        <v>5.4</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
       </c>
       <c r="H262" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I262" t="n">
         <v>0</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.283</v>
+        <v>0.287</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,23 +13564,23 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="E263" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="F263" t="n">
-        <v>1.3</v>
+        <v>7.6</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
       </c>
       <c r="H263" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.284</v>
+        <v>0.287</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,23 +13614,23 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="E264" t="n">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="F264" t="n">
-        <v>3.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
       </c>
       <c r="H264" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.284</v>
+        <v>0.287</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,23 +13664,23 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-14T11:03:18Z</t>
+          <t>2026-10-14T17:03:52Z</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>7.1</v>
+        <v>6.5</v>
       </c>
       <c r="E265" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="F265" t="n">
-        <v>4.2</v>
+        <v>7.2</v>
       </c>
       <c r="G265" t="n">
         <v>0</v>
       </c>
       <c r="H265" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.284</v>
+        <v>0.287</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13698,6 +13698,106 @@
         <v>0</v>
       </c>
       <c r="N265" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:03:52Z</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E266" t="n">
+        <v>79</v>
+      </c>
+      <c r="F266" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H266" t="n">
+        <v>0</v>
+      </c>
+      <c r="I266" t="n">
+        <v>0</v>
+      </c>
+      <c r="J266" t="n">
+        <v>0</v>
+      </c>
+      <c r="K266" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="L266" t="n">
+        <v>6</v>
+      </c>
+      <c r="M266" t="n">
+        <v>1</v>
+      </c>
+      <c r="N266" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:03:52Z</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E267" t="n">
+        <v>80</v>
+      </c>
+      <c r="F267" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G267" t="n">
+        <v>0</v>
+      </c>
+      <c r="H267" t="n">
+        <v>0</v>
+      </c>
+      <c r="I267" t="n">
+        <v>0</v>
+      </c>
+      <c r="J267" t="n">
+        <v>0</v>
+      </c>
+      <c r="K267" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="L267" t="n">
+        <v>6</v>
+      </c>
+      <c r="M267" t="n">
+        <v>1</v>
+      </c>
+      <c r="N267" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prognoza biciklista (zvanicna): 2026-10-15 01:03
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -664,7 +664,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -714,7 +714,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -764,7 +764,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -814,7 +814,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -914,7 +914,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -964,7 +964,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -11364,23 +11364,23 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="E219" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F219" t="n">
-        <v>8.300000000000001</v>
+        <v>6.8</v>
       </c>
       <c r="G219" t="n">
         <v>0</v>
       </c>
       <c r="H219" t="n">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="I219" t="n">
         <v>0</v>
@@ -11414,17 +11414,17 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="E220" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F220" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="G220" t="n">
         <v>0</v>
@@ -11439,7 +11439,7 @@
         <v>0</v>
       </c>
       <c r="K220" t="n">
-        <v>0.318</v>
+        <v>0.317</v>
       </c>
       <c r="L220" t="n">
         <v>4</v>
@@ -11464,23 +11464,23 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>9.800000000000001</v>
+        <v>10.2</v>
       </c>
       <c r="E221" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F221" t="n">
-        <v>9.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G221" t="n">
         <v>0</v>
       </c>
       <c r="H221" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="I221" t="n">
         <v>0</v>
@@ -11514,14 +11514,14 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="E222" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F222" t="n">
         <v>9.699999999999999</v>
@@ -11530,7 +11530,7 @@
         <v>0</v>
       </c>
       <c r="H222" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I222" t="n">
         <v>0</v>
@@ -11539,7 +11539,7 @@
         <v>0</v>
       </c>
       <c r="K222" t="n">
-        <v>0.317</v>
+        <v>0.316</v>
       </c>
       <c r="L222" t="n">
         <v>4</v>
@@ -11564,14 +11564,14 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>7.6</v>
+        <v>7.9</v>
       </c>
       <c r="E223" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F223" t="n">
         <v>9.699999999999999</v>
@@ -11580,7 +11580,7 @@
         <v>0</v>
       </c>
       <c r="H223" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="I223" t="n">
         <v>0</v>
@@ -11589,7 +11589,7 @@
         <v>0</v>
       </c>
       <c r="K223" t="n">
-        <v>0.317</v>
+        <v>0.316</v>
       </c>
       <c r="L223" t="n">
         <v>4</v>
@@ -11614,23 +11614,23 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="E224" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F224" t="n">
-        <v>10.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G224" t="n">
         <v>0</v>
       </c>
       <c r="H224" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I224" t="n">
         <v>0</v>
@@ -11664,17 +11664,17 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="E225" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F225" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G225" t="n">
         <v>0</v>
@@ -11714,20 +11714,20 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="E226" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F226" t="n">
-        <v>10.1</v>
+        <v>9.4</v>
       </c>
       <c r="G226" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H226" t="n">
         <v>100</v>
@@ -11739,7 +11739,7 @@
         <v>0</v>
       </c>
       <c r="K226" t="n">
-        <v>0.316</v>
+        <v>0.315</v>
       </c>
       <c r="L226" t="n">
         <v>4</v>
@@ -11764,23 +11764,23 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D227" t="n">
         <v>8.4</v>
       </c>
       <c r="E227" t="n">
+        <v>83</v>
+      </c>
+      <c r="F227" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G227" t="n">
+        <v>165</v>
+      </c>
+      <c r="H227" t="n">
         <v>85</v>
-      </c>
-      <c r="F227" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="G227" t="n">
-        <v>185</v>
-      </c>
-      <c r="H227" t="n">
-        <v>100</v>
       </c>
       <c r="I227" t="n">
         <v>0</v>
@@ -11814,23 +11814,23 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>11.2</v>
+        <v>10.8</v>
       </c>
       <c r="E228" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F228" t="n">
-        <v>10.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G228" t="n">
-        <v>342</v>
+        <v>297</v>
       </c>
       <c r="H228" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="I228" t="n">
         <v>0</v>
@@ -11864,23 +11864,23 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>14</v>
+        <v>12.9</v>
       </c>
       <c r="E229" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F229" t="n">
-        <v>10.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G229" t="n">
-        <v>474</v>
+        <v>290</v>
       </c>
       <c r="H229" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I229" t="n">
         <v>0</v>
@@ -11914,23 +11914,23 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>16.6</v>
+        <v>14.9</v>
       </c>
       <c r="E230" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F230" t="n">
-        <v>11.5</v>
+        <v>8.6</v>
       </c>
       <c r="G230" t="n">
-        <v>553</v>
+        <v>350</v>
       </c>
       <c r="H230" t="n">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="I230" t="n">
         <v>0</v>
@@ -11964,23 +11964,23 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>18.1</v>
+        <v>17</v>
       </c>
       <c r="E231" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F231" t="n">
-        <v>13.3</v>
+        <v>10.1</v>
       </c>
       <c r="G231" t="n">
-        <v>552</v>
+        <v>399</v>
       </c>
       <c r="H231" t="n">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
@@ -12014,23 +12014,23 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>18.8</v>
+        <v>18.1</v>
       </c>
       <c r="E232" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="F232" t="n">
-        <v>13.3</v>
+        <v>10.8</v>
       </c>
       <c r="G232" t="n">
-        <v>497</v>
+        <v>401</v>
       </c>
       <c r="H232" t="n">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
@@ -12064,23 +12064,23 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>19.1</v>
+        <v>18.7</v>
       </c>
       <c r="E233" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F233" t="n">
-        <v>13</v>
+        <v>11.5</v>
       </c>
       <c r="G233" t="n">
-        <v>395</v>
+        <v>347</v>
       </c>
       <c r="H233" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="I233" t="n">
         <v>0</v>
@@ -12114,23 +12114,23 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="E234" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F234" t="n">
-        <v>13.3</v>
+        <v>14</v>
       </c>
       <c r="G234" t="n">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="H234" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="I234" t="n">
         <v>0</v>
@@ -12164,23 +12164,23 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>18.4</v>
+        <v>18.1</v>
       </c>
       <c r="E235" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F235" t="n">
-        <v>15.8</v>
+        <v>14.4</v>
       </c>
       <c r="G235" t="n">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="H235" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
@@ -12214,23 +12214,23 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>16.8</v>
+        <v>16.2</v>
       </c>
       <c r="E236" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>9.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G236" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H236" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -12239,7 +12239,7 @@
         <v>0</v>
       </c>
       <c r="K236" t="n">
-        <v>0.301</v>
+        <v>0.302</v>
       </c>
       <c r="L236" t="n">
         <v>4</v>
@@ -12264,23 +12264,23 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>14.9</v>
+        <v>14.3</v>
       </c>
       <c r="E237" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F237" t="n">
-        <v>11.9</v>
+        <v>7.9</v>
       </c>
       <c r="G237" t="n">
         <v>0</v>
       </c>
       <c r="H237" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
@@ -12314,23 +12314,23 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>12.9</v>
+        <v>13.1</v>
       </c>
       <c r="E238" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F238" t="n">
-        <v>11.9</v>
+        <v>10.8</v>
       </c>
       <c r="G238" t="n">
         <v>0</v>
       </c>
       <c r="H238" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I238" t="n">
         <v>0</v>
@@ -12339,7 +12339,7 @@
         <v>0</v>
       </c>
       <c r="K238" t="n">
-        <v>0.3</v>
+        <v>0.301</v>
       </c>
       <c r="L238" t="n">
         <v>4</v>
@@ -12364,17 +12364,17 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="E239" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F239" t="n">
-        <v>11.9</v>
+        <v>13</v>
       </c>
       <c r="G239" t="n">
         <v>0</v>
@@ -12389,7 +12389,7 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>0.3</v>
+        <v>0.301</v>
       </c>
       <c r="L239" t="n">
         <v>4</v>
@@ -12414,17 +12414,17 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>9.699999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="E240" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F240" t="n">
-        <v>7.6</v>
+        <v>10.4</v>
       </c>
       <c r="G240" t="n">
         <v>0</v>
@@ -12464,17 +12464,17 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>8.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="E241" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F241" t="n">
-        <v>4.3</v>
+        <v>9</v>
       </c>
       <c r="G241" t="n">
         <v>0</v>
@@ -12489,7 +12489,7 @@
         <v>0</v>
       </c>
       <c r="K241" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L241" t="n">
         <v>4</v>
@@ -12514,17 +12514,17 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>7.1</v>
+        <v>7.6</v>
       </c>
       <c r="E242" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="F242" t="n">
-        <v>2.9</v>
+        <v>6.8</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -12539,7 +12539,7 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L242" t="n">
         <v>5</v>
@@ -12564,17 +12564,17 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D243" t="n">
         <v>6.5</v>
       </c>
       <c r="E243" t="n">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="F243" t="n">
-        <v>4.7</v>
+        <v>2.5</v>
       </c>
       <c r="G243" t="n">
         <v>0</v>
@@ -12589,7 +12589,7 @@
         <v>0</v>
       </c>
       <c r="K243" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L243" t="n">
         <v>5</v>
@@ -12614,17 +12614,17 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D244" t="n">
         <v>5.8</v>
       </c>
       <c r="E244" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F244" t="n">
-        <v>6.1</v>
+        <v>3.6</v>
       </c>
       <c r="G244" t="n">
         <v>0</v>
@@ -12639,7 +12639,7 @@
         <v>0</v>
       </c>
       <c r="K244" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L244" t="n">
         <v>5</v>
@@ -12664,17 +12664,17 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D245" t="n">
         <v>5.2</v>
       </c>
       <c r="E245" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F245" t="n">
-        <v>6.1</v>
+        <v>4</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -12689,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L245" t="n">
         <v>5</v>
@@ -12714,17 +12714,17 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D246" t="n">
         <v>4.6</v>
       </c>
       <c r="E246" t="n">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="F246" t="n">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="G246" t="n">
         <v>0</v>
@@ -12739,7 +12739,7 @@
         <v>0</v>
       </c>
       <c r="K246" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L246" t="n">
         <v>5</v>
@@ -12764,17 +12764,17 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>4.8</v>
+        <v>4.1</v>
       </c>
       <c r="E247" t="n">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="F247" t="n">
-        <v>7.9</v>
+        <v>5</v>
       </c>
       <c r="G247" t="n">
         <v>0</v>
@@ -12789,7 +12789,7 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L247" t="n">
         <v>5</v>
@@ -12814,17 +12814,17 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="E248" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F248" t="n">
-        <v>2.9</v>
+        <v>5</v>
       </c>
       <c r="G248" t="n">
         <v>0</v>
@@ -12839,7 +12839,7 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L248" t="n">
         <v>5</v>
@@ -12864,17 +12864,17 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="E249" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F249" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="G249" t="n">
         <v>0</v>
@@ -12889,7 +12889,7 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L249" t="n">
         <v>5</v>
@@ -12914,17 +12914,17 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="E250" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F250" t="n">
-        <v>4.7</v>
+        <v>6.8</v>
       </c>
       <c r="G250" t="n">
         <v>54</v>
@@ -12939,7 +12939,7 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>0.299</v>
+        <v>0.3</v>
       </c>
       <c r="L250" t="n">
         <v>5</v>
@@ -12964,20 +12964,20 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="E251" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F251" t="n">
-        <v>3.6</v>
+        <v>2.5</v>
       </c>
       <c r="G251" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H251" t="n">
         <v>0</v>
@@ -13014,20 +13014,20 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="E252" t="n">
         <v>65</v>
       </c>
       <c r="F252" t="n">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="G252" t="n">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H252" t="n">
         <v>0</v>
@@ -13039,7 +13039,7 @@
         <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>0.298</v>
+        <v>0.299</v>
       </c>
       <c r="L252" t="n">
         <v>5</v>
@@ -13064,23 +13064,23 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>13.7</v>
+        <v>14.2</v>
       </c>
       <c r="E253" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F253" t="n">
-        <v>7.2</v>
+        <v>9.4</v>
       </c>
       <c r="G253" t="n">
         <v>475</v>
       </c>
       <c r="H253" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I253" t="n">
         <v>0</v>
@@ -13114,23 +13114,23 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>14.6</v>
+        <v>15.4</v>
       </c>
       <c r="E254" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F254" t="n">
-        <v>14.8</v>
+        <v>12.6</v>
       </c>
       <c r="G254" t="n">
-        <v>420</v>
+        <v>503</v>
       </c>
       <c r="H254" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="I254" t="n">
         <v>0</v>
@@ -13139,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="K254" t="n">
-        <v>0.295</v>
+        <v>0.296</v>
       </c>
       <c r="L254" t="n">
         <v>5</v>
@@ -13164,23 +13164,23 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>14.5</v>
+        <v>16.2</v>
       </c>
       <c r="E255" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="F255" t="n">
-        <v>10.8</v>
+        <v>16.6</v>
       </c>
       <c r="G255" t="n">
-        <v>405</v>
+        <v>544</v>
       </c>
       <c r="H255" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13214,23 +13214,23 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D256" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="E256" t="n">
+        <v>38</v>
+      </c>
+      <c r="F256" t="n">
         <v>15.8</v>
       </c>
-      <c r="E256" t="n">
-        <v>41</v>
-      </c>
-      <c r="F256" t="n">
-        <v>14</v>
-      </c>
       <c r="G256" t="n">
-        <v>537</v>
+        <v>493</v>
       </c>
       <c r="H256" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="I256" t="n">
         <v>0</v>
@@ -13264,11 +13264,11 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>16</v>
+        <v>16.5</v>
       </c>
       <c r="E257" t="n">
         <v>39</v>
@@ -13277,10 +13277,10 @@
         <v>16.2</v>
       </c>
       <c r="G257" t="n">
-        <v>360</v>
+        <v>373</v>
       </c>
       <c r="H257" t="n">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -13314,23 +13314,23 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>16</v>
+        <v>16.3</v>
       </c>
       <c r="E258" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F258" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="G258" t="n">
-        <v>237</v>
+        <v>263</v>
       </c>
       <c r="H258" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -13339,7 +13339,7 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
-        <v>0.289</v>
+        <v>0.288</v>
       </c>
       <c r="L258" t="n">
         <v>5</v>
@@ -13364,23 +13364,23 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>15.3</v>
+        <v>15.8</v>
       </c>
       <c r="E259" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F259" t="n">
-        <v>16.6</v>
+        <v>16.9</v>
       </c>
       <c r="G259" t="n">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="H259" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="I259" t="n">
         <v>0</v>
@@ -13389,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>0.288</v>
+        <v>0.287</v>
       </c>
       <c r="L259" t="n">
         <v>5</v>
@@ -13414,20 +13414,20 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>13.7</v>
+        <v>14</v>
       </c>
       <c r="E260" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F260" t="n">
-        <v>10.4</v>
+        <v>9</v>
       </c>
       <c r="G260" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H260" t="n">
         <v>0</v>
@@ -13464,14 +13464,14 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="E261" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F261" t="n">
         <v>5.8</v>
@@ -13514,17 +13514,17 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>9.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E262" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F262" t="n">
-        <v>5.4</v>
+        <v>7.9</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.287</v>
+        <v>0.286</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,23 +13564,23 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8</v>
+        <v>8.4</v>
       </c>
       <c r="E263" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="F263" t="n">
-        <v>7.6</v>
+        <v>6.8</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
       </c>
       <c r="H263" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.287</v>
+        <v>0.286</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,23 +13614,23 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="E264" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F264" t="n">
-        <v>9.699999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
       </c>
       <c r="H264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.287</v>
+        <v>0.286</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,17 +13664,17 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D265" t="n">
         <v>6.5</v>
       </c>
       <c r="E265" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F265" t="n">
-        <v>7.2</v>
+        <v>6.5</v>
       </c>
       <c r="G265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.287</v>
+        <v>0.286</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13714,17 +13714,17 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D266" t="n">
         <v>5.8</v>
       </c>
       <c r="E266" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="F266" t="n">
-        <v>6.1</v>
+        <v>4</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -13739,7 +13739,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>0.287</v>
+        <v>0.286</v>
       </c>
       <c r="L266" t="n">
         <v>6</v>
@@ -13764,17 +13764,17 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-14T17:03:52Z</t>
+          <t>2026-10-14T23:03:38Z</t>
         </is>
       </c>
       <c r="D267" t="n">
         <v>5.4</v>
       </c>
       <c r="E267" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F267" t="n">
-        <v>2.9</v>
+        <v>5</v>
       </c>
       <c r="G267" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-15 07:04
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N267"/>
+  <dimension ref="A1:N291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -11664,17 +11664,17 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>5.8</v>
+        <v>5.1</v>
       </c>
       <c r="E225" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F225" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="G225" t="n">
         <v>0</v>
@@ -11689,7 +11689,7 @@
         <v>0</v>
       </c>
       <c r="K225" t="n">
-        <v>0.316</v>
+        <v>0.312</v>
       </c>
       <c r="L225" t="n">
         <v>4</v>
@@ -11714,20 +11714,20 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>6.3</v>
+        <v>5.7</v>
       </c>
       <c r="E226" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F226" t="n">
-        <v>9.4</v>
+        <v>9</v>
       </c>
       <c r="G226" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="H226" t="n">
         <v>100</v>
@@ -11739,7 +11739,7 @@
         <v>0</v>
       </c>
       <c r="K226" t="n">
-        <v>0.315</v>
+        <v>0.312</v>
       </c>
       <c r="L226" t="n">
         <v>4</v>
@@ -11764,23 +11764,23 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>8.4</v>
+        <v>7.9</v>
       </c>
       <c r="E227" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F227" t="n">
         <v>9.4</v>
       </c>
       <c r="G227" t="n">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="H227" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="I227" t="n">
         <v>0</v>
@@ -11789,7 +11789,7 @@
         <v>0</v>
       </c>
       <c r="K227" t="n">
-        <v>0.315</v>
+        <v>0.311</v>
       </c>
       <c r="L227" t="n">
         <v>4</v>
@@ -11814,20 +11814,20 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="E228" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F228" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="G228" t="n">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="H228" t="n">
         <v>100</v>
@@ -11839,7 +11839,7 @@
         <v>0</v>
       </c>
       <c r="K228" t="n">
-        <v>0.314</v>
+        <v>0.31</v>
       </c>
       <c r="L228" t="n">
         <v>4</v>
@@ -11864,20 +11864,20 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>12.9</v>
+        <v>13.5</v>
       </c>
       <c r="E229" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F229" t="n">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G229" t="n">
-        <v>290</v>
+        <v>387</v>
       </c>
       <c r="H229" t="n">
         <v>100</v>
@@ -11889,7 +11889,7 @@
         <v>0</v>
       </c>
       <c r="K229" t="n">
-        <v>0.313</v>
+        <v>0.309</v>
       </c>
       <c r="L229" t="n">
         <v>4</v>
@@ -11914,20 +11914,20 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>14.9</v>
+        <v>15.9</v>
       </c>
       <c r="E230" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F230" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G230" t="n">
-        <v>350</v>
+        <v>422</v>
       </c>
       <c r="H230" t="n">
         <v>100</v>
@@ -11939,7 +11939,7 @@
         <v>0</v>
       </c>
       <c r="K230" t="n">
-        <v>0.311</v>
+        <v>0.307</v>
       </c>
       <c r="L230" t="n">
         <v>4</v>
@@ -11964,23 +11964,23 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>17</v>
+        <v>17.8</v>
       </c>
       <c r="E231" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F231" t="n">
-        <v>10.1</v>
+        <v>13.3</v>
       </c>
       <c r="G231" t="n">
-        <v>399</v>
+        <v>438</v>
       </c>
       <c r="H231" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
@@ -11989,7 +11989,7 @@
         <v>0</v>
       </c>
       <c r="K231" t="n">
-        <v>0.309</v>
+        <v>0.305</v>
       </c>
       <c r="L231" t="n">
         <v>4</v>
@@ -12014,20 +12014,20 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>18.1</v>
+        <v>18.6</v>
       </c>
       <c r="E232" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F232" t="n">
-        <v>10.8</v>
+        <v>13.7</v>
       </c>
       <c r="G232" t="n">
-        <v>401</v>
+        <v>418</v>
       </c>
       <c r="H232" t="n">
         <v>85</v>
@@ -12039,7 +12039,7 @@
         <v>0</v>
       </c>
       <c r="K232" t="n">
-        <v>0.307</v>
+        <v>0.302</v>
       </c>
       <c r="L232" t="n">
         <v>4</v>
@@ -12064,23 +12064,23 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>18.7</v>
+        <v>19.1</v>
       </c>
       <c r="E233" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F233" t="n">
-        <v>11.5</v>
+        <v>14.4</v>
       </c>
       <c r="G233" t="n">
-        <v>347</v>
+        <v>358</v>
       </c>
       <c r="H233" t="n">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="I233" t="n">
         <v>0</v>
@@ -12089,7 +12089,7 @@
         <v>0</v>
       </c>
       <c r="K233" t="n">
-        <v>0.305</v>
+        <v>0.3</v>
       </c>
       <c r="L233" t="n">
         <v>4</v>
@@ -12114,23 +12114,23 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D234" t="n">
         <v>18.9</v>
       </c>
       <c r="E234" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F234" t="n">
-        <v>14</v>
+        <v>16.2</v>
       </c>
       <c r="G234" t="n">
-        <v>304</v>
+        <v>268</v>
       </c>
       <c r="H234" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="I234" t="n">
         <v>0</v>
@@ -12139,7 +12139,7 @@
         <v>0</v>
       </c>
       <c r="K234" t="n">
-        <v>0.303</v>
+        <v>0.298</v>
       </c>
       <c r="L234" t="n">
         <v>4</v>
@@ -12164,23 +12164,23 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>18.1</v>
+        <v>18.4</v>
       </c>
       <c r="E235" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F235" t="n">
-        <v>14.4</v>
+        <v>14.8</v>
       </c>
       <c r="G235" t="n">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H235" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
@@ -12189,7 +12189,7 @@
         <v>0</v>
       </c>
       <c r="K235" t="n">
-        <v>0.302</v>
+        <v>0.297</v>
       </c>
       <c r="L235" t="n">
         <v>4</v>
@@ -12214,23 +12214,23 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>16.2</v>
+        <v>16.5</v>
       </c>
       <c r="E236" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F236" t="n">
-        <v>10.4</v>
+        <v>11.2</v>
       </c>
       <c r="G236" t="n">
         <v>40</v>
       </c>
       <c r="H236" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -12239,7 +12239,7 @@
         <v>0</v>
       </c>
       <c r="K236" t="n">
-        <v>0.302</v>
+        <v>0.296</v>
       </c>
       <c r="L236" t="n">
         <v>4</v>
@@ -12264,23 +12264,23 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>14.3</v>
+        <v>14.6</v>
       </c>
       <c r="E237" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F237" t="n">
-        <v>7.9</v>
+        <v>11.2</v>
       </c>
       <c r="G237" t="n">
         <v>0</v>
       </c>
       <c r="H237" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
@@ -12289,7 +12289,7 @@
         <v>0</v>
       </c>
       <c r="K237" t="n">
-        <v>0.301</v>
+        <v>0.296</v>
       </c>
       <c r="L237" t="n">
         <v>4</v>
@@ -12314,23 +12314,23 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>13.1</v>
+        <v>13.6</v>
       </c>
       <c r="E238" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>10.8</v>
+        <v>11.2</v>
       </c>
       <c r="G238" t="n">
         <v>0</v>
       </c>
       <c r="H238" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="I238" t="n">
         <v>0</v>
@@ -12339,7 +12339,7 @@
         <v>0</v>
       </c>
       <c r="K238" t="n">
-        <v>0.301</v>
+        <v>0.296</v>
       </c>
       <c r="L238" t="n">
         <v>4</v>
@@ -12364,17 +12364,17 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="E239" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F239" t="n">
-        <v>13</v>
+        <v>10.8</v>
       </c>
       <c r="G239" t="n">
         <v>0</v>
@@ -12389,7 +12389,7 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>0.301</v>
+        <v>0.296</v>
       </c>
       <c r="L239" t="n">
         <v>4</v>
@@ -12414,14 +12414,14 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D240" t="n">
         <v>10.3</v>
       </c>
       <c r="E240" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F240" t="n">
         <v>10.4</v>
@@ -12439,7 +12439,7 @@
         <v>0</v>
       </c>
       <c r="K240" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L240" t="n">
         <v>4</v>
@@ -12464,17 +12464,17 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E241" t="n">
         <v>62</v>
       </c>
       <c r="F241" t="n">
-        <v>9</v>
+        <v>7.9</v>
       </c>
       <c r="G241" t="n">
         <v>0</v>
@@ -12489,7 +12489,7 @@
         <v>0</v>
       </c>
       <c r="K241" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L241" t="n">
         <v>4</v>
@@ -12514,17 +12514,17 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="E242" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F242" t="n">
-        <v>6.8</v>
+        <v>4.3</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -12539,7 +12539,7 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L242" t="n">
         <v>5</v>
@@ -12564,17 +12564,17 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D243" t="n">
         <v>6.5</v>
       </c>
       <c r="E243" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F243" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="G243" t="n">
         <v>0</v>
@@ -12589,7 +12589,7 @@
         <v>0</v>
       </c>
       <c r="K243" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L243" t="n">
         <v>5</v>
@@ -12614,17 +12614,17 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="E244" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F244" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="G244" t="n">
         <v>0</v>
@@ -12639,7 +12639,7 @@
         <v>0</v>
       </c>
       <c r="K244" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L244" t="n">
         <v>5</v>
@@ -12664,17 +12664,17 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="E245" t="n">
         <v>82</v>
       </c>
       <c r="F245" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -12689,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L245" t="n">
         <v>5</v>
@@ -12714,17 +12714,17 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="E246" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F246" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="G246" t="n">
         <v>0</v>
@@ -12739,7 +12739,7 @@
         <v>0</v>
       </c>
       <c r="K246" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L246" t="n">
         <v>5</v>
@@ -12764,17 +12764,17 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="E247" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F247" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="G247" t="n">
         <v>0</v>
@@ -12789,7 +12789,7 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L247" t="n">
         <v>5</v>
@@ -12814,7 +12814,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -12824,7 +12824,7 @@
         <v>89</v>
       </c>
       <c r="F248" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="G248" t="n">
         <v>0</v>
@@ -12839,7 +12839,7 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L248" t="n">
         <v>5</v>
@@ -12864,17 +12864,17 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="E249" t="n">
         <v>91</v>
       </c>
       <c r="F249" t="n">
-        <v>4.7</v>
+        <v>5.4</v>
       </c>
       <c r="G249" t="n">
         <v>0</v>
@@ -12889,7 +12889,7 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L249" t="n">
         <v>5</v>
@@ -12914,7 +12914,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -12924,10 +12924,10 @@
         <v>90</v>
       </c>
       <c r="F250" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="G250" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H250" t="n">
         <v>0</v>
@@ -12939,7 +12939,7 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>0.3</v>
+        <v>0.295</v>
       </c>
       <c r="L250" t="n">
         <v>5</v>
@@ -12964,20 +12964,20 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
       <c r="E251" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F251" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="G251" t="n">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H251" t="n">
         <v>0</v>
@@ -12989,7 +12989,7 @@
         <v>0</v>
       </c>
       <c r="K251" t="n">
-        <v>0.299</v>
+        <v>0.294</v>
       </c>
       <c r="L251" t="n">
         <v>5</v>
@@ -13014,23 +13014,23 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>11.2</v>
+        <v>11.9</v>
       </c>
       <c r="E252" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F252" t="n">
-        <v>4.3</v>
+        <v>6.8</v>
       </c>
       <c r="G252" t="n">
         <v>352</v>
       </c>
       <c r="H252" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I252" t="n">
         <v>0</v>
@@ -13039,7 +13039,7 @@
         <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>0.299</v>
+        <v>0.294</v>
       </c>
       <c r="L252" t="n">
         <v>5</v>
@@ -13064,23 +13064,23 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>14.2</v>
+        <v>13.9</v>
       </c>
       <c r="E253" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F253" t="n">
-        <v>9.4</v>
+        <v>11.5</v>
       </c>
       <c r="G253" t="n">
-        <v>475</v>
+        <v>312</v>
       </c>
       <c r="H253" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I253" t="n">
         <v>0</v>
@@ -13089,7 +13089,7 @@
         <v>0</v>
       </c>
       <c r="K253" t="n">
-        <v>0.297</v>
+        <v>0.292</v>
       </c>
       <c r="L253" t="n">
         <v>5</v>
@@ -13114,23 +13114,23 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>15.4</v>
+        <v>15.5</v>
       </c>
       <c r="E254" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F254" t="n">
-        <v>12.6</v>
+        <v>15.1</v>
       </c>
       <c r="G254" t="n">
-        <v>503</v>
+        <v>541</v>
       </c>
       <c r="H254" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="I254" t="n">
         <v>0</v>
@@ -13139,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="K254" t="n">
-        <v>0.296</v>
+        <v>0.291</v>
       </c>
       <c r="L254" t="n">
         <v>5</v>
@@ -13164,7 +13164,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -13174,13 +13174,13 @@
         <v>41</v>
       </c>
       <c r="F255" t="n">
-        <v>16.6</v>
+        <v>16.2</v>
       </c>
       <c r="G255" t="n">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="H255" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13189,7 +13189,7 @@
         <v>0</v>
       </c>
       <c r="K255" t="n">
-        <v>0.294</v>
+        <v>0.289</v>
       </c>
       <c r="L255" t="n">
         <v>5</v>
@@ -13214,23 +13214,23 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D256" t="n">
         <v>16.5</v>
       </c>
       <c r="E256" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F256" t="n">
-        <v>15.8</v>
+        <v>17.6</v>
       </c>
       <c r="G256" t="n">
-        <v>493</v>
+        <v>475</v>
       </c>
       <c r="H256" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I256" t="n">
         <v>0</v>
@@ -13239,7 +13239,7 @@
         <v>0</v>
       </c>
       <c r="K256" t="n">
-        <v>0.292</v>
+        <v>0.287</v>
       </c>
       <c r="L256" t="n">
         <v>5</v>
@@ -13264,7 +13264,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -13274,13 +13274,13 @@
         <v>39</v>
       </c>
       <c r="F257" t="n">
-        <v>16.2</v>
+        <v>18.4</v>
       </c>
       <c r="G257" t="n">
-        <v>373</v>
+        <v>386</v>
       </c>
       <c r="H257" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -13289,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="K257" t="n">
-        <v>0.29</v>
+        <v>0.285</v>
       </c>
       <c r="L257" t="n">
         <v>5</v>
@@ -13314,23 +13314,23 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>16.3</v>
+        <v>16.4</v>
       </c>
       <c r="E258" t="n">
         <v>38</v>
       </c>
       <c r="F258" t="n">
-        <v>17.3</v>
+        <v>16.9</v>
       </c>
       <c r="G258" t="n">
-        <v>263</v>
+        <v>287</v>
       </c>
       <c r="H258" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -13339,7 +13339,7 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
-        <v>0.288</v>
+        <v>0.284</v>
       </c>
       <c r="L258" t="n">
         <v>5</v>
@@ -13364,20 +13364,20 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>15.8</v>
+        <v>15.9</v>
       </c>
       <c r="E259" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F259" t="n">
-        <v>16.9</v>
+        <v>14</v>
       </c>
       <c r="G259" t="n">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="H259" t="n">
         <v>0</v>
@@ -13389,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>0.287</v>
+        <v>0.283</v>
       </c>
       <c r="L259" t="n">
         <v>5</v>
@@ -13414,17 +13414,17 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D260" t="n">
         <v>14</v>
       </c>
       <c r="E260" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F260" t="n">
-        <v>9</v>
+        <v>6.8</v>
       </c>
       <c r="G260" t="n">
         <v>38</v>
@@ -13439,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>0.287</v>
+        <v>0.282</v>
       </c>
       <c r="L260" t="n">
         <v>5</v>
@@ -13464,17 +13464,17 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D261" t="n">
         <v>11.5</v>
       </c>
       <c r="E261" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F261" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -13489,7 +13489,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>0.287</v>
+        <v>0.282</v>
       </c>
       <c r="L261" t="n">
         <v>5</v>
@@ -13514,23 +13514,23 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E262" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F262" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
       </c>
       <c r="H262" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I262" t="n">
         <v>0</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.286</v>
+        <v>0.282</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,23 +13564,23 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8.4</v>
+        <v>8.6</v>
       </c>
       <c r="E263" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F263" t="n">
-        <v>6.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
       </c>
       <c r="H263" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.286</v>
+        <v>0.282</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,23 +13614,23 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>7.3</v>
+        <v>7.7</v>
       </c>
       <c r="E264" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F264" t="n">
-        <v>7.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
       </c>
       <c r="H264" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.286</v>
+        <v>0.282</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,17 +13664,17 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6.5</v>
+        <v>6.9</v>
       </c>
       <c r="E265" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F265" t="n">
-        <v>6.5</v>
+        <v>9.4</v>
       </c>
       <c r="G265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.286</v>
+        <v>0.282</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13714,17 +13714,17 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
       <c r="E266" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F266" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -13739,7 +13739,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>0.286</v>
+        <v>0.282</v>
       </c>
       <c r="L266" t="n">
         <v>6</v>
@@ -13764,23 +13764,23 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-14T23:03:38Z</t>
+          <t>2026-10-15T05:03:41Z</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="E267" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F267" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G267" t="n">
         <v>0</v>
       </c>
       <c r="H267" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -13789,7 +13789,7 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>0.287</v>
+        <v>0.282</v>
       </c>
       <c r="L267" t="n">
         <v>6</v>
@@ -13798,6 +13798,1206 @@
         <v>1</v>
       </c>
       <c r="N267" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E268" t="n">
+        <v>70</v>
+      </c>
+      <c r="F268" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G268" t="n">
+        <v>0</v>
+      </c>
+      <c r="H268" t="n">
+        <v>100</v>
+      </c>
+      <c r="I268" t="n">
+        <v>0</v>
+      </c>
+      <c r="J268" t="n">
+        <v>0</v>
+      </c>
+      <c r="K268" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L268" t="n">
+        <v>6</v>
+      </c>
+      <c r="M268" t="n">
+        <v>1</v>
+      </c>
+      <c r="N268" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="E269" t="n">
+        <v>65</v>
+      </c>
+      <c r="F269" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G269" t="n">
+        <v>0</v>
+      </c>
+      <c r="H269" t="n">
+        <v>100</v>
+      </c>
+      <c r="I269" t="n">
+        <v>0</v>
+      </c>
+      <c r="J269" t="n">
+        <v>0</v>
+      </c>
+      <c r="K269" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L269" t="n">
+        <v>6</v>
+      </c>
+      <c r="M269" t="n">
+        <v>1</v>
+      </c>
+      <c r="N269" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E270" t="n">
+        <v>62</v>
+      </c>
+      <c r="F270" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G270" t="n">
+        <v>0</v>
+      </c>
+      <c r="H270" t="n">
+        <v>100</v>
+      </c>
+      <c r="I270" t="n">
+        <v>0</v>
+      </c>
+      <c r="J270" t="n">
+        <v>0</v>
+      </c>
+      <c r="K270" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L270" t="n">
+        <v>6</v>
+      </c>
+      <c r="M270" t="n">
+        <v>1</v>
+      </c>
+      <c r="N270" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E271" t="n">
+        <v>62</v>
+      </c>
+      <c r="F271" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G271" t="n">
+        <v>0</v>
+      </c>
+      <c r="H271" t="n">
+        <v>100</v>
+      </c>
+      <c r="I271" t="n">
+        <v>0</v>
+      </c>
+      <c r="J271" t="n">
+        <v>0</v>
+      </c>
+      <c r="K271" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L271" t="n">
+        <v>6</v>
+      </c>
+      <c r="M271" t="n">
+        <v>1</v>
+      </c>
+      <c r="N271" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E272" t="n">
+        <v>60</v>
+      </c>
+      <c r="F272" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" t="n">
+        <v>100</v>
+      </c>
+      <c r="I272" t="n">
+        <v>0</v>
+      </c>
+      <c r="J272" t="n">
+        <v>0</v>
+      </c>
+      <c r="K272" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L272" t="n">
+        <v>6</v>
+      </c>
+      <c r="M272" t="n">
+        <v>1</v>
+      </c>
+      <c r="N272" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="E273" t="n">
+        <v>59</v>
+      </c>
+      <c r="F273" t="n">
+        <v>5</v>
+      </c>
+      <c r="G273" t="n">
+        <v>0</v>
+      </c>
+      <c r="H273" t="n">
+        <v>100</v>
+      </c>
+      <c r="I273" t="n">
+        <v>0</v>
+      </c>
+      <c r="J273" t="n">
+        <v>0</v>
+      </c>
+      <c r="K273" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L273" t="n">
+        <v>6</v>
+      </c>
+      <c r="M273" t="n">
+        <v>1</v>
+      </c>
+      <c r="N273" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="E274" t="n">
+        <v>59</v>
+      </c>
+      <c r="F274" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G274" t="n">
+        <v>7</v>
+      </c>
+      <c r="H274" t="n">
+        <v>100</v>
+      </c>
+      <c r="I274" t="n">
+        <v>0</v>
+      </c>
+      <c r="J274" t="n">
+        <v>0</v>
+      </c>
+      <c r="K274" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L274" t="n">
+        <v>6</v>
+      </c>
+      <c r="M274" t="n">
+        <v>1</v>
+      </c>
+      <c r="N274" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E275" t="n">
+        <v>57</v>
+      </c>
+      <c r="F275" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G275" t="n">
+        <v>51</v>
+      </c>
+      <c r="H275" t="n">
+        <v>100</v>
+      </c>
+      <c r="I275" t="n">
+        <v>0</v>
+      </c>
+      <c r="J275" t="n">
+        <v>0</v>
+      </c>
+      <c r="K275" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L275" t="n">
+        <v>6</v>
+      </c>
+      <c r="M275" t="n">
+        <v>1</v>
+      </c>
+      <c r="N275" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>11</v>
+      </c>
+      <c r="E276" t="n">
+        <v>52</v>
+      </c>
+      <c r="F276" t="n">
+        <v>9</v>
+      </c>
+      <c r="G276" t="n">
+        <v>94</v>
+      </c>
+      <c r="H276" t="n">
+        <v>100</v>
+      </c>
+      <c r="I276" t="n">
+        <v>0</v>
+      </c>
+      <c r="J276" t="n">
+        <v>0</v>
+      </c>
+      <c r="K276" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="L276" t="n">
+        <v>6</v>
+      </c>
+      <c r="M276" t="n">
+        <v>1</v>
+      </c>
+      <c r="N276" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="E277" t="n">
+        <v>53</v>
+      </c>
+      <c r="F277" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G277" t="n">
+        <v>157.3</v>
+      </c>
+      <c r="H277" t="n">
+        <v>97</v>
+      </c>
+      <c r="I277" t="n">
+        <v>0</v>
+      </c>
+      <c r="J277" t="n">
+        <v>0</v>
+      </c>
+      <c r="K277" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="L277" t="n">
+        <v>6</v>
+      </c>
+      <c r="M277" t="n">
+        <v>1</v>
+      </c>
+      <c r="N277" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="E278" t="n">
+        <v>52</v>
+      </c>
+      <c r="F278" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G278" t="n">
+        <v>305</v>
+      </c>
+      <c r="H278" t="n">
+        <v>81</v>
+      </c>
+      <c r="I278" t="n">
+        <v>0</v>
+      </c>
+      <c r="J278" t="n">
+        <v>0</v>
+      </c>
+      <c r="K278" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="L278" t="n">
+        <v>6</v>
+      </c>
+      <c r="M278" t="n">
+        <v>1</v>
+      </c>
+      <c r="N278" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E279" t="n">
+        <v>53</v>
+      </c>
+      <c r="F279" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G279" t="n">
+        <v>361.8</v>
+      </c>
+      <c r="H279" t="n">
+        <v>84</v>
+      </c>
+      <c r="I279" t="n">
+        <v>0</v>
+      </c>
+      <c r="J279" t="n">
+        <v>0</v>
+      </c>
+      <c r="K279" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="L279" t="n">
+        <v>6</v>
+      </c>
+      <c r="M279" t="n">
+        <v>1</v>
+      </c>
+      <c r="N279" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="E280" t="n">
+        <v>56</v>
+      </c>
+      <c r="F280" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G280" t="n">
+        <v>274</v>
+      </c>
+      <c r="H280" t="n">
+        <v>100</v>
+      </c>
+      <c r="I280" t="n">
+        <v>0</v>
+      </c>
+      <c r="J280" t="n">
+        <v>0</v>
+      </c>
+      <c r="K280" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="L280" t="n">
+        <v>6</v>
+      </c>
+      <c r="M280" t="n">
+        <v>1</v>
+      </c>
+      <c r="N280" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="E281" t="n">
+        <v>55</v>
+      </c>
+      <c r="F281" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G281" t="n">
+        <v>189</v>
+      </c>
+      <c r="H281" t="n">
+        <v>98</v>
+      </c>
+      <c r="I281" t="n">
+        <v>0</v>
+      </c>
+      <c r="J281" t="n">
+        <v>0</v>
+      </c>
+      <c r="K281" t="n">
+        <v>0.276</v>
+      </c>
+      <c r="L281" t="n">
+        <v>6</v>
+      </c>
+      <c r="M281" t="n">
+        <v>1</v>
+      </c>
+      <c r="N281" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="E282" t="n">
+        <v>54</v>
+      </c>
+      <c r="F282" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G282" t="n">
+        <v>165</v>
+      </c>
+      <c r="H282" t="n">
+        <v>52</v>
+      </c>
+      <c r="I282" t="n">
+        <v>0</v>
+      </c>
+      <c r="J282" t="n">
+        <v>0</v>
+      </c>
+      <c r="K282" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="L282" t="n">
+        <v>6</v>
+      </c>
+      <c r="M282" t="n">
+        <v>1</v>
+      </c>
+      <c r="N282" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>14</v>
+      </c>
+      <c r="E283" t="n">
+        <v>60</v>
+      </c>
+      <c r="F283" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G283" t="n">
+        <v>101</v>
+      </c>
+      <c r="H283" t="n">
+        <v>76</v>
+      </c>
+      <c r="I283" t="n">
+        <v>0</v>
+      </c>
+      <c r="J283" t="n">
+        <v>0</v>
+      </c>
+      <c r="K283" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="L283" t="n">
+        <v>6</v>
+      </c>
+      <c r="M283" t="n">
+        <v>1</v>
+      </c>
+      <c r="N283" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="E284" t="n">
+        <v>66</v>
+      </c>
+      <c r="F284" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G284" t="n">
+        <v>19</v>
+      </c>
+      <c r="H284" t="n">
+        <v>80</v>
+      </c>
+      <c r="I284" t="n">
+        <v>0</v>
+      </c>
+      <c r="J284" t="n">
+        <v>0</v>
+      </c>
+      <c r="K284" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="L284" t="n">
+        <v>6</v>
+      </c>
+      <c r="M284" t="n">
+        <v>1</v>
+      </c>
+      <c r="N284" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="E285" t="n">
+        <v>67</v>
+      </c>
+      <c r="F285" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G285" t="n">
+        <v>0</v>
+      </c>
+      <c r="H285" t="n">
+        <v>64</v>
+      </c>
+      <c r="I285" t="n">
+        <v>0</v>
+      </c>
+      <c r="J285" t="n">
+        <v>0</v>
+      </c>
+      <c r="K285" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="L285" t="n">
+        <v>6</v>
+      </c>
+      <c r="M285" t="n">
+        <v>1</v>
+      </c>
+      <c r="N285" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="E286" t="n">
+        <v>67</v>
+      </c>
+      <c r="F286" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G286" t="n">
+        <v>0</v>
+      </c>
+      <c r="H286" t="n">
+        <v>98</v>
+      </c>
+      <c r="I286" t="n">
+        <v>0</v>
+      </c>
+      <c r="J286" t="n">
+        <v>0</v>
+      </c>
+      <c r="K286" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="L286" t="n">
+        <v>6</v>
+      </c>
+      <c r="M286" t="n">
+        <v>1</v>
+      </c>
+      <c r="N286" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E287" t="n">
+        <v>70</v>
+      </c>
+      <c r="F287" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="G287" t="n">
+        <v>0</v>
+      </c>
+      <c r="H287" t="n">
+        <v>73</v>
+      </c>
+      <c r="I287" t="n">
+        <v>0</v>
+      </c>
+      <c r="J287" t="n">
+        <v>0</v>
+      </c>
+      <c r="K287" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="L287" t="n">
+        <v>6</v>
+      </c>
+      <c r="M287" t="n">
+        <v>1</v>
+      </c>
+      <c r="N287" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="E288" t="n">
+        <v>73</v>
+      </c>
+      <c r="F288" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G288" t="n">
+        <v>0</v>
+      </c>
+      <c r="H288" t="n">
+        <v>46</v>
+      </c>
+      <c r="I288" t="n">
+        <v>0</v>
+      </c>
+      <c r="J288" t="n">
+        <v>0</v>
+      </c>
+      <c r="K288" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="L288" t="n">
+        <v>6</v>
+      </c>
+      <c r="M288" t="n">
+        <v>1</v>
+      </c>
+      <c r="N288" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="E289" t="n">
+        <v>73</v>
+      </c>
+      <c r="F289" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G289" t="n">
+        <v>0</v>
+      </c>
+      <c r="H289" t="n">
+        <v>73</v>
+      </c>
+      <c r="I289" t="n">
+        <v>0</v>
+      </c>
+      <c r="J289" t="n">
+        <v>0</v>
+      </c>
+      <c r="K289" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="L289" t="n">
+        <v>6</v>
+      </c>
+      <c r="M289" t="n">
+        <v>1</v>
+      </c>
+      <c r="N289" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="E290" t="n">
+        <v>74</v>
+      </c>
+      <c r="F290" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="G290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H290" t="n">
+        <v>100</v>
+      </c>
+      <c r="I290" t="n">
+        <v>0</v>
+      </c>
+      <c r="J290" t="n">
+        <v>0</v>
+      </c>
+      <c r="K290" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="L290" t="n">
+        <v>7</v>
+      </c>
+      <c r="M290" t="n">
+        <v>1</v>
+      </c>
+      <c r="N290" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>2026-10-15T05:03:41Z</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="E291" t="n">
+        <v>73</v>
+      </c>
+      <c r="F291" t="n">
+        <v>7</v>
+      </c>
+      <c r="G291" t="n">
+        <v>0</v>
+      </c>
+      <c r="H291" t="n">
+        <v>100</v>
+      </c>
+      <c r="I291" t="n">
+        <v>0</v>
+      </c>
+      <c r="J291" t="n">
+        <v>0</v>
+      </c>
+      <c r="K291" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="L291" t="n">
+        <v>7</v>
+      </c>
+      <c r="M291" t="n">
+        <v>1</v>
+      </c>
+      <c r="N291" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-15 13:04
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -11964,23 +11964,23 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>17.8</v>
+        <v>16.5</v>
       </c>
       <c r="E231" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F231" t="n">
-        <v>13.3</v>
+        <v>9</v>
       </c>
       <c r="G231" t="n">
-        <v>438</v>
+        <v>399</v>
       </c>
       <c r="H231" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
@@ -11989,7 +11989,7 @@
         <v>0</v>
       </c>
       <c r="K231" t="n">
-        <v>0.305</v>
+        <v>0.308</v>
       </c>
       <c r="L231" t="n">
         <v>4</v>
@@ -12014,23 +12014,23 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>18.6</v>
+        <v>17.6</v>
       </c>
       <c r="E232" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F232" t="n">
-        <v>13.7</v>
+        <v>10.4</v>
       </c>
       <c r="G232" t="n">
-        <v>418</v>
+        <v>395</v>
       </c>
       <c r="H232" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
@@ -12039,7 +12039,7 @@
         <v>0</v>
       </c>
       <c r="K232" t="n">
-        <v>0.302</v>
+        <v>0.305</v>
       </c>
       <c r="L232" t="n">
         <v>4</v>
@@ -12064,23 +12064,23 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>19.1</v>
+        <v>18.2</v>
       </c>
       <c r="E233" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F233" t="n">
-        <v>14.4</v>
+        <v>10.4</v>
       </c>
       <c r="G233" t="n">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="H233" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="I233" t="n">
         <v>0</v>
@@ -12089,7 +12089,7 @@
         <v>0</v>
       </c>
       <c r="K233" t="n">
-        <v>0.3</v>
+        <v>0.303</v>
       </c>
       <c r="L233" t="n">
         <v>4</v>
@@ -12114,23 +12114,23 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>18.9</v>
+        <v>18.4</v>
       </c>
       <c r="E234" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F234" t="n">
-        <v>16.2</v>
+        <v>10.4</v>
       </c>
       <c r="G234" t="n">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="H234" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="I234" t="n">
         <v>0</v>
@@ -12139,7 +12139,7 @@
         <v>0</v>
       </c>
       <c r="K234" t="n">
-        <v>0.298</v>
+        <v>0.301</v>
       </c>
       <c r="L234" t="n">
         <v>4</v>
@@ -12164,23 +12164,23 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>18.4</v>
+        <v>18.1</v>
       </c>
       <c r="E235" t="n">
         <v>33</v>
       </c>
       <c r="F235" t="n">
-        <v>14.8</v>
+        <v>13.3</v>
       </c>
       <c r="G235" t="n">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="H235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
@@ -12189,7 +12189,7 @@
         <v>0</v>
       </c>
       <c r="K235" t="n">
-        <v>0.297</v>
+        <v>0.3</v>
       </c>
       <c r="L235" t="n">
         <v>4</v>
@@ -12214,23 +12214,23 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>16.5</v>
+        <v>16.2</v>
       </c>
       <c r="E236" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F236" t="n">
-        <v>11.2</v>
+        <v>9.4</v>
       </c>
       <c r="G236" t="n">
         <v>40</v>
       </c>
       <c r="H236" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -12239,7 +12239,7 @@
         <v>0</v>
       </c>
       <c r="K236" t="n">
-        <v>0.296</v>
+        <v>0.3</v>
       </c>
       <c r="L236" t="n">
         <v>4</v>
@@ -12264,14 +12264,14 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>14.6</v>
+        <v>14.7</v>
       </c>
       <c r="E237" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F237" t="n">
         <v>11.2</v>
@@ -12280,7 +12280,7 @@
         <v>0</v>
       </c>
       <c r="H237" t="n">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
@@ -12289,7 +12289,7 @@
         <v>0</v>
       </c>
       <c r="K237" t="n">
-        <v>0.296</v>
+        <v>0.299</v>
       </c>
       <c r="L237" t="n">
         <v>4</v>
@@ -12314,23 +12314,23 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>13.6</v>
+        <v>13.4</v>
       </c>
       <c r="E238" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F238" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="G238" t="n">
         <v>0</v>
       </c>
       <c r="H238" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I238" t="n">
         <v>0</v>
@@ -12339,7 +12339,7 @@
         <v>0</v>
       </c>
       <c r="K238" t="n">
-        <v>0.296</v>
+        <v>0.299</v>
       </c>
       <c r="L238" t="n">
         <v>4</v>
@@ -12364,17 +12364,17 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="E239" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F239" t="n">
-        <v>10.8</v>
+        <v>11.9</v>
       </c>
       <c r="G239" t="n">
         <v>0</v>
@@ -12389,7 +12389,7 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>0.296</v>
+        <v>0.298</v>
       </c>
       <c r="L239" t="n">
         <v>4</v>
@@ -12414,17 +12414,17 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="E240" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F240" t="n">
-        <v>10.4</v>
+        <v>13.3</v>
       </c>
       <c r="G240" t="n">
         <v>0</v>
@@ -12439,7 +12439,7 @@
         <v>0</v>
       </c>
       <c r="K240" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L240" t="n">
         <v>4</v>
@@ -12464,17 +12464,17 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D241" t="n">
         <v>8.800000000000001</v>
       </c>
       <c r="E241" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F241" t="n">
-        <v>7.9</v>
+        <v>7.6</v>
       </c>
       <c r="G241" t="n">
         <v>0</v>
@@ -12489,7 +12489,7 @@
         <v>0</v>
       </c>
       <c r="K241" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L241" t="n">
         <v>4</v>
@@ -12514,17 +12514,17 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="E242" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F242" t="n">
-        <v>4.3</v>
+        <v>6.1</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -12539,7 +12539,7 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L242" t="n">
         <v>5</v>
@@ -12564,17 +12564,17 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="E243" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F243" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="G243" t="n">
         <v>0</v>
@@ -12589,7 +12589,7 @@
         <v>0</v>
       </c>
       <c r="K243" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L243" t="n">
         <v>5</v>
@@ -12614,17 +12614,17 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
       <c r="E244" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F244" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="G244" t="n">
         <v>0</v>
@@ -12639,7 +12639,7 @@
         <v>0</v>
       </c>
       <c r="K244" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L244" t="n">
         <v>5</v>
@@ -12664,17 +12664,17 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="E245" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F245" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -12689,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L245" t="n">
         <v>5</v>
@@ -12714,17 +12714,17 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="E246" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F246" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="G246" t="n">
         <v>0</v>
@@ -12739,7 +12739,7 @@
         <v>0</v>
       </c>
       <c r="K246" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L246" t="n">
         <v>5</v>
@@ -12764,14 +12764,14 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="E247" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F247" t="n">
         <v>4.7</v>
@@ -12789,7 +12789,7 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L247" t="n">
         <v>5</v>
@@ -12814,17 +12814,17 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="E248" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F248" t="n">
-        <v>5.8</v>
+        <v>7.2</v>
       </c>
       <c r="G248" t="n">
         <v>0</v>
@@ -12839,7 +12839,7 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L248" t="n">
         <v>5</v>
@@ -12864,17 +12864,17 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="E249" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F249" t="n">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="G249" t="n">
         <v>0</v>
@@ -12889,7 +12889,7 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L249" t="n">
         <v>5</v>
@@ -12914,23 +12914,23 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="E250" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F250" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="G250" t="n">
         <v>53</v>
       </c>
       <c r="H250" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="I250" t="n">
         <v>0</v>
@@ -12939,7 +12939,7 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>0.295</v>
+        <v>0.298</v>
       </c>
       <c r="L250" t="n">
         <v>5</v>
@@ -12964,20 +12964,20 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="E251" t="n">
         <v>76</v>
       </c>
       <c r="F251" t="n">
-        <v>3.2</v>
+        <v>5.8</v>
       </c>
       <c r="G251" t="n">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="H251" t="n">
         <v>0</v>
@@ -12989,7 +12989,7 @@
         <v>0</v>
       </c>
       <c r="K251" t="n">
-        <v>0.294</v>
+        <v>0.297</v>
       </c>
       <c r="L251" t="n">
         <v>5</v>
@@ -13014,23 +13014,23 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>11.9</v>
+        <v>11.6</v>
       </c>
       <c r="E252" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F252" t="n">
-        <v>6.8</v>
+        <v>7.9</v>
       </c>
       <c r="G252" t="n">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="H252" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I252" t="n">
         <v>0</v>
@@ -13039,7 +13039,7 @@
         <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>0.294</v>
+        <v>0.297</v>
       </c>
       <c r="L252" t="n">
         <v>5</v>
@@ -13064,23 +13064,23 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="E253" t="n">
         <v>53</v>
       </c>
       <c r="F253" t="n">
-        <v>11.5</v>
+        <v>12.2</v>
       </c>
       <c r="G253" t="n">
-        <v>312</v>
+        <v>459</v>
       </c>
       <c r="H253" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I253" t="n">
         <v>0</v>
@@ -13089,7 +13089,7 @@
         <v>0</v>
       </c>
       <c r="K253" t="n">
-        <v>0.292</v>
+        <v>0.295</v>
       </c>
       <c r="L253" t="n">
         <v>5</v>
@@ -13114,23 +13114,23 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>15.5</v>
+        <v>15.6</v>
       </c>
       <c r="E254" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F254" t="n">
-        <v>15.1</v>
+        <v>16.2</v>
       </c>
       <c r="G254" t="n">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="H254" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="I254" t="n">
         <v>0</v>
@@ -13139,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="K254" t="n">
-        <v>0.291</v>
+        <v>0.295</v>
       </c>
       <c r="L254" t="n">
         <v>5</v>
@@ -13164,23 +13164,23 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>16.2</v>
+        <v>16</v>
       </c>
       <c r="E255" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>16.2</v>
+        <v>16.9</v>
       </c>
       <c r="G255" t="n">
-        <v>542</v>
+        <v>513</v>
       </c>
       <c r="H255" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13189,7 +13189,7 @@
         <v>0</v>
       </c>
       <c r="K255" t="n">
-        <v>0.289</v>
+        <v>0.293</v>
       </c>
       <c r="L255" t="n">
         <v>5</v>
@@ -13214,23 +13214,23 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>16.5</v>
+        <v>16.2</v>
       </c>
       <c r="E256" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F256" t="n">
-        <v>17.6</v>
+        <v>16.2</v>
       </c>
       <c r="G256" t="n">
         <v>475</v>
       </c>
       <c r="H256" t="n">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="I256" t="n">
         <v>0</v>
@@ -13239,7 +13239,7 @@
         <v>0</v>
       </c>
       <c r="K256" t="n">
-        <v>0.287</v>
+        <v>0.291</v>
       </c>
       <c r="L256" t="n">
         <v>5</v>
@@ -13264,23 +13264,23 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>16.5</v>
+        <v>16.3</v>
       </c>
       <c r="E257" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F257" t="n">
-        <v>18.4</v>
+        <v>17.3</v>
       </c>
       <c r="G257" t="n">
-        <v>386</v>
+        <v>359</v>
       </c>
       <c r="H257" t="n">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -13289,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="K257" t="n">
-        <v>0.285</v>
+        <v>0.289</v>
       </c>
       <c r="L257" t="n">
         <v>5</v>
@@ -13314,23 +13314,23 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>16.4</v>
+        <v>16.2</v>
       </c>
       <c r="E258" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F258" t="n">
-        <v>16.9</v>
+        <v>15.8</v>
       </c>
       <c r="G258" t="n">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="H258" t="n">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -13339,7 +13339,7 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
-        <v>0.284</v>
+        <v>0.288</v>
       </c>
       <c r="L258" t="n">
         <v>5</v>
@@ -13364,20 +13364,20 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
       <c r="E259" t="n">
         <v>38</v>
       </c>
       <c r="F259" t="n">
-        <v>14</v>
+        <v>13.3</v>
       </c>
       <c r="G259" t="n">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="H259" t="n">
         <v>0</v>
@@ -13389,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>0.283</v>
+        <v>0.287</v>
       </c>
       <c r="L259" t="n">
         <v>5</v>
@@ -13414,20 +13414,20 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D260" t="n">
         <v>14</v>
       </c>
       <c r="E260" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F260" t="n">
-        <v>6.8</v>
+        <v>7.9</v>
       </c>
       <c r="G260" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H260" t="n">
         <v>0</v>
@@ -13439,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L260" t="n">
         <v>5</v>
@@ -13464,17 +13464,17 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D261" t="n">
         <v>11.5</v>
       </c>
       <c r="E261" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F261" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -13489,7 +13489,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L261" t="n">
         <v>5</v>
@@ -13514,7 +13514,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -13524,13 +13524,13 @@
         <v>57</v>
       </c>
       <c r="F262" t="n">
-        <v>8.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
       </c>
       <c r="H262" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="I262" t="n">
         <v>0</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,17 +13564,17 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E263" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F263" t="n">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,17 +13614,17 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D264" t="n">
         <v>7.7</v>
       </c>
       <c r="E264" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F264" t="n">
-        <v>9.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,17 +13664,17 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="E265" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F265" t="n">
-        <v>9.4</v>
+        <v>7.9</v>
       </c>
       <c r="G265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13714,17 +13714,17 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>6.4</v>
+        <v>5.9</v>
       </c>
       <c r="E266" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F266" t="n">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -13739,7 +13739,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L266" t="n">
         <v>6</v>
@@ -13764,23 +13764,23 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="E267" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F267" t="n">
-        <v>4</v>
+        <v>6.1</v>
       </c>
       <c r="G267" t="n">
         <v>0</v>
       </c>
       <c r="H267" t="n">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -13789,7 +13789,7 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L267" t="n">
         <v>6</v>
@@ -13814,23 +13814,23 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="E268" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F268" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
       </c>
       <c r="H268" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -13839,7 +13839,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L268" t="n">
         <v>6</v>
@@ -13864,23 +13864,23 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>7.7</v>
+        <v>7</v>
       </c>
       <c r="E269" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F269" t="n">
-        <v>7.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G269" t="n">
         <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I269" t="n">
         <v>0</v>
@@ -13889,7 +13889,7 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L269" t="n">
         <v>6</v>
@@ -13914,17 +13914,17 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="E270" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F270" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="G270" t="n">
         <v>0</v>
@@ -13939,7 +13939,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L270" t="n">
         <v>6</v>
@@ -13964,17 +13964,17 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>8.5</v>
+        <v>7.8</v>
       </c>
       <c r="E271" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F271" t="n">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
       <c r="G271" t="n">
         <v>0</v>
@@ -13989,7 +13989,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L271" t="n">
         <v>6</v>
@@ -14014,17 +14014,17 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>8.699999999999999</v>
+        <v>8</v>
       </c>
       <c r="E272" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F272" t="n">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
@@ -14039,7 +14039,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L272" t="n">
         <v>6</v>
@@ -14064,17 +14064,17 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>8.800000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E273" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="F273" t="n">
-        <v>5</v>
+        <v>6.1</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
@@ -14089,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>0.282</v>
+        <v>0.286</v>
       </c>
       <c r="L273" t="n">
         <v>6</v>
@@ -14114,20 +14114,20 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>9.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E274" t="n">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="F274" t="n">
-        <v>7.9</v>
+        <v>5</v>
       </c>
       <c r="G274" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H274" t="n">
         <v>100</v>
@@ -14139,7 +14139,7 @@
         <v>0</v>
       </c>
       <c r="K274" t="n">
-        <v>0.282</v>
+        <v>0.287</v>
       </c>
       <c r="L274" t="n">
         <v>6</v>
@@ -14164,20 +14164,20 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>9.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="E275" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F275" t="n">
-        <v>9.4</v>
+        <v>7.2</v>
       </c>
       <c r="G275" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="H275" t="n">
         <v>100</v>
@@ -14189,7 +14189,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>0.282</v>
+        <v>0.287</v>
       </c>
       <c r="L275" t="n">
         <v>6</v>
@@ -14214,20 +14214,20 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="E276" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F276" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="G276" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H276" t="n">
         <v>100</v>
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>0.281</v>
+        <v>0.288</v>
       </c>
       <c r="L276" t="n">
         <v>6</v>
@@ -14264,23 +14264,23 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>12.1</v>
+        <v>12.4</v>
       </c>
       <c r="E277" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F277" t="n">
-        <v>8.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G277" t="n">
-        <v>157.3</v>
+        <v>135</v>
       </c>
       <c r="H277" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="I277" t="n">
         <v>0</v>
@@ -14289,7 +14289,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>0.281</v>
+        <v>0.288</v>
       </c>
       <c r="L277" t="n">
         <v>6</v>
@@ -14314,23 +14314,23 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>13.7</v>
+        <v>13.1</v>
       </c>
       <c r="E278" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F278" t="n">
-        <v>7.5</v>
+        <v>12.6</v>
       </c>
       <c r="G278" t="n">
-        <v>305</v>
+        <v>103</v>
       </c>
       <c r="H278" t="n">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="I278" t="n">
         <v>0</v>
@@ -14339,7 +14339,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>0.28</v>
+        <v>0.287</v>
       </c>
       <c r="L278" t="n">
         <v>6</v>
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="E279" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="F279" t="n">
-        <v>7.3</v>
+        <v>12.6</v>
       </c>
       <c r="G279" t="n">
-        <v>361.8</v>
+        <v>162</v>
       </c>
       <c r="H279" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.279</v>
+        <v>0.286</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,23 +14414,23 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>14.3</v>
+        <v>14.9</v>
       </c>
       <c r="E280" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="F280" t="n">
-        <v>6.5</v>
+        <v>10.1</v>
       </c>
       <c r="G280" t="n">
-        <v>274</v>
+        <v>198</v>
       </c>
       <c r="H280" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="I280" t="n">
         <v>0</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.277</v>
+        <v>0.285</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,23 +14464,23 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>14.4</v>
+        <v>15.8</v>
       </c>
       <c r="E281" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="F281" t="n">
-        <v>7.6</v>
+        <v>9</v>
       </c>
       <c r="G281" t="n">
-        <v>189</v>
+        <v>309</v>
       </c>
       <c r="H281" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I281" t="n">
         <v>0</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.276</v>
+        <v>0.284</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,23 +14514,23 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>14.6</v>
+        <v>16.1</v>
       </c>
       <c r="E282" t="n">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="F282" t="n">
-        <v>7.6</v>
+        <v>7.9</v>
       </c>
       <c r="G282" t="n">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="H282" t="n">
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="I282" t="n">
         <v>0</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.275</v>
+        <v>0.283</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,23 +14564,23 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>14</v>
+        <v>15.2</v>
       </c>
       <c r="E283" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="F283" t="n">
         <v>5.6</v>
       </c>
       <c r="G283" t="n">
-        <v>101</v>
+        <v>55.3</v>
       </c>
       <c r="H283" t="n">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -14589,7 +14589,7 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0.275</v>
+        <v>0.282</v>
       </c>
       <c r="L283" t="n">
         <v>6</v>
@@ -14614,23 +14614,23 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>12.6</v>
+        <v>13.5</v>
       </c>
       <c r="E284" t="n">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F284" t="n">
-        <v>7.4</v>
+        <v>4.2</v>
       </c>
       <c r="G284" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H284" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I284" t="n">
         <v>0</v>
@@ -14639,7 +14639,7 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0.275</v>
+        <v>0.282</v>
       </c>
       <c r="L284" t="n">
         <v>6</v>
@@ -14664,23 +14664,23 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>12.3</v>
+        <v>11.4</v>
       </c>
       <c r="E285" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F285" t="n">
-        <v>9.199999999999999</v>
+        <v>5</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
       </c>
       <c r="H285" t="n">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -14689,7 +14689,7 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
-        <v>0.274</v>
+        <v>0.282</v>
       </c>
       <c r="L285" t="n">
         <v>6</v>
@@ -14714,23 +14714,23 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>11.9</v>
+        <v>10.4</v>
       </c>
       <c r="E286" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="F286" t="n">
-        <v>8.6</v>
+        <v>5.5</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14739,7 +14739,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0.274</v>
+        <v>0.281</v>
       </c>
       <c r="L286" t="n">
         <v>6</v>
@@ -14764,23 +14764,23 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>11.2</v>
+        <v>10.2</v>
       </c>
       <c r="E287" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="F287" t="n">
-        <v>7.7</v>
+        <v>5.6</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>73</v>
+        <v>16</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>0.274</v>
+        <v>0.281</v>
       </c>
       <c r="L287" t="n">
         <v>6</v>
@@ -14814,23 +14814,23 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>10.7</v>
+        <v>9.5</v>
       </c>
       <c r="E288" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="F288" t="n">
-        <v>6.9</v>
+        <v>5.3</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
       </c>
       <c r="H288" t="n">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.274</v>
+        <v>0.281</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,23 +14864,23 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>10.7</v>
+        <v>8.9</v>
       </c>
       <c r="E289" t="n">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="F289" t="n">
-        <v>6.4</v>
+        <v>4.6</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
       </c>
       <c r="H289" t="n">
-        <v>73</v>
+        <v>16</v>
       </c>
       <c r="I289" t="n">
         <v>0</v>
@@ -14889,7 +14889,7 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>0.274</v>
+        <v>0.281</v>
       </c>
       <c r="L289" t="n">
         <v>6</v>
@@ -14914,23 +14914,23 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>10.7</v>
+        <v>8.5</v>
       </c>
       <c r="E290" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F290" t="n">
-        <v>6.3</v>
+        <v>4.1</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
       </c>
       <c r="H290" t="n">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="I290" t="n">
         <v>0</v>
@@ -14939,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="K290" t="n">
-        <v>0.274</v>
+        <v>0.281</v>
       </c>
       <c r="L290" t="n">
         <v>7</v>
@@ -14964,23 +14964,23 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-15T05:03:41Z</t>
+          <t>2026-10-15T11:03:48Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>10.8</v>
+        <v>8</v>
       </c>
       <c r="E291" t="n">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="F291" t="n">
-        <v>7</v>
+        <v>4.9</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
       </c>
       <c r="H291" t="n">
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="I291" t="n">
         <v>0</v>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>0.274</v>
+        <v>0.281</v>
       </c>
       <c r="L291" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-15 19:04
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -12264,23 +12264,23 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>14.7</v>
+        <v>14.1</v>
       </c>
       <c r="E237" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F237" t="n">
-        <v>11.2</v>
+        <v>5.8</v>
       </c>
       <c r="G237" t="n">
         <v>0</v>
       </c>
       <c r="H237" t="n">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
@@ -12289,7 +12289,7 @@
         <v>0</v>
       </c>
       <c r="K237" t="n">
-        <v>0.299</v>
+        <v>0.301</v>
       </c>
       <c r="L237" t="n">
         <v>4</v>
@@ -12314,23 +12314,23 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>13.4</v>
+        <v>12.7</v>
       </c>
       <c r="E238" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="F238" t="n">
-        <v>11.5</v>
+        <v>6.5</v>
       </c>
       <c r="G238" t="n">
         <v>0</v>
       </c>
       <c r="H238" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I238" t="n">
         <v>0</v>
@@ -12339,7 +12339,7 @@
         <v>0</v>
       </c>
       <c r="K238" t="n">
-        <v>0.299</v>
+        <v>0.301</v>
       </c>
       <c r="L238" t="n">
         <v>4</v>
@@ -12364,17 +12364,17 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>11.8</v>
+        <v>10.9</v>
       </c>
       <c r="E239" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F239" t="n">
-        <v>11.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G239" t="n">
         <v>0</v>
@@ -12389,7 +12389,7 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L239" t="n">
         <v>4</v>
@@ -12414,17 +12414,17 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="E240" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F240" t="n">
-        <v>13.3</v>
+        <v>9.4</v>
       </c>
       <c r="G240" t="n">
         <v>0</v>
@@ -12439,7 +12439,7 @@
         <v>0</v>
       </c>
       <c r="K240" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L240" t="n">
         <v>4</v>
@@ -12464,17 +12464,17 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>8.800000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="E241" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F241" t="n">
-        <v>7.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G241" t="n">
         <v>0</v>
@@ -12489,7 +12489,7 @@
         <v>0</v>
       </c>
       <c r="K241" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L241" t="n">
         <v>4</v>
@@ -12514,17 +12514,17 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>7.4</v>
+        <v>6.8</v>
       </c>
       <c r="E242" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F242" t="n">
-        <v>6.1</v>
+        <v>9</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -12539,7 +12539,7 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L242" t="n">
         <v>5</v>
@@ -12564,17 +12564,17 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="E243" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="F243" t="n">
-        <v>4.3</v>
+        <v>6.8</v>
       </c>
       <c r="G243" t="n">
         <v>0</v>
@@ -12589,7 +12589,7 @@
         <v>0</v>
       </c>
       <c r="K243" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L243" t="n">
         <v>5</v>
@@ -12614,17 +12614,17 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>5.5</v>
+        <v>5.1</v>
       </c>
       <c r="E244" t="n">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="F244" t="n">
-        <v>4.7</v>
+        <v>4.3</v>
       </c>
       <c r="G244" t="n">
         <v>0</v>
@@ -12639,7 +12639,7 @@
         <v>0</v>
       </c>
       <c r="K244" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L244" t="n">
         <v>5</v>
@@ -12664,17 +12664,17 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="E245" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F245" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -12689,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L245" t="n">
         <v>5</v>
@@ -12714,17 +12714,17 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="E246" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F246" t="n">
-        <v>4.7</v>
+        <v>3.2</v>
       </c>
       <c r="G246" t="n">
         <v>0</v>
@@ -12739,7 +12739,7 @@
         <v>0</v>
       </c>
       <c r="K246" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L246" t="n">
         <v>5</v>
@@ -12764,17 +12764,17 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="E247" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F247" t="n">
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="G247" t="n">
         <v>0</v>
@@ -12789,7 +12789,7 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L247" t="n">
         <v>5</v>
@@ -12814,17 +12814,17 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>3.7</v>
+        <v>3.4</v>
       </c>
       <c r="E248" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F248" t="n">
-        <v>7.2</v>
+        <v>4.3</v>
       </c>
       <c r="G248" t="n">
         <v>0</v>
@@ -12839,7 +12839,7 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L248" t="n">
         <v>5</v>
@@ -12864,14 +12864,14 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="E249" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F249" t="n">
         <v>6.1</v>
@@ -12889,7 +12889,7 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L249" t="n">
         <v>5</v>
@@ -12914,23 +12914,23 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="E250" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F250" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G250" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H250" t="n">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="I250" t="n">
         <v>0</v>
@@ -12939,7 +12939,7 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>0.298</v>
+        <v>0.3</v>
       </c>
       <c r="L250" t="n">
         <v>5</v>
@@ -12964,20 +12964,20 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>7.3</v>
+        <v>6.9</v>
       </c>
       <c r="E251" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F251" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="G251" t="n">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="H251" t="n">
         <v>0</v>
@@ -12989,7 +12989,7 @@
         <v>0</v>
       </c>
       <c r="K251" t="n">
-        <v>0.297</v>
+        <v>0.299</v>
       </c>
       <c r="L251" t="n">
         <v>5</v>
@@ -13014,23 +13014,23 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>11.6</v>
+        <v>11.1</v>
       </c>
       <c r="E252" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F252" t="n">
         <v>7.9</v>
       </c>
       <c r="G252" t="n">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H252" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I252" t="n">
         <v>0</v>
@@ -13039,7 +13039,7 @@
         <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>0.297</v>
+        <v>0.298</v>
       </c>
       <c r="L252" t="n">
         <v>5</v>
@@ -13064,20 +13064,20 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>14</v>
+        <v>13.8</v>
       </c>
       <c r="E253" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F253" t="n">
-        <v>12.2</v>
+        <v>13.3</v>
       </c>
       <c r="G253" t="n">
-        <v>459</v>
+        <v>474</v>
       </c>
       <c r="H253" t="n">
         <v>0</v>
@@ -13089,7 +13089,7 @@
         <v>0</v>
       </c>
       <c r="K253" t="n">
-        <v>0.295</v>
+        <v>0.297</v>
       </c>
       <c r="L253" t="n">
         <v>5</v>
@@ -13114,20 +13114,20 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>15.6</v>
+        <v>15.2</v>
       </c>
       <c r="E254" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F254" t="n">
-        <v>16.2</v>
+        <v>15.5</v>
       </c>
       <c r="G254" t="n">
-        <v>554</v>
+        <v>549</v>
       </c>
       <c r="H254" t="n">
         <v>36</v>
@@ -13139,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="K254" t="n">
-        <v>0.295</v>
+        <v>0.296</v>
       </c>
       <c r="L254" t="n">
         <v>5</v>
@@ -13164,23 +13164,23 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>16</v>
+        <v>15.8</v>
       </c>
       <c r="E255" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F255" t="n">
-        <v>16.9</v>
+        <v>16.6</v>
       </c>
       <c r="G255" t="n">
-        <v>513</v>
+        <v>498</v>
       </c>
       <c r="H255" t="n">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13189,7 +13189,7 @@
         <v>0</v>
       </c>
       <c r="K255" t="n">
-        <v>0.293</v>
+        <v>0.295</v>
       </c>
       <c r="L255" t="n">
         <v>5</v>
@@ -13214,23 +13214,23 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="E256" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F256" t="n">
-        <v>16.2</v>
+        <v>17.6</v>
       </c>
       <c r="G256" t="n">
-        <v>475</v>
+        <v>427</v>
       </c>
       <c r="H256" t="n">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="I256" t="n">
         <v>0</v>
@@ -13239,7 +13239,7 @@
         <v>0</v>
       </c>
       <c r="K256" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L256" t="n">
         <v>5</v>
@@ -13264,20 +13264,20 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="E257" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F257" t="n">
-        <v>17.3</v>
+        <v>16.6</v>
       </c>
       <c r="G257" t="n">
-        <v>359</v>
+        <v>379</v>
       </c>
       <c r="H257" t="n">
         <v>77</v>
@@ -13289,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="K257" t="n">
-        <v>0.289</v>
+        <v>0.29</v>
       </c>
       <c r="L257" t="n">
         <v>5</v>
@@ -13314,23 +13314,23 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>16.2</v>
+        <v>16.3</v>
       </c>
       <c r="E258" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F258" t="n">
         <v>15.8</v>
       </c>
       <c r="G258" t="n">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="H258" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="I258" t="n">
         <v>0</v>
@@ -13339,7 +13339,7 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
-        <v>0.288</v>
+        <v>0.289</v>
       </c>
       <c r="L258" t="n">
         <v>5</v>
@@ -13364,20 +13364,20 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>15.8</v>
+        <v>15.9</v>
       </c>
       <c r="E259" t="n">
         <v>38</v>
       </c>
       <c r="F259" t="n">
-        <v>13.3</v>
+        <v>14.8</v>
       </c>
       <c r="G259" t="n">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="H259" t="n">
         <v>0</v>
@@ -13389,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>0.287</v>
+        <v>0.288</v>
       </c>
       <c r="L259" t="n">
         <v>5</v>
@@ -13414,20 +13414,20 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>14</v>
+        <v>14.1</v>
       </c>
       <c r="E260" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>7.9</v>
+        <v>9.4</v>
       </c>
       <c r="G260" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H260" t="n">
         <v>0</v>
@@ -13439,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L260" t="n">
         <v>5</v>
@@ -13464,17 +13464,17 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="E261" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F261" t="n">
-        <v>6.1</v>
+        <v>7.6</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -13489,7 +13489,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L261" t="n">
         <v>5</v>
@@ -13514,23 +13514,23 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D262" t="n">
         <v>9.800000000000001</v>
       </c>
       <c r="E262" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F262" t="n">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
       </c>
       <c r="H262" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="I262" t="n">
         <v>0</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,17 +13564,17 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E263" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F263" t="n">
-        <v>9.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,17 +13614,17 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="E264" t="n">
         <v>64</v>
       </c>
       <c r="F264" t="n">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,17 +13664,17 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="E265" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F265" t="n">
-        <v>7.9</v>
+        <v>7.6</v>
       </c>
       <c r="G265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13714,17 +13714,17 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="E266" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F266" t="n">
-        <v>6.5</v>
+        <v>7.2</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -13739,7 +13739,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L266" t="n">
         <v>6</v>
@@ -13764,23 +13764,23 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
       <c r="E267" t="n">
         <v>76</v>
       </c>
       <c r="F267" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="G267" t="n">
         <v>0</v>
       </c>
       <c r="H267" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -13789,7 +13789,7 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L267" t="n">
         <v>6</v>
@@ -13814,23 +13814,23 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>6.2</v>
+        <v>5</v>
       </c>
       <c r="E268" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F268" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
       </c>
       <c r="H268" t="n">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -13839,7 +13839,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L268" t="n">
         <v>6</v>
@@ -13864,23 +13864,23 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>7</v>
+        <v>4.7</v>
       </c>
       <c r="E269" t="n">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="F269" t="n">
-        <v>8.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="G269" t="n">
         <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="I269" t="n">
         <v>0</v>
@@ -13889,7 +13889,7 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L269" t="n">
         <v>6</v>
@@ -13914,23 +13914,23 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D270" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E270" t="n">
+        <v>83</v>
+      </c>
+      <c r="F270" t="n">
         <v>7.6</v>
       </c>
-      <c r="E270" t="n">
-        <v>67</v>
-      </c>
-      <c r="F270" t="n">
-        <v>6.1</v>
-      </c>
       <c r="G270" t="n">
         <v>0</v>
       </c>
       <c r="H270" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I270" t="n">
         <v>0</v>
@@ -13939,7 +13939,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L270" t="n">
         <v>6</v>
@@ -13964,23 +13964,23 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>7.8</v>
+        <v>4</v>
       </c>
       <c r="E271" t="n">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="F271" t="n">
-        <v>5.4</v>
+        <v>7.2</v>
       </c>
       <c r="G271" t="n">
         <v>0</v>
       </c>
       <c r="H271" t="n">
-        <v>100</v>
+        <v>57</v>
       </c>
       <c r="I271" t="n">
         <v>0</v>
@@ -13989,7 +13989,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L271" t="n">
         <v>6</v>
@@ -14014,23 +14014,23 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>8</v>
+        <v>4.1</v>
       </c>
       <c r="E272" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="F272" t="n">
-        <v>5.8</v>
+        <v>9</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
       </c>
       <c r="H272" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="I272" t="n">
         <v>0</v>
@@ -14039,7 +14039,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L272" t="n">
         <v>6</v>
@@ -14064,17 +14064,17 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>8.199999999999999</v>
+        <v>4.9</v>
       </c>
       <c r="E273" t="n">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="F273" t="n">
-        <v>6.1</v>
+        <v>6.8</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
@@ -14089,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L273" t="n">
         <v>6</v>
@@ -14114,23 +14114,23 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>8.300000000000001</v>
+        <v>5.9</v>
       </c>
       <c r="E274" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="F274" t="n">
-        <v>5</v>
+        <v>6.1</v>
       </c>
       <c r="G274" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="H274" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I274" t="n">
         <v>0</v>
@@ -14164,23 +14164,23 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>9.1</v>
+        <v>7.9</v>
       </c>
       <c r="E275" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F275" t="n">
-        <v>7.2</v>
+        <v>6.5</v>
       </c>
       <c r="G275" t="n">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="H275" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="I275" t="n">
         <v>0</v>
@@ -14214,20 +14214,20 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="E276" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F276" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="G276" t="n">
-        <v>103</v>
+        <v>237</v>
       </c>
       <c r="H276" t="n">
         <v>100</v>
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>0.288</v>
+        <v>0.287</v>
       </c>
       <c r="L276" t="n">
         <v>6</v>
@@ -14264,20 +14264,20 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>12.4</v>
+        <v>13.1</v>
       </c>
       <c r="E277" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="F277" t="n">
-        <v>8.300000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="G277" t="n">
-        <v>135</v>
+        <v>262</v>
       </c>
       <c r="H277" t="n">
         <v>100</v>
@@ -14289,7 +14289,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>0.288</v>
+        <v>0.286</v>
       </c>
       <c r="L277" t="n">
         <v>6</v>
@@ -14314,20 +14314,20 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>13.1</v>
+        <v>14.5</v>
       </c>
       <c r="E278" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F278" t="n">
-        <v>12.6</v>
+        <v>10.8</v>
       </c>
       <c r="G278" t="n">
-        <v>103</v>
+        <v>264</v>
       </c>
       <c r="H278" t="n">
         <v>100</v>
@@ -14339,7 +14339,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>0.287</v>
+        <v>0.284</v>
       </c>
       <c r="L278" t="n">
         <v>6</v>
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>14.2</v>
+        <v>16</v>
       </c>
       <c r="E279" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="F279" t="n">
-        <v>12.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G279" t="n">
-        <v>162</v>
+        <v>348</v>
       </c>
       <c r="H279" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.286</v>
+        <v>0.283</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,23 +14414,23 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>14.9</v>
+        <v>16.8</v>
       </c>
       <c r="E280" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F280" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
       <c r="G280" t="n">
-        <v>198</v>
+        <v>414</v>
       </c>
       <c r="H280" t="n">
-        <v>95</v>
+        <v>72</v>
       </c>
       <c r="I280" t="n">
         <v>0</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.285</v>
+        <v>0.282</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,23 +14464,23 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>15.8</v>
+        <v>17.2</v>
       </c>
       <c r="E281" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F281" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="G281" t="n">
-        <v>309</v>
+        <v>359</v>
       </c>
       <c r="H281" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="I281" t="n">
         <v>0</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.284</v>
+        <v>0.281</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,23 +14514,23 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>16.1</v>
+        <v>17.1</v>
       </c>
       <c r="E282" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F282" t="n">
-        <v>7.9</v>
+        <v>4.7</v>
       </c>
       <c r="G282" t="n">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="H282" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I282" t="n">
         <v>0</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.283</v>
+        <v>0.28</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,23 +14564,23 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>15.2</v>
+        <v>16.9</v>
       </c>
       <c r="E283" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F283" t="n">
-        <v>5.6</v>
+        <v>1.8</v>
       </c>
       <c r="G283" t="n">
-        <v>55.3</v>
+        <v>74</v>
       </c>
       <c r="H283" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -14589,7 +14589,7 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0.282</v>
+        <v>0.28</v>
       </c>
       <c r="L283" t="n">
         <v>6</v>
@@ -14614,23 +14614,23 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>13.5</v>
+        <v>14.7</v>
       </c>
       <c r="E284" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="F284" t="n">
-        <v>4.2</v>
+        <v>11.2</v>
       </c>
       <c r="G284" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="H284" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="I284" t="n">
         <v>0</v>
@@ -14639,7 +14639,7 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0.282</v>
+        <v>0.28</v>
       </c>
       <c r="L284" t="n">
         <v>6</v>
@@ -14664,23 +14664,23 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>11.4</v>
+        <v>12.5</v>
       </c>
       <c r="E285" t="n">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="F285" t="n">
-        <v>5</v>
+        <v>8.6</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
       </c>
       <c r="H285" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -14689,7 +14689,7 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
-        <v>0.282</v>
+        <v>0.28</v>
       </c>
       <c r="L285" t="n">
         <v>6</v>
@@ -14714,23 +14714,23 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>10.4</v>
+        <v>11.3</v>
       </c>
       <c r="E286" t="n">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="F286" t="n">
-        <v>5.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14739,7 +14739,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0.281</v>
+        <v>0.28</v>
       </c>
       <c r="L286" t="n">
         <v>6</v>
@@ -14764,23 +14764,23 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>10.2</v>
+        <v>10.5</v>
       </c>
       <c r="E287" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="F287" t="n">
-        <v>5.6</v>
+        <v>10.1</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>16</v>
+        <v>70</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>0.281</v>
+        <v>0.28</v>
       </c>
       <c r="L287" t="n">
         <v>6</v>
@@ -14814,23 +14814,23 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="E288" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="F288" t="n">
-        <v>5.3</v>
+        <v>10.4</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
       </c>
       <c r="H288" t="n">
-        <v>6</v>
+        <v>74</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.281</v>
+        <v>0.28</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,23 +14864,23 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>8.9</v>
+        <v>10.4</v>
       </c>
       <c r="E289" t="n">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="F289" t="n">
-        <v>4.6</v>
+        <v>7.2</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
       </c>
       <c r="H289" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="I289" t="n">
         <v>0</v>
@@ -14889,7 +14889,7 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>0.281</v>
+        <v>0.28</v>
       </c>
       <c r="L289" t="n">
         <v>6</v>
@@ -14914,23 +14914,23 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>8.5</v>
+        <v>9.4</v>
       </c>
       <c r="E290" t="n">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="F290" t="n">
-        <v>4.1</v>
+        <v>2.5</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
       </c>
       <c r="H290" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="I290" t="n">
         <v>0</v>
@@ -14939,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="K290" t="n">
-        <v>0.281</v>
+        <v>0.28</v>
       </c>
       <c r="L290" t="n">
         <v>7</v>
@@ -14964,23 +14964,23 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-15T11:03:48Z</t>
+          <t>2026-10-15T17:03:40Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="E291" t="n">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="F291" t="n">
-        <v>4.9</v>
+        <v>5.8</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
       </c>
       <c r="H291" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="I291" t="n">
         <v>0</v>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>0.281</v>
+        <v>0.28</v>
       </c>
       <c r="L291" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
prognoza biciklista (zvanicna): 2026-10-16 01:04
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -12564,17 +12564,17 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="E243" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F243" t="n">
-        <v>6.8</v>
+        <v>1.4</v>
       </c>
       <c r="G243" t="n">
         <v>0</v>
@@ -12589,7 +12589,7 @@
         <v>0</v>
       </c>
       <c r="K243" t="n">
-        <v>0.3</v>
+        <v>0.303</v>
       </c>
       <c r="L243" t="n">
         <v>5</v>
@@ -12614,17 +12614,17 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="E244" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F244" t="n">
-        <v>4.3</v>
+        <v>1.4</v>
       </c>
       <c r="G244" t="n">
         <v>0</v>
@@ -12639,7 +12639,7 @@
         <v>0</v>
       </c>
       <c r="K244" t="n">
-        <v>0.3</v>
+        <v>0.303</v>
       </c>
       <c r="L244" t="n">
         <v>5</v>
@@ -12664,17 +12664,17 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="E245" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F245" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -12689,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
-        <v>0.3</v>
+        <v>0.303</v>
       </c>
       <c r="L245" t="n">
         <v>5</v>
@@ -12714,17 +12714,17 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="E246" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F246" t="n">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
       <c r="G246" t="n">
         <v>0</v>
@@ -12739,7 +12739,7 @@
         <v>0</v>
       </c>
       <c r="K246" t="n">
-        <v>0.3</v>
+        <v>0.302</v>
       </c>
       <c r="L246" t="n">
         <v>5</v>
@@ -12764,17 +12764,17 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="E247" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F247" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G247" t="n">
         <v>0</v>
@@ -12789,7 +12789,7 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>0.3</v>
+        <v>0.302</v>
       </c>
       <c r="L247" t="n">
         <v>5</v>
@@ -12814,14 +12814,14 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="E248" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F248" t="n">
         <v>4.3</v>
@@ -12839,7 +12839,7 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
-        <v>0.3</v>
+        <v>0.302</v>
       </c>
       <c r="L248" t="n">
         <v>5</v>
@@ -12864,14 +12864,14 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
       <c r="E249" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F249" t="n">
         <v>6.1</v>
@@ -12889,7 +12889,7 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>0.3</v>
+        <v>0.302</v>
       </c>
       <c r="L249" t="n">
         <v>5</v>
@@ -12914,11 +12914,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>3.9</v>
+        <v>3.3</v>
       </c>
       <c r="E250" t="n">
         <v>94</v>
@@ -12927,10 +12927,10 @@
         <v>6.8</v>
       </c>
       <c r="G250" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H250" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="I250" t="n">
         <v>0</v>
@@ -12939,7 +12939,7 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>0.3</v>
+        <v>0.302</v>
       </c>
       <c r="L250" t="n">
         <v>5</v>
@@ -12964,20 +12964,20 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="E251" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F251" t="n">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="G251" t="n">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="H251" t="n">
         <v>0</v>
@@ -12989,7 +12989,7 @@
         <v>0</v>
       </c>
       <c r="K251" t="n">
-        <v>0.299</v>
+        <v>0.302</v>
       </c>
       <c r="L251" t="n">
         <v>5</v>
@@ -13014,20 +13014,20 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>11.1</v>
+        <v>10.8</v>
       </c>
       <c r="E252" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F252" t="n">
-        <v>7.9</v>
+        <v>7.2</v>
       </c>
       <c r="G252" t="n">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H252" t="n">
         <v>0</v>
@@ -13039,7 +13039,7 @@
         <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>0.298</v>
+        <v>0.301</v>
       </c>
       <c r="L252" t="n">
         <v>5</v>
@@ -13064,20 +13064,20 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>13.8</v>
+        <v>13.7</v>
       </c>
       <c r="E253" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F253" t="n">
-        <v>13.3</v>
+        <v>12.6</v>
       </c>
       <c r="G253" t="n">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="H253" t="n">
         <v>0</v>
@@ -13089,7 +13089,7 @@
         <v>0</v>
       </c>
       <c r="K253" t="n">
-        <v>0.297</v>
+        <v>0.3</v>
       </c>
       <c r="L253" t="n">
         <v>5</v>
@@ -13114,23 +13114,23 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
       <c r="E254" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F254" t="n">
-        <v>15.5</v>
+        <v>14</v>
       </c>
       <c r="G254" t="n">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="H254" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="I254" t="n">
         <v>0</v>
@@ -13139,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="K254" t="n">
-        <v>0.296</v>
+        <v>0.298</v>
       </c>
       <c r="L254" t="n">
         <v>5</v>
@@ -13164,23 +13164,23 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D255" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="E255" t="n">
+        <v>40</v>
+      </c>
+      <c r="F255" t="n">
         <v>15.8</v>
       </c>
-      <c r="E255" t="n">
-        <v>41</v>
-      </c>
-      <c r="F255" t="n">
-        <v>16.6</v>
-      </c>
       <c r="G255" t="n">
-        <v>498</v>
+        <v>576</v>
       </c>
       <c r="H255" t="n">
-        <v>64</v>
+        <v>23</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13189,7 +13189,7 @@
         <v>0</v>
       </c>
       <c r="K255" t="n">
-        <v>0.295</v>
+        <v>0.297</v>
       </c>
       <c r="L255" t="n">
         <v>5</v>
@@ -13214,23 +13214,23 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="E256" t="n">
         <v>39</v>
       </c>
       <c r="F256" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="G256" t="n">
-        <v>427</v>
+        <v>475</v>
       </c>
       <c r="H256" t="n">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="I256" t="n">
         <v>0</v>
@@ -13239,7 +13239,7 @@
         <v>0</v>
       </c>
       <c r="K256" t="n">
-        <v>0.292</v>
+        <v>0.294</v>
       </c>
       <c r="L256" t="n">
         <v>5</v>
@@ -13264,23 +13264,23 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>16.2</v>
+        <v>16.4</v>
       </c>
       <c r="E257" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F257" t="n">
-        <v>16.6</v>
+        <v>17.3</v>
       </c>
       <c r="G257" t="n">
-        <v>379</v>
+        <v>422</v>
       </c>
       <c r="H257" t="n">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -13289,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="K257" t="n">
-        <v>0.29</v>
+        <v>0.292</v>
       </c>
       <c r="L257" t="n">
         <v>5</v>
@@ -13314,20 +13314,20 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>16.3</v>
+        <v>16.4</v>
       </c>
       <c r="E258" t="n">
         <v>38</v>
       </c>
       <c r="F258" t="n">
-        <v>15.8</v>
+        <v>15.1</v>
       </c>
       <c r="G258" t="n">
-        <v>278</v>
+        <v>324</v>
       </c>
       <c r="H258" t="n">
         <v>0</v>
@@ -13339,7 +13339,7 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
-        <v>0.289</v>
+        <v>0.29</v>
       </c>
       <c r="L258" t="n">
         <v>5</v>
@@ -13364,20 +13364,20 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D259" t="n">
         <v>15.9</v>
       </c>
       <c r="E259" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F259" t="n">
-        <v>14.8</v>
+        <v>14</v>
       </c>
       <c r="G259" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="H259" t="n">
         <v>0</v>
@@ -13389,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>0.288</v>
+        <v>0.289</v>
       </c>
       <c r="L259" t="n">
         <v>5</v>
@@ -13414,17 +13414,17 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>14.1</v>
+        <v>14</v>
       </c>
       <c r="E260" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F260" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="G260" t="n">
         <v>38</v>
@@ -13439,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L260" t="n">
         <v>5</v>
@@ -13464,17 +13464,17 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="E261" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F261" t="n">
-        <v>7.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -13489,7 +13489,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L261" t="n">
         <v>5</v>
@@ -13514,17 +13514,17 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="E262" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F262" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,17 +13564,17 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="E263" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F263" t="n">
-        <v>9.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,17 +13614,17 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D264" t="n">
         <v>7.6</v>
       </c>
       <c r="E264" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F264" t="n">
-        <v>9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,17 +13664,17 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="E265" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F265" t="n">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
       <c r="G265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13714,17 +13714,17 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="E266" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F266" t="n">
-        <v>7.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -13739,7 +13739,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L266" t="n">
         <v>6</v>
@@ -13764,17 +13764,17 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D267" t="n">
         <v>5.3</v>
       </c>
       <c r="E267" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F267" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="G267" t="n">
         <v>0</v>
@@ -13789,7 +13789,7 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L267" t="n">
         <v>6</v>
@@ -13814,23 +13814,23 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="E268" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F268" t="n">
-        <v>7.6</v>
+        <v>6.8</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
       </c>
       <c r="H268" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -13839,7 +13839,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L268" t="n">
         <v>6</v>
@@ -13864,23 +13864,23 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="E269" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F269" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="G269" t="n">
         <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I269" t="n">
         <v>0</v>
@@ -13889,7 +13889,7 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L269" t="n">
         <v>6</v>
@@ -13914,23 +13914,23 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>4.3</v>
+        <v>4.9</v>
       </c>
       <c r="E270" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F270" t="n">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
       <c r="G270" t="n">
         <v>0</v>
       </c>
       <c r="H270" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I270" t="n">
         <v>0</v>
@@ -13939,7 +13939,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L270" t="n">
         <v>6</v>
@@ -13964,23 +13964,23 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="E271" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="F271" t="n">
-        <v>7.2</v>
+        <v>9</v>
       </c>
       <c r="G271" t="n">
         <v>0</v>
       </c>
       <c r="H271" t="n">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="I271" t="n">
         <v>0</v>
@@ -13989,7 +13989,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L271" t="n">
         <v>6</v>
@@ -14014,23 +14014,23 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="E272" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F272" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
       </c>
       <c r="H272" t="n">
-        <v>92</v>
+        <v>5</v>
       </c>
       <c r="I272" t="n">
         <v>0</v>
@@ -14039,7 +14039,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L272" t="n">
         <v>6</v>
@@ -14064,17 +14064,17 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="E273" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F273" t="n">
-        <v>6.8</v>
+        <v>7.6</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
@@ -14089,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L273" t="n">
         <v>6</v>
@@ -14114,23 +14114,23 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="E274" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F274" t="n">
-        <v>6.1</v>
+        <v>8.6</v>
       </c>
       <c r="G274" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="H274" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I274" t="n">
         <v>0</v>
@@ -14139,7 +14139,7 @@
         <v>0</v>
       </c>
       <c r="K274" t="n">
-        <v>0.287</v>
+        <v>0.288</v>
       </c>
       <c r="L274" t="n">
         <v>6</v>
@@ -14164,23 +14164,23 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>7.9</v>
+        <v>7</v>
       </c>
       <c r="E275" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F275" t="n">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="G275" t="n">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="H275" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="I275" t="n">
         <v>0</v>
@@ -14189,7 +14189,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>0.287</v>
+        <v>0.288</v>
       </c>
       <c r="L275" t="n">
         <v>6</v>
@@ -14214,20 +14214,20 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>11.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E276" t="n">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="F276" t="n">
-        <v>7.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G276" t="n">
-        <v>237</v>
+        <v>66</v>
       </c>
       <c r="H276" t="n">
         <v>100</v>
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>0.287</v>
+        <v>0.288</v>
       </c>
       <c r="L276" t="n">
         <v>6</v>
@@ -14264,23 +14264,23 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>13.1</v>
+        <v>10.9</v>
       </c>
       <c r="E277" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F277" t="n">
-        <v>10.4</v>
+        <v>7.6</v>
       </c>
       <c r="G277" t="n">
-        <v>262</v>
+        <v>201</v>
       </c>
       <c r="H277" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="I277" t="n">
         <v>0</v>
@@ -14289,7 +14289,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L277" t="n">
         <v>6</v>
@@ -14314,20 +14314,20 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>14.5</v>
+        <v>13</v>
       </c>
       <c r="E278" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F278" t="n">
-        <v>10.8</v>
+        <v>8.6</v>
       </c>
       <c r="G278" t="n">
-        <v>264</v>
+        <v>219</v>
       </c>
       <c r="H278" t="n">
         <v>100</v>
@@ -14339,7 +14339,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>0.284</v>
+        <v>0.287</v>
       </c>
       <c r="L278" t="n">
         <v>6</v>
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>16</v>
+        <v>14.5</v>
       </c>
       <c r="E279" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F279" t="n">
-        <v>9.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="G279" t="n">
-        <v>348</v>
+        <v>285</v>
       </c>
       <c r="H279" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.283</v>
+        <v>0.286</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,23 +14414,23 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>16.8</v>
+        <v>15.6</v>
       </c>
       <c r="E280" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F280" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="G280" t="n">
-        <v>414</v>
+        <v>337</v>
       </c>
       <c r="H280" t="n">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="I280" t="n">
         <v>0</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.282</v>
+        <v>0.285</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,23 +14464,23 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>17.2</v>
+        <v>16</v>
       </c>
       <c r="E281" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F281" t="n">
-        <v>7.2</v>
+        <v>4.3</v>
       </c>
       <c r="G281" t="n">
-        <v>359</v>
+        <v>241</v>
       </c>
       <c r="H281" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I281" t="n">
         <v>0</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.281</v>
+        <v>0.284</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,23 +14514,23 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>17.1</v>
+        <v>15.9</v>
       </c>
       <c r="E282" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F282" t="n">
-        <v>4.7</v>
+        <v>2.2</v>
       </c>
       <c r="G282" t="n">
-        <v>182</v>
+        <v>67</v>
       </c>
       <c r="H282" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I282" t="n">
         <v>0</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.28</v>
+        <v>0.284</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,23 +14564,23 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>16.9</v>
+        <v>15.4</v>
       </c>
       <c r="E283" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F283" t="n">
         <v>1.8</v>
       </c>
       <c r="G283" t="n">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="H283" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -14589,7 +14589,7 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L283" t="n">
         <v>6</v>
@@ -14614,23 +14614,23 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>14.7</v>
+        <v>14.1</v>
       </c>
       <c r="E284" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F284" t="n">
-        <v>11.2</v>
+        <v>5.8</v>
       </c>
       <c r="G284" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="H284" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="I284" t="n">
         <v>0</v>
@@ -14639,7 +14639,7 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L284" t="n">
         <v>6</v>
@@ -14664,23 +14664,23 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>12.5</v>
+        <v>12.9</v>
       </c>
       <c r="E285" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F285" t="n">
-        <v>8.6</v>
+        <v>5.4</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
       </c>
       <c r="H285" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -14689,7 +14689,7 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L285" t="n">
         <v>6</v>
@@ -14714,23 +14714,23 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="E286" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F286" t="n">
-        <v>9.699999999999999</v>
+        <v>5.8</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14739,7 +14739,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L286" t="n">
         <v>6</v>
@@ -14764,23 +14764,23 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>10.5</v>
+        <v>9.9</v>
       </c>
       <c r="E287" t="n">
         <v>55</v>
       </c>
       <c r="F287" t="n">
-        <v>10.1</v>
+        <v>6.5</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L287" t="n">
         <v>6</v>
@@ -14814,23 +14814,23 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>10.5</v>
+        <v>8</v>
       </c>
       <c r="E288" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F288" t="n">
-        <v>10.4</v>
+        <v>7.9</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
       </c>
       <c r="H288" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,23 +14864,23 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>10.4</v>
+        <v>6.8</v>
       </c>
       <c r="E289" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="F289" t="n">
-        <v>7.2</v>
+        <v>5.4</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
       </c>
       <c r="H289" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="I289" t="n">
         <v>0</v>
@@ -14889,7 +14889,7 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L289" t="n">
         <v>6</v>
@@ -14914,23 +14914,23 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>9.4</v>
+        <v>6.7</v>
       </c>
       <c r="E290" t="n">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="F290" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
       </c>
       <c r="H290" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="I290" t="n">
         <v>0</v>
@@ -14939,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="K290" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L290" t="n">
         <v>7</v>
@@ -14964,23 +14964,23 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-15T17:03:40Z</t>
+          <t>2026-10-15T23:03:44Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="E291" t="n">
         <v>66</v>
       </c>
       <c r="F291" t="n">
-        <v>5.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
       </c>
       <c r="H291" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I291" t="n">
         <v>0</v>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>0.28</v>
+        <v>0.283</v>
       </c>
       <c r="L291" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-16 07:04
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N291"/>
+  <dimension ref="A1:N315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -12864,14 +12864,14 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D249" t="n">
         <v>2.7</v>
       </c>
       <c r="E249" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F249" t="n">
         <v>6.1</v>
@@ -12889,7 +12889,7 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
-        <v>0.302</v>
+        <v>0.301</v>
       </c>
       <c r="L249" t="n">
         <v>5</v>
@@ -12914,11 +12914,11 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="E250" t="n">
         <v>94</v>
@@ -12939,7 +12939,7 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
-        <v>0.302</v>
+        <v>0.301</v>
       </c>
       <c r="L250" t="n">
         <v>5</v>
@@ -12964,20 +12964,20 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="E251" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F251" t="n">
         <v>6.1</v>
       </c>
       <c r="G251" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H251" t="n">
         <v>0</v>
@@ -12989,7 +12989,7 @@
         <v>0</v>
       </c>
       <c r="K251" t="n">
-        <v>0.302</v>
+        <v>0.301</v>
       </c>
       <c r="L251" t="n">
         <v>5</v>
@@ -13014,17 +13014,17 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D252" t="n">
         <v>10.8</v>
       </c>
       <c r="E252" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F252" t="n">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="G252" t="n">
         <v>350</v>
@@ -13039,7 +13039,7 @@
         <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>0.301</v>
+        <v>0.3</v>
       </c>
       <c r="L252" t="n">
         <v>5</v>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>13.7</v>
+        <v>13.3</v>
       </c>
       <c r="E253" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F253" t="n">
-        <v>12.6</v>
+        <v>10.4</v>
       </c>
       <c r="G253" t="n">
         <v>473</v>
@@ -13089,7 +13089,7 @@
         <v>0</v>
       </c>
       <c r="K253" t="n">
-        <v>0.3</v>
+        <v>0.298</v>
       </c>
       <c r="L253" t="n">
         <v>5</v>
@@ -13114,23 +13114,23 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>15.1</v>
+        <v>15</v>
       </c>
       <c r="E254" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F254" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G254" t="n">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="H254" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I254" t="n">
         <v>0</v>
@@ -13139,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="K254" t="n">
-        <v>0.298</v>
+        <v>0.296</v>
       </c>
       <c r="L254" t="n">
         <v>5</v>
@@ -13164,23 +13164,23 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D255" t="n">
         <v>16.1</v>
       </c>
       <c r="E255" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F255" t="n">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="G255" t="n">
-        <v>576</v>
+        <v>559</v>
       </c>
       <c r="H255" t="n">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13189,7 +13189,7 @@
         <v>0</v>
       </c>
       <c r="K255" t="n">
-        <v>0.297</v>
+        <v>0.294</v>
       </c>
       <c r="L255" t="n">
         <v>5</v>
@@ -13214,23 +13214,23 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
       <c r="E256" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F256" t="n">
-        <v>18.7</v>
+        <v>17.6</v>
       </c>
       <c r="G256" t="n">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="H256" t="n">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="I256" t="n">
         <v>0</v>
@@ -13239,7 +13239,7 @@
         <v>0</v>
       </c>
       <c r="K256" t="n">
-        <v>0.294</v>
+        <v>0.292</v>
       </c>
       <c r="L256" t="n">
         <v>5</v>
@@ -13264,23 +13264,23 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D257" t="n">
         <v>16.4</v>
       </c>
       <c r="E257" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F257" t="n">
-        <v>17.3</v>
+        <v>17.6</v>
       </c>
       <c r="G257" t="n">
-        <v>422</v>
+        <v>397</v>
       </c>
       <c r="H257" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -13289,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="K257" t="n">
-        <v>0.292</v>
+        <v>0.29</v>
       </c>
       <c r="L257" t="n">
         <v>5</v>
@@ -13314,20 +13314,20 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D258" t="n">
         <v>16.4</v>
       </c>
       <c r="E258" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F258" t="n">
-        <v>15.1</v>
+        <v>15.5</v>
       </c>
       <c r="G258" t="n">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="H258" t="n">
         <v>0</v>
@@ -13339,7 +13339,7 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
-        <v>0.29</v>
+        <v>0.288</v>
       </c>
       <c r="L258" t="n">
         <v>5</v>
@@ -13364,14 +13364,14 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>15.9</v>
+        <v>16</v>
       </c>
       <c r="E259" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F259" t="n">
         <v>14</v>
@@ -13389,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>0.289</v>
+        <v>0.287</v>
       </c>
       <c r="L259" t="n">
         <v>5</v>
@@ -13414,20 +13414,20 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>14</v>
+        <v>14.1</v>
       </c>
       <c r="E260" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F260" t="n">
-        <v>8.6</v>
+        <v>9.4</v>
       </c>
       <c r="G260" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H260" t="n">
         <v>0</v>
@@ -13439,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>0.289</v>
+        <v>0.287</v>
       </c>
       <c r="L260" t="n">
         <v>5</v>
@@ -13464,17 +13464,17 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="E261" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F261" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -13489,7 +13489,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L261" t="n">
         <v>5</v>
@@ -13514,14 +13514,14 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D262" t="n">
         <v>9.6</v>
       </c>
       <c r="E262" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F262" t="n">
         <v>8.6</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,17 +13564,17 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E263" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F263" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,17 +13614,17 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="E264" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F264" t="n">
-        <v>9.699999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,23 +13664,23 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D265" t="n">
         <v>6.8</v>
       </c>
       <c r="E265" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F265" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="G265" t="n">
         <v>0</v>
       </c>
       <c r="H265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13714,17 +13714,17 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="E266" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F266" t="n">
-        <v>8.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -13739,7 +13739,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L266" t="n">
         <v>6</v>
@@ -13764,14 +13764,14 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="E267" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F267" t="n">
         <v>5</v>
@@ -13789,7 +13789,7 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L267" t="n">
         <v>6</v>
@@ -13814,23 +13814,23 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
       <c r="E268" t="n">
         <v>74</v>
       </c>
       <c r="F268" t="n">
-        <v>6.8</v>
+        <v>9.4</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
       </c>
       <c r="H268" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -13839,7 +13839,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L268" t="n">
         <v>6</v>
@@ -13864,23 +13864,23 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="E269" t="n">
         <v>76</v>
       </c>
       <c r="F269" t="n">
-        <v>7.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G269" t="n">
         <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="I269" t="n">
         <v>0</v>
@@ -13889,7 +13889,7 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L269" t="n">
         <v>6</v>
@@ -13914,23 +13914,23 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="E270" t="n">
         <v>77</v>
       </c>
       <c r="F270" t="n">
-        <v>9.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G270" t="n">
         <v>0</v>
       </c>
       <c r="H270" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="I270" t="n">
         <v>0</v>
@@ -13939,7 +13939,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L270" t="n">
         <v>6</v>
@@ -13964,23 +13964,23 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>4.3</v>
+        <v>4.8</v>
       </c>
       <c r="E271" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F271" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="G271" t="n">
         <v>0</v>
       </c>
       <c r="H271" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I271" t="n">
         <v>0</v>
@@ -13989,7 +13989,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L271" t="n">
         <v>6</v>
@@ -14014,14 +14014,14 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>4</v>
+        <v>5.1</v>
       </c>
       <c r="E272" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F272" t="n">
         <v>8.300000000000001</v>
@@ -14030,7 +14030,7 @@
         <v>0</v>
       </c>
       <c r="H272" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I272" t="n">
         <v>0</v>
@@ -14039,7 +14039,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L272" t="n">
         <v>6</v>
@@ -14064,17 +14064,17 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>4.7</v>
+        <v>6</v>
       </c>
       <c r="E273" t="n">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F273" t="n">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
@@ -14089,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L273" t="n">
         <v>6</v>
@@ -14114,20 +14114,20 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="E274" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F274" t="n">
-        <v>8.6</v>
+        <v>11.2</v>
       </c>
       <c r="G274" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H274" t="n">
         <v>100</v>
@@ -14139,7 +14139,7 @@
         <v>0</v>
       </c>
       <c r="K274" t="n">
-        <v>0.288</v>
+        <v>0.286</v>
       </c>
       <c r="L274" t="n">
         <v>6</v>
@@ -14164,20 +14164,20 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="E275" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F275" t="n">
-        <v>6.8</v>
+        <v>9.4</v>
       </c>
       <c r="G275" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="H275" t="n">
         <v>100</v>
@@ -14189,7 +14189,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>0.288</v>
+        <v>0.286</v>
       </c>
       <c r="L275" t="n">
         <v>6</v>
@@ -14214,7 +14214,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D276" t="n">
@@ -14224,10 +14224,10 @@
         <v>63</v>
       </c>
       <c r="F276" t="n">
-        <v>8.300000000000001</v>
+        <v>6.8</v>
       </c>
       <c r="G276" t="n">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="H276" t="n">
         <v>100</v>
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>0.288</v>
+        <v>0.286</v>
       </c>
       <c r="L276" t="n">
         <v>6</v>
@@ -14264,23 +14264,23 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>10.9</v>
+        <v>10.2</v>
       </c>
       <c r="E277" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F277" t="n">
-        <v>7.6</v>
+        <v>9.4</v>
       </c>
       <c r="G277" t="n">
-        <v>201</v>
+        <v>153</v>
       </c>
       <c r="H277" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I277" t="n">
         <v>0</v>
@@ -14289,7 +14289,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>0.287</v>
+        <v>0.285</v>
       </c>
       <c r="L277" t="n">
         <v>6</v>
@@ -14314,23 +14314,23 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E278" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F278" t="n">
-        <v>8.6</v>
+        <v>10.1</v>
       </c>
       <c r="G278" t="n">
-        <v>219</v>
+        <v>403</v>
       </c>
       <c r="H278" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="I278" t="n">
         <v>0</v>
@@ -14339,7 +14339,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>0.287</v>
+        <v>0.284</v>
       </c>
       <c r="L278" t="n">
         <v>6</v>
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>14.5</v>
+        <v>16</v>
       </c>
       <c r="E279" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F279" t="n">
-        <v>9</v>
+        <v>10.4</v>
       </c>
       <c r="G279" t="n">
-        <v>285</v>
+        <v>539</v>
       </c>
       <c r="H279" t="n">
-        <v>100</v>
+        <v>13</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.286</v>
+        <v>0.283</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,20 +14414,20 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>15.6</v>
+        <v>16.9</v>
       </c>
       <c r="E280" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F280" t="n">
-        <v>7.2</v>
+        <v>13</v>
       </c>
       <c r="G280" t="n">
-        <v>337</v>
+        <v>505</v>
       </c>
       <c r="H280" t="n">
         <v>99</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.285</v>
+        <v>0.283</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,20 +14464,20 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>16</v>
+        <v>16.4</v>
       </c>
       <c r="E281" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F281" t="n">
-        <v>4.3</v>
+        <v>12.2</v>
       </c>
       <c r="G281" t="n">
-        <v>241</v>
+        <v>194</v>
       </c>
       <c r="H281" t="n">
         <v>100</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.284</v>
+        <v>0.282</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,20 +14514,20 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>15.9</v>
+        <v>16.2</v>
       </c>
       <c r="E282" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F282" t="n">
-        <v>2.2</v>
+        <v>9</v>
       </c>
       <c r="G282" t="n">
-        <v>67</v>
+        <v>84</v>
       </c>
       <c r="H282" t="n">
         <v>100</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.284</v>
+        <v>0.281</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,23 +14564,23 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>15.4</v>
+        <v>15.8</v>
       </c>
       <c r="E283" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F283" t="n">
-        <v>1.8</v>
+        <v>4.7</v>
       </c>
       <c r="G283" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="H283" t="n">
-        <v>85</v>
+        <v>3</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -14589,7 +14589,7 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L283" t="n">
         <v>6</v>
@@ -14614,23 +14614,23 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>14.1</v>
+        <v>13.9</v>
       </c>
       <c r="E284" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F284" t="n">
-        <v>5.8</v>
+        <v>1.4</v>
       </c>
       <c r="G284" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="H284" t="n">
-        <v>100</v>
+        <v>32</v>
       </c>
       <c r="I284" t="n">
         <v>0</v>
@@ -14639,7 +14639,7 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L284" t="n">
         <v>6</v>
@@ -14664,23 +14664,23 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>12.9</v>
+        <v>12.1</v>
       </c>
       <c r="E285" t="n">
         <v>45</v>
       </c>
       <c r="F285" t="n">
-        <v>5.4</v>
+        <v>4.7</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
       </c>
       <c r="H285" t="n">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -14689,7 +14689,7 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L285" t="n">
         <v>6</v>
@@ -14714,23 +14714,23 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="E286" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F286" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14739,7 +14739,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L286" t="n">
         <v>6</v>
@@ -14764,23 +14764,23 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>9.9</v>
+        <v>11.3</v>
       </c>
       <c r="E287" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="F287" t="n">
-        <v>6.5</v>
+        <v>3.6</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L287" t="n">
         <v>6</v>
@@ -14814,17 +14814,17 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>8</v>
+        <v>9.9</v>
       </c>
       <c r="E288" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F288" t="n">
-        <v>7.9</v>
+        <v>6.5</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,23 +14864,23 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>6.8</v>
+        <v>8.6</v>
       </c>
       <c r="E289" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="F289" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
       </c>
       <c r="H289" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I289" t="n">
         <v>0</v>
@@ -14889,7 +14889,7 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L289" t="n">
         <v>6</v>
@@ -14914,17 +14914,17 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>6.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E290" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="F290" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
@@ -14939,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="K290" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L290" t="n">
         <v>7</v>
@@ -14964,17 +14964,17 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-15T23:03:44Z</t>
+          <t>2026-10-16T05:03:20Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="E291" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F291" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>0.283</v>
+        <v>0.281</v>
       </c>
       <c r="L291" t="n">
         <v>7</v>
@@ -14998,6 +14998,1206 @@
         <v>1</v>
       </c>
       <c r="N291" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E292" t="n">
+        <v>56</v>
+      </c>
+      <c r="F292" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0</v>
+      </c>
+      <c r="H292" t="n">
+        <v>86</v>
+      </c>
+      <c r="I292" t="n">
+        <v>0</v>
+      </c>
+      <c r="J292" t="n">
+        <v>0</v>
+      </c>
+      <c r="K292" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="L292" t="n">
+        <v>7</v>
+      </c>
+      <c r="M292" t="n">
+        <v>1</v>
+      </c>
+      <c r="N292" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E293" t="n">
+        <v>55</v>
+      </c>
+      <c r="F293" t="n">
+        <v>9</v>
+      </c>
+      <c r="G293" t="n">
+        <v>0</v>
+      </c>
+      <c r="H293" t="n">
+        <v>100</v>
+      </c>
+      <c r="I293" t="n">
+        <v>0</v>
+      </c>
+      <c r="J293" t="n">
+        <v>0</v>
+      </c>
+      <c r="K293" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="L293" t="n">
+        <v>7</v>
+      </c>
+      <c r="M293" t="n">
+        <v>1</v>
+      </c>
+      <c r="N293" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E294" t="n">
+        <v>52</v>
+      </c>
+      <c r="F294" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0</v>
+      </c>
+      <c r="H294" t="n">
+        <v>100</v>
+      </c>
+      <c r="I294" t="n">
+        <v>0</v>
+      </c>
+      <c r="J294" t="n">
+        <v>0</v>
+      </c>
+      <c r="K294" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="L294" t="n">
+        <v>7</v>
+      </c>
+      <c r="M294" t="n">
+        <v>1</v>
+      </c>
+      <c r="N294" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="E295" t="n">
+        <v>51</v>
+      </c>
+      <c r="F295" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0</v>
+      </c>
+      <c r="H295" t="n">
+        <v>95</v>
+      </c>
+      <c r="I295" t="n">
+        <v>0</v>
+      </c>
+      <c r="J295" t="n">
+        <v>0</v>
+      </c>
+      <c r="K295" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="L295" t="n">
+        <v>7</v>
+      </c>
+      <c r="M295" t="n">
+        <v>1</v>
+      </c>
+      <c r="N295" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="E296" t="n">
+        <v>52</v>
+      </c>
+      <c r="F296" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="n">
+        <v>100</v>
+      </c>
+      <c r="I296" t="n">
+        <v>0</v>
+      </c>
+      <c r="J296" t="n">
+        <v>0</v>
+      </c>
+      <c r="K296" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="L296" t="n">
+        <v>7</v>
+      </c>
+      <c r="M296" t="n">
+        <v>1</v>
+      </c>
+      <c r="N296" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E297" t="n">
+        <v>53</v>
+      </c>
+      <c r="F297" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G297" t="n">
+        <v>0</v>
+      </c>
+      <c r="H297" t="n">
+        <v>100</v>
+      </c>
+      <c r="I297" t="n">
+        <v>0</v>
+      </c>
+      <c r="J297" t="n">
+        <v>0</v>
+      </c>
+      <c r="K297" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="L297" t="n">
+        <v>7</v>
+      </c>
+      <c r="M297" t="n">
+        <v>1</v>
+      </c>
+      <c r="N297" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="E298" t="n">
+        <v>54</v>
+      </c>
+      <c r="F298" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G298" t="n">
+        <v>13</v>
+      </c>
+      <c r="H298" t="n">
+        <v>99</v>
+      </c>
+      <c r="I298" t="n">
+        <v>0</v>
+      </c>
+      <c r="J298" t="n">
+        <v>0</v>
+      </c>
+      <c r="K298" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="L298" t="n">
+        <v>7</v>
+      </c>
+      <c r="M298" t="n">
+        <v>1</v>
+      </c>
+      <c r="N298" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>11</v>
+      </c>
+      <c r="E299" t="n">
+        <v>51</v>
+      </c>
+      <c r="F299" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G299" t="n">
+        <v>166</v>
+      </c>
+      <c r="H299" t="n">
+        <v>0</v>
+      </c>
+      <c r="I299" t="n">
+        <v>0</v>
+      </c>
+      <c r="J299" t="n">
+        <v>0</v>
+      </c>
+      <c r="K299" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="L299" t="n">
+        <v>7</v>
+      </c>
+      <c r="M299" t="n">
+        <v>1</v>
+      </c>
+      <c r="N299" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="E300" t="n">
+        <v>42</v>
+      </c>
+      <c r="F300" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G300" t="n">
+        <v>341</v>
+      </c>
+      <c r="H300" t="n">
+        <v>6</v>
+      </c>
+      <c r="I300" t="n">
+        <v>0</v>
+      </c>
+      <c r="J300" t="n">
+        <v>0</v>
+      </c>
+      <c r="K300" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="L300" t="n">
+        <v>7</v>
+      </c>
+      <c r="M300" t="n">
+        <v>1</v>
+      </c>
+      <c r="N300" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="E301" t="n">
+        <v>42</v>
+      </c>
+      <c r="F301" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G301" t="n">
+        <v>445</v>
+      </c>
+      <c r="H301" t="n">
+        <v>18</v>
+      </c>
+      <c r="I301" t="n">
+        <v>0</v>
+      </c>
+      <c r="J301" t="n">
+        <v>0</v>
+      </c>
+      <c r="K301" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="L301" t="n">
+        <v>7</v>
+      </c>
+      <c r="M301" t="n">
+        <v>1</v>
+      </c>
+      <c r="N301" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="E302" t="n">
+        <v>43</v>
+      </c>
+      <c r="F302" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G302" t="n">
+        <v>500</v>
+      </c>
+      <c r="H302" t="n">
+        <v>33</v>
+      </c>
+      <c r="I302" t="n">
+        <v>0</v>
+      </c>
+      <c r="J302" t="n">
+        <v>0</v>
+      </c>
+      <c r="K302" t="n">
+        <v>0.276</v>
+      </c>
+      <c r="L302" t="n">
+        <v>7</v>
+      </c>
+      <c r="M302" t="n">
+        <v>1</v>
+      </c>
+      <c r="N302" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="E303" t="n">
+        <v>45</v>
+      </c>
+      <c r="F303" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G303" t="n">
+        <v>447.5</v>
+      </c>
+      <c r="H303" t="n">
+        <v>36</v>
+      </c>
+      <c r="I303" t="n">
+        <v>0</v>
+      </c>
+      <c r="J303" t="n">
+        <v>0</v>
+      </c>
+      <c r="K303" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="L303" t="n">
+        <v>7</v>
+      </c>
+      <c r="M303" t="n">
+        <v>1</v>
+      </c>
+      <c r="N303" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E304" t="n">
+        <v>48</v>
+      </c>
+      <c r="F304" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="G304" t="n">
+        <v>496</v>
+      </c>
+      <c r="H304" t="n">
+        <v>51</v>
+      </c>
+      <c r="I304" t="n">
+        <v>0</v>
+      </c>
+      <c r="J304" t="n">
+        <v>0</v>
+      </c>
+      <c r="K304" t="n">
+        <v>0.272</v>
+      </c>
+      <c r="L304" t="n">
+        <v>7</v>
+      </c>
+      <c r="M304" t="n">
+        <v>1</v>
+      </c>
+      <c r="N304" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="E305" t="n">
+        <v>48</v>
+      </c>
+      <c r="F305" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G305" t="n">
+        <v>386</v>
+      </c>
+      <c r="H305" t="n">
+        <v>45</v>
+      </c>
+      <c r="I305" t="n">
+        <v>0</v>
+      </c>
+      <c r="J305" t="n">
+        <v>0</v>
+      </c>
+      <c r="K305" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="L305" t="n">
+        <v>7</v>
+      </c>
+      <c r="M305" t="n">
+        <v>1</v>
+      </c>
+      <c r="N305" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E306" t="n">
+        <v>48</v>
+      </c>
+      <c r="F306" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G306" t="n">
+        <v>295</v>
+      </c>
+      <c r="H306" t="n">
+        <v>45</v>
+      </c>
+      <c r="I306" t="n">
+        <v>0</v>
+      </c>
+      <c r="J306" t="n">
+        <v>0</v>
+      </c>
+      <c r="K306" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="L306" t="n">
+        <v>7</v>
+      </c>
+      <c r="M306" t="n">
+        <v>1</v>
+      </c>
+      <c r="N306" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="E307" t="n">
+        <v>57</v>
+      </c>
+      <c r="F307" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G307" t="n">
+        <v>157</v>
+      </c>
+      <c r="H307" t="n">
+        <v>45</v>
+      </c>
+      <c r="I307" t="n">
+        <v>0</v>
+      </c>
+      <c r="J307" t="n">
+        <v>0</v>
+      </c>
+      <c r="K307" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="L307" t="n">
+        <v>7</v>
+      </c>
+      <c r="M307" t="n">
+        <v>1</v>
+      </c>
+      <c r="N307" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>14</v>
+      </c>
+      <c r="E308" t="n">
+        <v>65</v>
+      </c>
+      <c r="F308" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G308" t="n">
+        <v>28</v>
+      </c>
+      <c r="H308" t="n">
+        <v>31</v>
+      </c>
+      <c r="I308" t="n">
+        <v>0</v>
+      </c>
+      <c r="J308" t="n">
+        <v>0</v>
+      </c>
+      <c r="K308" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="L308" t="n">
+        <v>7</v>
+      </c>
+      <c r="M308" t="n">
+        <v>1</v>
+      </c>
+      <c r="N308" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="E309" t="n">
+        <v>68</v>
+      </c>
+      <c r="F309" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="n">
+        <v>12</v>
+      </c>
+      <c r="I309" t="n">
+        <v>0</v>
+      </c>
+      <c r="J309" t="n">
+        <v>0</v>
+      </c>
+      <c r="K309" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L309" t="n">
+        <v>7</v>
+      </c>
+      <c r="M309" t="n">
+        <v>1</v>
+      </c>
+      <c r="N309" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="E310" t="n">
+        <v>71</v>
+      </c>
+      <c r="F310" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H310" t="n">
+        <v>25</v>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0</v>
+      </c>
+      <c r="K310" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L310" t="n">
+        <v>7</v>
+      </c>
+      <c r="M310" t="n">
+        <v>1</v>
+      </c>
+      <c r="N310" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E311" t="n">
+        <v>75</v>
+      </c>
+      <c r="F311" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0</v>
+      </c>
+      <c r="H311" t="n">
+        <v>20</v>
+      </c>
+      <c r="I311" t="n">
+        <v>0</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0</v>
+      </c>
+      <c r="K311" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L311" t="n">
+        <v>7</v>
+      </c>
+      <c r="M311" t="n">
+        <v>1</v>
+      </c>
+      <c r="N311" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E312" t="n">
+        <v>79</v>
+      </c>
+      <c r="F312" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="G312" t="n">
+        <v>0</v>
+      </c>
+      <c r="H312" t="n">
+        <v>5</v>
+      </c>
+      <c r="I312" t="n">
+        <v>0</v>
+      </c>
+      <c r="J312" t="n">
+        <v>0</v>
+      </c>
+      <c r="K312" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L312" t="n">
+        <v>7</v>
+      </c>
+      <c r="M312" t="n">
+        <v>1</v>
+      </c>
+      <c r="N312" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>10</v>
+      </c>
+      <c r="E313" t="n">
+        <v>81</v>
+      </c>
+      <c r="F313" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" t="n">
+        <v>5</v>
+      </c>
+      <c r="I313" t="n">
+        <v>0</v>
+      </c>
+      <c r="J313" t="n">
+        <v>0</v>
+      </c>
+      <c r="K313" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L313" t="n">
+        <v>7</v>
+      </c>
+      <c r="M313" t="n">
+        <v>1</v>
+      </c>
+      <c r="N313" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="E314" t="n">
+        <v>84</v>
+      </c>
+      <c r="F314" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0</v>
+      </c>
+      <c r="H314" t="n">
+        <v>1</v>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L314" t="n">
+        <v>1</v>
+      </c>
+      <c r="M314" t="n">
+        <v>0</v>
+      </c>
+      <c r="N314" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>2026-10-16T05:03:20Z</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E315" t="n">
+        <v>86</v>
+      </c>
+      <c r="F315" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0</v>
+      </c>
+      <c r="H315" t="n">
+        <v>5</v>
+      </c>
+      <c r="I315" t="n">
+        <v>0</v>
+      </c>
+      <c r="J315" t="n">
+        <v>0</v>
+      </c>
+      <c r="K315" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="L315" t="n">
+        <v>1</v>
+      </c>
+      <c r="M315" t="n">
+        <v>0</v>
+      </c>
+      <c r="N315" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-16 13:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -13164,23 +13164,23 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>16.1</v>
+        <v>15.9</v>
       </c>
       <c r="E255" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>16.2</v>
+        <v>15.5</v>
       </c>
       <c r="G255" t="n">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="H255" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="I255" t="n">
         <v>0</v>
@@ -13189,7 +13189,7 @@
         <v>0</v>
       </c>
       <c r="K255" t="n">
-        <v>0.294</v>
+        <v>0.299</v>
       </c>
       <c r="L255" t="n">
         <v>5</v>
@@ -13214,7 +13214,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -13224,13 +13224,13 @@
         <v>40</v>
       </c>
       <c r="F256" t="n">
-        <v>17.6</v>
+        <v>16.9</v>
       </c>
       <c r="G256" t="n">
-        <v>478</v>
+        <v>496</v>
       </c>
       <c r="H256" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="I256" t="n">
         <v>0</v>
@@ -13239,7 +13239,7 @@
         <v>0</v>
       </c>
       <c r="K256" t="n">
-        <v>0.292</v>
+        <v>0.296</v>
       </c>
       <c r="L256" t="n">
         <v>5</v>
@@ -13264,23 +13264,23 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="E257" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F257" t="n">
-        <v>17.6</v>
+        <v>16.6</v>
       </c>
       <c r="G257" t="n">
-        <v>397</v>
+        <v>421</v>
       </c>
       <c r="H257" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="I257" t="n">
         <v>0</v>
@@ -13289,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="K257" t="n">
-        <v>0.29</v>
+        <v>0.294</v>
       </c>
       <c r="L257" t="n">
         <v>5</v>
@@ -13314,20 +13314,20 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>16.4</v>
+        <v>16.6</v>
       </c>
       <c r="E258" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F258" t="n">
-        <v>15.5</v>
+        <v>14.8</v>
       </c>
       <c r="G258" t="n">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="H258" t="n">
         <v>0</v>
@@ -13339,7 +13339,7 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
-        <v>0.288</v>
+        <v>0.292</v>
       </c>
       <c r="L258" t="n">
         <v>5</v>
@@ -13364,17 +13364,17 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>16</v>
+        <v>16.1</v>
       </c>
       <c r="E259" t="n">
         <v>35</v>
       </c>
       <c r="F259" t="n">
-        <v>14</v>
+        <v>14.4</v>
       </c>
       <c r="G259" t="n">
         <v>182</v>
@@ -13389,7 +13389,7 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
-        <v>0.287</v>
+        <v>0.291</v>
       </c>
       <c r="L259" t="n">
         <v>5</v>
@@ -13414,11 +13414,11 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="E260" t="n">
         <v>40</v>
@@ -13427,7 +13427,7 @@
         <v>9.4</v>
       </c>
       <c r="G260" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H260" t="n">
         <v>0</v>
@@ -13439,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
-        <v>0.287</v>
+        <v>0.291</v>
       </c>
       <c r="L260" t="n">
         <v>5</v>
@@ -13464,17 +13464,17 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="E261" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F261" t="n">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -13489,7 +13489,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>0.286</v>
+        <v>0.291</v>
       </c>
       <c r="L261" t="n">
         <v>5</v>
@@ -13514,17 +13514,17 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="E262" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F262" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.286</v>
+        <v>0.291</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,17 +13564,17 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="E263" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F263" t="n">
-        <v>10.1</v>
+        <v>9.4</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.286</v>
+        <v>0.291</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,23 +13614,23 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="E264" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F264" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
       </c>
       <c r="H264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.286</v>
+        <v>0.291</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,17 +13664,17 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6.8</v>
+        <v>6.7</v>
       </c>
       <c r="E265" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F265" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="G265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.286</v>
+        <v>0.291</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13714,23 +13714,23 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D266" t="n">
         <v>6.1</v>
       </c>
       <c r="E266" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F266" t="n">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
       </c>
       <c r="H266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I266" t="n">
         <v>0</v>
@@ -13739,7 +13739,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>0.286</v>
+        <v>0.291</v>
       </c>
       <c r="L266" t="n">
         <v>6</v>
@@ -13764,23 +13764,23 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="E267" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F267" t="n">
-        <v>5</v>
+        <v>7.2</v>
       </c>
       <c r="G267" t="n">
         <v>0</v>
       </c>
       <c r="H267" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -13789,7 +13789,7 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>0.286</v>
+        <v>0.291</v>
       </c>
       <c r="L267" t="n">
         <v>6</v>
@@ -13814,23 +13814,23 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>5.2</v>
+        <v>7</v>
       </c>
       <c r="E268" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="F268" t="n">
-        <v>9.4</v>
+        <v>7.9</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
       </c>
       <c r="H268" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -13839,7 +13839,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>0.286</v>
+        <v>0.291</v>
       </c>
       <c r="L268" t="n">
         <v>6</v>
@@ -13864,23 +13864,23 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>5</v>
+        <v>7.4</v>
       </c>
       <c r="E269" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="F269" t="n">
-        <v>9.699999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="G269" t="n">
         <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="I269" t="n">
         <v>0</v>
@@ -13889,7 +13889,7 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
-        <v>0.286</v>
+        <v>0.29</v>
       </c>
       <c r="L269" t="n">
         <v>6</v>
@@ -13914,14 +13914,14 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>4.8</v>
+        <v>7.7</v>
       </c>
       <c r="E270" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="F270" t="n">
         <v>8.300000000000001</v>
@@ -13930,7 +13930,7 @@
         <v>0</v>
       </c>
       <c r="H270" t="n">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="I270" t="n">
         <v>0</v>
@@ -13939,7 +13939,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>0.286</v>
+        <v>0.29</v>
       </c>
       <c r="L270" t="n">
         <v>6</v>
@@ -13964,23 +13964,23 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>4.8</v>
+        <v>7.8</v>
       </c>
       <c r="E271" t="n">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="F271" t="n">
-        <v>7.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G271" t="n">
         <v>0</v>
       </c>
       <c r="H271" t="n">
-        <v>26</v>
+        <v>100</v>
       </c>
       <c r="I271" t="n">
         <v>0</v>
@@ -13989,7 +13989,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>0.286</v>
+        <v>0.29</v>
       </c>
       <c r="L271" t="n">
         <v>6</v>
@@ -14014,17 +14014,17 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>5.1</v>
+        <v>8.1</v>
       </c>
       <c r="E272" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="F272" t="n">
-        <v>8.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
@@ -14039,7 +14039,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>0.286</v>
+        <v>0.29</v>
       </c>
       <c r="L272" t="n">
         <v>6</v>
@@ -14064,17 +14064,17 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E273" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F273" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
@@ -14089,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>0.286</v>
+        <v>0.29</v>
       </c>
       <c r="L273" t="n">
         <v>6</v>
@@ -14114,20 +14114,20 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>6.8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E274" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F274" t="n">
-        <v>11.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G274" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H274" t="n">
         <v>100</v>
@@ -14139,7 +14139,7 @@
         <v>0</v>
       </c>
       <c r="K274" t="n">
-        <v>0.286</v>
+        <v>0.29</v>
       </c>
       <c r="L274" t="n">
         <v>6</v>
@@ -14164,20 +14164,20 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>7.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E275" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F275" t="n">
-        <v>9.4</v>
+        <v>6.5</v>
       </c>
       <c r="G275" t="n">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="H275" t="n">
         <v>100</v>
@@ -14189,7 +14189,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>0.286</v>
+        <v>0.29</v>
       </c>
       <c r="L275" t="n">
         <v>6</v>
@@ -14214,23 +14214,23 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>8.199999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="E276" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="F276" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="G276" t="n">
-        <v>51</v>
+        <v>190</v>
       </c>
       <c r="H276" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="I276" t="n">
         <v>0</v>
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>0.286</v>
+        <v>0.289</v>
       </c>
       <c r="L276" t="n">
         <v>6</v>
@@ -14264,23 +14264,23 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>10.2</v>
+        <v>13.5</v>
       </c>
       <c r="E277" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="F277" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="G277" t="n">
-        <v>153</v>
+        <v>342</v>
       </c>
       <c r="H277" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="I277" t="n">
         <v>0</v>
@@ -14289,7 +14289,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>0.285</v>
+        <v>0.289</v>
       </c>
       <c r="L277" t="n">
         <v>6</v>
@@ -14314,23 +14314,23 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>14</v>
+        <v>15.7</v>
       </c>
       <c r="E278" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F278" t="n">
-        <v>10.1</v>
+        <v>10.8</v>
       </c>
       <c r="G278" t="n">
-        <v>403</v>
+        <v>449</v>
       </c>
       <c r="H278" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="I278" t="n">
         <v>0</v>
@@ -14339,7 +14339,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>0.284</v>
+        <v>0.287</v>
       </c>
       <c r="L278" t="n">
         <v>6</v>
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>16</v>
+        <v>16.8</v>
       </c>
       <c r="E279" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F279" t="n">
-        <v>10.4</v>
+        <v>14</v>
       </c>
       <c r="G279" t="n">
-        <v>539</v>
+        <v>489</v>
       </c>
       <c r="H279" t="n">
-        <v>13</v>
+        <v>99</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.283</v>
+        <v>0.286</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,7 +14414,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -14424,13 +14424,13 @@
         <v>34</v>
       </c>
       <c r="F280" t="n">
-        <v>13</v>
+        <v>13.3</v>
       </c>
       <c r="G280" t="n">
-        <v>505</v>
+        <v>251</v>
       </c>
       <c r="H280" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I280" t="n">
         <v>0</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.283</v>
+        <v>0.284</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,20 +14464,20 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>16.4</v>
+        <v>16.9</v>
       </c>
       <c r="E281" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F281" t="n">
-        <v>12.2</v>
+        <v>12.6</v>
       </c>
       <c r="G281" t="n">
-        <v>194</v>
+        <v>161</v>
       </c>
       <c r="H281" t="n">
         <v>100</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,20 +14514,20 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>16.2</v>
+        <v>16.5</v>
       </c>
       <c r="E282" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F282" t="n">
-        <v>9</v>
+        <v>7.9</v>
       </c>
       <c r="G282" t="n">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="H282" t="n">
         <v>100</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,23 +14564,23 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D283" t="n">
         <v>15.8</v>
       </c>
       <c r="E283" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F283" t="n">
         <v>4.7</v>
       </c>
       <c r="G283" t="n">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="H283" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -14614,23 +14614,23 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>13.9</v>
+        <v>14.9</v>
       </c>
       <c r="E284" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F284" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
       <c r="G284" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="H284" t="n">
-        <v>32</v>
+        <v>100</v>
       </c>
       <c r="I284" t="n">
         <v>0</v>
@@ -14664,23 +14664,23 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>12.1</v>
+        <v>13.1</v>
       </c>
       <c r="E285" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F285" t="n">
-        <v>4.7</v>
+        <v>10.1</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
       </c>
       <c r="H285" t="n">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -14714,23 +14714,23 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="E286" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F286" t="n">
-        <v>5.4</v>
+        <v>9</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14764,23 +14764,23 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="E287" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F287" t="n">
-        <v>3.6</v>
+        <v>9</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -14814,17 +14814,17 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>9.9</v>
+        <v>10.5</v>
       </c>
       <c r="E288" t="n">
         <v>55</v>
       </c>
       <c r="F288" t="n">
-        <v>6.5</v>
+        <v>10.8</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
@@ -14864,23 +14864,23 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>8.6</v>
+        <v>9.4</v>
       </c>
       <c r="E289" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F289" t="n">
-        <v>4.3</v>
+        <v>9.4</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
       </c>
       <c r="H289" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I289" t="n">
         <v>0</v>
@@ -14914,17 +14914,17 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>8.300000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E290" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F290" t="n">
-        <v>4.7</v>
+        <v>7.6</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
@@ -14964,17 +14964,17 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E291" t="n">
         <v>59</v>
       </c>
       <c r="F291" t="n">
-        <v>7.6</v>
+        <v>7.9</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
@@ -15014,23 +15014,23 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="E292" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F292" t="n">
-        <v>6.8</v>
+        <v>4.3</v>
       </c>
       <c r="G292" t="n">
         <v>0</v>
       </c>
       <c r="H292" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I292" t="n">
         <v>0</v>
@@ -15064,17 +15064,17 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>9.4</v>
+        <v>9.9</v>
       </c>
       <c r="E293" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F293" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G293" t="n">
         <v>0</v>
@@ -15114,17 +15114,17 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>9.9</v>
+        <v>10</v>
       </c>
       <c r="E294" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F294" t="n">
-        <v>8.6</v>
+        <v>6.5</v>
       </c>
       <c r="G294" t="n">
         <v>0</v>
@@ -15139,7 +15139,7 @@
         <v>0</v>
       </c>
       <c r="K294" t="n">
-        <v>0.281</v>
+        <v>0.28</v>
       </c>
       <c r="L294" t="n">
         <v>7</v>
@@ -15164,23 +15164,23 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="E295" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F295" t="n">
-        <v>8.300000000000001</v>
+        <v>6.5</v>
       </c>
       <c r="G295" t="n">
         <v>0</v>
       </c>
       <c r="H295" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I295" t="n">
         <v>0</v>
@@ -15214,17 +15214,17 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>9.699999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="E296" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F296" t="n">
-        <v>10.8</v>
+        <v>11.5</v>
       </c>
       <c r="G296" t="n">
         <v>0</v>
@@ -15264,17 +15264,17 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E297" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F297" t="n">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="G297" t="n">
         <v>0</v>
@@ -15314,23 +15314,23 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>9.699999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="E298" t="n">
         <v>54</v>
       </c>
       <c r="F298" t="n">
-        <v>6.8</v>
+        <v>3.6</v>
       </c>
       <c r="G298" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H298" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I298" t="n">
         <v>0</v>
@@ -15364,23 +15364,23 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="E299" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F299" t="n">
-        <v>7.6</v>
+        <v>6.8</v>
       </c>
       <c r="G299" t="n">
-        <v>166</v>
+        <v>63</v>
       </c>
       <c r="H299" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I299" t="n">
         <v>0</v>
@@ -15414,23 +15414,23 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>13.6</v>
+        <v>12.8</v>
       </c>
       <c r="E300" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F300" t="n">
-        <v>9.4</v>
+        <v>5.4</v>
       </c>
       <c r="G300" t="n">
-        <v>341</v>
+        <v>251</v>
       </c>
       <c r="H300" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="I300" t="n">
         <v>0</v>
@@ -15464,23 +15464,23 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>15.6</v>
+        <v>14.5</v>
       </c>
       <c r="E301" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F301" t="n">
-        <v>8.800000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G301" t="n">
-        <v>445</v>
+        <v>157</v>
       </c>
       <c r="H301" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="I301" t="n">
         <v>0</v>
@@ -15514,23 +15514,23 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>17.1</v>
+        <v>14.9</v>
       </c>
       <c r="E302" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F302" t="n">
-        <v>8.300000000000001</v>
+        <v>5.4</v>
       </c>
       <c r="G302" t="n">
-        <v>500</v>
+        <v>76</v>
       </c>
       <c r="H302" t="n">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="I302" t="n">
         <v>0</v>
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>17.4</v>
+        <v>16.4</v>
       </c>
       <c r="E303" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="F303" t="n">
-        <v>7.8</v>
+        <v>4.7</v>
       </c>
       <c r="G303" t="n">
-        <v>447.5</v>
+        <v>334</v>
       </c>
       <c r="H303" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15614,23 +15614,23 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>17.5</v>
+        <v>18.5</v>
       </c>
       <c r="E304" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="F304" t="n">
-        <v>6.6</v>
+        <v>5.8</v>
       </c>
       <c r="G304" t="n">
-        <v>496</v>
+        <v>537</v>
       </c>
       <c r="H304" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -15664,23 +15664,23 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>17.6</v>
+        <v>19.5</v>
       </c>
       <c r="E305" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="F305" t="n">
         <v>6.5</v>
       </c>
       <c r="G305" t="n">
-        <v>386</v>
+        <v>451</v>
       </c>
       <c r="H305" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -15689,7 +15689,7 @@
         <v>0</v>
       </c>
       <c r="K305" t="n">
-        <v>0.271</v>
+        <v>0.27</v>
       </c>
       <c r="L305" t="n">
         <v>7</v>
@@ -15714,23 +15714,23 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>17.5</v>
+        <v>19.8</v>
       </c>
       <c r="E306" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="F306" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="G306" t="n">
-        <v>295</v>
+        <v>323</v>
       </c>
       <c r="H306" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>16.3</v>
+        <v>18.7</v>
       </c>
       <c r="E307" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="F307" t="n">
-        <v>5.6</v>
+        <v>6.1</v>
       </c>
       <c r="G307" t="n">
-        <v>157</v>
+        <v>163.3</v>
       </c>
       <c r="H307" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15789,7 +15789,7 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0.269</v>
+        <v>0.268</v>
       </c>
       <c r="L307" t="n">
         <v>7</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>14</v>
+        <v>15.7</v>
       </c>
       <c r="E308" t="n">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="F308" t="n">
-        <v>6.5</v>
+        <v>4.7</v>
       </c>
       <c r="G308" t="n">
-        <v>28</v>
+        <v>29.5</v>
       </c>
       <c r="H308" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15839,7 +15839,7 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0.269</v>
+        <v>0.268</v>
       </c>
       <c r="L308" t="n">
         <v>7</v>
@@ -15864,23 +15864,23 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>13.1</v>
+        <v>13.3</v>
       </c>
       <c r="E309" t="n">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="F309" t="n">
-        <v>7.1</v>
+        <v>4.7</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15914,7 +15914,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -15924,13 +15924,13 @@
         <v>71</v>
       </c>
       <c r="F310" t="n">
-        <v>6.5</v>
+        <v>1.8</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15964,23 +15964,23 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="E311" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F311" t="n">
-        <v>5.8</v>
+        <v>0.7</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I311" t="n">
         <v>0</v>
@@ -16014,23 +16014,23 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>10.4</v>
+        <v>10.7</v>
       </c>
       <c r="E312" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F312" t="n">
-        <v>3.8</v>
+        <v>2</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
       </c>
       <c r="H312" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="I312" t="n">
         <v>0</v>
@@ -16064,14 +16064,14 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>10</v>
+        <v>10.1</v>
       </c>
       <c r="E313" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F313" t="n">
         <v>3.9</v>
@@ -16080,7 +16080,7 @@
         <v>0</v>
       </c>
       <c r="H313" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="I313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.268</v>
+        <v>0.269</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,23 +16114,23 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E314" t="n">
         <v>84</v>
       </c>
       <c r="F314" t="n">
-        <v>4.3</v>
+        <v>4.9</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
       </c>
       <c r="H314" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I314" t="n">
         <v>0</v>
@@ -16139,7 +16139,7 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0.268</v>
+        <v>0.269</v>
       </c>
       <c r="L314" t="n">
         <v>1</v>
@@ -16164,23 +16164,23 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-16T05:03:20Z</t>
+          <t>2026-10-16T11:03:42Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>9.199999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="E315" t="n">
         <v>86</v>
       </c>
       <c r="F315" t="n">
-        <v>4.2</v>
+        <v>5.6</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
       </c>
       <c r="H315" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I315" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-16 19:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -13464,17 +13464,17 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>11.7</v>
+        <v>11.3</v>
       </c>
       <c r="E261" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="F261" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -13489,7 +13489,7 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L261" t="n">
         <v>5</v>
@@ -13514,17 +13514,17 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>9.9</v>
+        <v>9.5</v>
       </c>
       <c r="E262" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F262" t="n">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
@@ -13539,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L262" t="n">
         <v>5</v>
@@ -13564,17 +13564,17 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>8.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E263" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F263" t="n">
-        <v>9.4</v>
+        <v>9</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
@@ -13589,7 +13589,7 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L263" t="n">
         <v>5</v>
@@ -13614,23 +13614,23 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="E264" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F264" t="n">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
       </c>
       <c r="H264" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="I264" t="n">
         <v>0</v>
@@ -13639,7 +13639,7 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L264" t="n">
         <v>5</v>
@@ -13664,14 +13664,14 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="E265" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F265" t="n">
         <v>9.4</v>
@@ -13680,7 +13680,7 @@
         <v>0</v>
       </c>
       <c r="H265" t="n">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="I265" t="n">
         <v>0</v>
@@ -13689,7 +13689,7 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L265" t="n">
         <v>5</v>
@@ -13714,23 +13714,23 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>6.1</v>
+        <v>6.7</v>
       </c>
       <c r="E266" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F266" t="n">
-        <v>9.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
       </c>
       <c r="H266" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="I266" t="n">
         <v>0</v>
@@ -13739,7 +13739,7 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L266" t="n">
         <v>6</v>
@@ -13764,23 +13764,23 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>6.3</v>
+        <v>6.2</v>
       </c>
       <c r="E267" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F267" t="n">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="G267" t="n">
         <v>0</v>
       </c>
       <c r="H267" t="n">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -13789,7 +13789,7 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L267" t="n">
         <v>6</v>
@@ -13814,23 +13814,23 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>7</v>
+        <v>6.6</v>
       </c>
       <c r="E268" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="F268" t="n">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
       </c>
       <c r="H268" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -13839,7 +13839,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>0.291</v>
+        <v>0.292</v>
       </c>
       <c r="L268" t="n">
         <v>6</v>
@@ -13864,23 +13864,23 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="E269" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F269" t="n">
-        <v>7.6</v>
+        <v>6.8</v>
       </c>
       <c r="G269" t="n">
         <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I269" t="n">
         <v>0</v>
@@ -13889,7 +13889,7 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
-        <v>0.29</v>
+        <v>0.292</v>
       </c>
       <c r="L269" t="n">
         <v>6</v>
@@ -13914,23 +13914,23 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
       <c r="E270" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F270" t="n">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="G270" t="n">
         <v>0</v>
       </c>
       <c r="H270" t="n">
-        <v>55</v>
+        <v>99</v>
       </c>
       <c r="I270" t="n">
         <v>0</v>
@@ -13939,7 +13939,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>0.29</v>
+        <v>0.292</v>
       </c>
       <c r="L270" t="n">
         <v>6</v>
@@ -13964,23 +13964,23 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>7.8</v>
+        <v>7.2</v>
       </c>
       <c r="E271" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F271" t="n">
-        <v>8.300000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="G271" t="n">
         <v>0</v>
       </c>
       <c r="H271" t="n">
-        <v>100</v>
+        <v>37</v>
       </c>
       <c r="I271" t="n">
         <v>0</v>
@@ -13989,7 +13989,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>0.29</v>
+        <v>0.292</v>
       </c>
       <c r="L271" t="n">
         <v>6</v>
@@ -14014,23 +14014,23 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>8.1</v>
+        <v>6.6</v>
       </c>
       <c r="E272" t="n">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="F272" t="n">
-        <v>9.4</v>
+        <v>9</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
       </c>
       <c r="H272" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="I272" t="n">
         <v>0</v>
@@ -14039,7 +14039,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>0.29</v>
+        <v>0.291</v>
       </c>
       <c r="L272" t="n">
         <v>6</v>
@@ -14064,17 +14064,17 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>8.199999999999999</v>
+        <v>6.7</v>
       </c>
       <c r="E273" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="F273" t="n">
-        <v>10.4</v>
+        <v>11.5</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
@@ -14089,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>0.29</v>
+        <v>0.291</v>
       </c>
       <c r="L273" t="n">
         <v>6</v>
@@ -14114,20 +14114,20 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>8.199999999999999</v>
+        <v>6.9</v>
       </c>
       <c r="E274" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="F274" t="n">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="G274" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H274" t="n">
         <v>100</v>
@@ -14139,7 +14139,7 @@
         <v>0</v>
       </c>
       <c r="K274" t="n">
-        <v>0.29</v>
+        <v>0.291</v>
       </c>
       <c r="L274" t="n">
         <v>6</v>
@@ -14164,23 +14164,23 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>8.800000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="E275" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F275" t="n">
-        <v>6.5</v>
+        <v>10.1</v>
       </c>
       <c r="G275" t="n">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="H275" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="I275" t="n">
         <v>0</v>
@@ -14189,7 +14189,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>0.29</v>
+        <v>0.291</v>
       </c>
       <c r="L275" t="n">
         <v>6</v>
@@ -14214,23 +14214,23 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>10.6</v>
+        <v>10.5</v>
       </c>
       <c r="E276" t="n">
         <v>54</v>
       </c>
       <c r="F276" t="n">
-        <v>6.1</v>
+        <v>10.1</v>
       </c>
       <c r="G276" t="n">
-        <v>190</v>
+        <v>232</v>
       </c>
       <c r="H276" t="n">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="I276" t="n">
         <v>0</v>
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>0.289</v>
+        <v>0.29</v>
       </c>
       <c r="L276" t="n">
         <v>6</v>
@@ -14264,23 +14264,23 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>13.5</v>
+        <v>13.1</v>
       </c>
       <c r="E277" t="n">
         <v>45</v>
       </c>
       <c r="F277" t="n">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G277" t="n">
-        <v>342</v>
+        <v>407</v>
       </c>
       <c r="H277" t="n">
-        <v>95</v>
+        <v>63</v>
       </c>
       <c r="I277" t="n">
         <v>0</v>
@@ -14289,7 +14289,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>0.289</v>
+        <v>0.29</v>
       </c>
       <c r="L277" t="n">
         <v>6</v>
@@ -14314,23 +14314,23 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>15.7</v>
+        <v>15.5</v>
       </c>
       <c r="E278" t="n">
         <v>39</v>
       </c>
       <c r="F278" t="n">
-        <v>10.8</v>
+        <v>11.5</v>
       </c>
       <c r="G278" t="n">
-        <v>449</v>
+        <v>495</v>
       </c>
       <c r="H278" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I278" t="n">
         <v>0</v>
@@ -14339,7 +14339,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L278" t="n">
         <v>6</v>
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>16.8</v>
+        <v>16.7</v>
       </c>
       <c r="E279" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F279" t="n">
-        <v>14</v>
+        <v>11.9</v>
       </c>
       <c r="G279" t="n">
-        <v>489</v>
+        <v>555</v>
       </c>
       <c r="H279" t="n">
-        <v>99</v>
+        <v>25</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.286</v>
+        <v>0.287</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,23 +14414,23 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>16.9</v>
+        <v>17.3</v>
       </c>
       <c r="E280" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F280" t="n">
-        <v>13.3</v>
+        <v>11.2</v>
       </c>
       <c r="G280" t="n">
-        <v>251</v>
+        <v>458</v>
       </c>
       <c r="H280" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="I280" t="n">
         <v>0</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.284</v>
+        <v>0.286</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,7 +14464,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -14474,10 +14474,10 @@
         <v>33</v>
       </c>
       <c r="F281" t="n">
-        <v>12.6</v>
+        <v>11.2</v>
       </c>
       <c r="G281" t="n">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="H281" t="n">
         <v>100</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.283</v>
+        <v>0.284</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,23 +14514,23 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>16.5</v>
+        <v>16.7</v>
       </c>
       <c r="E282" t="n">
         <v>33</v>
       </c>
       <c r="F282" t="n">
-        <v>7.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G282" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="H282" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="I282" t="n">
         <v>0</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,20 +14564,20 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>15.8</v>
+        <v>16.7</v>
       </c>
       <c r="E283" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F283" t="n">
-        <v>4.7</v>
+        <v>10.1</v>
       </c>
       <c r="G283" t="n">
-        <v>34</v>
+        <v>118</v>
       </c>
       <c r="H283" t="n">
         <v>100</v>
@@ -14589,7 +14589,7 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0.281</v>
+        <v>0.283</v>
       </c>
       <c r="L283" t="n">
         <v>6</v>
@@ -14614,20 +14614,20 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>14.9</v>
+        <v>14.3</v>
       </c>
       <c r="E284" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F284" t="n">
-        <v>2.9</v>
+        <v>10.4</v>
       </c>
       <c r="G284" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H284" t="n">
         <v>100</v>
@@ -14639,7 +14639,7 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0.281</v>
+        <v>0.283</v>
       </c>
       <c r="L284" t="n">
         <v>6</v>
@@ -14664,23 +14664,23 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>13.1</v>
+        <v>13.3</v>
       </c>
       <c r="E285" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F285" t="n">
-        <v>10.1</v>
+        <v>10.8</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
       </c>
       <c r="H285" t="n">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -14689,7 +14689,7 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
-        <v>0.281</v>
+        <v>0.283</v>
       </c>
       <c r="L285" t="n">
         <v>6</v>
@@ -14714,23 +14714,23 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>12</v>
+        <v>12.9</v>
       </c>
       <c r="E286" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F286" t="n">
-        <v>9</v>
+        <v>10.4</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14739,7 +14739,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L286" t="n">
         <v>6</v>
@@ -14764,23 +14764,23 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>11.4</v>
+        <v>12.4</v>
       </c>
       <c r="E287" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F287" t="n">
-        <v>9</v>
+        <v>13.3</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L287" t="n">
         <v>6</v>
@@ -14814,14 +14814,14 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>10.5</v>
+        <v>11.8</v>
       </c>
       <c r="E288" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F288" t="n">
         <v>10.8</v>
@@ -14830,7 +14830,7 @@
         <v>0</v>
       </c>
       <c r="H288" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,23 +14864,23 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>9.4</v>
+        <v>11.5</v>
       </c>
       <c r="E289" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="F289" t="n">
-        <v>9.4</v>
+        <v>9</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
       </c>
       <c r="H289" t="n">
-        <v>14</v>
+        <v>100</v>
       </c>
       <c r="I289" t="n">
         <v>0</v>
@@ -14889,7 +14889,7 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L289" t="n">
         <v>6</v>
@@ -14914,17 +14914,17 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>9.300000000000001</v>
+        <v>11.6</v>
       </c>
       <c r="E290" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="F290" t="n">
-        <v>7.6</v>
+        <v>6.5</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
@@ -14939,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="K290" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L290" t="n">
         <v>7</v>
@@ -14964,17 +14964,17 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>9.800000000000001</v>
+        <v>11.6</v>
       </c>
       <c r="E291" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="F291" t="n">
-        <v>7.9</v>
+        <v>8.6</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L291" t="n">
         <v>7</v>
@@ -15014,23 +15014,23 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>10</v>
+        <v>11.6</v>
       </c>
       <c r="E292" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="F292" t="n">
-        <v>4.3</v>
+        <v>7.9</v>
       </c>
       <c r="G292" t="n">
         <v>0</v>
       </c>
       <c r="H292" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="I292" t="n">
         <v>0</v>
@@ -15039,7 +15039,7 @@
         <v>0</v>
       </c>
       <c r="K292" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L292" t="n">
         <v>7</v>
@@ -15064,17 +15064,17 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>9.9</v>
+        <v>11.3</v>
       </c>
       <c r="E293" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F293" t="n">
-        <v>4</v>
+        <v>6.1</v>
       </c>
       <c r="G293" t="n">
         <v>0</v>
@@ -15089,7 +15089,7 @@
         <v>0</v>
       </c>
       <c r="K293" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L293" t="n">
         <v>7</v>
@@ -15114,17 +15114,17 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>10</v>
+        <v>11.4</v>
       </c>
       <c r="E294" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F294" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="G294" t="n">
         <v>0</v>
@@ -15139,7 +15139,7 @@
         <v>0</v>
       </c>
       <c r="K294" t="n">
-        <v>0.28</v>
+        <v>0.282</v>
       </c>
       <c r="L294" t="n">
         <v>7</v>
@@ -15164,17 +15164,17 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>10.4</v>
+        <v>11.3</v>
       </c>
       <c r="E295" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F295" t="n">
-        <v>6.5</v>
+        <v>2.9</v>
       </c>
       <c r="G295" t="n">
         <v>0</v>
@@ -15189,7 +15189,7 @@
         <v>0</v>
       </c>
       <c r="K295" t="n">
-        <v>0.28</v>
+        <v>0.281</v>
       </c>
       <c r="L295" t="n">
         <v>7</v>
@@ -15214,17 +15214,17 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>10.6</v>
+        <v>11.3</v>
       </c>
       <c r="E296" t="n">
         <v>51</v>
       </c>
       <c r="F296" t="n">
-        <v>11.5</v>
+        <v>3.2</v>
       </c>
       <c r="G296" t="n">
         <v>0</v>
@@ -15239,7 +15239,7 @@
         <v>0</v>
       </c>
       <c r="K296" t="n">
-        <v>0.28</v>
+        <v>0.281</v>
       </c>
       <c r="L296" t="n">
         <v>7</v>
@@ -15264,17 +15264,17 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>9.699999999999999</v>
+        <v>11.2</v>
       </c>
       <c r="E297" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F297" t="n">
-        <v>5.8</v>
+        <v>4</v>
       </c>
       <c r="G297" t="n">
         <v>0</v>
@@ -15289,7 +15289,7 @@
         <v>0</v>
       </c>
       <c r="K297" t="n">
-        <v>0.28</v>
+        <v>0.281</v>
       </c>
       <c r="L297" t="n">
         <v>7</v>
@@ -15314,20 +15314,20 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>9.9</v>
+        <v>11.2</v>
       </c>
       <c r="E298" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F298" t="n">
-        <v>3.6</v>
+        <v>2.5</v>
       </c>
       <c r="G298" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H298" t="n">
         <v>100</v>
@@ -15339,7 +15339,7 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
-        <v>0.28</v>
+        <v>0.281</v>
       </c>
       <c r="L298" t="n">
         <v>7</v>
@@ -15364,20 +15364,20 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>10.6</v>
+        <v>12.1</v>
       </c>
       <c r="E299" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="F299" t="n">
-        <v>6.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G299" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="H299" t="n">
         <v>100</v>
@@ -15389,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="K299" t="n">
-        <v>0.28</v>
+        <v>0.281</v>
       </c>
       <c r="L299" t="n">
         <v>7</v>
@@ -15414,23 +15414,23 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>12.8</v>
+        <v>12.6</v>
       </c>
       <c r="E300" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F300" t="n">
-        <v>5.4</v>
+        <v>7.9</v>
       </c>
       <c r="G300" t="n">
-        <v>251</v>
+        <v>56</v>
       </c>
       <c r="H300" t="n">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="I300" t="n">
         <v>0</v>
@@ -15439,7 +15439,7 @@
         <v>0</v>
       </c>
       <c r="K300" t="n">
-        <v>0.279</v>
+        <v>0.28</v>
       </c>
       <c r="L300" t="n">
         <v>7</v>
@@ -15464,20 +15464,20 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>14.5</v>
+        <v>13.2</v>
       </c>
       <c r="E301" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="F301" t="n">
-        <v>7.6</v>
+        <v>3.6</v>
       </c>
       <c r="G301" t="n">
-        <v>157</v>
+        <v>90</v>
       </c>
       <c r="H301" t="n">
         <v>100</v>
@@ -15489,7 +15489,7 @@
         <v>0</v>
       </c>
       <c r="K301" t="n">
-        <v>0.278</v>
+        <v>0.279</v>
       </c>
       <c r="L301" t="n">
         <v>7</v>
@@ -15514,23 +15514,23 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D302" t="n">
         <v>14.9</v>
       </c>
       <c r="E302" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F302" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="G302" t="n">
-        <v>76</v>
+        <v>304</v>
       </c>
       <c r="H302" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I302" t="n">
         <v>0</v>
@@ -15539,7 +15539,7 @@
         <v>0</v>
       </c>
       <c r="K302" t="n">
-        <v>0.276</v>
+        <v>0.278</v>
       </c>
       <c r="L302" t="n">
         <v>7</v>
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>16.4</v>
+        <v>17.4</v>
       </c>
       <c r="E303" t="n">
         <v>36</v>
       </c>
       <c r="F303" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="G303" t="n">
-        <v>334</v>
+        <v>556</v>
       </c>
       <c r="H303" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15589,7 +15589,7 @@
         <v>0</v>
       </c>
       <c r="K303" t="n">
-        <v>0.274</v>
+        <v>0.276</v>
       </c>
       <c r="L303" t="n">
         <v>7</v>
@@ -15614,20 +15614,20 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>18.5</v>
+        <v>19.3</v>
       </c>
       <c r="E304" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F304" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="G304" t="n">
-        <v>537</v>
+        <v>526</v>
       </c>
       <c r="H304" t="n">
         <v>0</v>
@@ -15639,7 +15639,7 @@
         <v>0</v>
       </c>
       <c r="K304" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="L304" t="n">
         <v>7</v>
@@ -15664,20 +15664,20 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>19.5</v>
+        <v>20.1</v>
       </c>
       <c r="E305" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F305" t="n">
-        <v>6.5</v>
+        <v>7.2</v>
       </c>
       <c r="G305" t="n">
-        <v>451</v>
+        <v>443</v>
       </c>
       <c r="H305" t="n">
         <v>0</v>
@@ -15689,7 +15689,7 @@
         <v>0</v>
       </c>
       <c r="K305" t="n">
-        <v>0.27</v>
+        <v>0.272</v>
       </c>
       <c r="L305" t="n">
         <v>7</v>
@@ -15714,20 +15714,20 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>19.8</v>
+        <v>20.3</v>
       </c>
       <c r="E306" t="n">
         <v>26</v>
       </c>
       <c r="F306" t="n">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="G306" t="n">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="H306" t="n">
         <v>0</v>
@@ -15739,7 +15739,7 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>0.269</v>
+        <v>0.271</v>
       </c>
       <c r="L306" t="n">
         <v>7</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>18.7</v>
+        <v>19.9</v>
       </c>
       <c r="E307" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="F307" t="n">
-        <v>6.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G307" t="n">
-        <v>163.3</v>
+        <v>165</v>
       </c>
       <c r="H307" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15789,7 +15789,7 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0.268</v>
+        <v>0.27</v>
       </c>
       <c r="L307" t="n">
         <v>7</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>15.7</v>
+        <v>17.6</v>
       </c>
       <c r="E308" t="n">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F308" t="n">
-        <v>4.7</v>
+        <v>6.8</v>
       </c>
       <c r="G308" t="n">
-        <v>29.5</v>
+        <v>31</v>
       </c>
       <c r="H308" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15839,7 +15839,7 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0.268</v>
+        <v>0.27</v>
       </c>
       <c r="L308" t="n">
         <v>7</v>
@@ -15864,23 +15864,23 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>13.3</v>
+        <v>15</v>
       </c>
       <c r="E309" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="F309" t="n">
-        <v>4.7</v>
+        <v>7.2</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>0.268</v>
+        <v>0.27</v>
       </c>
       <c r="L309" t="n">
         <v>7</v>
@@ -15914,23 +15914,23 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>12.1</v>
+        <v>13.2</v>
       </c>
       <c r="E310" t="n">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="F310" t="n">
-        <v>1.8</v>
+        <v>7.6</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15939,7 +15939,7 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>0.268</v>
+        <v>0.27</v>
       </c>
       <c r="L310" t="n">
         <v>7</v>
@@ -15964,23 +15964,23 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="E311" t="n">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="F311" t="n">
-        <v>0.7</v>
+        <v>4</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="I311" t="n">
         <v>0</v>
@@ -15989,7 +15989,7 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>0.268</v>
+        <v>0.271</v>
       </c>
       <c r="L311" t="n">
         <v>7</v>
@@ -16014,23 +16014,23 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="E312" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="F312" t="n">
-        <v>2</v>
+        <v>3.6</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
       </c>
       <c r="H312" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="I312" t="n">
         <v>0</v>
@@ -16039,7 +16039,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0.268</v>
+        <v>0.271</v>
       </c>
       <c r="L312" t="n">
         <v>7</v>
@@ -16064,23 +16064,23 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D313" t="n">
         <v>10.1</v>
       </c>
       <c r="E313" t="n">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="F313" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
       </c>
       <c r="H313" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="I313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.269</v>
+        <v>0.271</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,17 +16114,17 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="E314" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="F314" t="n">
-        <v>4.9</v>
+        <v>3.6</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -16139,7 +16139,7 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0.269</v>
+        <v>0.271</v>
       </c>
       <c r="L314" t="n">
         <v>1</v>
@@ -16164,24 +16164,24 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-16T11:03:42Z</t>
+          <t>2026-10-16T17:03:41Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>9.5</v>
+        <v>8.4</v>
       </c>
       <c r="E315" t="n">
+        <v>60</v>
+      </c>
+      <c r="F315" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0</v>
+      </c>
+      <c r="H315" t="n">
         <v>86</v>
       </c>
-      <c r="F315" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="G315" t="n">
-        <v>0</v>
-      </c>
-      <c r="H315" t="n">
-        <v>2</v>
-      </c>
       <c r="I315" t="n">
         <v>0</v>
       </c>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0.269</v>
+        <v>0.271</v>
       </c>
       <c r="L315" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
prognoza biciklista (zvanicna): 2026-10-17 01:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -3014,7 +3014,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -13764,23 +13764,23 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="E267" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F267" t="n">
-        <v>7.9</v>
+        <v>9.4</v>
       </c>
       <c r="G267" t="n">
         <v>0</v>
       </c>
       <c r="H267" t="n">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -13789,7 +13789,7 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
-        <v>0.292</v>
+        <v>0.289</v>
       </c>
       <c r="L267" t="n">
         <v>6</v>
@@ -13814,23 +13814,23 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="E268" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F268" t="n">
-        <v>8.6</v>
+        <v>9.4</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
       </c>
       <c r="H268" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -13839,7 +13839,7 @@
         <v>0</v>
       </c>
       <c r="K268" t="n">
-        <v>0.292</v>
+        <v>0.289</v>
       </c>
       <c r="L268" t="n">
         <v>6</v>
@@ -13864,23 +13864,23 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>7.1</v>
+        <v>6.3</v>
       </c>
       <c r="E269" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F269" t="n">
-        <v>6.8</v>
+        <v>7.6</v>
       </c>
       <c r="G269" t="n">
         <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I269" t="n">
         <v>0</v>
@@ -13889,7 +13889,7 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
-        <v>0.292</v>
+        <v>0.289</v>
       </c>
       <c r="L269" t="n">
         <v>6</v>
@@ -13914,14 +13914,14 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>7.3</v>
+        <v>6.7</v>
       </c>
       <c r="E270" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F270" t="n">
         <v>7.9</v>
@@ -13930,7 +13930,7 @@
         <v>0</v>
       </c>
       <c r="H270" t="n">
-        <v>99</v>
+        <v>53</v>
       </c>
       <c r="I270" t="n">
         <v>0</v>
@@ -13939,7 +13939,7 @@
         <v>0</v>
       </c>
       <c r="K270" t="n">
-        <v>0.292</v>
+        <v>0.289</v>
       </c>
       <c r="L270" t="n">
         <v>6</v>
@@ -13964,23 +13964,23 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>7.2</v>
+        <v>6.5</v>
       </c>
       <c r="E271" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F271" t="n">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="G271" t="n">
         <v>0</v>
       </c>
       <c r="H271" t="n">
-        <v>37</v>
+        <v>88</v>
       </c>
       <c r="I271" t="n">
         <v>0</v>
@@ -13989,7 +13989,7 @@
         <v>0</v>
       </c>
       <c r="K271" t="n">
-        <v>0.292</v>
+        <v>0.289</v>
       </c>
       <c r="L271" t="n">
         <v>6</v>
@@ -14014,23 +14014,23 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="E272" t="n">
         <v>73</v>
       </c>
       <c r="F272" t="n">
-        <v>9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
       </c>
       <c r="H272" t="n">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="I272" t="n">
         <v>0</v>
@@ -14039,7 +14039,7 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>0.291</v>
+        <v>0.289</v>
       </c>
       <c r="L272" t="n">
         <v>6</v>
@@ -14064,23 +14064,23 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>6.7</v>
+        <v>5.9</v>
       </c>
       <c r="E273" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F273" t="n">
-        <v>11.5</v>
+        <v>11.2</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
       </c>
       <c r="H273" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="I273" t="n">
         <v>0</v>
@@ -14089,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>0.291</v>
+        <v>0.289</v>
       </c>
       <c r="L273" t="n">
         <v>6</v>
@@ -14114,11 +14114,11 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="E274" t="n">
         <v>71</v>
@@ -14127,7 +14127,7 @@
         <v>9.4</v>
       </c>
       <c r="G274" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="H274" t="n">
         <v>100</v>
@@ -14139,7 +14139,7 @@
         <v>0</v>
       </c>
       <c r="K274" t="n">
-        <v>0.291</v>
+        <v>0.289</v>
       </c>
       <c r="L274" t="n">
         <v>6</v>
@@ -14164,23 +14164,23 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>7.9</v>
+        <v>8</v>
       </c>
       <c r="E275" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F275" t="n">
         <v>10.1</v>
       </c>
       <c r="G275" t="n">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="H275" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="I275" t="n">
         <v>0</v>
@@ -14189,7 +14189,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>0.291</v>
+        <v>0.288</v>
       </c>
       <c r="L275" t="n">
         <v>6</v>
@@ -14214,23 +14214,23 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>10.5</v>
+        <v>9.5</v>
       </c>
       <c r="E276" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F276" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G276" t="n">
-        <v>232</v>
+        <v>114</v>
       </c>
       <c r="H276" t="n">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="I276" t="n">
         <v>0</v>
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>0.29</v>
+        <v>0.288</v>
       </c>
       <c r="L276" t="n">
         <v>6</v>
@@ -14264,23 +14264,23 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>13.1</v>
+        <v>10.8</v>
       </c>
       <c r="E277" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F277" t="n">
         <v>8.300000000000001</v>
       </c>
       <c r="G277" t="n">
-        <v>407</v>
+        <v>118</v>
       </c>
       <c r="H277" t="n">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="I277" t="n">
         <v>0</v>
@@ -14289,7 +14289,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>0.29</v>
+        <v>0.287</v>
       </c>
       <c r="L277" t="n">
         <v>6</v>
@@ -14314,23 +14314,23 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>15.5</v>
+        <v>13.6</v>
       </c>
       <c r="E278" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F278" t="n">
-        <v>11.5</v>
+        <v>9.4</v>
       </c>
       <c r="G278" t="n">
-        <v>495</v>
+        <v>389</v>
       </c>
       <c r="H278" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="I278" t="n">
         <v>0</v>
@@ -14339,7 +14339,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>0.289</v>
+        <v>0.286</v>
       </c>
       <c r="L278" t="n">
         <v>6</v>
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>16.7</v>
+        <v>15.7</v>
       </c>
       <c r="E279" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F279" t="n">
-        <v>11.9</v>
+        <v>7.6</v>
       </c>
       <c r="G279" t="n">
-        <v>555</v>
+        <v>544</v>
       </c>
       <c r="H279" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.287</v>
+        <v>0.285</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,23 +14414,23 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>17.3</v>
+        <v>16.8</v>
       </c>
       <c r="E280" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F280" t="n">
-        <v>11.2</v>
+        <v>7.6</v>
       </c>
       <c r="G280" t="n">
-        <v>458</v>
+        <v>448</v>
       </c>
       <c r="H280" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="I280" t="n">
         <v>0</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.286</v>
+        <v>0.284</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,20 +14464,20 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>16.9</v>
+        <v>16.5</v>
       </c>
       <c r="E281" t="n">
         <v>33</v>
       </c>
       <c r="F281" t="n">
-        <v>11.2</v>
+        <v>8.6</v>
       </c>
       <c r="G281" t="n">
-        <v>170</v>
+        <v>102</v>
       </c>
       <c r="H281" t="n">
         <v>100</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.284</v>
+        <v>0.283</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,23 +14514,23 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>16.7</v>
+        <v>16.4</v>
       </c>
       <c r="E282" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F282" t="n">
-        <v>9.699999999999999</v>
+        <v>5.8</v>
       </c>
       <c r="G282" t="n">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="H282" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="I282" t="n">
         <v>0</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.284</v>
+        <v>0.282</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,20 +14564,20 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>16.7</v>
+        <v>15.7</v>
       </c>
       <c r="E283" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F283" t="n">
-        <v>10.1</v>
+        <v>2.9</v>
       </c>
       <c r="G283" t="n">
-        <v>118</v>
+        <v>20</v>
       </c>
       <c r="H283" t="n">
         <v>100</v>
@@ -14589,7 +14589,7 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0.283</v>
+        <v>0.282</v>
       </c>
       <c r="L283" t="n">
         <v>6</v>
@@ -14614,11 +14614,11 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>14.3</v>
+        <v>13.7</v>
       </c>
       <c r="E284" t="n">
         <v>42</v>
@@ -14627,7 +14627,7 @@
         <v>10.4</v>
       </c>
       <c r="G284" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H284" t="n">
         <v>100</v>
@@ -14639,7 +14639,7 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0.283</v>
+        <v>0.282</v>
       </c>
       <c r="L284" t="n">
         <v>6</v>
@@ -14664,23 +14664,23 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>13.3</v>
+        <v>12.5</v>
       </c>
       <c r="E285" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F285" t="n">
-        <v>10.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
       </c>
       <c r="H285" t="n">
-        <v>100</v>
+        <v>23</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -14689,7 +14689,7 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
-        <v>0.283</v>
+        <v>0.282</v>
       </c>
       <c r="L285" t="n">
         <v>6</v>
@@ -14714,23 +14714,23 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>12.9</v>
+        <v>11.1</v>
       </c>
       <c r="E286" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F286" t="n">
-        <v>10.4</v>
+        <v>5.8</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>100</v>
+        <v>21</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14764,23 +14764,23 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>12.4</v>
+        <v>10.3</v>
       </c>
       <c r="E287" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F287" t="n">
-        <v>13.3</v>
+        <v>4.7</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -14814,23 +14814,23 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>11.8</v>
+        <v>9.5</v>
       </c>
       <c r="E288" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="F288" t="n">
-        <v>10.8</v>
+        <v>7.2</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
       </c>
       <c r="H288" t="n">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.282</v>
+        <v>0.281</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,17 +14864,17 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>11.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E289" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F289" t="n">
-        <v>9</v>
+        <v>5.4</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
@@ -14889,7 +14889,7 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>0.282</v>
+        <v>0.281</v>
       </c>
       <c r="L289" t="n">
         <v>6</v>
@@ -14914,23 +14914,23 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>11.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E290" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="F290" t="n">
-        <v>6.5</v>
+        <v>0.4</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
       </c>
       <c r="H290" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I290" t="n">
         <v>0</v>
@@ -14964,17 +14964,17 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>11.6</v>
+        <v>10.2</v>
       </c>
       <c r="E291" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F291" t="n">
-        <v>8.6</v>
+        <v>3.6</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
@@ -15014,17 +15014,17 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>11.6</v>
+        <v>9.4</v>
       </c>
       <c r="E292" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="F292" t="n">
-        <v>7.9</v>
+        <v>6.5</v>
       </c>
       <c r="G292" t="n">
         <v>0</v>
@@ -15064,17 +15064,17 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>11.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E293" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="F293" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="G293" t="n">
         <v>0</v>
@@ -15114,17 +15114,17 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>11.4</v>
+        <v>10.1</v>
       </c>
       <c r="E294" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F294" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="G294" t="n">
         <v>0</v>
@@ -15164,24 +15164,24 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>11.3</v>
+        <v>10.2</v>
       </c>
       <c r="E295" t="n">
+        <v>56</v>
+      </c>
+      <c r="F295" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0</v>
+      </c>
+      <c r="H295" t="n">
         <v>52</v>
       </c>
-      <c r="F295" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G295" t="n">
-        <v>0</v>
-      </c>
-      <c r="H295" t="n">
-        <v>100</v>
-      </c>
       <c r="I295" t="n">
         <v>0</v>
       </c>
@@ -15189,7 +15189,7 @@
         <v>0</v>
       </c>
       <c r="K295" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L295" t="n">
         <v>7</v>
@@ -15214,23 +15214,23 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>11.3</v>
+        <v>9.4</v>
       </c>
       <c r="E296" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F296" t="n">
-        <v>3.2</v>
+        <v>10.1</v>
       </c>
       <c r="G296" t="n">
         <v>0</v>
       </c>
       <c r="H296" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="I296" t="n">
         <v>0</v>
@@ -15239,7 +15239,7 @@
         <v>0</v>
       </c>
       <c r="K296" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L296" t="n">
         <v>7</v>
@@ -15264,23 +15264,23 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>11.2</v>
+        <v>9</v>
       </c>
       <c r="E297" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="F297" t="n">
-        <v>4</v>
+        <v>6.1</v>
       </c>
       <c r="G297" t="n">
         <v>0</v>
       </c>
       <c r="H297" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I297" t="n">
         <v>0</v>
@@ -15289,7 +15289,7 @@
         <v>0</v>
       </c>
       <c r="K297" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L297" t="n">
         <v>7</v>
@@ -15314,23 +15314,23 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>11.2</v>
+        <v>8.9</v>
       </c>
       <c r="E298" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="F298" t="n">
-        <v>2.5</v>
+        <v>4.7</v>
       </c>
       <c r="G298" t="n">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="H298" t="n">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="I298" t="n">
         <v>0</v>
@@ -15339,7 +15339,7 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L298" t="n">
         <v>7</v>
@@ -15364,23 +15364,23 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>12.1</v>
+        <v>10.2</v>
       </c>
       <c r="E299" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="F299" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G299" t="n">
-        <v>54</v>
+        <v>184</v>
       </c>
       <c r="H299" t="n">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="I299" t="n">
         <v>0</v>
@@ -15414,23 +15414,23 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D300" t="n">
         <v>12.6</v>
       </c>
       <c r="E300" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F300" t="n">
-        <v>7.9</v>
+        <v>7.6</v>
       </c>
       <c r="G300" t="n">
-        <v>56</v>
+        <v>328</v>
       </c>
       <c r="H300" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="I300" t="n">
         <v>0</v>
@@ -15439,7 +15439,7 @@
         <v>0</v>
       </c>
       <c r="K300" t="n">
-        <v>0.28</v>
+        <v>0.281</v>
       </c>
       <c r="L300" t="n">
         <v>7</v>
@@ -15464,20 +15464,20 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>13.2</v>
+        <v>14</v>
       </c>
       <c r="E301" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F301" t="n">
-        <v>3.6</v>
+        <v>6.8</v>
       </c>
       <c r="G301" t="n">
-        <v>90</v>
+        <v>204</v>
       </c>
       <c r="H301" t="n">
         <v>100</v>
@@ -15489,7 +15489,7 @@
         <v>0</v>
       </c>
       <c r="K301" t="n">
-        <v>0.279</v>
+        <v>0.28</v>
       </c>
       <c r="L301" t="n">
         <v>7</v>
@@ -15514,23 +15514,23 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>14.9</v>
+        <v>15.3</v>
       </c>
       <c r="E302" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F302" t="n">
-        <v>4.3</v>
+        <v>5.4</v>
       </c>
       <c r="G302" t="n">
-        <v>304</v>
+        <v>220</v>
       </c>
       <c r="H302" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I302" t="n">
         <v>0</v>
@@ -15539,7 +15539,7 @@
         <v>0</v>
       </c>
       <c r="K302" t="n">
-        <v>0.278</v>
+        <v>0.279</v>
       </c>
       <c r="L302" t="n">
         <v>7</v>
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>17.4</v>
+        <v>16.9</v>
       </c>
       <c r="E303" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F303" t="n">
-        <v>5</v>
+        <v>7.9</v>
       </c>
       <c r="G303" t="n">
-        <v>556</v>
+        <v>338</v>
       </c>
       <c r="H303" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15589,7 +15589,7 @@
         <v>0</v>
       </c>
       <c r="K303" t="n">
-        <v>0.276</v>
+        <v>0.277</v>
       </c>
       <c r="L303" t="n">
         <v>7</v>
@@ -15614,23 +15614,23 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>19.3</v>
+        <v>18.2</v>
       </c>
       <c r="E304" t="n">
         <v>31</v>
       </c>
       <c r="F304" t="n">
-        <v>6.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G304" t="n">
-        <v>526</v>
+        <v>510</v>
       </c>
       <c r="H304" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -15639,7 +15639,7 @@
         <v>0</v>
       </c>
       <c r="K304" t="n">
-        <v>0.274</v>
+        <v>0.275</v>
       </c>
       <c r="L304" t="n">
         <v>7</v>
@@ -15664,23 +15664,23 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>20.1</v>
+        <v>18.8</v>
       </c>
       <c r="E305" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F305" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="G305" t="n">
-        <v>443</v>
+        <v>416</v>
       </c>
       <c r="H305" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -15689,7 +15689,7 @@
         <v>0</v>
       </c>
       <c r="K305" t="n">
-        <v>0.272</v>
+        <v>0.273</v>
       </c>
       <c r="L305" t="n">
         <v>7</v>
@@ -15714,23 +15714,23 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>20.3</v>
+        <v>19.1</v>
       </c>
       <c r="E306" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F306" t="n">
-        <v>7.9</v>
+        <v>7.2</v>
       </c>
       <c r="G306" t="n">
-        <v>316</v>
+        <v>296</v>
       </c>
       <c r="H306" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
@@ -15739,7 +15739,7 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="L306" t="n">
         <v>7</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>19.9</v>
+        <v>18.6</v>
       </c>
       <c r="E307" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F307" t="n">
-        <v>8.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="G307" t="n">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H307" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15789,7 +15789,7 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0.27</v>
+        <v>0.271</v>
       </c>
       <c r="L307" t="n">
         <v>7</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>17.6</v>
+        <v>16.5</v>
       </c>
       <c r="E308" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F308" t="n">
-        <v>6.8</v>
+        <v>7.9</v>
       </c>
       <c r="G308" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H308" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15839,7 +15839,7 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0.27</v>
+        <v>0.271</v>
       </c>
       <c r="L308" t="n">
         <v>7</v>
@@ -15864,23 +15864,23 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E309" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="F309" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>0.27</v>
+        <v>0.271</v>
       </c>
       <c r="L309" t="n">
         <v>7</v>
@@ -15914,23 +15914,23 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>13.2</v>
+        <v>12.1</v>
       </c>
       <c r="E310" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="F310" t="n">
-        <v>7.6</v>
+        <v>4.7</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15939,7 +15939,7 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>0.27</v>
+        <v>0.271</v>
       </c>
       <c r="L310" t="n">
         <v>7</v>
@@ -15964,17 +15964,17 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>11.8</v>
+        <v>10.7</v>
       </c>
       <c r="E311" t="n">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="F311" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
@@ -16014,23 +16014,23 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>10.9</v>
+        <v>9.9</v>
       </c>
       <c r="E312" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="F312" t="n">
-        <v>3.6</v>
+        <v>2.2</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
       </c>
       <c r="H312" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I312" t="n">
         <v>0</v>
@@ -16064,17 +16064,17 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>10.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E313" t="n">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="F313" t="n">
-        <v>2.9</v>
+        <v>1.8</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -16114,23 +16114,23 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9.4</v>
+        <v>8.5</v>
       </c>
       <c r="E314" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="F314" t="n">
-        <v>3.6</v>
+        <v>2.5</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
       </c>
       <c r="H314" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I314" t="n">
         <v>0</v>
@@ -16164,23 +16164,23 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-16T17:03:41Z</t>
+          <t>2026-10-16T23:03:44Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>8.4</v>
+        <v>7.8</v>
       </c>
       <c r="E315" t="n">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="F315" t="n">
-        <v>9.699999999999999</v>
+        <v>4.7</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
       </c>
       <c r="H315" t="n">
-        <v>86</v>
+        <v>0</v>
       </c>
       <c r="I315" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-17 07:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N315"/>
+  <dimension ref="A1:N339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -14064,23 +14064,23 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>5.9</v>
+        <v>6.7</v>
       </c>
       <c r="E273" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F273" t="n">
-        <v>11.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
       </c>
       <c r="H273" t="n">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="I273" t="n">
         <v>0</v>
@@ -14089,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="K273" t="n">
-        <v>0.289</v>
+        <v>0.291</v>
       </c>
       <c r="L273" t="n">
         <v>6</v>
@@ -14114,20 +14114,20 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>6.6</v>
+        <v>7.3</v>
       </c>
       <c r="E274" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F274" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="G274" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H274" t="n">
         <v>100</v>
@@ -14139,7 +14139,7 @@
         <v>0</v>
       </c>
       <c r="K274" t="n">
-        <v>0.289</v>
+        <v>0.291</v>
       </c>
       <c r="L274" t="n">
         <v>6</v>
@@ -14164,20 +14164,20 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E275" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F275" t="n">
-        <v>10.1</v>
+        <v>9.4</v>
       </c>
       <c r="G275" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H275" t="n">
         <v>100</v>
@@ -14189,7 +14189,7 @@
         <v>0</v>
       </c>
       <c r="K275" t="n">
-        <v>0.288</v>
+        <v>0.29</v>
       </c>
       <c r="L275" t="n">
         <v>6</v>
@@ -14214,23 +14214,23 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>9.5</v>
+        <v>10.4</v>
       </c>
       <c r="E276" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F276" t="n">
-        <v>9.699999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="G276" t="n">
-        <v>114</v>
+        <v>209</v>
       </c>
       <c r="H276" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="I276" t="n">
         <v>0</v>
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="K276" t="n">
-        <v>0.288</v>
+        <v>0.29</v>
       </c>
       <c r="L276" t="n">
         <v>6</v>
@@ -14264,23 +14264,23 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>10.8</v>
+        <v>11.9</v>
       </c>
       <c r="E277" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F277" t="n">
-        <v>8.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="G277" t="n">
-        <v>118</v>
+        <v>201</v>
       </c>
       <c r="H277" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="I277" t="n">
         <v>0</v>
@@ -14289,7 +14289,7 @@
         <v>0</v>
       </c>
       <c r="K277" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="L277" t="n">
         <v>6</v>
@@ -14314,23 +14314,23 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>13.6</v>
+        <v>14.3</v>
       </c>
       <c r="E278" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F278" t="n">
-        <v>9.4</v>
+        <v>10.8</v>
       </c>
       <c r="G278" t="n">
-        <v>389</v>
+        <v>500</v>
       </c>
       <c r="H278" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I278" t="n">
         <v>0</v>
@@ -14339,7 +14339,7 @@
         <v>0</v>
       </c>
       <c r="K278" t="n">
-        <v>0.286</v>
+        <v>0.288</v>
       </c>
       <c r="L278" t="n">
         <v>6</v>
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>15.7</v>
+        <v>16</v>
       </c>
       <c r="E279" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F279" t="n">
-        <v>7.6</v>
+        <v>10.1</v>
       </c>
       <c r="G279" t="n">
-        <v>544</v>
+        <v>523</v>
       </c>
       <c r="H279" t="n">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.285</v>
+        <v>0.287</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,20 +14414,20 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>16.8</v>
+        <v>16.1</v>
       </c>
       <c r="E280" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F280" t="n">
         <v>7.6</v>
       </c>
       <c r="G280" t="n">
-        <v>448</v>
+        <v>184</v>
       </c>
       <c r="H280" t="n">
         <v>100</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.284</v>
+        <v>0.286</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,20 +14464,20 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>16.5</v>
+        <v>16.2</v>
       </c>
       <c r="E281" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F281" t="n">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G281" t="n">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="H281" t="n">
         <v>100</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.283</v>
+        <v>0.285</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,20 +14514,20 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>16.4</v>
+        <v>16.2</v>
       </c>
       <c r="E282" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F282" t="n">
-        <v>5.8</v>
+        <v>10.1</v>
       </c>
       <c r="G282" t="n">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="H282" t="n">
         <v>100</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,20 +14564,20 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="E283" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F283" t="n">
-        <v>2.9</v>
+        <v>7.6</v>
       </c>
       <c r="G283" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="H283" t="n">
         <v>100</v>
@@ -14589,7 +14589,7 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
       <c r="L283" t="n">
         <v>6</v>
@@ -14614,20 +14614,20 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>13.7</v>
+        <v>14.5</v>
       </c>
       <c r="E284" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F284" t="n">
-        <v>10.4</v>
+        <v>5.4</v>
       </c>
       <c r="G284" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H284" t="n">
         <v>100</v>
@@ -14639,7 +14639,7 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
       <c r="L284" t="n">
         <v>6</v>
@@ -14664,23 +14664,23 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>12.5</v>
+        <v>13.6</v>
       </c>
       <c r="E285" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="F285" t="n">
-        <v>8.300000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
       </c>
       <c r="H285" t="n">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -14689,7 +14689,7 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L285" t="n">
         <v>6</v>
@@ -14714,14 +14714,14 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>11.1</v>
+        <v>12.4</v>
       </c>
       <c r="E286" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="F286" t="n">
         <v>5.8</v>
@@ -14730,7 +14730,7 @@
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14739,7 +14739,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L286" t="n">
         <v>6</v>
@@ -14764,23 +14764,23 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
       <c r="E287" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="F287" t="n">
-        <v>4.7</v>
+        <v>1.8</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L287" t="n">
         <v>6</v>
@@ -14814,23 +14814,23 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>9.5</v>
+        <v>10.7</v>
       </c>
       <c r="E288" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F288" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
       </c>
       <c r="H288" t="n">
-        <v>42</v>
+        <v>100</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.281</v>
+        <v>0.283</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,17 +14864,17 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>8.800000000000001</v>
+        <v>10.7</v>
       </c>
       <c r="E289" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="F289" t="n">
-        <v>5.4</v>
+        <v>4.7</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
@@ -14889,7 +14889,7 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>0.281</v>
+        <v>0.283</v>
       </c>
       <c r="L289" t="n">
         <v>6</v>
@@ -14914,23 +14914,23 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>9.300000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="E290" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F290" t="n">
-        <v>0.4</v>
+        <v>4</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
       </c>
       <c r="H290" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I290" t="n">
         <v>0</v>
@@ -14939,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="K290" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L290" t="n">
         <v>7</v>
@@ -14964,17 +14964,17 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="E291" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F291" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L291" t="n">
         <v>7</v>
@@ -15014,17 +15014,17 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="E292" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F292" t="n">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="G292" t="n">
         <v>0</v>
@@ -15039,7 +15039,7 @@
         <v>0</v>
       </c>
       <c r="K292" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L292" t="n">
         <v>7</v>
@@ -15064,17 +15064,17 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>9.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="E293" t="n">
         <v>57</v>
       </c>
       <c r="F293" t="n">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="G293" t="n">
         <v>0</v>
@@ -15089,7 +15089,7 @@
         <v>0</v>
       </c>
       <c r="K293" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L293" t="n">
         <v>7</v>
@@ -15114,17 +15114,17 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>10.1</v>
+        <v>10.9</v>
       </c>
       <c r="E294" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F294" t="n">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="G294" t="n">
         <v>0</v>
@@ -15139,7 +15139,7 @@
         <v>0</v>
       </c>
       <c r="K294" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L294" t="n">
         <v>7</v>
@@ -15164,23 +15164,23 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>10.2</v>
+        <v>10.6</v>
       </c>
       <c r="E295" t="n">
         <v>56</v>
       </c>
       <c r="F295" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="G295" t="n">
         <v>0</v>
       </c>
       <c r="H295" t="n">
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="I295" t="n">
         <v>0</v>
@@ -15189,7 +15189,7 @@
         <v>0</v>
       </c>
       <c r="K295" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L295" t="n">
         <v>7</v>
@@ -15214,23 +15214,23 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>9.4</v>
+        <v>11</v>
       </c>
       <c r="E296" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F296" t="n">
-        <v>10.1</v>
+        <v>8.6</v>
       </c>
       <c r="G296" t="n">
         <v>0</v>
       </c>
       <c r="H296" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="I296" t="n">
         <v>0</v>
@@ -15239,7 +15239,7 @@
         <v>0</v>
       </c>
       <c r="K296" t="n">
-        <v>0.282</v>
+        <v>0.283</v>
       </c>
       <c r="L296" t="n">
         <v>7</v>
@@ -15264,23 +15264,23 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>9</v>
+        <v>10.6</v>
       </c>
       <c r="E297" t="n">
         <v>58</v>
       </c>
       <c r="F297" t="n">
-        <v>6.1</v>
+        <v>3.2</v>
       </c>
       <c r="G297" t="n">
         <v>0</v>
       </c>
       <c r="H297" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I297" t="n">
         <v>0</v>
@@ -15314,23 +15314,23 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>8.9</v>
+        <v>10.6</v>
       </c>
       <c r="E298" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F298" t="n">
-        <v>4.7</v>
+        <v>1.4</v>
       </c>
       <c r="G298" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="H298" t="n">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="I298" t="n">
         <v>0</v>
@@ -15364,23 +15364,23 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>10.2</v>
+        <v>11.4</v>
       </c>
       <c r="E299" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F299" t="n">
-        <v>7.6</v>
+        <v>4.3</v>
       </c>
       <c r="G299" t="n">
-        <v>184</v>
+        <v>66</v>
       </c>
       <c r="H299" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="I299" t="n">
         <v>0</v>
@@ -15389,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="K299" t="n">
-        <v>0.281</v>
+        <v>0.282</v>
       </c>
       <c r="L299" t="n">
         <v>7</v>
@@ -15414,23 +15414,23 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D300" t="n">
         <v>12.6</v>
       </c>
       <c r="E300" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F300" t="n">
-        <v>7.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G300" t="n">
-        <v>328</v>
+        <v>96</v>
       </c>
       <c r="H300" t="n">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="I300" t="n">
         <v>0</v>
@@ -15464,20 +15464,20 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>14</v>
+        <v>13.1</v>
       </c>
       <c r="E301" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="F301" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="G301" t="n">
-        <v>204</v>
+        <v>84</v>
       </c>
       <c r="H301" t="n">
         <v>100</v>
@@ -15514,20 +15514,20 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>15.3</v>
+        <v>13.8</v>
       </c>
       <c r="E302" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="F302" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="G302" t="n">
-        <v>220</v>
+        <v>115</v>
       </c>
       <c r="H302" t="n">
         <v>100</v>
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>16.9</v>
+        <v>14.7</v>
       </c>
       <c r="E303" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="F303" t="n">
-        <v>7.9</v>
+        <v>4.3</v>
       </c>
       <c r="G303" t="n">
-        <v>338</v>
+        <v>248</v>
       </c>
       <c r="H303" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15614,23 +15614,23 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>18.2</v>
+        <v>17.1</v>
       </c>
       <c r="E304" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="F304" t="n">
-        <v>8.300000000000001</v>
+        <v>4.7</v>
       </c>
       <c r="G304" t="n">
-        <v>510</v>
+        <v>523</v>
       </c>
       <c r="H304" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -15664,23 +15664,23 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="E305" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F305" t="n">
-        <v>7.6</v>
+        <v>5.8</v>
       </c>
       <c r="G305" t="n">
-        <v>416</v>
+        <v>438</v>
       </c>
       <c r="H305" t="n">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -15689,7 +15689,7 @@
         <v>0</v>
       </c>
       <c r="K305" t="n">
-        <v>0.273</v>
+        <v>0.274</v>
       </c>
       <c r="L305" t="n">
         <v>7</v>
@@ -15714,23 +15714,23 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D306" t="n">
         <v>19.1</v>
       </c>
       <c r="E306" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F306" t="n">
-        <v>7.2</v>
+        <v>6.5</v>
       </c>
       <c r="G306" t="n">
-        <v>296</v>
+        <v>311</v>
       </c>
       <c r="H306" t="n">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="E307" t="n">
         <v>31</v>
       </c>
       <c r="F307" t="n">
-        <v>9.4</v>
+        <v>7.6</v>
       </c>
       <c r="G307" t="n">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="H307" t="n">
-        <v>5</v>
+        <v>88</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15789,7 +15789,7 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="L307" t="n">
         <v>7</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>16.5</v>
+        <v>16.7</v>
       </c>
       <c r="E308" t="n">
         <v>37</v>
       </c>
       <c r="F308" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G308" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H308" t="n">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15839,7 +15839,7 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="L308" t="n">
         <v>7</v>
@@ -15864,23 +15864,23 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>14</v>
+        <v>14.1</v>
       </c>
       <c r="E309" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F309" t="n">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="L309" t="n">
         <v>7</v>
@@ -15914,23 +15914,23 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="E310" t="n">
         <v>51</v>
       </c>
       <c r="F310" t="n">
-        <v>4.7</v>
+        <v>5.4</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15939,7 +15939,7 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="L310" t="n">
         <v>7</v>
@@ -15964,17 +15964,17 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="E311" t="n">
         <v>57</v>
       </c>
       <c r="F311" t="n">
-        <v>4.3</v>
+        <v>6.1</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
@@ -15989,7 +15989,7 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="L311" t="n">
         <v>7</v>
@@ -16014,17 +16014,17 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>9.9</v>
+        <v>10.2</v>
       </c>
       <c r="E312" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F312" t="n">
-        <v>2.2</v>
+        <v>4.7</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -16039,7 +16039,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="L312" t="n">
         <v>7</v>
@@ -16064,17 +16064,17 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>9.199999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="E313" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F313" t="n">
-        <v>1.8</v>
+        <v>3.6</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,17 +16114,17 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="E314" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F314" t="n">
-        <v>2.5</v>
+        <v>5.8</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -16139,7 +16139,7 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0.271</v>
+        <v>0.273</v>
       </c>
       <c r="L314" t="n">
         <v>1</v>
@@ -16164,17 +16164,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-16T23:03:44Z</t>
+          <t>2026-10-17T05:03:19Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>7.8</v>
+        <v>7.6</v>
       </c>
       <c r="E315" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F315" t="n">
-        <v>4.7</v>
+        <v>6.1</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0.271</v>
+        <v>0.273</v>
       </c>
       <c r="L315" t="n">
         <v>1</v>
@@ -16198,6 +16198,1206 @@
         <v>0</v>
       </c>
       <c r="N315" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E316" t="n">
+        <v>75</v>
+      </c>
+      <c r="F316" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G316" t="n">
+        <v>0</v>
+      </c>
+      <c r="H316" t="n">
+        <v>0</v>
+      </c>
+      <c r="I316" t="n">
+        <v>0</v>
+      </c>
+      <c r="J316" t="n">
+        <v>0</v>
+      </c>
+      <c r="K316" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L316" t="n">
+        <v>1</v>
+      </c>
+      <c r="M316" t="n">
+        <v>0</v>
+      </c>
+      <c r="N316" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E317" t="n">
+        <v>77</v>
+      </c>
+      <c r="F317" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G317" t="n">
+        <v>0</v>
+      </c>
+      <c r="H317" t="n">
+        <v>3</v>
+      </c>
+      <c r="I317" t="n">
+        <v>0</v>
+      </c>
+      <c r="J317" t="n">
+        <v>0</v>
+      </c>
+      <c r="K317" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L317" t="n">
+        <v>1</v>
+      </c>
+      <c r="M317" t="n">
+        <v>0</v>
+      </c>
+      <c r="N317" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E318" t="n">
+        <v>79</v>
+      </c>
+      <c r="F318" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0</v>
+      </c>
+      <c r="H318" t="n">
+        <v>0</v>
+      </c>
+      <c r="I318" t="n">
+        <v>0</v>
+      </c>
+      <c r="J318" t="n">
+        <v>0</v>
+      </c>
+      <c r="K318" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L318" t="n">
+        <v>1</v>
+      </c>
+      <c r="M318" t="n">
+        <v>0</v>
+      </c>
+      <c r="N318" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E319" t="n">
+        <v>85</v>
+      </c>
+      <c r="F319" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G319" t="n">
+        <v>0</v>
+      </c>
+      <c r="H319" t="n">
+        <v>0</v>
+      </c>
+      <c r="I319" t="n">
+        <v>0</v>
+      </c>
+      <c r="J319" t="n">
+        <v>0</v>
+      </c>
+      <c r="K319" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L319" t="n">
+        <v>1</v>
+      </c>
+      <c r="M319" t="n">
+        <v>0</v>
+      </c>
+      <c r="N319" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>6</v>
+      </c>
+      <c r="E320" t="n">
+        <v>92</v>
+      </c>
+      <c r="F320" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G320" t="n">
+        <v>0</v>
+      </c>
+      <c r="H320" t="n">
+        <v>0</v>
+      </c>
+      <c r="I320" t="n">
+        <v>0</v>
+      </c>
+      <c r="J320" t="n">
+        <v>0</v>
+      </c>
+      <c r="K320" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L320" t="n">
+        <v>1</v>
+      </c>
+      <c r="M320" t="n">
+        <v>0</v>
+      </c>
+      <c r="N320" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E321" t="n">
+        <v>95</v>
+      </c>
+      <c r="F321" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G321" t="n">
+        <v>0</v>
+      </c>
+      <c r="H321" t="n">
+        <v>0</v>
+      </c>
+      <c r="I321" t="n">
+        <v>0</v>
+      </c>
+      <c r="J321" t="n">
+        <v>0</v>
+      </c>
+      <c r="K321" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L321" t="n">
+        <v>1</v>
+      </c>
+      <c r="M321" t="n">
+        <v>0</v>
+      </c>
+      <c r="N321" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E322" t="n">
+        <v>92</v>
+      </c>
+      <c r="F322" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G322" t="n">
+        <v>44</v>
+      </c>
+      <c r="H322" t="n">
+        <v>0</v>
+      </c>
+      <c r="I322" t="n">
+        <v>0</v>
+      </c>
+      <c r="J322" t="n">
+        <v>0</v>
+      </c>
+      <c r="K322" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L322" t="n">
+        <v>1</v>
+      </c>
+      <c r="M322" t="n">
+        <v>0</v>
+      </c>
+      <c r="N322" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E323" t="n">
+        <v>79</v>
+      </c>
+      <c r="F323" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G323" t="n">
+        <v>183</v>
+      </c>
+      <c r="H323" t="n">
+        <v>0</v>
+      </c>
+      <c r="I323" t="n">
+        <v>0</v>
+      </c>
+      <c r="J323" t="n">
+        <v>0</v>
+      </c>
+      <c r="K323" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L323" t="n">
+        <v>1</v>
+      </c>
+      <c r="M323" t="n">
+        <v>0</v>
+      </c>
+      <c r="N323" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="E324" t="n">
+        <v>67</v>
+      </c>
+      <c r="F324" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G324" t="n">
+        <v>329</v>
+      </c>
+      <c r="H324" t="n">
+        <v>0</v>
+      </c>
+      <c r="I324" t="n">
+        <v>0</v>
+      </c>
+      <c r="J324" t="n">
+        <v>0</v>
+      </c>
+      <c r="K324" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="L324" t="n">
+        <v>1</v>
+      </c>
+      <c r="M324" t="n">
+        <v>0</v>
+      </c>
+      <c r="N324" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E325" t="n">
+        <v>62</v>
+      </c>
+      <c r="F325" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G325" t="n">
+        <v>442.8</v>
+      </c>
+      <c r="H325" t="n">
+        <v>2</v>
+      </c>
+      <c r="I325" t="n">
+        <v>0</v>
+      </c>
+      <c r="J325" t="n">
+        <v>0</v>
+      </c>
+      <c r="K325" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="L325" t="n">
+        <v>1</v>
+      </c>
+      <c r="M325" t="n">
+        <v>0</v>
+      </c>
+      <c r="N325" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="E326" t="n">
+        <v>59</v>
+      </c>
+      <c r="F326" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G326" t="n">
+        <v>517</v>
+      </c>
+      <c r="H326" t="n">
+        <v>5</v>
+      </c>
+      <c r="I326" t="n">
+        <v>0</v>
+      </c>
+      <c r="J326" t="n">
+        <v>0</v>
+      </c>
+      <c r="K326" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="L326" t="n">
+        <v>1</v>
+      </c>
+      <c r="M326" t="n">
+        <v>0</v>
+      </c>
+      <c r="N326" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E327" t="n">
+        <v>57</v>
+      </c>
+      <c r="F327" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="G327" t="n">
+        <v>534.5</v>
+      </c>
+      <c r="H327" t="n">
+        <v>25</v>
+      </c>
+      <c r="I327" t="n">
+        <v>0</v>
+      </c>
+      <c r="J327" t="n">
+        <v>0</v>
+      </c>
+      <c r="K327" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L327" t="n">
+        <v>1</v>
+      </c>
+      <c r="M327" t="n">
+        <v>0</v>
+      </c>
+      <c r="N327" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="E328" t="n">
+        <v>55</v>
+      </c>
+      <c r="F328" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="G328" t="n">
+        <v>504</v>
+      </c>
+      <c r="H328" t="n">
+        <v>55</v>
+      </c>
+      <c r="I328" t="n">
+        <v>0</v>
+      </c>
+      <c r="J328" t="n">
+        <v>0</v>
+      </c>
+      <c r="K328" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="L328" t="n">
+        <v>1</v>
+      </c>
+      <c r="M328" t="n">
+        <v>0</v>
+      </c>
+      <c r="N328" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="E329" t="n">
+        <v>53</v>
+      </c>
+      <c r="F329" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="G329" t="n">
+        <v>397</v>
+      </c>
+      <c r="H329" t="n">
+        <v>33</v>
+      </c>
+      <c r="I329" t="n">
+        <v>0</v>
+      </c>
+      <c r="J329" t="n">
+        <v>0</v>
+      </c>
+      <c r="K329" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="L329" t="n">
+        <v>1</v>
+      </c>
+      <c r="M329" t="n">
+        <v>0</v>
+      </c>
+      <c r="N329" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="E330" t="n">
+        <v>55</v>
+      </c>
+      <c r="F330" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G330" t="n">
+        <v>296</v>
+      </c>
+      <c r="H330" t="n">
+        <v>12</v>
+      </c>
+      <c r="I330" t="n">
+        <v>0</v>
+      </c>
+      <c r="J330" t="n">
+        <v>0</v>
+      </c>
+      <c r="K330" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="L330" t="n">
+        <v>1</v>
+      </c>
+      <c r="M330" t="n">
+        <v>0</v>
+      </c>
+      <c r="N330" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="E331" t="n">
+        <v>62</v>
+      </c>
+      <c r="F331" t="n">
+        <v>6</v>
+      </c>
+      <c r="G331" t="n">
+        <v>152</v>
+      </c>
+      <c r="H331" t="n">
+        <v>7</v>
+      </c>
+      <c r="I331" t="n">
+        <v>0</v>
+      </c>
+      <c r="J331" t="n">
+        <v>0</v>
+      </c>
+      <c r="K331" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="L331" t="n">
+        <v>1</v>
+      </c>
+      <c r="M331" t="n">
+        <v>0</v>
+      </c>
+      <c r="N331" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>14</v>
+      </c>
+      <c r="E332" t="n">
+        <v>73</v>
+      </c>
+      <c r="F332" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G332" t="n">
+        <v>25</v>
+      </c>
+      <c r="H332" t="n">
+        <v>13</v>
+      </c>
+      <c r="I332" t="n">
+        <v>0</v>
+      </c>
+      <c r="J332" t="n">
+        <v>0</v>
+      </c>
+      <c r="K332" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="L332" t="n">
+        <v>1</v>
+      </c>
+      <c r="M332" t="n">
+        <v>0</v>
+      </c>
+      <c r="N332" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="E333" t="n">
+        <v>79</v>
+      </c>
+      <c r="F333" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="n">
+        <v>73</v>
+      </c>
+      <c r="I333" t="n">
+        <v>0</v>
+      </c>
+      <c r="J333" t="n">
+        <v>0</v>
+      </c>
+      <c r="K333" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="L333" t="n">
+        <v>1</v>
+      </c>
+      <c r="M333" t="n">
+        <v>0</v>
+      </c>
+      <c r="N333" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>12</v>
+      </c>
+      <c r="E334" t="n">
+        <v>83</v>
+      </c>
+      <c r="F334" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
+      <c r="H334" t="n">
+        <v>100</v>
+      </c>
+      <c r="I334" t="n">
+        <v>0</v>
+      </c>
+      <c r="J334" t="n">
+        <v>0</v>
+      </c>
+      <c r="K334" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="L334" t="n">
+        <v>1</v>
+      </c>
+      <c r="M334" t="n">
+        <v>0</v>
+      </c>
+      <c r="N334" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="E335" t="n">
+        <v>83</v>
+      </c>
+      <c r="F335" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0</v>
+      </c>
+      <c r="H335" t="n">
+        <v>96</v>
+      </c>
+      <c r="I335" t="n">
+        <v>0</v>
+      </c>
+      <c r="J335" t="n">
+        <v>0</v>
+      </c>
+      <c r="K335" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="L335" t="n">
+        <v>1</v>
+      </c>
+      <c r="M335" t="n">
+        <v>0</v>
+      </c>
+      <c r="N335" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="E336" t="n">
+        <v>83</v>
+      </c>
+      <c r="F336" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0</v>
+      </c>
+      <c r="H336" t="n">
+        <v>96</v>
+      </c>
+      <c r="I336" t="n">
+        <v>0</v>
+      </c>
+      <c r="J336" t="n">
+        <v>0</v>
+      </c>
+      <c r="K336" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="L336" t="n">
+        <v>1</v>
+      </c>
+      <c r="M336" t="n">
+        <v>0</v>
+      </c>
+      <c r="N336" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="E337" t="n">
+        <v>86</v>
+      </c>
+      <c r="F337" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0</v>
+      </c>
+      <c r="H337" t="n">
+        <v>88</v>
+      </c>
+      <c r="I337" t="n">
+        <v>0</v>
+      </c>
+      <c r="J337" t="n">
+        <v>0</v>
+      </c>
+      <c r="K337" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="L337" t="n">
+        <v>1</v>
+      </c>
+      <c r="M337" t="n">
+        <v>0</v>
+      </c>
+      <c r="N337" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="E338" t="n">
+        <v>88</v>
+      </c>
+      <c r="F338" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0</v>
+      </c>
+      <c r="H338" t="n">
+        <v>84</v>
+      </c>
+      <c r="I338" t="n">
+        <v>0</v>
+      </c>
+      <c r="J338" t="n">
+        <v>0</v>
+      </c>
+      <c r="K338" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="L338" t="n">
+        <v>2</v>
+      </c>
+      <c r="M338" t="n">
+        <v>0</v>
+      </c>
+      <c r="N338" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>2026-10-17T05:03:19Z</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="E339" t="n">
+        <v>89</v>
+      </c>
+      <c r="F339" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0</v>
+      </c>
+      <c r="H339" t="n">
+        <v>89</v>
+      </c>
+      <c r="I339" t="n">
+        <v>0</v>
+      </c>
+      <c r="J339" t="n">
+        <v>0</v>
+      </c>
+      <c r="K339" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="L339" t="n">
+        <v>2</v>
+      </c>
+      <c r="M339" t="n">
+        <v>0</v>
+      </c>
+      <c r="N339" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-17 13:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -14364,23 +14364,23 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>16</v>
+        <v>15.3</v>
       </c>
       <c r="E279" t="n">
         <v>37</v>
       </c>
       <c r="F279" t="n">
-        <v>10.1</v>
+        <v>11.2</v>
       </c>
       <c r="G279" t="n">
-        <v>523</v>
+        <v>561</v>
       </c>
       <c r="H279" t="n">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
@@ -14389,7 +14389,7 @@
         <v>0</v>
       </c>
       <c r="K279" t="n">
-        <v>0.287</v>
+        <v>0.29</v>
       </c>
       <c r="L279" t="n">
         <v>6</v>
@@ -14414,20 +14414,20 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>16.1</v>
+        <v>16.2</v>
       </c>
       <c r="E280" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F280" t="n">
-        <v>7.6</v>
+        <v>10.1</v>
       </c>
       <c r="G280" t="n">
-        <v>184</v>
+        <v>463</v>
       </c>
       <c r="H280" t="n">
         <v>100</v>
@@ -14439,7 +14439,7 @@
         <v>0</v>
       </c>
       <c r="K280" t="n">
-        <v>0.286</v>
+        <v>0.289</v>
       </c>
       <c r="L280" t="n">
         <v>6</v>
@@ -14464,20 +14464,20 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>16.2</v>
+        <v>15.8</v>
       </c>
       <c r="E281" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F281" t="n">
-        <v>8.300000000000001</v>
+        <v>10.8</v>
       </c>
       <c r="G281" t="n">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="H281" t="n">
         <v>100</v>
@@ -14489,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="K281" t="n">
-        <v>0.285</v>
+        <v>0.287</v>
       </c>
       <c r="L281" t="n">
         <v>6</v>
@@ -14514,20 +14514,20 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>16.2</v>
+        <v>15.5</v>
       </c>
       <c r="E282" t="n">
         <v>35</v>
       </c>
       <c r="F282" t="n">
-        <v>10.1</v>
+        <v>10.8</v>
       </c>
       <c r="G282" t="n">
-        <v>144</v>
+        <v>61</v>
       </c>
       <c r="H282" t="n">
         <v>100</v>
@@ -14539,7 +14539,7 @@
         <v>0</v>
       </c>
       <c r="K282" t="n">
-        <v>0.284</v>
+        <v>0.287</v>
       </c>
       <c r="L282" t="n">
         <v>6</v>
@@ -14564,20 +14564,20 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>15.6</v>
+        <v>14.7</v>
       </c>
       <c r="E283" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F283" t="n">
-        <v>7.6</v>
+        <v>6.5</v>
       </c>
       <c r="G283" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="H283" t="n">
         <v>100</v>
@@ -14589,7 +14589,7 @@
         <v>0</v>
       </c>
       <c r="K283" t="n">
-        <v>0.284</v>
+        <v>0.286</v>
       </c>
       <c r="L283" t="n">
         <v>6</v>
@@ -14614,20 +14614,20 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>14.5</v>
+        <v>13.8</v>
       </c>
       <c r="E284" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F284" t="n">
-        <v>5.4</v>
+        <v>2.9</v>
       </c>
       <c r="G284" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H284" t="n">
         <v>100</v>
@@ -14639,7 +14639,7 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
-        <v>0.284</v>
+        <v>0.286</v>
       </c>
       <c r="L284" t="n">
         <v>6</v>
@@ -14664,17 +14664,17 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>13.6</v>
+        <v>13.2</v>
       </c>
       <c r="E285" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F285" t="n">
-        <v>5.8</v>
+        <v>4</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
@@ -14689,7 +14689,7 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
-        <v>0.283</v>
+        <v>0.286</v>
       </c>
       <c r="L285" t="n">
         <v>6</v>
@@ -14714,23 +14714,23 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>12.4</v>
+        <v>12.8</v>
       </c>
       <c r="E286" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F286" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
       </c>
       <c r="H286" t="n">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -14739,7 +14739,7 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
-        <v>0.283</v>
+        <v>0.286</v>
       </c>
       <c r="L286" t="n">
         <v>6</v>
@@ -14764,17 +14764,17 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>11.7</v>
+        <v>12.5</v>
       </c>
       <c r="E287" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="F287" t="n">
-        <v>1.8</v>
+        <v>4.3</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>0.283</v>
+        <v>0.286</v>
       </c>
       <c r="L287" t="n">
         <v>6</v>
@@ -14814,17 +14814,17 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>10.7</v>
+        <v>12.1</v>
       </c>
       <c r="E288" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="F288" t="n">
-        <v>6.8</v>
+        <v>3.6</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.283</v>
+        <v>0.286</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,17 +14864,17 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>10.7</v>
+        <v>12</v>
       </c>
       <c r="E289" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="F289" t="n">
-        <v>4.7</v>
+        <v>4.3</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
@@ -14889,7 +14889,7 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
-        <v>0.283</v>
+        <v>0.285</v>
       </c>
       <c r="L289" t="n">
         <v>6</v>
@@ -14914,17 +14914,17 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="E290" t="n">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="F290" t="n">
-        <v>4</v>
+        <v>1.8</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
@@ -14939,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="K290" t="n">
-        <v>0.283</v>
+        <v>0.285</v>
       </c>
       <c r="L290" t="n">
         <v>7</v>
@@ -14964,17 +14964,17 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>10.4</v>
+        <v>11.2</v>
       </c>
       <c r="E291" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="F291" t="n">
-        <v>4.7</v>
+        <v>1.8</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>0.283</v>
+        <v>0.285</v>
       </c>
       <c r="L291" t="n">
         <v>7</v>
@@ -15014,17 +15014,17 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>10.4</v>
+        <v>10.9</v>
       </c>
       <c r="E292" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="F292" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="G292" t="n">
         <v>0</v>
@@ -15039,7 +15039,7 @@
         <v>0</v>
       </c>
       <c r="K292" t="n">
-        <v>0.283</v>
+        <v>0.285</v>
       </c>
       <c r="L292" t="n">
         <v>7</v>
@@ -15064,17 +15064,17 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>10.4</v>
+        <v>10.8</v>
       </c>
       <c r="E293" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F293" t="n">
-        <v>5.8</v>
+        <v>2.9</v>
       </c>
       <c r="G293" t="n">
         <v>0</v>
@@ -15089,7 +15089,7 @@
         <v>0</v>
       </c>
       <c r="K293" t="n">
-        <v>0.283</v>
+        <v>0.285</v>
       </c>
       <c r="L293" t="n">
         <v>7</v>
@@ -15114,17 +15114,17 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D294" t="n">
         <v>10.9</v>
       </c>
       <c r="E294" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F294" t="n">
-        <v>6.5</v>
+        <v>4</v>
       </c>
       <c r="G294" t="n">
         <v>0</v>
@@ -15139,7 +15139,7 @@
         <v>0</v>
       </c>
       <c r="K294" t="n">
-        <v>0.283</v>
+        <v>0.285</v>
       </c>
       <c r="L294" t="n">
         <v>7</v>
@@ -15164,17 +15164,17 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>10.6</v>
+        <v>11</v>
       </c>
       <c r="E295" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="F295" t="n">
-        <v>5.8</v>
+        <v>11.9</v>
       </c>
       <c r="G295" t="n">
         <v>0</v>
@@ -15189,7 +15189,7 @@
         <v>0</v>
       </c>
       <c r="K295" t="n">
-        <v>0.283</v>
+        <v>0.284</v>
       </c>
       <c r="L295" t="n">
         <v>7</v>
@@ -15214,17 +15214,17 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>11</v>
+        <v>10.8</v>
       </c>
       <c r="E296" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F296" t="n">
-        <v>8.6</v>
+        <v>7.9</v>
       </c>
       <c r="G296" t="n">
         <v>0</v>
@@ -15239,7 +15239,7 @@
         <v>0</v>
       </c>
       <c r="K296" t="n">
-        <v>0.283</v>
+        <v>0.284</v>
       </c>
       <c r="L296" t="n">
         <v>7</v>
@@ -15264,17 +15264,17 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D297" t="n">
         <v>10.6</v>
       </c>
       <c r="E297" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F297" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="G297" t="n">
         <v>0</v>
@@ -15289,7 +15289,7 @@
         <v>0</v>
       </c>
       <c r="K297" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
       <c r="L297" t="n">
         <v>7</v>
@@ -15314,23 +15314,23 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>10.6</v>
+        <v>10.7</v>
       </c>
       <c r="E298" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F298" t="n">
-        <v>1.4</v>
+        <v>6.1</v>
       </c>
       <c r="G298" t="n">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="H298" t="n">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="I298" t="n">
         <v>0</v>
@@ -15339,7 +15339,7 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
       <c r="L298" t="n">
         <v>7</v>
@@ -15364,20 +15364,20 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>11.4</v>
+        <v>12</v>
       </c>
       <c r="E299" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F299" t="n">
-        <v>4.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G299" t="n">
-        <v>66</v>
+        <v>135</v>
       </c>
       <c r="H299" t="n">
         <v>100</v>
@@ -15389,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="K299" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
       <c r="L299" t="n">
         <v>7</v>
@@ -15414,20 +15414,20 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D300" t="n">
         <v>12.6</v>
       </c>
       <c r="E300" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F300" t="n">
-        <v>9.699999999999999</v>
+        <v>11.5</v>
       </c>
       <c r="G300" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="H300" t="n">
         <v>100</v>
@@ -15439,7 +15439,7 @@
         <v>0</v>
       </c>
       <c r="K300" t="n">
-        <v>0.281</v>
+        <v>0.283</v>
       </c>
       <c r="L300" t="n">
         <v>7</v>
@@ -15464,7 +15464,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -15474,10 +15474,10 @@
         <v>50</v>
       </c>
       <c r="F301" t="n">
-        <v>7.2</v>
+        <v>9</v>
       </c>
       <c r="G301" t="n">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="H301" t="n">
         <v>100</v>
@@ -15489,7 +15489,7 @@
         <v>0</v>
       </c>
       <c r="K301" t="n">
-        <v>0.28</v>
+        <v>0.282</v>
       </c>
       <c r="L301" t="n">
         <v>7</v>
@@ -15514,23 +15514,23 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>13.8</v>
+        <v>15.9</v>
       </c>
       <c r="E302" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F302" t="n">
-        <v>4.3</v>
+        <v>5</v>
       </c>
       <c r="G302" t="n">
-        <v>115</v>
+        <v>388</v>
       </c>
       <c r="H302" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="I302" t="n">
         <v>0</v>
@@ -15539,7 +15539,7 @@
         <v>0</v>
       </c>
       <c r="K302" t="n">
-        <v>0.279</v>
+        <v>0.281</v>
       </c>
       <c r="L302" t="n">
         <v>7</v>
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>14.7</v>
+        <v>17.8</v>
       </c>
       <c r="E303" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F303" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="G303" t="n">
-        <v>248</v>
+        <v>520</v>
       </c>
       <c r="H303" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15589,7 +15589,7 @@
         <v>0</v>
       </c>
       <c r="K303" t="n">
-        <v>0.277</v>
+        <v>0.279</v>
       </c>
       <c r="L303" t="n">
         <v>7</v>
@@ -15614,23 +15614,23 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>17.1</v>
+        <v>19.1</v>
       </c>
       <c r="E304" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F304" t="n">
-        <v>4.7</v>
+        <v>3.6</v>
       </c>
       <c r="G304" t="n">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="H304" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -15639,7 +15639,7 @@
         <v>0</v>
       </c>
       <c r="K304" t="n">
-        <v>0.275</v>
+        <v>0.278</v>
       </c>
       <c r="L304" t="n">
         <v>7</v>
@@ -15664,23 +15664,23 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>18.7</v>
+        <v>20.1</v>
       </c>
       <c r="E305" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F305" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="G305" t="n">
-        <v>438</v>
+        <v>431</v>
       </c>
       <c r="H305" t="n">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -15689,7 +15689,7 @@
         <v>0</v>
       </c>
       <c r="K305" t="n">
-        <v>0.274</v>
+        <v>0.276</v>
       </c>
       <c r="L305" t="n">
         <v>7</v>
@@ -15714,23 +15714,23 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>19.1</v>
+        <v>20.6</v>
       </c>
       <c r="E306" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F306" t="n">
-        <v>6.5</v>
+        <v>11.2</v>
       </c>
       <c r="G306" t="n">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="H306" t="n">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
@@ -15739,7 +15739,7 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>0.272</v>
+        <v>0.275</v>
       </c>
       <c r="L306" t="n">
         <v>7</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>18.8</v>
+        <v>20</v>
       </c>
       <c r="E307" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F307" t="n">
-        <v>7.6</v>
+        <v>10.8</v>
       </c>
       <c r="G307" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H307" t="n">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15789,7 +15789,7 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="L307" t="n">
         <v>7</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>16.7</v>
+        <v>17.6</v>
       </c>
       <c r="E308" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F308" t="n">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G308" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H308" t="n">
-        <v>9</v>
+        <v>72</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15839,7 +15839,7 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="L308" t="n">
         <v>7</v>
@@ -15864,23 +15864,23 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>14.1</v>
+        <v>15</v>
       </c>
       <c r="E309" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F309" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="L309" t="n">
         <v>7</v>
@@ -15914,23 +15914,23 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>12.2</v>
+        <v>13.1</v>
       </c>
       <c r="E310" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F310" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15939,7 +15939,7 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="L310" t="n">
         <v>7</v>
@@ -15964,17 +15964,17 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>10.8</v>
+        <v>11.8</v>
       </c>
       <c r="E311" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F311" t="n">
-        <v>6.1</v>
+        <v>0.7</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
@@ -15989,7 +15989,7 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="L311" t="n">
         <v>7</v>
@@ -16014,17 +16014,17 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D312" t="n">
         <v>10.2</v>
       </c>
       <c r="E312" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F312" t="n">
-        <v>4.7</v>
+        <v>9</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -16039,7 +16039,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="L312" t="n">
         <v>7</v>
@@ -16064,17 +16064,17 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>9.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E313" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F313" t="n">
-        <v>3.6</v>
+        <v>5.4</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,17 +16114,17 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="E314" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F314" t="n">
-        <v>5.8</v>
+        <v>5</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -16139,7 +16139,7 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0.273</v>
+        <v>0.274</v>
       </c>
       <c r="L314" t="n">
         <v>1</v>
@@ -16164,17 +16164,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>7.6</v>
+        <v>8.6</v>
       </c>
       <c r="E315" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F315" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L315" t="n">
         <v>1</v>
@@ -16214,23 +16214,23 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
       <c r="E316" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="F316" t="n">
-        <v>3.2</v>
+        <v>5.4</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I316" t="n">
         <v>0</v>
@@ -16239,7 +16239,7 @@
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L316" t="n">
         <v>1</v>
@@ -16264,23 +16264,23 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>7.1</v>
+        <v>7.6</v>
       </c>
       <c r="E317" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F317" t="n">
-        <v>5.4</v>
+        <v>5</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I317" t="n">
         <v>0</v>
@@ -16289,7 +16289,7 @@
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L317" t="n">
         <v>1</v>
@@ -16314,17 +16314,17 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="E318" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F318" t="n">
-        <v>8.300000000000001</v>
+        <v>6.1</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
@@ -16339,7 +16339,7 @@
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L318" t="n">
         <v>1</v>
@@ -16364,17 +16364,17 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="E319" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F319" t="n">
-        <v>8.6</v>
+        <v>4.7</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
@@ -16389,7 +16389,7 @@
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L319" t="n">
         <v>1</v>
@@ -16414,17 +16414,17 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>6</v>
+        <v>6.4</v>
       </c>
       <c r="E320" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F320" t="n">
-        <v>7.2</v>
+        <v>3.6</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
@@ -16439,7 +16439,7 @@
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L320" t="n">
         <v>1</v>
@@ -16464,17 +16464,17 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.6</v>
+        <v>6.2</v>
       </c>
       <c r="E321" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F321" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
@@ -16489,7 +16489,7 @@
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L321" t="n">
         <v>1</v>
@@ -16514,17 +16514,17 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D322" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E322" t="n">
+        <v>90</v>
+      </c>
+      <c r="F322" t="n">
         <v>6.5</v>
-      </c>
-      <c r="E322" t="n">
-        <v>92</v>
-      </c>
-      <c r="F322" t="n">
-        <v>7.2</v>
       </c>
       <c r="G322" t="n">
         <v>44</v>
@@ -16539,7 +16539,7 @@
         <v>0</v>
       </c>
       <c r="K322" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L322" t="n">
         <v>1</v>
@@ -16564,20 +16564,20 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D323" t="n">
         <v>9.4</v>
       </c>
       <c r="E323" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F323" t="n">
-        <v>7.6</v>
+        <v>6.1</v>
       </c>
       <c r="G323" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H323" t="n">
         <v>0</v>
@@ -16589,7 +16589,7 @@
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>0.273</v>
+        <v>0.275</v>
       </c>
       <c r="L323" t="n">
         <v>1</v>
@@ -16614,20 +16614,20 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
       <c r="E324" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F324" t="n">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="G324" t="n">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -16639,7 +16639,7 @@
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0.273</v>
+        <v>0.274</v>
       </c>
       <c r="L324" t="n">
         <v>1</v>
@@ -16664,23 +16664,23 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>14.5</v>
+        <v>14.7</v>
       </c>
       <c r="E325" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F325" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="G325" t="n">
-        <v>442.8</v>
+        <v>452</v>
       </c>
       <c r="H325" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -16689,7 +16689,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>0.271</v>
+        <v>0.273</v>
       </c>
       <c r="L325" t="n">
         <v>1</v>
@@ -16714,23 +16714,23 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>16.4</v>
+        <v>17</v>
       </c>
       <c r="E326" t="n">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="F326" t="n">
-        <v>7.8</v>
+        <v>8.6</v>
       </c>
       <c r="G326" t="n">
-        <v>517</v>
+        <v>487</v>
       </c>
       <c r="H326" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I326" t="n">
         <v>0</v>
@@ -16739,7 +16739,7 @@
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>0.27</v>
+        <v>0.272</v>
       </c>
       <c r="L326" t="n">
         <v>1</v>
@@ -16764,23 +16764,23 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>17.5</v>
+        <v>18.5</v>
       </c>
       <c r="E327" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="F327" t="n">
-        <v>9.300000000000001</v>
+        <v>9</v>
       </c>
       <c r="G327" t="n">
-        <v>534.5</v>
+        <v>504</v>
       </c>
       <c r="H327" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I327" t="n">
         <v>0</v>
@@ -16789,7 +16789,7 @@
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>0.268</v>
+        <v>0.27</v>
       </c>
       <c r="L327" t="n">
         <v>1</v>
@@ -16814,23 +16814,23 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>18.2</v>
+        <v>19.5</v>
       </c>
       <c r="E328" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="F328" t="n">
-        <v>12.3</v>
+        <v>10.1</v>
       </c>
       <c r="G328" t="n">
-        <v>504</v>
+        <v>520</v>
       </c>
       <c r="H328" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="I328" t="n">
         <v>0</v>
@@ -16839,7 +16839,7 @@
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0.266</v>
+        <v>0.268</v>
       </c>
       <c r="L328" t="n">
         <v>1</v>
@@ -16864,23 +16864,23 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>18.2</v>
+        <v>20</v>
       </c>
       <c r="E329" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="F329" t="n">
-        <v>12.1</v>
+        <v>10.4</v>
       </c>
       <c r="G329" t="n">
-        <v>397</v>
+        <v>437</v>
       </c>
       <c r="H329" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="I329" t="n">
         <v>0</v>
@@ -16889,7 +16889,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>0.264</v>
+        <v>0.267</v>
       </c>
       <c r="L329" t="n">
         <v>1</v>
@@ -16914,23 +16914,23 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>17.8</v>
+        <v>20</v>
       </c>
       <c r="E330" t="n">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="F330" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="G330" t="n">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="H330" t="n">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="I330" t="n">
         <v>0</v>
@@ -16939,7 +16939,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>0.263</v>
+        <v>0.265</v>
       </c>
       <c r="L330" t="n">
         <v>1</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>16.6</v>
+        <v>18.6</v>
       </c>
       <c r="E331" t="n">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="F331" t="n">
-        <v>6</v>
+        <v>8.9</v>
       </c>
       <c r="G331" t="n">
-        <v>152</v>
+        <v>138.8</v>
       </c>
       <c r="H331" t="n">
-        <v>7</v>
+        <v>86</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -16989,7 +16989,7 @@
         <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>0.262</v>
+        <v>0.265</v>
       </c>
       <c r="L331" t="n">
         <v>1</v>
@@ -17014,23 +17014,23 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>14</v>
+        <v>15.7</v>
       </c>
       <c r="E332" t="n">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="F332" t="n">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="G332" t="n">
-        <v>25</v>
+        <v>22.5</v>
       </c>
       <c r="H332" t="n">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -17039,7 +17039,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>0.262</v>
+        <v>0.265</v>
       </c>
       <c r="L332" t="n">
         <v>1</v>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>12.8</v>
+        <v>14</v>
       </c>
       <c r="E333" t="n">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="F333" t="n">
-        <v>5.6</v>
+        <v>8.9</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>73</v>
+        <v>100</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17089,7 +17089,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>0.262</v>
+        <v>0.265</v>
       </c>
       <c r="L333" t="n">
         <v>1</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>12</v>
+        <v>12.8</v>
       </c>
       <c r="E334" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F334" t="n">
-        <v>5.5</v>
+        <v>6.4</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17139,7 +17139,7 @@
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>0.262</v>
+        <v>0.265</v>
       </c>
       <c r="L334" t="n">
         <v>1</v>
@@ -17164,23 +17164,23 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D335" t="n">
         <v>11.9</v>
       </c>
       <c r="E335" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F335" t="n">
-        <v>4.5</v>
+        <v>5.3</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I335" t="n">
         <v>0</v>
@@ -17189,7 +17189,7 @@
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>0.262</v>
+        <v>0.265</v>
       </c>
       <c r="L335" t="n">
         <v>1</v>
@@ -17214,23 +17214,23 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="E336" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F336" t="n">
-        <v>3.6</v>
+        <v>5.2</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17239,7 +17239,7 @@
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0.263</v>
+        <v>0.265</v>
       </c>
       <c r="L336" t="n">
         <v>1</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>10.8</v>
+        <v>11</v>
       </c>
       <c r="E337" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F337" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17289,7 +17289,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>0.263</v>
+        <v>0.265</v>
       </c>
       <c r="L337" t="n">
         <v>1</v>
@@ -17314,23 +17314,23 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>10.2</v>
+        <v>10.5</v>
       </c>
       <c r="E338" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F338" t="n">
-        <v>4.7</v>
+        <v>5.4</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17339,7 +17339,7 @@
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0.263</v>
+        <v>0.265</v>
       </c>
       <c r="L338" t="n">
         <v>2</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-17T05:03:19Z</t>
+          <t>2026-10-17T11:03:36Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E339" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F339" t="n">
-        <v>3.5</v>
+        <v>4.9</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.263</v>
+        <v>0.265</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-17 19:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -14664,17 +14664,17 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>13.2</v>
+        <v>12.3</v>
       </c>
       <c r="E285" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F285" t="n">
-        <v>4</v>
+        <v>5.8</v>
       </c>
       <c r="G285" t="n">
         <v>0</v>
@@ -14714,17 +14714,17 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>12.8</v>
+        <v>11.9</v>
       </c>
       <c r="E286" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F286" t="n">
-        <v>5.4</v>
+        <v>5</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
@@ -14764,17 +14764,17 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>12.5</v>
+        <v>11.6</v>
       </c>
       <c r="E287" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F287" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="G287" t="n">
         <v>0</v>
@@ -14789,7 +14789,7 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
-        <v>0.286</v>
+        <v>0.285</v>
       </c>
       <c r="L287" t="n">
         <v>6</v>
@@ -14814,17 +14814,17 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>12.1</v>
+        <v>11.2</v>
       </c>
       <c r="E288" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F288" t="n">
-        <v>3.6</v>
+        <v>5.8</v>
       </c>
       <c r="G288" t="n">
         <v>0</v>
@@ -14839,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
-        <v>0.286</v>
+        <v>0.285</v>
       </c>
       <c r="L288" t="n">
         <v>6</v>
@@ -14864,17 +14864,17 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="E289" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F289" t="n">
-        <v>4.3</v>
+        <v>6.1</v>
       </c>
       <c r="G289" t="n">
         <v>0</v>
@@ -14914,17 +14914,17 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="E290" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F290" t="n">
-        <v>1.8</v>
+        <v>6.1</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
@@ -14964,17 +14964,17 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="E291" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F291" t="n">
-        <v>1.8</v>
+        <v>7.6</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
@@ -15014,17 +15014,17 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>10.9</v>
+        <v>11.4</v>
       </c>
       <c r="E292" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F292" t="n">
-        <v>4.3</v>
+        <v>7.9</v>
       </c>
       <c r="G292" t="n">
         <v>0</v>
@@ -15064,17 +15064,17 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>10.8</v>
+        <v>11.4</v>
       </c>
       <c r="E293" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="F293" t="n">
-        <v>2.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G293" t="n">
         <v>0</v>
@@ -15114,17 +15114,17 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>10.9</v>
+        <v>11.2</v>
       </c>
       <c r="E294" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="F294" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G294" t="n">
         <v>0</v>
@@ -15164,17 +15164,17 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="E295" t="n">
         <v>47</v>
       </c>
       <c r="F295" t="n">
-        <v>11.9</v>
+        <v>11.5</v>
       </c>
       <c r="G295" t="n">
         <v>0</v>
@@ -15214,17 +15214,17 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D296" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E296" t="n">
+        <v>51</v>
+      </c>
+      <c r="F296" t="n">
         <v>10.8</v>
-      </c>
-      <c r="E296" t="n">
-        <v>52</v>
-      </c>
-      <c r="F296" t="n">
-        <v>7.9</v>
       </c>
       <c r="G296" t="n">
         <v>0</v>
@@ -15264,17 +15264,17 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>10.6</v>
+        <v>10.9</v>
       </c>
       <c r="E297" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F297" t="n">
-        <v>4.3</v>
+        <v>6.8</v>
       </c>
       <c r="G297" t="n">
         <v>0</v>
@@ -15314,23 +15314,23 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="E298" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F298" t="n">
         <v>6.1</v>
       </c>
       <c r="G298" t="n">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="H298" t="n">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="I298" t="n">
         <v>0</v>
@@ -15364,20 +15364,20 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="E299" t="n">
         <v>52</v>
       </c>
       <c r="F299" t="n">
-        <v>8.300000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="G299" t="n">
-        <v>135</v>
+        <v>51</v>
       </c>
       <c r="H299" t="n">
         <v>100</v>
@@ -15389,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="K299" t="n">
-        <v>0.284</v>
+        <v>0.283</v>
       </c>
       <c r="L299" t="n">
         <v>7</v>
@@ -15414,20 +15414,20 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>12.6</v>
+        <v>12.2</v>
       </c>
       <c r="E300" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="F300" t="n">
-        <v>11.5</v>
+        <v>10.4</v>
       </c>
       <c r="G300" t="n">
-        <v>108</v>
+        <v>73</v>
       </c>
       <c r="H300" t="n">
         <v>100</v>
@@ -15464,20 +15464,20 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="E301" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F301" t="n">
-        <v>9</v>
+        <v>10.1</v>
       </c>
       <c r="G301" t="n">
-        <v>99</v>
+        <v>61</v>
       </c>
       <c r="H301" t="n">
         <v>100</v>
@@ -15514,23 +15514,23 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>15.9</v>
+        <v>15.1</v>
       </c>
       <c r="E302" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F302" t="n">
-        <v>5</v>
+        <v>8.6</v>
       </c>
       <c r="G302" t="n">
-        <v>388</v>
+        <v>331</v>
       </c>
       <c r="H302" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="I302" t="n">
         <v>0</v>
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>17.8</v>
+        <v>17.3</v>
       </c>
       <c r="E303" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F303" t="n">
-        <v>3.2</v>
+        <v>6.8</v>
       </c>
       <c r="G303" t="n">
-        <v>520</v>
+        <v>547</v>
       </c>
       <c r="H303" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15614,23 +15614,23 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>19.1</v>
+        <v>18.7</v>
       </c>
       <c r="E304" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F304" t="n">
-        <v>3.6</v>
+        <v>5.8</v>
       </c>
       <c r="G304" t="n">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H304" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -15639,7 +15639,7 @@
         <v>0</v>
       </c>
       <c r="K304" t="n">
-        <v>0.278</v>
+        <v>0.277</v>
       </c>
       <c r="L304" t="n">
         <v>7</v>
@@ -15664,23 +15664,23 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>20.1</v>
+        <v>19.7</v>
       </c>
       <c r="E305" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F305" t="n">
-        <v>5.4</v>
+        <v>6.5</v>
       </c>
       <c r="G305" t="n">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="H305" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -15714,23 +15714,23 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>20.6</v>
+        <v>20</v>
       </c>
       <c r="E306" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F306" t="n">
-        <v>11.2</v>
+        <v>6.5</v>
       </c>
       <c r="G306" t="n">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="H306" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
@@ -15739,7 +15739,7 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L306" t="n">
         <v>7</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>20</v>
+        <v>19.9</v>
       </c>
       <c r="E307" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F307" t="n">
-        <v>10.8</v>
+        <v>6.8</v>
       </c>
       <c r="G307" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H307" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>17.6</v>
+        <v>17.5</v>
       </c>
       <c r="E308" t="n">
         <v>36</v>
       </c>
       <c r="F308" t="n">
-        <v>9.699999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="G308" t="n">
         <v>30</v>
       </c>
       <c r="H308" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15839,7 +15839,7 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0.274</v>
+        <v>0.273</v>
       </c>
       <c r="L308" t="n">
         <v>7</v>
@@ -15864,23 +15864,23 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D309" t="n">
         <v>15</v>
       </c>
       <c r="E309" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F309" t="n">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>0.274</v>
+        <v>0.273</v>
       </c>
       <c r="L309" t="n">
         <v>7</v>
@@ -15914,23 +15914,23 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D310" t="n">
         <v>13.1</v>
       </c>
       <c r="E310" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F310" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15939,7 +15939,7 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>0.274</v>
+        <v>0.273</v>
       </c>
       <c r="L310" t="n">
         <v>7</v>
@@ -15964,23 +15964,23 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="E311" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F311" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I311" t="n">
         <v>0</v>
@@ -15989,7 +15989,7 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>0.274</v>
+        <v>0.273</v>
       </c>
       <c r="L311" t="n">
         <v>7</v>
@@ -16014,17 +16014,17 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>10.2</v>
+        <v>10.5</v>
       </c>
       <c r="E312" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F312" t="n">
-        <v>9</v>
+        <v>5.4</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -16039,7 +16039,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0.274</v>
+        <v>0.273</v>
       </c>
       <c r="L312" t="n">
         <v>7</v>
@@ -16064,17 +16064,17 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>9.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="E313" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F313" t="n">
-        <v>5.4</v>
+        <v>7.2</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.274</v>
+        <v>0.273</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,14 +16114,14 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9.5</v>
+        <v>9.1</v>
       </c>
       <c r="E314" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F314" t="n">
         <v>5</v>
@@ -16164,17 +16164,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="E315" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F315" t="n">
-        <v>6.5</v>
+        <v>2.9</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L315" t="n">
         <v>1</v>
@@ -16214,23 +16214,23 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E316" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="F316" t="n">
-        <v>5.4</v>
+        <v>2.9</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I316" t="n">
         <v>0</v>
@@ -16239,7 +16239,7 @@
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L316" t="n">
         <v>1</v>
@@ -16264,17 +16264,17 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>7.6</v>
+        <v>8.1</v>
       </c>
       <c r="E317" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F317" t="n">
-        <v>5</v>
+        <v>2.9</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
@@ -16289,7 +16289,7 @@
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L317" t="n">
         <v>1</v>
@@ -16314,17 +16314,17 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>7.1</v>
+        <v>7.6</v>
       </c>
       <c r="E318" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F318" t="n">
-        <v>6.1</v>
+        <v>3.6</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
@@ -16339,7 +16339,7 @@
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L318" t="n">
         <v>1</v>
@@ -16364,17 +16364,17 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="E319" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="F319" t="n">
-        <v>4.7</v>
+        <v>9</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
@@ -16389,7 +16389,7 @@
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L319" t="n">
         <v>1</v>
@@ -16414,17 +16414,17 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="E320" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="F320" t="n">
-        <v>3.6</v>
+        <v>7.2</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
@@ -16439,7 +16439,7 @@
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L320" t="n">
         <v>1</v>
@@ -16464,17 +16464,17 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="E321" t="n">
         <v>92</v>
       </c>
       <c r="F321" t="n">
-        <v>5</v>
+        <v>2.9</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
@@ -16489,7 +16489,7 @@
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L321" t="n">
         <v>1</v>
@@ -16514,20 +16514,20 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="E322" t="n">
         <v>90</v>
       </c>
       <c r="F322" t="n">
-        <v>6.5</v>
+        <v>0.4</v>
       </c>
       <c r="G322" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H322" t="n">
         <v>0</v>
@@ -16539,7 +16539,7 @@
         <v>0</v>
       </c>
       <c r="K322" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L322" t="n">
         <v>1</v>
@@ -16564,20 +16564,20 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="E323" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F323" t="n">
-        <v>6.1</v>
+        <v>1.8</v>
       </c>
       <c r="G323" t="n">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H323" t="n">
         <v>0</v>
@@ -16589,7 +16589,7 @@
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L323" t="n">
         <v>1</v>
@@ -16614,20 +16614,20 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>11.9</v>
+        <v>11.2</v>
       </c>
       <c r="E324" t="n">
         <v>64</v>
       </c>
       <c r="F324" t="n">
-        <v>4.7</v>
+        <v>2.5</v>
       </c>
       <c r="G324" t="n">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -16639,7 +16639,7 @@
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0.274</v>
+        <v>0.273</v>
       </c>
       <c r="L324" t="n">
         <v>1</v>
@@ -16664,23 +16664,23 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>14.7</v>
+        <v>14.4</v>
       </c>
       <c r="E325" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F325" t="n">
-        <v>6.5</v>
+        <v>3.2</v>
       </c>
       <c r="G325" t="n">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="H325" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -16689,7 +16689,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>0.273</v>
+        <v>0.272</v>
       </c>
       <c r="L325" t="n">
         <v>1</v>
@@ -16714,23 +16714,23 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>17</v>
+        <v>16.9</v>
       </c>
       <c r="E326" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F326" t="n">
-        <v>8.6</v>
+        <v>4</v>
       </c>
       <c r="G326" t="n">
-        <v>487</v>
+        <v>533</v>
       </c>
       <c r="H326" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I326" t="n">
         <v>0</v>
@@ -16739,7 +16739,7 @@
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>0.272</v>
+        <v>0.271</v>
       </c>
       <c r="L326" t="n">
         <v>1</v>
@@ -16764,23 +16764,23 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>18.5</v>
+        <v>18.4</v>
       </c>
       <c r="E327" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F327" t="n">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="G327" t="n">
-        <v>504</v>
+        <v>556</v>
       </c>
       <c r="H327" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="I327" t="n">
         <v>0</v>
@@ -16789,7 +16789,7 @@
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>0.27</v>
+        <v>0.269</v>
       </c>
       <c r="L327" t="n">
         <v>1</v>
@@ -16814,20 +16814,20 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>19.5</v>
+        <v>19.9</v>
       </c>
       <c r="E328" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F328" t="n">
-        <v>10.1</v>
+        <v>7.2</v>
       </c>
       <c r="G328" t="n">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
@@ -16839,7 +16839,7 @@
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0.268</v>
+        <v>0.267</v>
       </c>
       <c r="L328" t="n">
         <v>1</v>
@@ -16864,23 +16864,23 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>20</v>
+        <v>20.3</v>
       </c>
       <c r="E329" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F329" t="n">
-        <v>10.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G329" t="n">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="H329" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I329" t="n">
         <v>0</v>
@@ -16889,7 +16889,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>0.267</v>
+        <v>0.265</v>
       </c>
       <c r="L329" t="n">
         <v>1</v>
@@ -16914,23 +16914,23 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>20</v>
+        <v>20.2</v>
       </c>
       <c r="E330" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F330" t="n">
-        <v>10.1</v>
+        <v>6.8</v>
       </c>
       <c r="G330" t="n">
-        <v>305</v>
+        <v>315</v>
       </c>
       <c r="H330" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="I330" t="n">
         <v>0</v>
@@ -16939,7 +16939,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>0.265</v>
+        <v>0.264</v>
       </c>
       <c r="L330" t="n">
         <v>1</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>18.6</v>
+        <v>19.7</v>
       </c>
       <c r="E331" t="n">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="F331" t="n">
-        <v>8.9</v>
+        <v>6.8</v>
       </c>
       <c r="G331" t="n">
-        <v>138.8</v>
+        <v>163</v>
       </c>
       <c r="H331" t="n">
-        <v>86</v>
+        <v>0</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -16989,7 +16989,7 @@
         <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>0.265</v>
+        <v>0.264</v>
       </c>
       <c r="L331" t="n">
         <v>1</v>
@@ -17014,23 +17014,23 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>15.7</v>
+        <v>17.4</v>
       </c>
       <c r="E332" t="n">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="F332" t="n">
-        <v>7.5</v>
+        <v>6.8</v>
       </c>
       <c r="G332" t="n">
-        <v>22.5</v>
+        <v>30</v>
       </c>
       <c r="H332" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -17039,7 +17039,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>0.265</v>
+        <v>0.263</v>
       </c>
       <c r="L332" t="n">
         <v>1</v>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>14</v>
+        <v>14.8</v>
       </c>
       <c r="E333" t="n">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="F333" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17089,7 +17089,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>0.265</v>
+        <v>0.263</v>
       </c>
       <c r="L333" t="n">
         <v>1</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="E334" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="F334" t="n">
-        <v>6.4</v>
+        <v>9.4</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17139,7 +17139,7 @@
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>0.265</v>
+        <v>0.263</v>
       </c>
       <c r="L334" t="n">
         <v>1</v>
@@ -17164,23 +17164,23 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11.9</v>
+        <v>11.6</v>
       </c>
       <c r="E335" t="n">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="F335" t="n">
-        <v>5.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="I335" t="n">
         <v>0</v>
@@ -17189,7 +17189,7 @@
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>0.265</v>
+        <v>0.263</v>
       </c>
       <c r="L335" t="n">
         <v>1</v>
@@ -17214,23 +17214,23 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>11.5</v>
+        <v>10.4</v>
       </c>
       <c r="E336" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="F336" t="n">
-        <v>5.2</v>
+        <v>9.4</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17239,7 +17239,7 @@
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0.265</v>
+        <v>0.263</v>
       </c>
       <c r="L336" t="n">
         <v>1</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="E337" t="n">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="F337" t="n">
-        <v>5.4</v>
+        <v>7.2</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17289,7 +17289,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>0.265</v>
+        <v>0.264</v>
       </c>
       <c r="L337" t="n">
         <v>1</v>
@@ -17314,23 +17314,23 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="E338" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="F338" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17339,7 +17339,7 @@
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0.265</v>
+        <v>0.264</v>
       </c>
       <c r="L338" t="n">
         <v>2</v>
@@ -17364,17 +17364,17 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-17T11:03:36Z</t>
+          <t>2026-10-17T17:03:21Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>9.800000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="E339" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="F339" t="n">
-        <v>4.9</v>
+        <v>6.5</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.265</v>
+        <v>0.264</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
prognoza biciklista (zvanicna): 2026-10-18 01:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -5014,7 +5014,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -14964,11 +14964,11 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="E291" t="n">
         <v>43</v>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
-        <v>0.285</v>
+        <v>0.284</v>
       </c>
       <c r="L291" t="n">
         <v>7</v>
@@ -15014,17 +15014,17 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="E292" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F292" t="n">
-        <v>7.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G292" t="n">
         <v>0</v>
@@ -15039,7 +15039,7 @@
         <v>0</v>
       </c>
       <c r="K292" t="n">
-        <v>0.285</v>
+        <v>0.284</v>
       </c>
       <c r="L292" t="n">
         <v>7</v>
@@ -15064,17 +15064,17 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
       <c r="E293" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F293" t="n">
-        <v>8.300000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="G293" t="n">
         <v>0</v>
@@ -15089,7 +15089,7 @@
         <v>0</v>
       </c>
       <c r="K293" t="n">
-        <v>0.285</v>
+        <v>0.283</v>
       </c>
       <c r="L293" t="n">
         <v>7</v>
@@ -15114,14 +15114,14 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="E294" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F294" t="n">
         <v>9</v>
@@ -15139,7 +15139,7 @@
         <v>0</v>
       </c>
       <c r="K294" t="n">
-        <v>0.285</v>
+        <v>0.283</v>
       </c>
       <c r="L294" t="n">
         <v>7</v>
@@ -15164,17 +15164,17 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D295" t="n">
         <v>11.2</v>
       </c>
       <c r="E295" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F295" t="n">
-        <v>11.5</v>
+        <v>7.9</v>
       </c>
       <c r="G295" t="n">
         <v>0</v>
@@ -15189,7 +15189,7 @@
         <v>0</v>
       </c>
       <c r="K295" t="n">
-        <v>0.284</v>
+        <v>0.283</v>
       </c>
       <c r="L295" t="n">
         <v>7</v>
@@ -15214,17 +15214,17 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>11.3</v>
+        <v>11.1</v>
       </c>
       <c r="E296" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F296" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
       <c r="G296" t="n">
         <v>0</v>
@@ -15239,7 +15239,7 @@
         <v>0</v>
       </c>
       <c r="K296" t="n">
-        <v>0.284</v>
+        <v>0.283</v>
       </c>
       <c r="L296" t="n">
         <v>7</v>
@@ -15264,17 +15264,17 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D297" t="n">
         <v>10.9</v>
       </c>
       <c r="E297" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F297" t="n">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="G297" t="n">
         <v>0</v>
@@ -15289,7 +15289,7 @@
         <v>0</v>
       </c>
       <c r="K297" t="n">
-        <v>0.284</v>
+        <v>0.282</v>
       </c>
       <c r="L297" t="n">
         <v>7</v>
@@ -15314,20 +15314,20 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>10.8</v>
+        <v>11</v>
       </c>
       <c r="E298" t="n">
         <v>53</v>
       </c>
       <c r="F298" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="G298" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="H298" t="n">
         <v>100</v>
@@ -15339,7 +15339,7 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
-        <v>0.284</v>
+        <v>0.282</v>
       </c>
       <c r="L298" t="n">
         <v>7</v>
@@ -15364,20 +15364,20 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="E299" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F299" t="n">
-        <v>5.8</v>
+        <v>9.4</v>
       </c>
       <c r="G299" t="n">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="H299" t="n">
         <v>100</v>
@@ -15389,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="K299" t="n">
-        <v>0.283</v>
+        <v>0.282</v>
       </c>
       <c r="L299" t="n">
         <v>7</v>
@@ -15414,20 +15414,20 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>12.2</v>
+        <v>12.1</v>
       </c>
       <c r="E300" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F300" t="n">
-        <v>10.4</v>
+        <v>6.5</v>
       </c>
       <c r="G300" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="H300" t="n">
         <v>100</v>
@@ -15439,7 +15439,7 @@
         <v>0</v>
       </c>
       <c r="K300" t="n">
-        <v>0.283</v>
+        <v>0.282</v>
       </c>
       <c r="L300" t="n">
         <v>7</v>
@@ -15464,23 +15464,23 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>12.6</v>
+        <v>13</v>
       </c>
       <c r="E301" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F301" t="n">
-        <v>10.1</v>
+        <v>4.7</v>
       </c>
       <c r="G301" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="H301" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I301" t="n">
         <v>0</v>
@@ -15489,7 +15489,7 @@
         <v>0</v>
       </c>
       <c r="K301" t="n">
-        <v>0.282</v>
+        <v>0.281</v>
       </c>
       <c r="L301" t="n">
         <v>7</v>
@@ -15514,23 +15514,23 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>15.1</v>
+        <v>16.2</v>
       </c>
       <c r="E302" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F302" t="n">
-        <v>8.6</v>
+        <v>7.2</v>
       </c>
       <c r="G302" t="n">
-        <v>331</v>
+        <v>460</v>
       </c>
       <c r="H302" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I302" t="n">
         <v>0</v>
@@ -15539,7 +15539,7 @@
         <v>0</v>
       </c>
       <c r="K302" t="n">
-        <v>0.281</v>
+        <v>0.28</v>
       </c>
       <c r="L302" t="n">
         <v>7</v>
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>17.3</v>
+        <v>18.2</v>
       </c>
       <c r="E303" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="F303" t="n">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="G303" t="n">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="H303" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15614,23 +15614,23 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>18.7</v>
+        <v>19.5</v>
       </c>
       <c r="E304" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="F304" t="n">
-        <v>5.8</v>
+        <v>7.9</v>
       </c>
       <c r="G304" t="n">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="H304" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -15664,23 +15664,23 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="E305" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="F305" t="n">
-        <v>6.5</v>
+        <v>9</v>
       </c>
       <c r="G305" t="n">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="H305" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -15714,23 +15714,23 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="E306" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F306" t="n">
-        <v>6.5</v>
+        <v>10.1</v>
       </c>
       <c r="G306" t="n">
         <v>311</v>
       </c>
       <c r="H306" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="E307" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F307" t="n">
-        <v>6.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G307" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H307" t="n">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15789,7 +15789,7 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0.274</v>
+        <v>0.273</v>
       </c>
       <c r="L307" t="n">
         <v>7</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>17.5</v>
+        <v>17.9</v>
       </c>
       <c r="E308" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F308" t="n">
-        <v>7.2</v>
+        <v>6.1</v>
       </c>
       <c r="G308" t="n">
         <v>30</v>
       </c>
       <c r="H308" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15864,23 +15864,23 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="E309" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F309" t="n">
-        <v>6.1</v>
+        <v>4</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15914,23 +15914,23 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>13.1</v>
+        <v>13.6</v>
       </c>
       <c r="E310" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F310" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H310" t="n">
         <v>4</v>
-      </c>
-      <c r="G310" t="n">
-        <v>0</v>
-      </c>
-      <c r="H310" t="n">
-        <v>23</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15964,23 +15964,23 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>11.9</v>
+        <v>12</v>
       </c>
       <c r="E311" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F311" t="n">
-        <v>0.4</v>
+        <v>6.1</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I311" t="n">
         <v>0</v>
@@ -16014,17 +16014,17 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="E312" t="n">
         <v>61</v>
       </c>
       <c r="F312" t="n">
-        <v>5.4</v>
+        <v>3.2</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -16039,7 +16039,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0.273</v>
+        <v>0.274</v>
       </c>
       <c r="L312" t="n">
         <v>7</v>
@@ -16064,17 +16064,17 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>9.5</v>
+        <v>10.2</v>
       </c>
       <c r="E313" t="n">
         <v>67</v>
       </c>
       <c r="F313" t="n">
-        <v>7.2</v>
+        <v>2.9</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.273</v>
+        <v>0.274</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,17 +16114,17 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9.1</v>
+        <v>9.6</v>
       </c>
       <c r="E314" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F314" t="n">
-        <v>5</v>
+        <v>1.1</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -16164,17 +16164,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D315" t="n">
         <v>9.1</v>
       </c>
       <c r="E315" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F315" t="n">
-        <v>2.9</v>
+        <v>1.1</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -16214,23 +16214,23 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>8.699999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E316" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F316" t="n">
-        <v>2.9</v>
+        <v>2.5</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="I316" t="n">
         <v>0</v>
@@ -16264,23 +16264,23 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>8.1</v>
+        <v>7.7</v>
       </c>
       <c r="E317" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="F317" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I317" t="n">
         <v>0</v>
@@ -16314,23 +16314,23 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>7.6</v>
+        <v>7</v>
       </c>
       <c r="E318" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="F318" t="n">
-        <v>3.6</v>
+        <v>6.8</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I318" t="n">
         <v>0</v>
@@ -16364,23 +16364,23 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>7</v>
+        <v>6.6</v>
       </c>
       <c r="E319" t="n">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="F319" t="n">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I319" t="n">
         <v>0</v>
@@ -16414,17 +16414,17 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="E320" t="n">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="F320" t="n">
-        <v>7.2</v>
+        <v>3.2</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
@@ -16464,17 +16464,17 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>6.1</v>
+        <v>5.6</v>
       </c>
       <c r="E321" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F321" t="n">
-        <v>2.9</v>
+        <v>1.1</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
@@ -16514,17 +16514,17 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>6.5</v>
+        <v>5.9</v>
       </c>
       <c r="E322" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F322" t="n">
-        <v>0.4</v>
+        <v>4.7</v>
       </c>
       <c r="G322" t="n">
         <v>45</v>
@@ -16564,17 +16564,17 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="E323" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F323" t="n">
-        <v>1.8</v>
+        <v>3.6</v>
       </c>
       <c r="G323" t="n">
         <v>186</v>
@@ -16614,20 +16614,20 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>11.2</v>
+        <v>11.7</v>
       </c>
       <c r="E324" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F324" t="n">
-        <v>2.5</v>
+        <v>5.8</v>
       </c>
       <c r="G324" t="n">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -16639,7 +16639,7 @@
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0.273</v>
+        <v>0.274</v>
       </c>
       <c r="L324" t="n">
         <v>1</v>
@@ -16664,23 +16664,23 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>14.4</v>
+        <v>14.2</v>
       </c>
       <c r="E325" t="n">
         <v>51</v>
       </c>
       <c r="F325" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="G325" t="n">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="H325" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -16689,7 +16689,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>0.272</v>
+        <v>0.273</v>
       </c>
       <c r="L325" t="n">
         <v>1</v>
@@ -16714,23 +16714,23 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>16.9</v>
+        <v>16.5</v>
       </c>
       <c r="E326" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F326" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G326" t="n">
-        <v>533</v>
+        <v>512</v>
       </c>
       <c r="H326" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="I326" t="n">
         <v>0</v>
@@ -16764,20 +16764,20 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>18.4</v>
+        <v>18.5</v>
       </c>
       <c r="E327" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F327" t="n">
-        <v>3.2</v>
+        <v>6.8</v>
       </c>
       <c r="G327" t="n">
-        <v>556</v>
+        <v>542</v>
       </c>
       <c r="H327" t="n">
         <v>0</v>
@@ -16814,17 +16814,17 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>19.9</v>
+        <v>19.4</v>
       </c>
       <c r="E328" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F328" t="n">
-        <v>7.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G328" t="n">
         <v>525</v>
@@ -16864,23 +16864,23 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>20.3</v>
+        <v>19.7</v>
       </c>
       <c r="E329" t="n">
         <v>34</v>
       </c>
       <c r="F329" t="n">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="G329" t="n">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="H329" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="I329" t="n">
         <v>0</v>
@@ -16889,7 +16889,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>0.265</v>
+        <v>0.266</v>
       </c>
       <c r="L329" t="n">
         <v>1</v>
@@ -16914,20 +16914,20 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>20.2</v>
+        <v>19.8</v>
       </c>
       <c r="E330" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F330" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="G330" t="n">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="H330" t="n">
         <v>0</v>
@@ -16939,7 +16939,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>0.264</v>
+        <v>0.265</v>
       </c>
       <c r="L330" t="n">
         <v>1</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>19.7</v>
+        <v>19.4</v>
       </c>
       <c r="E331" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F331" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="G331" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H331" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -17014,23 +17014,23 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>17.4</v>
+        <v>17.2</v>
       </c>
       <c r="E332" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F332" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="G332" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H332" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -17039,7 +17039,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>0.263</v>
+        <v>0.264</v>
       </c>
       <c r="L332" t="n">
         <v>1</v>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>14.8</v>
+        <v>15.1</v>
       </c>
       <c r="E333" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F333" t="n">
-        <v>9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17089,7 +17089,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>0.263</v>
+        <v>0.264</v>
       </c>
       <c r="L333" t="n">
         <v>1</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>13</v>
+        <v>13.6</v>
       </c>
       <c r="E334" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F334" t="n">
-        <v>9.4</v>
+        <v>11.2</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17139,7 +17139,7 @@
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>0.263</v>
+        <v>0.264</v>
       </c>
       <c r="L334" t="n">
         <v>1</v>
@@ -17164,23 +17164,23 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11.6</v>
+        <v>11.9</v>
       </c>
       <c r="E335" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F335" t="n">
-        <v>9.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I335" t="n">
         <v>0</v>
@@ -17189,7 +17189,7 @@
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>0.263</v>
+        <v>0.264</v>
       </c>
       <c r="L335" t="n">
         <v>1</v>
@@ -17214,23 +17214,23 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="E336" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F336" t="n">
-        <v>9.4</v>
+        <v>6.5</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17239,7 +17239,7 @@
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0.263</v>
+        <v>0.264</v>
       </c>
       <c r="L336" t="n">
         <v>1</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>9.5</v>
+        <v>9.6</v>
       </c>
       <c r="E337" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F337" t="n">
-        <v>7.2</v>
+        <v>6.1</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17314,23 +17314,23 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="E338" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F338" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-17T17:03:21Z</t>
+          <t>2026-10-17T23:03:48Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="E339" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F339" t="n">
-        <v>6.5</v>
+        <v>4.7</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.264</v>
+        <v>0.265</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-18 07:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N339"/>
+  <dimension ref="A1:N363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -15264,17 +15264,17 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="E297" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F297" t="n">
-        <v>5.8</v>
+        <v>7.9</v>
       </c>
       <c r="G297" t="n">
         <v>0</v>
@@ -15289,7 +15289,7 @@
         <v>0</v>
       </c>
       <c r="K297" t="n">
-        <v>0.282</v>
+        <v>0.281</v>
       </c>
       <c r="L297" t="n">
         <v>7</v>
@@ -15314,20 +15314,20 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="E298" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F298" t="n">
-        <v>5.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G298" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H298" t="n">
         <v>100</v>
@@ -15339,7 +15339,7 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
-        <v>0.282</v>
+        <v>0.281</v>
       </c>
       <c r="L298" t="n">
         <v>7</v>
@@ -15364,20 +15364,20 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="E299" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F299" t="n">
-        <v>9.4</v>
+        <v>6.8</v>
       </c>
       <c r="G299" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="H299" t="n">
         <v>100</v>
@@ -15389,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="K299" t="n">
-        <v>0.282</v>
+        <v>0.281</v>
       </c>
       <c r="L299" t="n">
         <v>7</v>
@@ -15414,20 +15414,20 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
       <c r="E300" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F300" t="n">
-        <v>6.5</v>
+        <v>10.8</v>
       </c>
       <c r="G300" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="H300" t="n">
         <v>100</v>
@@ -15439,7 +15439,7 @@
         <v>0</v>
       </c>
       <c r="K300" t="n">
-        <v>0.282</v>
+        <v>0.28</v>
       </c>
       <c r="L300" t="n">
         <v>7</v>
@@ -15464,23 +15464,23 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>13</v>
+        <v>11.9</v>
       </c>
       <c r="E301" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F301" t="n">
-        <v>4.7</v>
+        <v>9</v>
       </c>
       <c r="G301" t="n">
-        <v>69</v>
+        <v>32</v>
       </c>
       <c r="H301" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="I301" t="n">
         <v>0</v>
@@ -15489,7 +15489,7 @@
         <v>0</v>
       </c>
       <c r="K301" t="n">
-        <v>0.281</v>
+        <v>0.279</v>
       </c>
       <c r="L301" t="n">
         <v>7</v>
@@ -15514,23 +15514,23 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>16.2</v>
+        <v>14.7</v>
       </c>
       <c r="E302" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F302" t="n">
-        <v>7.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G302" t="n">
-        <v>460</v>
+        <v>407</v>
       </c>
       <c r="H302" t="n">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="I302" t="n">
         <v>0</v>
@@ -15539,7 +15539,7 @@
         <v>0</v>
       </c>
       <c r="K302" t="n">
-        <v>0.28</v>
+        <v>0.278</v>
       </c>
       <c r="L302" t="n">
         <v>7</v>
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>18.2</v>
+        <v>17.7</v>
       </c>
       <c r="E303" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F303" t="n">
-        <v>5.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G303" t="n">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="H303" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15589,7 +15589,7 @@
         <v>0</v>
       </c>
       <c r="K303" t="n">
-        <v>0.279</v>
+        <v>0.276</v>
       </c>
       <c r="L303" t="n">
         <v>7</v>
@@ -15614,23 +15614,23 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>19.5</v>
+        <v>19</v>
       </c>
       <c r="E304" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F304" t="n">
-        <v>7.9</v>
+        <v>7.6</v>
       </c>
       <c r="G304" t="n">
-        <v>521</v>
+        <v>515</v>
       </c>
       <c r="H304" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -15639,7 +15639,7 @@
         <v>0</v>
       </c>
       <c r="K304" t="n">
-        <v>0.277</v>
+        <v>0.274</v>
       </c>
       <c r="L304" t="n">
         <v>7</v>
@@ -15664,23 +15664,23 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>20.3</v>
+        <v>19.9</v>
       </c>
       <c r="E305" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F305" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G305" t="n">
-        <v>435</v>
+        <v>428</v>
       </c>
       <c r="H305" t="n">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -15689,7 +15689,7 @@
         <v>0</v>
       </c>
       <c r="K305" t="n">
-        <v>0.276</v>
+        <v>0.271</v>
       </c>
       <c r="L305" t="n">
         <v>7</v>
@@ -15714,23 +15714,23 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>20.5</v>
+        <v>20.3</v>
       </c>
       <c r="E306" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F306" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G306" t="n">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="H306" t="n">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="I306" t="n">
         <v>0</v>
@@ -15739,7 +15739,7 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>0.274</v>
+        <v>0.27</v>
       </c>
       <c r="L306" t="n">
         <v>7</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>20.1</v>
+        <v>20.2</v>
       </c>
       <c r="E307" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F307" t="n">
-        <v>9.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="G307" t="n">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H307" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15789,7 +15789,7 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0.273</v>
+        <v>0.269</v>
       </c>
       <c r="L307" t="n">
         <v>7</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="E308" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="F308" t="n">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="G308" t="n">
         <v>30</v>
       </c>
       <c r="H308" t="n">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15839,7 +15839,7 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0.273</v>
+        <v>0.269</v>
       </c>
       <c r="L308" t="n">
         <v>7</v>
@@ -15864,23 +15864,23 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D309" t="n">
         <v>15.5</v>
       </c>
       <c r="E309" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F309" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="G309" t="n">
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>0.273</v>
+        <v>0.269</v>
       </c>
       <c r="L309" t="n">
         <v>7</v>
@@ -15914,23 +15914,23 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>13.6</v>
+        <v>13.5</v>
       </c>
       <c r="E310" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="F310" t="n">
-        <v>3.6</v>
+        <v>5.4</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15939,7 +15939,7 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>0.273</v>
+        <v>0.269</v>
       </c>
       <c r="L310" t="n">
         <v>7</v>
@@ -15964,17 +15964,17 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="E311" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="F311" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
@@ -15989,7 +15989,7 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>0.273</v>
+        <v>0.269</v>
       </c>
       <c r="L311" t="n">
         <v>7</v>
@@ -16014,17 +16014,17 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="E312" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="F312" t="n">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -16039,7 +16039,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0.274</v>
+        <v>0.269</v>
       </c>
       <c r="L312" t="n">
         <v>7</v>
@@ -16064,17 +16064,17 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D313" t="n">
         <v>10.2</v>
       </c>
       <c r="E313" t="n">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="F313" t="n">
-        <v>2.9</v>
+        <v>6.5</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.274</v>
+        <v>0.269</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,17 +16114,17 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E314" t="n">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="F314" t="n">
-        <v>1.1</v>
+        <v>5.8</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -16139,7 +16139,7 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0.274</v>
+        <v>0.269</v>
       </c>
       <c r="L314" t="n">
         <v>1</v>
@@ -16164,17 +16164,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="E315" t="n">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="F315" t="n">
-        <v>1.1</v>
+        <v>5.8</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0.274</v>
+        <v>0.269</v>
       </c>
       <c r="L315" t="n">
         <v>1</v>
@@ -16214,23 +16214,23 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D316" t="n">
         <v>8.199999999999999</v>
       </c>
       <c r="E316" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="F316" t="n">
-        <v>2.5</v>
+        <v>5.8</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="I316" t="n">
         <v>0</v>
@@ -16239,7 +16239,7 @@
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>0.274</v>
+        <v>0.269</v>
       </c>
       <c r="L316" t="n">
         <v>1</v>
@@ -16264,23 +16264,23 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
       <c r="E317" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="F317" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I317" t="n">
         <v>0</v>
@@ -16289,7 +16289,7 @@
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0.274</v>
+        <v>0.269</v>
       </c>
       <c r="L317" t="n">
         <v>1</v>
@@ -16314,23 +16314,23 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
       <c r="E318" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="F318" t="n">
-        <v>6.8</v>
+        <v>4</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I318" t="n">
         <v>0</v>
@@ -16339,7 +16339,7 @@
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>0.274</v>
+        <v>0.27</v>
       </c>
       <c r="L318" t="n">
         <v>1</v>
@@ -16364,23 +16364,23 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="E319" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="F319" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="I319" t="n">
         <v>0</v>
@@ -16389,7 +16389,7 @@
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>0.274</v>
+        <v>0.27</v>
       </c>
       <c r="L319" t="n">
         <v>1</v>
@@ -16414,23 +16414,23 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>6</v>
+        <v>6.2</v>
       </c>
       <c r="E320" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F320" t="n">
-        <v>3.2</v>
+        <v>1.1</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I320" t="n">
         <v>0</v>
@@ -16439,7 +16439,7 @@
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>0.274</v>
+        <v>0.27</v>
       </c>
       <c r="L320" t="n">
         <v>1</v>
@@ -16464,17 +16464,17 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="E321" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F321" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
@@ -16489,7 +16489,7 @@
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>0.274</v>
+        <v>0.27</v>
       </c>
       <c r="L321" t="n">
         <v>1</v>
@@ -16514,17 +16514,17 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="E322" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="F322" t="n">
-        <v>4.7</v>
+        <v>6.1</v>
       </c>
       <c r="G322" t="n">
         <v>45</v>
@@ -16539,7 +16539,7 @@
         <v>0</v>
       </c>
       <c r="K322" t="n">
-        <v>0.274</v>
+        <v>0.27</v>
       </c>
       <c r="L322" t="n">
         <v>1</v>
@@ -16564,20 +16564,20 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E323" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F323" t="n">
         <v>3.6</v>
       </c>
       <c r="G323" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H323" t="n">
         <v>0</v>
@@ -16589,7 +16589,7 @@
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>0.274</v>
+        <v>0.27</v>
       </c>
       <c r="L323" t="n">
         <v>1</v>
@@ -16614,20 +16614,20 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="E324" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F324" t="n">
-        <v>5.8</v>
+        <v>5</v>
       </c>
       <c r="G324" t="n">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -16639,7 +16639,7 @@
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0.274</v>
+        <v>0.269</v>
       </c>
       <c r="L324" t="n">
         <v>1</v>
@@ -16664,23 +16664,23 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="E325" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F325" t="n">
-        <v>2.9</v>
+        <v>2.2</v>
       </c>
       <c r="G325" t="n">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="H325" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -16689,7 +16689,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>0.273</v>
+        <v>0.268</v>
       </c>
       <c r="L325" t="n">
         <v>1</v>
@@ -16714,23 +16714,23 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>16.5</v>
+        <v>16.6</v>
       </c>
       <c r="E326" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F326" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="G326" t="n">
-        <v>512</v>
+        <v>534</v>
       </c>
       <c r="H326" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="I326" t="n">
         <v>0</v>
@@ -16739,7 +16739,7 @@
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>0.271</v>
+        <v>0.267</v>
       </c>
       <c r="L326" t="n">
         <v>1</v>
@@ -16764,20 +16764,20 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>18.5</v>
+        <v>18.4</v>
       </c>
       <c r="E327" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F327" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="G327" t="n">
-        <v>542</v>
+        <v>557</v>
       </c>
       <c r="H327" t="n">
         <v>0</v>
@@ -16789,7 +16789,7 @@
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>0.269</v>
+        <v>0.265</v>
       </c>
       <c r="L327" t="n">
         <v>1</v>
@@ -16814,20 +16814,20 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D328" t="n">
         <v>19.4</v>
       </c>
       <c r="E328" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F328" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G328" t="n">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
@@ -16839,7 +16839,7 @@
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0.267</v>
+        <v>0.263</v>
       </c>
       <c r="L328" t="n">
         <v>1</v>
@@ -16864,23 +16864,23 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="E329" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F329" t="n">
-        <v>7.9</v>
+        <v>6.8</v>
       </c>
       <c r="G329" t="n">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="H329" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="I329" t="n">
         <v>0</v>
@@ -16889,7 +16889,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>0.266</v>
+        <v>0.261</v>
       </c>
       <c r="L329" t="n">
         <v>1</v>
@@ -16914,23 +16914,23 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="E330" t="n">
         <v>33</v>
       </c>
       <c r="F330" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="G330" t="n">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H330" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="I330" t="n">
         <v>0</v>
@@ -16939,7 +16939,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>0.265</v>
+        <v>0.26</v>
       </c>
       <c r="L330" t="n">
         <v>1</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>19.4</v>
+        <v>19.5</v>
       </c>
       <c r="E331" t="n">
         <v>33</v>
       </c>
       <c r="F331" t="n">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
       <c r="G331" t="n">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="H331" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -16989,7 +16989,7 @@
         <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="L331" t="n">
         <v>1</v>
@@ -17014,23 +17014,23 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>17.2</v>
+        <v>17.4</v>
       </c>
       <c r="E332" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F332" t="n">
-        <v>7.2</v>
+        <v>5</v>
       </c>
       <c r="G332" t="n">
         <v>29</v>
       </c>
       <c r="H332" t="n">
-        <v>99</v>
+        <v>36</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -17039,7 +17039,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="L332" t="n">
         <v>1</v>
@@ -17064,24 +17064,24 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>15.1</v>
+        <v>14.8</v>
       </c>
       <c r="E333" t="n">
+        <v>45</v>
+      </c>
+      <c r="F333" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="n">
         <v>41</v>
       </c>
-      <c r="F333" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="G333" t="n">
-        <v>0</v>
-      </c>
-      <c r="H333" t="n">
-        <v>98</v>
-      </c>
       <c r="I333" t="n">
         <v>0</v>
       </c>
@@ -17089,7 +17089,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="L333" t="n">
         <v>1</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>13.6</v>
+        <v>12.9</v>
       </c>
       <c r="E334" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F334" t="n">
-        <v>11.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>7</v>
+        <v>95</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17139,7 +17139,7 @@
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="L334" t="n">
         <v>1</v>
@@ -17164,14 +17164,14 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="E335" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F335" t="n">
         <v>9</v>
@@ -17180,7 +17180,7 @@
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="I335" t="n">
         <v>0</v>
@@ -17189,7 +17189,7 @@
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="L335" t="n">
         <v>1</v>
@@ -17214,23 +17214,23 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D336" t="n">
         <v>10.6</v>
       </c>
       <c r="E336" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="F336" t="n">
-        <v>6.5</v>
+        <v>7.9</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17239,7 +17239,7 @@
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="L336" t="n">
         <v>1</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="E337" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F337" t="n">
-        <v>6.1</v>
+        <v>5</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17289,7 +17289,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="L337" t="n">
         <v>1</v>
@@ -17314,14 +17314,14 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="E338" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F338" t="n">
         <v>4.7</v>
@@ -17330,7 +17330,7 @@
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>94</v>
+        <v>37</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17339,7 +17339,7 @@
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="L338" t="n">
         <v>2</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-17T23:03:48Z</t>
+          <t>2026-10-18T05:03:32Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="E339" t="n">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="F339" t="n">
-        <v>4.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.265</v>
+        <v>0.26</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>
@@ -17398,6 +17398,1206 @@
         <v>0</v>
       </c>
       <c r="N339" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="E340" t="n">
+        <v>70</v>
+      </c>
+      <c r="F340" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0</v>
+      </c>
+      <c r="H340" t="n">
+        <v>0</v>
+      </c>
+      <c r="I340" t="n">
+        <v>0</v>
+      </c>
+      <c r="J340" t="n">
+        <v>0</v>
+      </c>
+      <c r="K340" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L340" t="n">
+        <v>2</v>
+      </c>
+      <c r="M340" t="n">
+        <v>0</v>
+      </c>
+      <c r="N340" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E341" t="n">
+        <v>74</v>
+      </c>
+      <c r="F341" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G341" t="n">
+        <v>0</v>
+      </c>
+      <c r="H341" t="n">
+        <v>100</v>
+      </c>
+      <c r="I341" t="n">
+        <v>0</v>
+      </c>
+      <c r="J341" t="n">
+        <v>0</v>
+      </c>
+      <c r="K341" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L341" t="n">
+        <v>2</v>
+      </c>
+      <c r="M341" t="n">
+        <v>0</v>
+      </c>
+      <c r="N341" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="E342" t="n">
+        <v>72</v>
+      </c>
+      <c r="F342" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
+      <c r="H342" t="n">
+        <v>100</v>
+      </c>
+      <c r="I342" t="n">
+        <v>0</v>
+      </c>
+      <c r="J342" t="n">
+        <v>0</v>
+      </c>
+      <c r="K342" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L342" t="n">
+        <v>2</v>
+      </c>
+      <c r="M342" t="n">
+        <v>0</v>
+      </c>
+      <c r="N342" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>7</v>
+      </c>
+      <c r="E343" t="n">
+        <v>76</v>
+      </c>
+      <c r="F343" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0</v>
+      </c>
+      <c r="H343" t="n">
+        <v>94</v>
+      </c>
+      <c r="I343" t="n">
+        <v>0</v>
+      </c>
+      <c r="J343" t="n">
+        <v>0</v>
+      </c>
+      <c r="K343" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L343" t="n">
+        <v>2</v>
+      </c>
+      <c r="M343" t="n">
+        <v>0</v>
+      </c>
+      <c r="N343" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="E344" t="n">
+        <v>80</v>
+      </c>
+      <c r="F344" t="n">
+        <v>9</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0</v>
+      </c>
+      <c r="H344" t="n">
+        <v>0</v>
+      </c>
+      <c r="I344" t="n">
+        <v>0</v>
+      </c>
+      <c r="J344" t="n">
+        <v>0</v>
+      </c>
+      <c r="K344" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L344" t="n">
+        <v>2</v>
+      </c>
+      <c r="M344" t="n">
+        <v>0</v>
+      </c>
+      <c r="N344" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E345" t="n">
+        <v>84</v>
+      </c>
+      <c r="F345" t="n">
+        <v>9</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0</v>
+      </c>
+      <c r="H345" t="n">
+        <v>16</v>
+      </c>
+      <c r="I345" t="n">
+        <v>0</v>
+      </c>
+      <c r="J345" t="n">
+        <v>0</v>
+      </c>
+      <c r="K345" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="L345" t="n">
+        <v>2</v>
+      </c>
+      <c r="M345" t="n">
+        <v>0</v>
+      </c>
+      <c r="N345" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E346" t="n">
+        <v>79</v>
+      </c>
+      <c r="F346" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G346" t="n">
+        <v>42</v>
+      </c>
+      <c r="H346" t="n">
+        <v>0</v>
+      </c>
+      <c r="I346" t="n">
+        <v>0</v>
+      </c>
+      <c r="J346" t="n">
+        <v>0</v>
+      </c>
+      <c r="K346" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="L346" t="n">
+        <v>2</v>
+      </c>
+      <c r="M346" t="n">
+        <v>0</v>
+      </c>
+      <c r="N346" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E347" t="n">
+        <v>63</v>
+      </c>
+      <c r="F347" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G347" t="n">
+        <v>184</v>
+      </c>
+      <c r="H347" t="n">
+        <v>0</v>
+      </c>
+      <c r="I347" t="n">
+        <v>0</v>
+      </c>
+      <c r="J347" t="n">
+        <v>0</v>
+      </c>
+      <c r="K347" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="L347" t="n">
+        <v>2</v>
+      </c>
+      <c r="M347" t="n">
+        <v>0</v>
+      </c>
+      <c r="N347" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="E348" t="n">
+        <v>48</v>
+      </c>
+      <c r="F348" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G348" t="n">
+        <v>333</v>
+      </c>
+      <c r="H348" t="n">
+        <v>0</v>
+      </c>
+      <c r="I348" t="n">
+        <v>0</v>
+      </c>
+      <c r="J348" t="n">
+        <v>0</v>
+      </c>
+      <c r="K348" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L348" t="n">
+        <v>2</v>
+      </c>
+      <c r="M348" t="n">
+        <v>0</v>
+      </c>
+      <c r="N348" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="E349" t="n">
+        <v>48</v>
+      </c>
+      <c r="F349" t="n">
+        <v>12</v>
+      </c>
+      <c r="G349" t="n">
+        <v>451.8</v>
+      </c>
+      <c r="H349" t="n">
+        <v>0</v>
+      </c>
+      <c r="I349" t="n">
+        <v>0</v>
+      </c>
+      <c r="J349" t="n">
+        <v>0</v>
+      </c>
+      <c r="K349" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="L349" t="n">
+        <v>2</v>
+      </c>
+      <c r="M349" t="n">
+        <v>0</v>
+      </c>
+      <c r="N349" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="E350" t="n">
+        <v>48</v>
+      </c>
+      <c r="F350" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="G350" t="n">
+        <v>526.5</v>
+      </c>
+      <c r="H350" t="n">
+        <v>0</v>
+      </c>
+      <c r="I350" t="n">
+        <v>0</v>
+      </c>
+      <c r="J350" t="n">
+        <v>0</v>
+      </c>
+      <c r="K350" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="L350" t="n">
+        <v>2</v>
+      </c>
+      <c r="M350" t="n">
+        <v>0</v>
+      </c>
+      <c r="N350" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E351" t="n">
+        <v>49</v>
+      </c>
+      <c r="F351" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="G351" t="n">
+        <v>547.8</v>
+      </c>
+      <c r="H351" t="n">
+        <v>0</v>
+      </c>
+      <c r="I351" t="n">
+        <v>0</v>
+      </c>
+      <c r="J351" t="n">
+        <v>0</v>
+      </c>
+      <c r="K351" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="L351" t="n">
+        <v>2</v>
+      </c>
+      <c r="M351" t="n">
+        <v>0</v>
+      </c>
+      <c r="N351" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="E352" t="n">
+        <v>52</v>
+      </c>
+      <c r="F352" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G352" t="n">
+        <v>511</v>
+      </c>
+      <c r="H352" t="n">
+        <v>6</v>
+      </c>
+      <c r="I352" t="n">
+        <v>0</v>
+      </c>
+      <c r="J352" t="n">
+        <v>0</v>
+      </c>
+      <c r="K352" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="L352" t="n">
+        <v>2</v>
+      </c>
+      <c r="M352" t="n">
+        <v>0</v>
+      </c>
+      <c r="N352" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="E353" t="n">
+        <v>52</v>
+      </c>
+      <c r="F353" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="G353" t="n">
+        <v>426</v>
+      </c>
+      <c r="H353" t="n">
+        <v>15</v>
+      </c>
+      <c r="I353" t="n">
+        <v>0</v>
+      </c>
+      <c r="J353" t="n">
+        <v>0</v>
+      </c>
+      <c r="K353" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="L353" t="n">
+        <v>2</v>
+      </c>
+      <c r="M353" t="n">
+        <v>0</v>
+      </c>
+      <c r="N353" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="E354" t="n">
+        <v>53</v>
+      </c>
+      <c r="F354" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G354" t="n">
+        <v>302</v>
+      </c>
+      <c r="H354" t="n">
+        <v>21</v>
+      </c>
+      <c r="I354" t="n">
+        <v>0</v>
+      </c>
+      <c r="J354" t="n">
+        <v>0</v>
+      </c>
+      <c r="K354" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L354" t="n">
+        <v>2</v>
+      </c>
+      <c r="M354" t="n">
+        <v>0</v>
+      </c>
+      <c r="N354" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="E355" t="n">
+        <v>60</v>
+      </c>
+      <c r="F355" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="G355" t="n">
+        <v>151</v>
+      </c>
+      <c r="H355" t="n">
+        <v>2</v>
+      </c>
+      <c r="I355" t="n">
+        <v>0</v>
+      </c>
+      <c r="J355" t="n">
+        <v>0</v>
+      </c>
+      <c r="K355" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L355" t="n">
+        <v>2</v>
+      </c>
+      <c r="M355" t="n">
+        <v>0</v>
+      </c>
+      <c r="N355" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="E356" t="n">
+        <v>68</v>
+      </c>
+      <c r="F356" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G356" t="n">
+        <v>24</v>
+      </c>
+      <c r="H356" t="n">
+        <v>0</v>
+      </c>
+      <c r="I356" t="n">
+        <v>0</v>
+      </c>
+      <c r="J356" t="n">
+        <v>0</v>
+      </c>
+      <c r="K356" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L356" t="n">
+        <v>2</v>
+      </c>
+      <c r="M356" t="n">
+        <v>0</v>
+      </c>
+      <c r="N356" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="E357" t="n">
+        <v>71</v>
+      </c>
+      <c r="F357" t="n">
+        <v>12</v>
+      </c>
+      <c r="G357" t="n">
+        <v>0</v>
+      </c>
+      <c r="H357" t="n">
+        <v>0</v>
+      </c>
+      <c r="I357" t="n">
+        <v>0</v>
+      </c>
+      <c r="J357" t="n">
+        <v>0</v>
+      </c>
+      <c r="K357" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L357" t="n">
+        <v>2</v>
+      </c>
+      <c r="M357" t="n">
+        <v>0</v>
+      </c>
+      <c r="N357" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="E358" t="n">
+        <v>72</v>
+      </c>
+      <c r="F358" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G358" t="n">
+        <v>0</v>
+      </c>
+      <c r="H358" t="n">
+        <v>1</v>
+      </c>
+      <c r="I358" t="n">
+        <v>0</v>
+      </c>
+      <c r="J358" t="n">
+        <v>0</v>
+      </c>
+      <c r="K358" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L358" t="n">
+        <v>2</v>
+      </c>
+      <c r="M358" t="n">
+        <v>0</v>
+      </c>
+      <c r="N358" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>14</v>
+      </c>
+      <c r="E359" t="n">
+        <v>71</v>
+      </c>
+      <c r="F359" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0</v>
+      </c>
+      <c r="H359" t="n">
+        <v>3</v>
+      </c>
+      <c r="I359" t="n">
+        <v>0</v>
+      </c>
+      <c r="J359" t="n">
+        <v>0</v>
+      </c>
+      <c r="K359" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L359" t="n">
+        <v>2</v>
+      </c>
+      <c r="M359" t="n">
+        <v>0</v>
+      </c>
+      <c r="N359" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="E360" t="n">
+        <v>71</v>
+      </c>
+      <c r="F360" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="G360" t="n">
+        <v>0</v>
+      </c>
+      <c r="H360" t="n">
+        <v>0</v>
+      </c>
+      <c r="I360" t="n">
+        <v>0</v>
+      </c>
+      <c r="J360" t="n">
+        <v>0</v>
+      </c>
+      <c r="K360" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L360" t="n">
+        <v>2</v>
+      </c>
+      <c r="M360" t="n">
+        <v>0</v>
+      </c>
+      <c r="N360" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E361" t="n">
+        <v>71</v>
+      </c>
+      <c r="F361" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0</v>
+      </c>
+      <c r="H361" t="n">
+        <v>0</v>
+      </c>
+      <c r="I361" t="n">
+        <v>0</v>
+      </c>
+      <c r="J361" t="n">
+        <v>0</v>
+      </c>
+      <c r="K361" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L361" t="n">
+        <v>2</v>
+      </c>
+      <c r="M361" t="n">
+        <v>0</v>
+      </c>
+      <c r="N361" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="E362" t="n">
+        <v>70</v>
+      </c>
+      <c r="F362" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="G362" t="n">
+        <v>0</v>
+      </c>
+      <c r="H362" t="n">
+        <v>0</v>
+      </c>
+      <c r="I362" t="n">
+        <v>0</v>
+      </c>
+      <c r="J362" t="n">
+        <v>0</v>
+      </c>
+      <c r="K362" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L362" t="n">
+        <v>3</v>
+      </c>
+      <c r="M362" t="n">
+        <v>0</v>
+      </c>
+      <c r="N362" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>2026-10-18T05:03:32Z</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="E363" t="n">
+        <v>69</v>
+      </c>
+      <c r="F363" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="G363" t="n">
+        <v>0</v>
+      </c>
+      <c r="H363" t="n">
+        <v>0</v>
+      </c>
+      <c r="I363" t="n">
+        <v>0</v>
+      </c>
+      <c r="J363" t="n">
+        <v>0</v>
+      </c>
+      <c r="K363" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L363" t="n">
+        <v>3</v>
+      </c>
+      <c r="M363" t="n">
+        <v>0</v>
+      </c>
+      <c r="N363" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-18 13:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -15564,23 +15564,23 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>17.7</v>
+        <v>16.9</v>
       </c>
       <c r="E303" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F303" t="n">
         <v>8.300000000000001</v>
       </c>
       <c r="G303" t="n">
-        <v>547</v>
+        <v>457</v>
       </c>
       <c r="H303" t="n">
-        <v>19</v>
+        <v>99</v>
       </c>
       <c r="I303" t="n">
         <v>0</v>
@@ -15589,7 +15589,7 @@
         <v>0</v>
       </c>
       <c r="K303" t="n">
-        <v>0.276</v>
+        <v>0.285</v>
       </c>
       <c r="L303" t="n">
         <v>7</v>
@@ -15614,23 +15614,23 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>19</v>
+        <v>17.7</v>
       </c>
       <c r="E304" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F304" t="n">
-        <v>7.6</v>
+        <v>9</v>
       </c>
       <c r="G304" t="n">
-        <v>515</v>
+        <v>360</v>
       </c>
       <c r="H304" t="n">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="I304" t="n">
         <v>0</v>
@@ -15639,7 +15639,7 @@
         <v>0</v>
       </c>
       <c r="K304" t="n">
-        <v>0.274</v>
+        <v>0.284</v>
       </c>
       <c r="L304" t="n">
         <v>7</v>
@@ -15664,23 +15664,23 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>19.9</v>
+        <v>18.5</v>
       </c>
       <c r="E305" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F305" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G305" t="n">
         <v>428</v>
       </c>
       <c r="H305" t="n">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="I305" t="n">
         <v>0</v>
@@ -15689,7 +15689,7 @@
         <v>0</v>
       </c>
       <c r="K305" t="n">
-        <v>0.271</v>
+        <v>0.282</v>
       </c>
       <c r="L305" t="n">
         <v>7</v>
@@ -15714,24 +15714,24 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>20.3</v>
+        <v>19.2</v>
       </c>
       <c r="E306" t="n">
+        <v>31</v>
+      </c>
+      <c r="F306" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G306" t="n">
+        <v>307</v>
+      </c>
+      <c r="H306" t="n">
         <v>28</v>
       </c>
-      <c r="F306" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="G306" t="n">
-        <v>304</v>
-      </c>
-      <c r="H306" t="n">
-        <v>86</v>
-      </c>
       <c r="I306" t="n">
         <v>0</v>
       </c>
@@ -15739,7 +15739,7 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="L306" t="n">
         <v>7</v>
@@ -15764,23 +15764,23 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>20.2</v>
+        <v>19.1</v>
       </c>
       <c r="E307" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F307" t="n">
-        <v>8.6</v>
+        <v>6.8</v>
       </c>
       <c r="G307" t="n">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="H307" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="I307" t="n">
         <v>0</v>
@@ -15789,7 +15789,7 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L307" t="n">
         <v>7</v>
@@ -15814,23 +15814,23 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>18</v>
+        <v>17.2</v>
       </c>
       <c r="E308" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F308" t="n">
-        <v>4.7</v>
+        <v>2.9</v>
       </c>
       <c r="G308" t="n">
         <v>30</v>
       </c>
       <c r="H308" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -15839,7 +15839,7 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L308" t="n">
         <v>7</v>
@@ -15864,14 +15864,14 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>15.5</v>
+        <v>14.9</v>
       </c>
       <c r="E309" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F309" t="n">
         <v>4.7</v>
@@ -15880,7 +15880,7 @@
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L309" t="n">
         <v>7</v>
@@ -15914,17 +15914,17 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>13.5</v>
+        <v>12.9</v>
       </c>
       <c r="E310" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F310" t="n">
-        <v>5.4</v>
+        <v>6.8</v>
       </c>
       <c r="G310" t="n">
         <v>0</v>
@@ -15939,7 +15939,7 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L310" t="n">
         <v>7</v>
@@ -15964,17 +15964,17 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>12.1</v>
+        <v>11.6</v>
       </c>
       <c r="E311" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F311" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
@@ -15989,7 +15989,7 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L311" t="n">
         <v>7</v>
@@ -16014,17 +16014,17 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>11.1</v>
+        <v>10.5</v>
       </c>
       <c r="E312" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="F312" t="n">
-        <v>5</v>
+        <v>7.2</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -16039,7 +16039,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L312" t="n">
         <v>7</v>
@@ -16064,17 +16064,17 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>10.2</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E313" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="F313" t="n">
-        <v>6.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,17 +16114,17 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9.699999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E314" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F314" t="n">
-        <v>5.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -16139,7 +16139,7 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L314" t="n">
         <v>1</v>
@@ -16164,17 +16164,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="E315" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F315" t="n">
-        <v>5.8</v>
+        <v>8.6</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L315" t="n">
         <v>1</v>
@@ -16214,23 +16214,23 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D316" t="n">
         <v>8.199999999999999</v>
       </c>
       <c r="E316" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F316" t="n">
-        <v>5.8</v>
+        <v>6.8</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="I316" t="n">
         <v>0</v>
@@ -16239,7 +16239,7 @@
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L316" t="n">
         <v>1</v>
@@ -16264,23 +16264,23 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="E317" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F317" t="n">
-        <v>2.9</v>
+        <v>7.2</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I317" t="n">
         <v>0</v>
@@ -16289,7 +16289,7 @@
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0.269</v>
+        <v>0.28</v>
       </c>
       <c r="L317" t="n">
         <v>1</v>
@@ -16314,17 +16314,17 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="E318" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F318" t="n">
-        <v>4</v>
+        <v>5.4</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
@@ -16339,7 +16339,7 @@
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="L318" t="n">
         <v>1</v>
@@ -16364,23 +16364,23 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>6.7</v>
+        <v>6.4</v>
       </c>
       <c r="E319" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F319" t="n">
-        <v>1.8</v>
+        <v>4</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I319" t="n">
         <v>0</v>
@@ -16389,7 +16389,7 @@
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="L319" t="n">
         <v>1</v>
@@ -16414,23 +16414,23 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>6.2</v>
+        <v>5.9</v>
       </c>
       <c r="E320" t="n">
         <v>85</v>
       </c>
       <c r="F320" t="n">
-        <v>1.1</v>
+        <v>2.5</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I320" t="n">
         <v>0</v>
@@ -16439,7 +16439,7 @@
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="L320" t="n">
         <v>1</v>
@@ -16464,17 +16464,17 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>6</v>
+        <v>5.6</v>
       </c>
       <c r="E321" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F321" t="n">
-        <v>1.8</v>
+        <v>2.9</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
@@ -16489,7 +16489,7 @@
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="L321" t="n">
         <v>1</v>
@@ -16514,17 +16514,17 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="E322" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F322" t="n">
-        <v>6.1</v>
+        <v>3.6</v>
       </c>
       <c r="G322" t="n">
         <v>45</v>
@@ -16539,7 +16539,7 @@
         <v>0</v>
       </c>
       <c r="K322" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="L322" t="n">
         <v>1</v>
@@ -16564,20 +16564,20 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>8.800000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E323" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="F323" t="n">
-        <v>3.6</v>
+        <v>2.2</v>
       </c>
       <c r="G323" t="n">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H323" t="n">
         <v>0</v>
@@ -16589,7 +16589,7 @@
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="L323" t="n">
         <v>1</v>
@@ -16614,17 +16614,17 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>12</v>
+        <v>11.2</v>
       </c>
       <c r="E324" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F324" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="G324" t="n">
         <v>337</v>
@@ -16639,7 +16639,7 @@
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0.269</v>
+        <v>0.279</v>
       </c>
       <c r="L324" t="n">
         <v>1</v>
@@ -16664,17 +16664,17 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>14.3</v>
+        <v>13.8</v>
       </c>
       <c r="E325" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F325" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="G325" t="n">
         <v>459</v>
@@ -16689,7 +16689,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>0.268</v>
+        <v>0.278</v>
       </c>
       <c r="L325" t="n">
         <v>1</v>
@@ -16714,20 +16714,20 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>16.6</v>
+        <v>16.2</v>
       </c>
       <c r="E326" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F326" t="n">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="G326" t="n">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="H326" t="n">
         <v>0</v>
@@ -16739,7 +16739,7 @@
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>0.267</v>
+        <v>0.277</v>
       </c>
       <c r="L326" t="n">
         <v>1</v>
@@ -16764,17 +16764,17 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>18.4</v>
+        <v>18</v>
       </c>
       <c r="E327" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F327" t="n">
-        <v>6.5</v>
+        <v>7.6</v>
       </c>
       <c r="G327" t="n">
         <v>557</v>
@@ -16789,7 +16789,7 @@
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>0.265</v>
+        <v>0.275</v>
       </c>
       <c r="L327" t="n">
         <v>1</v>
@@ -16814,20 +16814,20 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>19.4</v>
+        <v>19</v>
       </c>
       <c r="E328" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F328" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="G328" t="n">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
@@ -16839,7 +16839,7 @@
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0.263</v>
+        <v>0.273</v>
       </c>
       <c r="L328" t="n">
         <v>1</v>
@@ -16864,20 +16864,20 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>19.9</v>
+        <v>19.5</v>
       </c>
       <c r="E329" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F329" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="G329" t="n">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
@@ -16889,7 +16889,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>0.261</v>
+        <v>0.271</v>
       </c>
       <c r="L329" t="n">
         <v>1</v>
@@ -16914,23 +16914,23 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="E330" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F330" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="G330" t="n">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="H330" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="I330" t="n">
         <v>0</v>
@@ -16939,7 +16939,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L330" t="n">
         <v>1</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>19.5</v>
+        <v>19.3</v>
       </c>
       <c r="E331" t="n">
         <v>33</v>
       </c>
       <c r="F331" t="n">
-        <v>5.4</v>
+        <v>6.8</v>
       </c>
       <c r="G331" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H331" t="n">
-        <v>27</v>
+        <v>100</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -16989,7 +16989,7 @@
         <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>0.26</v>
+        <v>0.269</v>
       </c>
       <c r="L331" t="n">
         <v>1</v>
@@ -17014,20 +17014,20 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>17.4</v>
+        <v>17.2</v>
       </c>
       <c r="E332" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F332" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="G332" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H332" t="n">
         <v>36</v>
@@ -17039,7 +17039,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>0.26</v>
+        <v>0.269</v>
       </c>
       <c r="L332" t="n">
         <v>1</v>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>14.8</v>
+        <v>14.6</v>
       </c>
       <c r="E333" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F333" t="n">
-        <v>6.8</v>
+        <v>8.6</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17089,7 +17089,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>0.26</v>
+        <v>0.269</v>
       </c>
       <c r="L333" t="n">
         <v>1</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="E334" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F334" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17139,7 +17139,7 @@
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>0.26</v>
+        <v>0.269</v>
       </c>
       <c r="L334" t="n">
         <v>1</v>
@@ -17164,23 +17164,23 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="E335" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F335" t="n">
-        <v>9</v>
+        <v>7.9</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="I335" t="n">
         <v>0</v>
@@ -17189,7 +17189,7 @@
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>0.26</v>
+        <v>0.269</v>
       </c>
       <c r="L335" t="n">
         <v>1</v>
@@ -17214,14 +17214,14 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>10.6</v>
+        <v>10.4</v>
       </c>
       <c r="E336" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F336" t="n">
         <v>7.9</v>
@@ -17230,7 +17230,7 @@
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>98</v>
+        <v>67</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17239,7 +17239,7 @@
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0.26</v>
+        <v>0.269</v>
       </c>
       <c r="L336" t="n">
         <v>1</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>9.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E337" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F337" t="n">
-        <v>5</v>
+        <v>2.2</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>97</v>
+        <v>20</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17289,7 +17289,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>0.26</v>
+        <v>0.269</v>
       </c>
       <c r="L337" t="n">
         <v>1</v>
@@ -17314,23 +17314,23 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D338" t="n">
         <v>8.5</v>
       </c>
       <c r="E338" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F338" t="n">
-        <v>4.7</v>
+        <v>4.3</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>37</v>
+        <v>84</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17339,7 +17339,7 @@
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L338" t="n">
         <v>2</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>7.9</v>
+        <v>7.7</v>
       </c>
       <c r="E339" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F339" t="n">
-        <v>8.300000000000001</v>
+        <v>4.7</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>
@@ -17414,23 +17414,23 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="E340" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F340" t="n">
-        <v>5.8</v>
+        <v>4.7</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I340" t="n">
         <v>0</v>
@@ -17439,7 +17439,7 @@
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L340" t="n">
         <v>2</v>
@@ -17464,23 +17464,23 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D341" t="n">
         <v>6.6</v>
       </c>
       <c r="E341" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F341" t="n">
-        <v>8.6</v>
+        <v>4.7</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="I341" t="n">
         <v>0</v>
@@ -17489,7 +17489,7 @@
         <v>0</v>
       </c>
       <c r="K341" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L341" t="n">
         <v>2</v>
@@ -17514,23 +17514,23 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>7.4</v>
+        <v>6</v>
       </c>
       <c r="E342" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="F342" t="n">
-        <v>11.5</v>
+        <v>6.1</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="I342" t="n">
         <v>0</v>
@@ -17539,7 +17539,7 @@
         <v>0</v>
       </c>
       <c r="K342" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L342" t="n">
         <v>2</v>
@@ -17564,23 +17564,23 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="E343" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F343" t="n">
-        <v>9.699999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="I343" t="n">
         <v>0</v>
@@ -17589,7 +17589,7 @@
         <v>0</v>
       </c>
       <c r="K343" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L343" t="n">
         <v>2</v>
@@ -17614,23 +17614,23 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>6.6</v>
+        <v>5.2</v>
       </c>
       <c r="E344" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F344" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I344" t="n">
         <v>0</v>
@@ -17639,7 +17639,7 @@
         <v>0</v>
       </c>
       <c r="K344" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L344" t="n">
         <v>2</v>
@@ -17664,23 +17664,23 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>6.1</v>
+        <v>4.9</v>
       </c>
       <c r="E345" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F345" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="I345" t="n">
         <v>0</v>
@@ -17689,7 +17689,7 @@
         <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>0.261</v>
+        <v>0.27</v>
       </c>
       <c r="L345" t="n">
         <v>2</v>
@@ -17714,20 +17714,20 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>6.7</v>
+        <v>5.8</v>
       </c>
       <c r="E346" t="n">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="F346" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="G346" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H346" t="n">
         <v>0</v>
@@ -17739,7 +17739,7 @@
         <v>0</v>
       </c>
       <c r="K346" t="n">
-        <v>0.261</v>
+        <v>0.27</v>
       </c>
       <c r="L346" t="n">
         <v>2</v>
@@ -17764,20 +17764,20 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>9.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E347" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F347" t="n">
-        <v>9.4</v>
+        <v>6.8</v>
       </c>
       <c r="G347" t="n">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H347" t="n">
         <v>0</v>
@@ -17789,7 +17789,7 @@
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>0.261</v>
+        <v>0.27</v>
       </c>
       <c r="L347" t="n">
         <v>2</v>
@@ -17814,20 +17814,20 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>14.1</v>
+        <v>13.1</v>
       </c>
       <c r="E348" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F348" t="n">
-        <v>10.8</v>
+        <v>7.2</v>
       </c>
       <c r="G348" t="n">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="H348" t="n">
         <v>0</v>
@@ -17839,7 +17839,7 @@
         <v>0</v>
       </c>
       <c r="K348" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="L348" t="n">
         <v>2</v>
@@ -17864,20 +17864,20 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D349" t="n">
         <v>16.6</v>
       </c>
       <c r="E349" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="F349" t="n">
-        <v>12</v>
+        <v>10.1</v>
       </c>
       <c r="G349" t="n">
-        <v>451.8</v>
+        <v>454</v>
       </c>
       <c r="H349" t="n">
         <v>0</v>
@@ -17889,7 +17889,7 @@
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>0.259</v>
+        <v>0.269</v>
       </c>
       <c r="L349" t="n">
         <v>2</v>
@@ -17914,20 +17914,20 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>17.9</v>
+        <v>18.6</v>
       </c>
       <c r="E350" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="F350" t="n">
-        <v>11.2</v>
+        <v>12.2</v>
       </c>
       <c r="G350" t="n">
-        <v>526.5</v>
+        <v>532</v>
       </c>
       <c r="H350" t="n">
         <v>0</v>
@@ -17939,7 +17939,7 @@
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>0.258</v>
+        <v>0.267</v>
       </c>
       <c r="L350" t="n">
         <v>2</v>
@@ -17964,20 +17964,20 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>18.5</v>
+        <v>20</v>
       </c>
       <c r="E351" t="n">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="F351" t="n">
-        <v>10.7</v>
+        <v>12.6</v>
       </c>
       <c r="G351" t="n">
-        <v>547.8</v>
+        <v>559</v>
       </c>
       <c r="H351" t="n">
         <v>0</v>
@@ -17989,7 +17989,7 @@
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>0.256</v>
+        <v>0.265</v>
       </c>
       <c r="L351" t="n">
         <v>2</v>
@@ -18014,23 +18014,23 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>18.7</v>
+        <v>21.1</v>
       </c>
       <c r="E352" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="F352" t="n">
-        <v>10.4</v>
+        <v>11.5</v>
       </c>
       <c r="G352" t="n">
-        <v>511</v>
+        <v>530</v>
       </c>
       <c r="H352" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -18039,7 +18039,7 @@
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>0.254</v>
+        <v>0.263</v>
       </c>
       <c r="L352" t="n">
         <v>2</v>
@@ -18064,23 +18064,23 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>19.1</v>
+        <v>21.9</v>
       </c>
       <c r="E353" t="n">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="F353" t="n">
-        <v>11.2</v>
+        <v>10.8</v>
       </c>
       <c r="G353" t="n">
-        <v>426</v>
+        <v>444</v>
       </c>
       <c r="H353" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -18089,7 +18089,7 @@
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>0.252</v>
+        <v>0.261</v>
       </c>
       <c r="L353" t="n">
         <v>2</v>
@@ -18114,23 +18114,23 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>18.9</v>
+        <v>22.3</v>
       </c>
       <c r="E354" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="F354" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="G354" t="n">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="H354" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="I354" t="n">
         <v>0</v>
@@ -18139,7 +18139,7 @@
         <v>0</v>
       </c>
       <c r="K354" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="L354" t="n">
         <v>2</v>
@@ -18164,23 +18164,23 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>17.7</v>
+        <v>20.8</v>
       </c>
       <c r="E355" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="F355" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
       <c r="G355" t="n">
-        <v>151</v>
+        <v>160.3</v>
       </c>
       <c r="H355" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I355" t="n">
         <v>0</v>
@@ -18189,7 +18189,7 @@
         <v>0</v>
       </c>
       <c r="K355" t="n">
-        <v>0.25</v>
+        <v>0.259</v>
       </c>
       <c r="L355" t="n">
         <v>2</v>
@@ -18214,20 +18214,20 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>15.6</v>
+        <v>17.1</v>
       </c>
       <c r="E356" t="n">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="F356" t="n">
-        <v>11.8</v>
+        <v>10.3</v>
       </c>
       <c r="G356" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H356" t="n">
         <v>0</v>
@@ -18239,7 +18239,7 @@
         <v>0</v>
       </c>
       <c r="K356" t="n">
-        <v>0.25</v>
+        <v>0.259</v>
       </c>
       <c r="L356" t="n">
         <v>2</v>
@@ -18264,17 +18264,17 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="E357" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F357" t="n">
-        <v>12</v>
+        <v>10.9</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
@@ -18289,7 +18289,7 @@
         <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>0.25</v>
+        <v>0.259</v>
       </c>
       <c r="L357" t="n">
         <v>2</v>
@@ -18314,23 +18314,23 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>14.3</v>
+        <v>13.7</v>
       </c>
       <c r="E358" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F358" t="n">
-        <v>11.8</v>
+        <v>10.4</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
       </c>
       <c r="H358" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I358" t="n">
         <v>0</v>
@@ -18339,7 +18339,7 @@
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>0.25</v>
+        <v>0.259</v>
       </c>
       <c r="L358" t="n">
         <v>2</v>
@@ -18364,23 +18364,23 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>14</v>
+        <v>13.5</v>
       </c>
       <c r="E359" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F359" t="n">
-        <v>12.4</v>
+        <v>11</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
       </c>
       <c r="H359" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I359" t="n">
         <v>0</v>
@@ -18389,7 +18389,7 @@
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>0.25</v>
+        <v>0.259</v>
       </c>
       <c r="L359" t="n">
         <v>2</v>
@@ -18414,17 +18414,17 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>13.6</v>
+        <v>13.4</v>
       </c>
       <c r="E360" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F360" t="n">
-        <v>14.2</v>
+        <v>12.2</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
@@ -18439,7 +18439,7 @@
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>0.25</v>
+        <v>0.259</v>
       </c>
       <c r="L360" t="n">
         <v>2</v>
@@ -18464,17 +18464,17 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>13.5</v>
+        <v>13.4</v>
       </c>
       <c r="E361" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F361" t="n">
-        <v>15.9</v>
+        <v>13.9</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
@@ -18489,7 +18489,7 @@
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>0.249</v>
+        <v>0.259</v>
       </c>
       <c r="L361" t="n">
         <v>2</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>13.4</v>
+        <v>13.2</v>
       </c>
       <c r="E362" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="F362" t="n">
-        <v>16.9</v>
+        <v>14.2</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18539,7 +18539,7 @@
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>0.249</v>
+        <v>0.259</v>
       </c>
       <c r="L362" t="n">
         <v>3</v>
@@ -18564,17 +18564,17 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-18T05:03:32Z</t>
+          <t>2026-10-18T11:03:28Z</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="E363" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F363" t="n">
-        <v>16.7</v>
+        <v>12.8</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -18589,7 +18589,7 @@
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>0.249</v>
+        <v>0.259</v>
       </c>
       <c r="L363" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-18 19:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -15864,14 +15864,14 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>14.9</v>
+        <v>15.2</v>
       </c>
       <c r="E309" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F309" t="n">
         <v>4.7</v>
@@ -15880,7 +15880,7 @@
         <v>0</v>
       </c>
       <c r="H309" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="I309" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L309" t="n">
         <v>7</v>
@@ -15914,14 +15914,14 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>12.9</v>
+        <v>13.4</v>
       </c>
       <c r="E310" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F310" t="n">
         <v>6.8</v>
@@ -15930,7 +15930,7 @@
         <v>0</v>
       </c>
       <c r="H310" t="n">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="I310" t="n">
         <v>0</v>
@@ -15939,7 +15939,7 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L310" t="n">
         <v>7</v>
@@ -15964,23 +15964,23 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="E311" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F311" t="n">
-        <v>6.8</v>
+        <v>3.6</v>
       </c>
       <c r="G311" t="n">
         <v>0</v>
       </c>
       <c r="H311" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I311" t="n">
         <v>0</v>
@@ -15989,7 +15989,7 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L311" t="n">
         <v>7</v>
@@ -16014,17 +16014,17 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>10.5</v>
+        <v>11.1</v>
       </c>
       <c r="E312" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F312" t="n">
-        <v>7.2</v>
+        <v>4.7</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -16039,7 +16039,7 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L312" t="n">
         <v>7</v>
@@ -16064,17 +16064,17 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="E313" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F313" t="n">
-        <v>8.300000000000001</v>
+        <v>6.8</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -16089,7 +16089,7 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L313" t="n">
         <v>7</v>
@@ -16114,17 +16114,17 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="E314" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F314" t="n">
-        <v>8.300000000000001</v>
+        <v>6.8</v>
       </c>
       <c r="G314" t="n">
         <v>0</v>
@@ -16139,7 +16139,7 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L314" t="n">
         <v>1</v>
@@ -16164,17 +16164,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D315" t="n">
         <v>8.9</v>
       </c>
       <c r="E315" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F315" t="n">
-        <v>8.6</v>
+        <v>7.6</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L315" t="n">
         <v>1</v>
@@ -16214,23 +16214,23 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D316" t="n">
         <v>8.199999999999999</v>
       </c>
       <c r="E316" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F316" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="I316" t="n">
         <v>0</v>
@@ -16239,7 +16239,7 @@
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L316" t="n">
         <v>1</v>
@@ -16264,23 +16264,23 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="E317" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F317" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I317" t="n">
         <v>0</v>
@@ -16289,7 +16289,7 @@
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L317" t="n">
         <v>1</v>
@@ -16314,23 +16314,23 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>7.1</v>
+        <v>7.5</v>
       </c>
       <c r="E318" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F318" t="n">
-        <v>5.4</v>
+        <v>1.4</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="I318" t="n">
         <v>0</v>
@@ -16339,7 +16339,7 @@
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L318" t="n">
         <v>1</v>
@@ -16364,23 +16364,23 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>6.4</v>
+        <v>7</v>
       </c>
       <c r="E319" t="n">
         <v>75</v>
       </c>
       <c r="F319" t="n">
-        <v>4</v>
+        <v>1.1</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="I319" t="n">
         <v>0</v>
@@ -16389,7 +16389,7 @@
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L319" t="n">
         <v>1</v>
@@ -16414,23 +16414,23 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="E320" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F320" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I320" t="n">
         <v>0</v>
@@ -16439,7 +16439,7 @@
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L320" t="n">
         <v>1</v>
@@ -16464,17 +16464,17 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="E321" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="F321" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
@@ -16514,17 +16514,17 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="E322" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F322" t="n">
-        <v>3.6</v>
+        <v>4.3</v>
       </c>
       <c r="G322" t="n">
         <v>45</v>
@@ -16564,20 +16564,20 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>8.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="E323" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="F323" t="n">
-        <v>2.2</v>
+        <v>5</v>
       </c>
       <c r="G323" t="n">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H323" t="n">
         <v>0</v>
@@ -16589,7 +16589,7 @@
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>0.28</v>
+        <v>0.279</v>
       </c>
       <c r="L323" t="n">
         <v>1</v>
@@ -16614,20 +16614,20 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>11.2</v>
+        <v>11.7</v>
       </c>
       <c r="E324" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F324" t="n">
-        <v>3.6</v>
+        <v>1.1</v>
       </c>
       <c r="G324" t="n">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -16664,20 +16664,20 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>13.8</v>
+        <v>14</v>
       </c>
       <c r="E325" t="n">
         <v>54</v>
       </c>
       <c r="F325" t="n">
-        <v>2.5</v>
+        <v>1.4</v>
       </c>
       <c r="G325" t="n">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="H325" t="n">
         <v>0</v>
@@ -16714,20 +16714,20 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>16.2</v>
+        <v>16.6</v>
       </c>
       <c r="E326" t="n">
         <v>47</v>
       </c>
       <c r="F326" t="n">
-        <v>4.7</v>
+        <v>4.3</v>
       </c>
       <c r="G326" t="n">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="H326" t="n">
         <v>0</v>
@@ -16739,7 +16739,7 @@
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>0.277</v>
+        <v>0.276</v>
       </c>
       <c r="L326" t="n">
         <v>1</v>
@@ -16764,20 +16764,20 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>18</v>
+        <v>18.2</v>
       </c>
       <c r="E327" t="n">
         <v>42</v>
       </c>
       <c r="F327" t="n">
-        <v>7.6</v>
+        <v>5.4</v>
       </c>
       <c r="G327" t="n">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="H327" t="n">
         <v>0</v>
@@ -16789,7 +16789,7 @@
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="L327" t="n">
         <v>1</v>
@@ -16814,20 +16814,20 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>19</v>
+        <v>19.2</v>
       </c>
       <c r="E328" t="n">
         <v>38</v>
       </c>
       <c r="F328" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="G328" t="n">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
@@ -16839,7 +16839,7 @@
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0.273</v>
+        <v>0.272</v>
       </c>
       <c r="L328" t="n">
         <v>1</v>
@@ -16864,20 +16864,20 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="E329" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F329" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="G329" t="n">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
@@ -16914,20 +16914,20 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="E330" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F330" t="n">
         <v>6.5</v>
       </c>
       <c r="G330" t="n">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H330" t="n">
         <v>0</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>19.3</v>
+        <v>19.5</v>
       </c>
       <c r="E331" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F331" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="G331" t="n">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="H331" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -17014,23 +17014,23 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>17.2</v>
+        <v>17.3</v>
       </c>
       <c r="E332" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F332" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="G332" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="H332" t="n">
-        <v>36</v>
+        <v>95</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>14.6</v>
+        <v>14.8</v>
       </c>
       <c r="E333" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F333" t="n">
-        <v>8.6</v>
+        <v>7.6</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="E334" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F334" t="n">
-        <v>8.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17164,23 +17164,23 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="E335" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F335" t="n">
-        <v>7.9</v>
+        <v>11.2</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="I335" t="n">
         <v>0</v>
@@ -17214,14 +17214,14 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
       <c r="E336" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F336" t="n">
         <v>7.9</v>
@@ -17230,7 +17230,7 @@
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="E337" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F337" t="n">
-        <v>2.2</v>
+        <v>1.4</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>20</v>
+        <v>87</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17314,23 +17314,23 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E338" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F338" t="n">
-        <v>4.3</v>
+        <v>2.2</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
       <c r="E339" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F339" t="n">
-        <v>4.7</v>
+        <v>2.9</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17414,23 +17414,23 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>7.1</v>
+        <v>7.6</v>
       </c>
       <c r="E340" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F340" t="n">
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I340" t="n">
         <v>0</v>
@@ -17464,23 +17464,23 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="E341" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F341" t="n">
-        <v>4.7</v>
+        <v>5.4</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="I341" t="n">
         <v>0</v>
@@ -17514,14 +17514,14 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="E342" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F342" t="n">
         <v>6.1</v>
@@ -17530,7 +17530,7 @@
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="I342" t="n">
         <v>0</v>
@@ -17564,23 +17564,23 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D343" t="n">
         <v>5.5</v>
       </c>
       <c r="E343" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F343" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="I343" t="n">
         <v>0</v>
@@ -17614,23 +17614,23 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D344" t="n">
         <v>5.2</v>
       </c>
       <c r="E344" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F344" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="I344" t="n">
         <v>0</v>
@@ -17664,23 +17664,23 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D345" t="n">
         <v>4.9</v>
       </c>
       <c r="E345" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F345" t="n">
-        <v>8.300000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="I345" t="n">
         <v>0</v>
@@ -17714,23 +17714,23 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
       <c r="E346" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F346" t="n">
-        <v>8.6</v>
+        <v>6.1</v>
       </c>
       <c r="G346" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H346" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I346" t="n">
         <v>0</v>
@@ -17764,20 +17764,20 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="E347" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F347" t="n">
         <v>6.8</v>
       </c>
       <c r="G347" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H347" t="n">
         <v>0</v>
@@ -17814,20 +17814,20 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>13.1</v>
+        <v>12.9</v>
       </c>
       <c r="E348" t="n">
         <v>51</v>
       </c>
       <c r="F348" t="n">
-        <v>7.2</v>
+        <v>8.6</v>
       </c>
       <c r="G348" t="n">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="H348" t="n">
         <v>0</v>
@@ -17864,20 +17864,20 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>16.6</v>
+        <v>16.2</v>
       </c>
       <c r="E349" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F349" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
       <c r="G349" t="n">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="H349" t="n">
         <v>0</v>
@@ -17914,7 +17914,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D350" t="n">
@@ -17924,10 +17924,10 @@
         <v>35</v>
       </c>
       <c r="F350" t="n">
-        <v>12.2</v>
+        <v>10.8</v>
       </c>
       <c r="G350" t="n">
-        <v>532</v>
+        <v>527</v>
       </c>
       <c r="H350" t="n">
         <v>0</v>
@@ -17964,20 +17964,20 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="E351" t="n">
         <v>31</v>
       </c>
       <c r="F351" t="n">
-        <v>12.6</v>
+        <v>11.9</v>
       </c>
       <c r="G351" t="n">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="H351" t="n">
         <v>0</v>
@@ -18014,11 +18014,11 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>21.1</v>
+        <v>21</v>
       </c>
       <c r="E352" t="n">
         <v>28</v>
@@ -18027,10 +18027,10 @@
         <v>11.5</v>
       </c>
       <c r="G352" t="n">
-        <v>530</v>
+        <v>521</v>
       </c>
       <c r="H352" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -18064,11 +18064,11 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>21.9</v>
+        <v>21.7</v>
       </c>
       <c r="E353" t="n">
         <v>27</v>
@@ -18077,7 +18077,7 @@
         <v>10.8</v>
       </c>
       <c r="G353" t="n">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="H353" t="n">
         <v>0</v>
@@ -18114,20 +18114,20 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>22.3</v>
+        <v>22</v>
       </c>
       <c r="E354" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F354" t="n">
-        <v>11.5</v>
+        <v>10.1</v>
       </c>
       <c r="G354" t="n">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="H354" t="n">
         <v>0</v>
@@ -18164,20 +18164,20 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>20.8</v>
+        <v>21.6</v>
       </c>
       <c r="E355" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F355" t="n">
-        <v>11.7</v>
+        <v>11.2</v>
       </c>
       <c r="G355" t="n">
-        <v>160.3</v>
+        <v>159</v>
       </c>
       <c r="H355" t="n">
         <v>0</v>
@@ -18214,20 +18214,20 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>17.1</v>
+        <v>19</v>
       </c>
       <c r="E356" t="n">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="F356" t="n">
-        <v>10.3</v>
+        <v>10.8</v>
       </c>
       <c r="G356" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H356" t="n">
         <v>0</v>
@@ -18264,17 +18264,17 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>14.8</v>
+        <v>16.6</v>
       </c>
       <c r="E357" t="n">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="F357" t="n">
-        <v>10.9</v>
+        <v>12.6</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
@@ -18314,17 +18314,17 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>13.7</v>
+        <v>15</v>
       </c>
       <c r="E358" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="F358" t="n">
-        <v>10.4</v>
+        <v>12.6</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
@@ -18364,17 +18364,17 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>13.5</v>
+        <v>14.1</v>
       </c>
       <c r="E359" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="F359" t="n">
-        <v>11</v>
+        <v>14.8</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
@@ -18414,17 +18414,17 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
       <c r="E360" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F360" t="n">
-        <v>12.2</v>
+        <v>14.4</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
@@ -18464,17 +18464,17 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>13.4</v>
+        <v>13</v>
       </c>
       <c r="E361" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F361" t="n">
-        <v>13.9</v>
+        <v>16.6</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>13.2</v>
+        <v>12.9</v>
       </c>
       <c r="E362" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="F362" t="n">
-        <v>14.2</v>
+        <v>18</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18564,17 +18564,17 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-18T11:03:28Z</t>
+          <t>2026-10-18T17:03:45Z</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="E363" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="F363" t="n">
-        <v>12.8</v>
+        <v>18.7</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
prognoza biciklista (zvanicna): 2026-10-19 01:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -16164,17 +16164,17 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="E315" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F315" t="n">
-        <v>7.6</v>
+        <v>7.9</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -16189,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
-        <v>0.279</v>
+        <v>0.269</v>
       </c>
       <c r="L315" t="n">
         <v>1</v>
@@ -16214,17 +16214,17 @@
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="E316" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F316" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="G316" t="n">
         <v>0</v>
@@ -16239,7 +16239,7 @@
         <v>0</v>
       </c>
       <c r="K316" t="n">
-        <v>0.279</v>
+        <v>0.269</v>
       </c>
       <c r="L316" t="n">
         <v>1</v>
@@ -16264,23 +16264,23 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="E317" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F317" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="G317" t="n">
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I317" t="n">
         <v>0</v>
@@ -16289,7 +16289,7 @@
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0.279</v>
+        <v>0.269</v>
       </c>
       <c r="L317" t="n">
         <v>1</v>
@@ -16314,23 +16314,23 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D318" t="n">
         <v>7.5</v>
       </c>
       <c r="E318" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F318" t="n">
-        <v>1.4</v>
+        <v>3.6</v>
       </c>
       <c r="G318" t="n">
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="I318" t="n">
         <v>0</v>
@@ -16339,7 +16339,7 @@
         <v>0</v>
       </c>
       <c r="K318" t="n">
-        <v>0.279</v>
+        <v>0.269</v>
       </c>
       <c r="L318" t="n">
         <v>1</v>
@@ -16364,14 +16364,14 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="E319" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F319" t="n">
         <v>1.1</v>
@@ -16380,7 +16380,7 @@
         <v>0</v>
       </c>
       <c r="H319" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="I319" t="n">
         <v>0</v>
@@ -16389,7 +16389,7 @@
         <v>0</v>
       </c>
       <c r="K319" t="n">
-        <v>0.279</v>
+        <v>0.269</v>
       </c>
       <c r="L319" t="n">
         <v>1</v>
@@ -16414,23 +16414,23 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="E320" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F320" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="G320" t="n">
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I320" t="n">
         <v>0</v>
@@ -16439,7 +16439,7 @@
         <v>0</v>
       </c>
       <c r="K320" t="n">
-        <v>0.279</v>
+        <v>0.269</v>
       </c>
       <c r="L320" t="n">
         <v>1</v>
@@ -16464,17 +16464,17 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="E321" t="n">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F321" t="n">
-        <v>3.6</v>
+        <v>2.2</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
@@ -16489,7 +16489,7 @@
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>0.28</v>
+        <v>0.269</v>
       </c>
       <c r="L321" t="n">
         <v>1</v>
@@ -16514,17 +16514,17 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="E322" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F322" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="G322" t="n">
         <v>45</v>
@@ -16539,7 +16539,7 @@
         <v>0</v>
       </c>
       <c r="K322" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="L322" t="n">
         <v>1</v>
@@ -16564,17 +16564,17 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D323" t="n">
         <v>8.9</v>
       </c>
       <c r="E323" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F323" t="n">
-        <v>5</v>
+        <v>0.7</v>
       </c>
       <c r="G323" t="n">
         <v>187</v>
@@ -16589,7 +16589,7 @@
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>0.279</v>
+        <v>0.269</v>
       </c>
       <c r="L323" t="n">
         <v>1</v>
@@ -16614,20 +16614,20 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D324" t="n">
         <v>11.7</v>
       </c>
       <c r="E324" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F324" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="G324" t="n">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="H324" t="n">
         <v>0</v>
@@ -16639,7 +16639,7 @@
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0.279</v>
+        <v>0.269</v>
       </c>
       <c r="L324" t="n">
         <v>1</v>
@@ -16664,23 +16664,23 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>14</v>
+        <v>14.2</v>
       </c>
       <c r="E325" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F325" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="G325" t="n">
         <v>458</v>
       </c>
       <c r="H325" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -16689,7 +16689,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>0.278</v>
+        <v>0.268</v>
       </c>
       <c r="L325" t="n">
         <v>1</v>
@@ -16714,23 +16714,23 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>16.6</v>
+        <v>16.7</v>
       </c>
       <c r="E326" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F326" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="G326" t="n">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="H326" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I326" t="n">
         <v>0</v>
@@ -16739,7 +16739,7 @@
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>0.276</v>
+        <v>0.266</v>
       </c>
       <c r="L326" t="n">
         <v>1</v>
@@ -16764,20 +16764,20 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>18.2</v>
+        <v>18.5</v>
       </c>
       <c r="E327" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F327" t="n">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="G327" t="n">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="H327" t="n">
         <v>0</v>
@@ -16789,7 +16789,7 @@
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>0.274</v>
+        <v>0.264</v>
       </c>
       <c r="L327" t="n">
         <v>1</v>
@@ -16814,20 +16814,20 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>19.2</v>
+        <v>19.5</v>
       </c>
       <c r="E328" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F328" t="n">
-        <v>7.6</v>
+        <v>6.8</v>
       </c>
       <c r="G328" t="n">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
@@ -16839,7 +16839,7 @@
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0.272</v>
+        <v>0.262</v>
       </c>
       <c r="L328" t="n">
         <v>1</v>
@@ -16864,20 +16864,20 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>19.6</v>
+        <v>19.9</v>
       </c>
       <c r="E329" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F329" t="n">
-        <v>6.1</v>
+        <v>6.8</v>
       </c>
       <c r="G329" t="n">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
@@ -16889,7 +16889,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>0.271</v>
+        <v>0.261</v>
       </c>
       <c r="L329" t="n">
         <v>1</v>
@@ -16914,20 +16914,20 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>19.8</v>
+        <v>20</v>
       </c>
       <c r="E330" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F330" t="n">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="G330" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H330" t="n">
         <v>0</v>
@@ -16939,7 +16939,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L330" t="n">
         <v>1</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="E331" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F331" t="n">
         <v>7.2</v>
       </c>
       <c r="G331" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H331" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -16989,7 +16989,7 @@
         <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>0.269</v>
+        <v>0.259</v>
       </c>
       <c r="L331" t="n">
         <v>1</v>
@@ -17014,23 +17014,23 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>17.3</v>
+        <v>17.5</v>
       </c>
       <c r="E332" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F332" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="G332" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H332" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -17039,7 +17039,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>0.269</v>
+        <v>0.259</v>
       </c>
       <c r="L332" t="n">
         <v>1</v>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>14.8</v>
+        <v>14.9</v>
       </c>
       <c r="E333" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F333" t="n">
-        <v>7.6</v>
+        <v>5.8</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17089,7 +17089,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>0.269</v>
+        <v>0.259</v>
       </c>
       <c r="L333" t="n">
         <v>1</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="E334" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F334" t="n">
-        <v>9.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17139,7 +17139,7 @@
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>0.269</v>
+        <v>0.259</v>
       </c>
       <c r="L334" t="n">
         <v>1</v>
@@ -17164,23 +17164,23 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="E335" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F335" t="n">
-        <v>11.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I335" t="n">
         <v>0</v>
@@ -17189,7 +17189,7 @@
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>0.269</v>
+        <v>0.259</v>
       </c>
       <c r="L335" t="n">
         <v>1</v>
@@ -17214,23 +17214,23 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>10.5</v>
+        <v>10.6</v>
       </c>
       <c r="E336" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F336" t="n">
-        <v>7.9</v>
+        <v>7.2</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17239,7 +17239,7 @@
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0.269</v>
+        <v>0.26</v>
       </c>
       <c r="L336" t="n">
         <v>1</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="E337" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F337" t="n">
-        <v>1.4</v>
+        <v>3.2</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>87</v>
+        <v>2</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17289,7 +17289,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>0.269</v>
+        <v>0.26</v>
       </c>
       <c r="L337" t="n">
         <v>1</v>
@@ -17314,14 +17314,14 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="E338" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F338" t="n">
         <v>2.2</v>
@@ -17330,7 +17330,7 @@
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17339,7 +17339,7 @@
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L338" t="n">
         <v>2</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E339" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F339" t="n">
-        <v>2.9</v>
+        <v>2.5</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>
@@ -17414,23 +17414,23 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>7.6</v>
+        <v>7.3</v>
       </c>
       <c r="E340" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F340" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I340" t="n">
         <v>0</v>
@@ -17439,7 +17439,7 @@
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L340" t="n">
         <v>2</v>
@@ -17464,23 +17464,23 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="E341" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F341" t="n">
-        <v>5.4</v>
+        <v>4.7</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I341" t="n">
         <v>0</v>
@@ -17489,7 +17489,7 @@
         <v>0</v>
       </c>
       <c r="K341" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L341" t="n">
         <v>2</v>
@@ -17514,23 +17514,23 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="E342" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F342" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I342" t="n">
         <v>0</v>
@@ -17539,7 +17539,7 @@
         <v>0</v>
       </c>
       <c r="K342" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L342" t="n">
         <v>2</v>
@@ -17564,23 +17564,23 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>5.5</v>
+        <v>6.2</v>
       </c>
       <c r="E343" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F343" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>7</v>
+        <v>74</v>
       </c>
       <c r="I343" t="n">
         <v>0</v>
@@ -17589,7 +17589,7 @@
         <v>0</v>
       </c>
       <c r="K343" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L343" t="n">
         <v>2</v>
@@ -17614,23 +17614,23 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>5.2</v>
+        <v>5.9</v>
       </c>
       <c r="E344" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F344" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="I344" t="n">
         <v>0</v>
@@ -17639,7 +17639,7 @@
         <v>0</v>
       </c>
       <c r="K344" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L344" t="n">
         <v>2</v>
@@ -17664,23 +17664,23 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>4.9</v>
+        <v>5.6</v>
       </c>
       <c r="E345" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F345" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="I345" t="n">
         <v>0</v>
@@ -17689,7 +17689,7 @@
         <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>0.27</v>
+        <v>0.261</v>
       </c>
       <c r="L345" t="n">
         <v>2</v>
@@ -17714,23 +17714,23 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>5.6</v>
+        <v>6.2</v>
       </c>
       <c r="E346" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F346" t="n">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
       <c r="G346" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H346" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I346" t="n">
         <v>0</v>
@@ -17739,7 +17739,7 @@
         <v>0</v>
       </c>
       <c r="K346" t="n">
-        <v>0.27</v>
+        <v>0.261</v>
       </c>
       <c r="L346" t="n">
         <v>2</v>
@@ -17764,20 +17764,20 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="E347" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F347" t="n">
-        <v>6.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G347" t="n">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H347" t="n">
         <v>0</v>
@@ -17789,7 +17789,7 @@
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>0.27</v>
+        <v>0.261</v>
       </c>
       <c r="L347" t="n">
         <v>2</v>
@@ -17814,20 +17814,20 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>12.9</v>
+        <v>13</v>
       </c>
       <c r="E348" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F348" t="n">
-        <v>8.6</v>
+        <v>10.1</v>
       </c>
       <c r="G348" t="n">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="H348" t="n">
         <v>0</v>
@@ -17839,7 +17839,7 @@
         <v>0</v>
       </c>
       <c r="K348" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="L348" t="n">
         <v>2</v>
@@ -17864,20 +17864,20 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D349" t="n">
         <v>16.2</v>
       </c>
       <c r="E349" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F349" t="n">
-        <v>9</v>
+        <v>10.4</v>
       </c>
       <c r="G349" t="n">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="H349" t="n">
         <v>0</v>
@@ -17889,7 +17889,7 @@
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>0.269</v>
+        <v>0.259</v>
       </c>
       <c r="L349" t="n">
         <v>2</v>
@@ -17914,23 +17914,23 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>18.6</v>
+        <v>18.5</v>
       </c>
       <c r="E350" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F350" t="n">
-        <v>10.8</v>
+        <v>10.4</v>
       </c>
       <c r="G350" t="n">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="H350" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I350" t="n">
         <v>0</v>
@@ -17939,7 +17939,7 @@
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>0.267</v>
+        <v>0.258</v>
       </c>
       <c r="L350" t="n">
         <v>2</v>
@@ -17964,23 +17964,23 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="E351" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F351" t="n">
-        <v>11.9</v>
+        <v>11.2</v>
       </c>
       <c r="G351" t="n">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="H351" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -17989,7 +17989,7 @@
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>0.265</v>
+        <v>0.256</v>
       </c>
       <c r="L351" t="n">
         <v>2</v>
@@ -18014,23 +18014,23 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D352" t="n">
         <v>21</v>
       </c>
       <c r="E352" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F352" t="n">
-        <v>11.5</v>
+        <v>10.8</v>
       </c>
       <c r="G352" t="n">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="H352" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -18039,7 +18039,7 @@
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>0.263</v>
+        <v>0.254</v>
       </c>
       <c r="L352" t="n">
         <v>2</v>
@@ -18064,20 +18064,20 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D353" t="n">
         <v>21.7</v>
       </c>
       <c r="E353" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F353" t="n">
         <v>10.8</v>
       </c>
       <c r="G353" t="n">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="H353" t="n">
         <v>0</v>
@@ -18089,7 +18089,7 @@
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>0.261</v>
+        <v>0.252</v>
       </c>
       <c r="L353" t="n">
         <v>2</v>
@@ -18114,7 +18114,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D354" t="n">
@@ -18124,10 +18124,10 @@
         <v>27</v>
       </c>
       <c r="F354" t="n">
-        <v>10.1</v>
+        <v>11.2</v>
       </c>
       <c r="G354" t="n">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H354" t="n">
         <v>0</v>
@@ -18139,7 +18139,7 @@
         <v>0</v>
       </c>
       <c r="K354" t="n">
-        <v>0.26</v>
+        <v>0.251</v>
       </c>
       <c r="L354" t="n">
         <v>2</v>
@@ -18164,17 +18164,17 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>21.6</v>
+        <v>21.5</v>
       </c>
       <c r="E355" t="n">
         <v>29</v>
       </c>
       <c r="F355" t="n">
-        <v>11.2</v>
+        <v>12.2</v>
       </c>
       <c r="G355" t="n">
         <v>159</v>
@@ -18189,7 +18189,7 @@
         <v>0</v>
       </c>
       <c r="K355" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L355" t="n">
         <v>2</v>
@@ -18214,17 +18214,17 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="E356" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F356" t="n">
-        <v>10.8</v>
+        <v>11.2</v>
       </c>
       <c r="G356" t="n">
         <v>27</v>
@@ -18239,7 +18239,7 @@
         <v>0</v>
       </c>
       <c r="K356" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L356" t="n">
         <v>2</v>
@@ -18264,17 +18264,17 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>16.6</v>
+        <v>16.4</v>
       </c>
       <c r="E357" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F357" t="n">
-        <v>12.6</v>
+        <v>11.2</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
@@ -18289,7 +18289,7 @@
         <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L357" t="n">
         <v>2</v>
@@ -18314,17 +18314,17 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="E358" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F358" t="n">
-        <v>12.6</v>
+        <v>11.9</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
@@ -18339,7 +18339,7 @@
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L358" t="n">
         <v>2</v>
@@ -18364,17 +18364,17 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>14.1</v>
+        <v>13.4</v>
       </c>
       <c r="E359" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F359" t="n">
-        <v>14.8</v>
+        <v>11.2</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
@@ -18389,7 +18389,7 @@
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L359" t="n">
         <v>2</v>
@@ -18414,17 +18414,17 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>13.5</v>
+        <v>12.7</v>
       </c>
       <c r="E360" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F360" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
@@ -18439,7 +18439,7 @@
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L360" t="n">
         <v>2</v>
@@ -18464,17 +18464,17 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>13</v>
+        <v>12.5</v>
       </c>
       <c r="E361" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F361" t="n">
-        <v>16.6</v>
+        <v>15.8</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
@@ -18489,7 +18489,7 @@
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L361" t="n">
         <v>2</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>12.9</v>
+        <v>12.5</v>
       </c>
       <c r="E362" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F362" t="n">
-        <v>18</v>
+        <v>16.9</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18539,7 +18539,7 @@
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L362" t="n">
         <v>3</v>
@@ -18564,17 +18564,17 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-18T17:03:45Z</t>
+          <t>2026-10-18T23:03:49Z</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>12.8</v>
+        <v>12.4</v>
       </c>
       <c r="E363" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F363" t="n">
-        <v>18.7</v>
+        <v>16.2</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -18589,7 +18589,7 @@
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>0.259</v>
+        <v>0.25</v>
       </c>
       <c r="L363" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-19 07:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N363"/>
+  <dimension ref="A1:N387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -16464,23 +16464,23 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>5.9</v>
+        <v>5.4</v>
       </c>
       <c r="E321" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="F321" t="n">
-        <v>2.2</v>
+        <v>4.7</v>
       </c>
       <c r="G321" t="n">
         <v>0</v>
       </c>
       <c r="H321" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="I321" t="n">
         <v>0</v>
@@ -16489,7 +16489,7 @@
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>0.269</v>
+        <v>0.268</v>
       </c>
       <c r="L321" t="n">
         <v>1</v>
@@ -16514,17 +16514,17 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="E322" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F322" t="n">
-        <v>3.2</v>
+        <v>6.5</v>
       </c>
       <c r="G322" t="n">
         <v>45</v>
@@ -16539,7 +16539,7 @@
         <v>0</v>
       </c>
       <c r="K322" t="n">
-        <v>0.27</v>
+        <v>0.268</v>
       </c>
       <c r="L322" t="n">
         <v>1</v>
@@ -16564,17 +16564,17 @@
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="E323" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="F323" t="n">
-        <v>0.7</v>
+        <v>5.4</v>
       </c>
       <c r="G323" t="n">
         <v>187</v>
@@ -16589,7 +16589,7 @@
         <v>0</v>
       </c>
       <c r="K323" t="n">
-        <v>0.269</v>
+        <v>0.268</v>
       </c>
       <c r="L323" t="n">
         <v>1</v>
@@ -16614,17 +16614,17 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D324" t="n">
         <v>11.7</v>
       </c>
       <c r="E324" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F324" t="n">
-        <v>0.7</v>
+        <v>6.1</v>
       </c>
       <c r="G324" t="n">
         <v>337</v>
@@ -16639,7 +16639,7 @@
         <v>0</v>
       </c>
       <c r="K324" t="n">
-        <v>0.269</v>
+        <v>0.267</v>
       </c>
       <c r="L324" t="n">
         <v>1</v>
@@ -16664,23 +16664,23 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>14.2</v>
+        <v>14.3</v>
       </c>
       <c r="E325" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F325" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G325" t="n">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="H325" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="I325" t="n">
         <v>0</v>
@@ -16689,7 +16689,7 @@
         <v>0</v>
       </c>
       <c r="K325" t="n">
-        <v>0.268</v>
+        <v>0.266</v>
       </c>
       <c r="L325" t="n">
         <v>1</v>
@@ -16714,23 +16714,23 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>16.7</v>
+        <v>16.8</v>
       </c>
       <c r="E326" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F326" t="n">
-        <v>3.2</v>
+        <v>6.5</v>
       </c>
       <c r="G326" t="n">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="H326" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I326" t="n">
         <v>0</v>
@@ -16739,7 +16739,7 @@
         <v>0</v>
       </c>
       <c r="K326" t="n">
-        <v>0.266</v>
+        <v>0.264</v>
       </c>
       <c r="L326" t="n">
         <v>1</v>
@@ -16764,17 +16764,17 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>18.5</v>
+        <v>18.7</v>
       </c>
       <c r="E327" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="F327" t="n">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="G327" t="n">
         <v>557</v>
@@ -16789,7 +16789,7 @@
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>0.264</v>
+        <v>0.262</v>
       </c>
       <c r="L327" t="n">
         <v>1</v>
@@ -16814,20 +16814,20 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="E328" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F328" t="n">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="G328" t="n">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
@@ -16839,7 +16839,7 @@
         <v>0</v>
       </c>
       <c r="K328" t="n">
-        <v>0.262</v>
+        <v>0.261</v>
       </c>
       <c r="L328" t="n">
         <v>1</v>
@@ -16864,20 +16864,20 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>19.9</v>
+        <v>20.2</v>
       </c>
       <c r="E329" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F329" t="n">
-        <v>6.8</v>
+        <v>5.8</v>
       </c>
       <c r="G329" t="n">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="H329" t="n">
         <v>0</v>
@@ -16889,7 +16889,7 @@
         <v>0</v>
       </c>
       <c r="K329" t="n">
-        <v>0.261</v>
+        <v>0.259</v>
       </c>
       <c r="L329" t="n">
         <v>1</v>
@@ -16914,20 +16914,20 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>20</v>
+        <v>20.4</v>
       </c>
       <c r="E330" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F330" t="n">
         <v>6.8</v>
       </c>
       <c r="G330" t="n">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H330" t="n">
         <v>0</v>
@@ -16939,7 +16939,7 @@
         <v>0</v>
       </c>
       <c r="K330" t="n">
-        <v>0.26</v>
+        <v>0.258</v>
       </c>
       <c r="L330" t="n">
         <v>1</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>19.6</v>
+        <v>19.9</v>
       </c>
       <c r="E331" t="n">
         <v>34</v>
       </c>
       <c r="F331" t="n">
-        <v>7.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G331" t="n">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="H331" t="n">
-        <v>52</v>
+        <v>98</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -16989,7 +16989,7 @@
         <v>0</v>
       </c>
       <c r="K331" t="n">
-        <v>0.259</v>
+        <v>0.258</v>
       </c>
       <c r="L331" t="n">
         <v>1</v>
@@ -17014,23 +17014,23 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
       <c r="E332" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F332" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="G332" t="n">
         <v>28</v>
       </c>
       <c r="H332" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -17039,7 +17039,7 @@
         <v>0</v>
       </c>
       <c r="K332" t="n">
-        <v>0.259</v>
+        <v>0.258</v>
       </c>
       <c r="L332" t="n">
         <v>1</v>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
       <c r="E333" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F333" t="n">
-        <v>5.8</v>
+        <v>7.9</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>66</v>
+        <v>99</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17089,7 +17089,7 @@
         <v>0</v>
       </c>
       <c r="K333" t="n">
-        <v>0.259</v>
+        <v>0.258</v>
       </c>
       <c r="L333" t="n">
         <v>1</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D334" t="n">
         <v>13.2</v>
       </c>
       <c r="E334" t="n">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F334" t="n">
-        <v>10.4</v>
+        <v>6.8</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>47</v>
+        <v>99</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17139,7 +17139,7 @@
         <v>0</v>
       </c>
       <c r="K334" t="n">
-        <v>0.259</v>
+        <v>0.258</v>
       </c>
       <c r="L334" t="n">
         <v>1</v>
@@ -17164,14 +17164,14 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11.8</v>
+        <v>12.1</v>
       </c>
       <c r="E335" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F335" t="n">
         <v>9.699999999999999</v>
@@ -17180,7 +17180,7 @@
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="I335" t="n">
         <v>0</v>
@@ -17189,7 +17189,7 @@
         <v>0</v>
       </c>
       <c r="K335" t="n">
-        <v>0.259</v>
+        <v>0.258</v>
       </c>
       <c r="L335" t="n">
         <v>1</v>
@@ -17214,23 +17214,23 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>10.6</v>
+        <v>11.5</v>
       </c>
       <c r="E336" t="n">
         <v>55</v>
       </c>
       <c r="F336" t="n">
-        <v>7.2</v>
+        <v>10.1</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>28</v>
+        <v>99</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17239,7 +17239,7 @@
         <v>0</v>
       </c>
       <c r="K336" t="n">
-        <v>0.26</v>
+        <v>0.258</v>
       </c>
       <c r="L336" t="n">
         <v>1</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>9.5</v>
+        <v>10.4</v>
       </c>
       <c r="E337" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F337" t="n">
-        <v>3.2</v>
+        <v>6.8</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17289,7 +17289,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>0.26</v>
+        <v>0.258</v>
       </c>
       <c r="L337" t="n">
         <v>1</v>
@@ -17314,23 +17314,23 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>8.9</v>
+        <v>9.4</v>
       </c>
       <c r="E338" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F338" t="n">
-        <v>2.2</v>
+        <v>1.4</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17339,7 +17339,7 @@
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0.26</v>
+        <v>0.258</v>
       </c>
       <c r="L338" t="n">
         <v>2</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>8.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E339" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F339" t="n">
-        <v>2.5</v>
+        <v>0.4</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.26</v>
+        <v>0.258</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>
@@ -17414,23 +17414,23 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>7.3</v>
+        <v>7.8</v>
       </c>
       <c r="E340" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F340" t="n">
-        <v>3.6</v>
+        <v>1.8</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="I340" t="n">
         <v>0</v>
@@ -17439,7 +17439,7 @@
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>0.26</v>
+        <v>0.258</v>
       </c>
       <c r="L340" t="n">
         <v>2</v>
@@ -17464,23 +17464,23 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>6.8</v>
+        <v>7.3</v>
       </c>
       <c r="E341" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F341" t="n">
-        <v>4.7</v>
+        <v>3.2</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="I341" t="n">
         <v>0</v>
@@ -17489,7 +17489,7 @@
         <v>0</v>
       </c>
       <c r="K341" t="n">
-        <v>0.26</v>
+        <v>0.259</v>
       </c>
       <c r="L341" t="n">
         <v>2</v>
@@ -17514,23 +17514,23 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>6.3</v>
+        <v>6.7</v>
       </c>
       <c r="E342" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F342" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="I342" t="n">
         <v>0</v>
@@ -17539,7 +17539,7 @@
         <v>0</v>
       </c>
       <c r="K342" t="n">
-        <v>0.26</v>
+        <v>0.259</v>
       </c>
       <c r="L342" t="n">
         <v>2</v>
@@ -17564,23 +17564,23 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="E343" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F343" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>74</v>
+        <v>6</v>
       </c>
       <c r="I343" t="n">
         <v>0</v>
@@ -17589,7 +17589,7 @@
         <v>0</v>
       </c>
       <c r="K343" t="n">
-        <v>0.26</v>
+        <v>0.259</v>
       </c>
       <c r="L343" t="n">
         <v>2</v>
@@ -17614,23 +17614,23 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>5.9</v>
+        <v>5.6</v>
       </c>
       <c r="E344" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F344" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="I344" t="n">
         <v>0</v>
@@ -17639,7 +17639,7 @@
         <v>0</v>
       </c>
       <c r="K344" t="n">
-        <v>0.26</v>
+        <v>0.259</v>
       </c>
       <c r="L344" t="n">
         <v>2</v>
@@ -17664,23 +17664,23 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="E345" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F345" t="n">
-        <v>7.6</v>
+        <v>6.5</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="I345" t="n">
         <v>0</v>
@@ -17689,7 +17689,7 @@
         <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>0.261</v>
+        <v>0.259</v>
       </c>
       <c r="L345" t="n">
         <v>2</v>
@@ -17714,14 +17714,14 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
       <c r="E346" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F346" t="n">
         <v>7.2</v>
@@ -17730,7 +17730,7 @@
         <v>41</v>
       </c>
       <c r="H346" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="I346" t="n">
         <v>0</v>
@@ -17739,7 +17739,7 @@
         <v>0</v>
       </c>
       <c r="K346" t="n">
-        <v>0.261</v>
+        <v>0.259</v>
       </c>
       <c r="L346" t="n">
         <v>2</v>
@@ -17764,23 +17764,23 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D347" t="n">
         <v>8.9</v>
       </c>
       <c r="E347" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F347" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G347" t="n">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="H347" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I347" t="n">
         <v>0</v>
@@ -17789,7 +17789,7 @@
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>0.261</v>
+        <v>0.259</v>
       </c>
       <c r="L347" t="n">
         <v>2</v>
@@ -17814,23 +17814,23 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>13</v>
+        <v>12.8</v>
       </c>
       <c r="E348" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F348" t="n">
-        <v>10.1</v>
+        <v>8.6</v>
       </c>
       <c r="G348" t="n">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="H348" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I348" t="n">
         <v>0</v>
@@ -17839,7 +17839,7 @@
         <v>0</v>
       </c>
       <c r="K348" t="n">
-        <v>0.26</v>
+        <v>0.259</v>
       </c>
       <c r="L348" t="n">
         <v>2</v>
@@ -17864,23 +17864,23 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>16.2</v>
+        <v>16.6</v>
       </c>
       <c r="E349" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F349" t="n">
-        <v>10.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G349" t="n">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="H349" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -17889,7 +17889,7 @@
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>0.259</v>
+        <v>0.258</v>
       </c>
       <c r="L349" t="n">
         <v>2</v>
@@ -17914,23 +17914,23 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
       <c r="E350" t="n">
         <v>36</v>
       </c>
       <c r="F350" t="n">
-        <v>10.4</v>
+        <v>10.8</v>
       </c>
       <c r="G350" t="n">
-        <v>525</v>
+        <v>515</v>
       </c>
       <c r="H350" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="I350" t="n">
         <v>0</v>
@@ -17939,7 +17939,7 @@
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>0.258</v>
+        <v>0.256</v>
       </c>
       <c r="L350" t="n">
         <v>2</v>
@@ -17964,23 +17964,23 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>20</v>
+        <v>20.4</v>
       </c>
       <c r="E351" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F351" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="G351" t="n">
-        <v>549</v>
+        <v>541</v>
       </c>
       <c r="H351" t="n">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -17989,7 +17989,7 @@
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>0.256</v>
+        <v>0.254</v>
       </c>
       <c r="L351" t="n">
         <v>2</v>
@@ -18014,23 +18014,23 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>21</v>
+        <v>21.3</v>
       </c>
       <c r="E352" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F352" t="n">
-        <v>10.8</v>
+        <v>11.5</v>
       </c>
       <c r="G352" t="n">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="H352" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -18039,7 +18039,7 @@
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>0.254</v>
+        <v>0.253</v>
       </c>
       <c r="L352" t="n">
         <v>2</v>
@@ -18064,23 +18064,23 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>21.7</v>
+        <v>21.9</v>
       </c>
       <c r="E353" t="n">
         <v>28</v>
       </c>
       <c r="F353" t="n">
-        <v>10.8</v>
+        <v>10.4</v>
       </c>
       <c r="G353" t="n">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="H353" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -18089,7 +18089,7 @@
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>0.252</v>
+        <v>0.251</v>
       </c>
       <c r="L353" t="n">
         <v>2</v>
@@ -18114,20 +18114,20 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>22</v>
+        <v>22.1</v>
       </c>
       <c r="E354" t="n">
         <v>27</v>
       </c>
       <c r="F354" t="n">
-        <v>11.2</v>
+        <v>10.1</v>
       </c>
       <c r="G354" t="n">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="H354" t="n">
         <v>0</v>
@@ -18139,7 +18139,7 @@
         <v>0</v>
       </c>
       <c r="K354" t="n">
-        <v>0.251</v>
+        <v>0.25</v>
       </c>
       <c r="L354" t="n">
         <v>2</v>
@@ -18164,20 +18164,20 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="E355" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F355" t="n">
-        <v>12.2</v>
+        <v>10.8</v>
       </c>
       <c r="G355" t="n">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H355" t="n">
         <v>0</v>
@@ -18189,7 +18189,7 @@
         <v>0</v>
       </c>
       <c r="K355" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L355" t="n">
         <v>2</v>
@@ -18214,11 +18214,11 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="E356" t="n">
         <v>35</v>
@@ -18239,7 +18239,7 @@
         <v>0</v>
       </c>
       <c r="K356" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L356" t="n">
         <v>2</v>
@@ -18264,17 +18264,17 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>16.4</v>
+        <v>16.5</v>
       </c>
       <c r="E357" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F357" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
@@ -18289,7 +18289,7 @@
         <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L357" t="n">
         <v>2</v>
@@ -18314,17 +18314,17 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D358" t="n">
         <v>14.9</v>
       </c>
       <c r="E358" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F358" t="n">
-        <v>11.9</v>
+        <v>12.2</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
@@ -18339,7 +18339,7 @@
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L358" t="n">
         <v>2</v>
@@ -18364,17 +18364,17 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="E359" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F359" t="n">
-        <v>11.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
@@ -18389,7 +18389,7 @@
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L359" t="n">
         <v>2</v>
@@ -18414,17 +18414,17 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="E360" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F360" t="n">
-        <v>13.3</v>
+        <v>11.9</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
@@ -18439,7 +18439,7 @@
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L360" t="n">
         <v>2</v>
@@ -18464,17 +18464,17 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>12.5</v>
+        <v>12.3</v>
       </c>
       <c r="E361" t="n">
         <v>72</v>
       </c>
       <c r="F361" t="n">
-        <v>15.8</v>
+        <v>15.5</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
@@ -18489,7 +18489,7 @@
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L361" t="n">
         <v>2</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>12.5</v>
+        <v>12.3</v>
       </c>
       <c r="E362" t="n">
         <v>72</v>
       </c>
       <c r="F362" t="n">
-        <v>16.9</v>
+        <v>16.2</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18539,7 +18539,7 @@
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L362" t="n">
         <v>3</v>
@@ -18564,7 +18564,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-18T23:03:49Z</t>
+          <t>2026-10-19T05:03:39Z</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -18574,7 +18574,7 @@
         <v>71</v>
       </c>
       <c r="F363" t="n">
-        <v>16.2</v>
+        <v>16.9</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -18589,7 +18589,7 @@
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>0.25</v>
+        <v>0.249</v>
       </c>
       <c r="L363" t="n">
         <v>3</v>
@@ -18598,6 +18598,1206 @@
         <v>0</v>
       </c>
       <c r="N363" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E364" t="n">
+        <v>70</v>
+      </c>
+      <c r="F364" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="G364" t="n">
+        <v>0</v>
+      </c>
+      <c r="H364" t="n">
+        <v>0</v>
+      </c>
+      <c r="I364" t="n">
+        <v>0</v>
+      </c>
+      <c r="J364" t="n">
+        <v>0</v>
+      </c>
+      <c r="K364" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L364" t="n">
+        <v>3</v>
+      </c>
+      <c r="M364" t="n">
+        <v>0</v>
+      </c>
+      <c r="N364" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="E365" t="n">
+        <v>68</v>
+      </c>
+      <c r="F365" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0</v>
+      </c>
+      <c r="H365" t="n">
+        <v>0</v>
+      </c>
+      <c r="I365" t="n">
+        <v>0</v>
+      </c>
+      <c r="J365" t="n">
+        <v>0</v>
+      </c>
+      <c r="K365" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L365" t="n">
+        <v>3</v>
+      </c>
+      <c r="M365" t="n">
+        <v>0</v>
+      </c>
+      <c r="N365" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>12</v>
+      </c>
+      <c r="E366" t="n">
+        <v>69</v>
+      </c>
+      <c r="F366" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0</v>
+      </c>
+      <c r="H366" t="n">
+        <v>0</v>
+      </c>
+      <c r="I366" t="n">
+        <v>0</v>
+      </c>
+      <c r="J366" t="n">
+        <v>0</v>
+      </c>
+      <c r="K366" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L366" t="n">
+        <v>3</v>
+      </c>
+      <c r="M366" t="n">
+        <v>0</v>
+      </c>
+      <c r="N366" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="E367" t="n">
+        <v>71</v>
+      </c>
+      <c r="F367" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0</v>
+      </c>
+      <c r="H367" t="n">
+        <v>0</v>
+      </c>
+      <c r="I367" t="n">
+        <v>0</v>
+      </c>
+      <c r="J367" t="n">
+        <v>0</v>
+      </c>
+      <c r="K367" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L367" t="n">
+        <v>3</v>
+      </c>
+      <c r="M367" t="n">
+        <v>0</v>
+      </c>
+      <c r="N367" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="E368" t="n">
+        <v>72</v>
+      </c>
+      <c r="F368" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0</v>
+      </c>
+      <c r="H368" t="n">
+        <v>68</v>
+      </c>
+      <c r="I368" t="n">
+        <v>0</v>
+      </c>
+      <c r="J368" t="n">
+        <v>0</v>
+      </c>
+      <c r="K368" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L368" t="n">
+        <v>3</v>
+      </c>
+      <c r="M368" t="n">
+        <v>0</v>
+      </c>
+      <c r="N368" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="E369" t="n">
+        <v>75</v>
+      </c>
+      <c r="F369" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="G369" t="n">
+        <v>0</v>
+      </c>
+      <c r="H369" t="n">
+        <v>98</v>
+      </c>
+      <c r="I369" t="n">
+        <v>0</v>
+      </c>
+      <c r="J369" t="n">
+        <v>0</v>
+      </c>
+      <c r="K369" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L369" t="n">
+        <v>3</v>
+      </c>
+      <c r="M369" t="n">
+        <v>0</v>
+      </c>
+      <c r="N369" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="E370" t="n">
+        <v>75</v>
+      </c>
+      <c r="F370" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="G370" t="n">
+        <v>39</v>
+      </c>
+      <c r="H370" t="n">
+        <v>22</v>
+      </c>
+      <c r="I370" t="n">
+        <v>0</v>
+      </c>
+      <c r="J370" t="n">
+        <v>0</v>
+      </c>
+      <c r="K370" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L370" t="n">
+        <v>3</v>
+      </c>
+      <c r="M370" t="n">
+        <v>0</v>
+      </c>
+      <c r="N370" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="E371" t="n">
+        <v>65</v>
+      </c>
+      <c r="F371" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="G371" t="n">
+        <v>178</v>
+      </c>
+      <c r="H371" t="n">
+        <v>0</v>
+      </c>
+      <c r="I371" t="n">
+        <v>0</v>
+      </c>
+      <c r="J371" t="n">
+        <v>0</v>
+      </c>
+      <c r="K371" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L371" t="n">
+        <v>3</v>
+      </c>
+      <c r="M371" t="n">
+        <v>0</v>
+      </c>
+      <c r="N371" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="E372" t="n">
+        <v>53</v>
+      </c>
+      <c r="F372" t="n">
+        <v>18</v>
+      </c>
+      <c r="G372" t="n">
+        <v>325</v>
+      </c>
+      <c r="H372" t="n">
+        <v>0</v>
+      </c>
+      <c r="I372" t="n">
+        <v>0</v>
+      </c>
+      <c r="J372" t="n">
+        <v>0</v>
+      </c>
+      <c r="K372" t="n">
+        <v>0.248</v>
+      </c>
+      <c r="L372" t="n">
+        <v>3</v>
+      </c>
+      <c r="M372" t="n">
+        <v>0</v>
+      </c>
+      <c r="N372" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="E373" t="n">
+        <v>47</v>
+      </c>
+      <c r="F373" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="G373" t="n">
+        <v>444</v>
+      </c>
+      <c r="H373" t="n">
+        <v>7</v>
+      </c>
+      <c r="I373" t="n">
+        <v>0</v>
+      </c>
+      <c r="J373" t="n">
+        <v>0</v>
+      </c>
+      <c r="K373" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L373" t="n">
+        <v>3</v>
+      </c>
+      <c r="M373" t="n">
+        <v>0</v>
+      </c>
+      <c r="N373" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="E374" t="n">
+        <v>45</v>
+      </c>
+      <c r="F374" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="G374" t="n">
+        <v>517</v>
+      </c>
+      <c r="H374" t="n">
+        <v>23</v>
+      </c>
+      <c r="I374" t="n">
+        <v>0</v>
+      </c>
+      <c r="J374" t="n">
+        <v>0</v>
+      </c>
+      <c r="K374" t="n">
+        <v>0.244</v>
+      </c>
+      <c r="L374" t="n">
+        <v>3</v>
+      </c>
+      <c r="M374" t="n">
+        <v>0</v>
+      </c>
+      <c r="N374" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E375" t="n">
+        <v>45</v>
+      </c>
+      <c r="F375" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="G375" t="n">
+        <v>533.8</v>
+      </c>
+      <c r="H375" t="n">
+        <v>37</v>
+      </c>
+      <c r="I375" t="n">
+        <v>0</v>
+      </c>
+      <c r="J375" t="n">
+        <v>0</v>
+      </c>
+      <c r="K375" t="n">
+        <v>0.242</v>
+      </c>
+      <c r="L375" t="n">
+        <v>3</v>
+      </c>
+      <c r="M375" t="n">
+        <v>0</v>
+      </c>
+      <c r="N375" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="E376" t="n">
+        <v>48</v>
+      </c>
+      <c r="F376" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="G376" t="n">
+        <v>497</v>
+      </c>
+      <c r="H376" t="n">
+        <v>30</v>
+      </c>
+      <c r="I376" t="n">
+        <v>0</v>
+      </c>
+      <c r="J376" t="n">
+        <v>0</v>
+      </c>
+      <c r="K376" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="L376" t="n">
+        <v>3</v>
+      </c>
+      <c r="M376" t="n">
+        <v>0</v>
+      </c>
+      <c r="N376" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="E377" t="n">
+        <v>47</v>
+      </c>
+      <c r="F377" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G377" t="n">
+        <v>406</v>
+      </c>
+      <c r="H377" t="n">
+        <v>62</v>
+      </c>
+      <c r="I377" t="n">
+        <v>0</v>
+      </c>
+      <c r="J377" t="n">
+        <v>0</v>
+      </c>
+      <c r="K377" t="n">
+        <v>0.238</v>
+      </c>
+      <c r="L377" t="n">
+        <v>3</v>
+      </c>
+      <c r="M377" t="n">
+        <v>0</v>
+      </c>
+      <c r="N377" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="E378" t="n">
+        <v>50</v>
+      </c>
+      <c r="F378" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G378" t="n">
+        <v>270</v>
+      </c>
+      <c r="H378" t="n">
+        <v>76</v>
+      </c>
+      <c r="I378" t="n">
+        <v>0</v>
+      </c>
+      <c r="J378" t="n">
+        <v>0</v>
+      </c>
+      <c r="K378" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="L378" t="n">
+        <v>3</v>
+      </c>
+      <c r="M378" t="n">
+        <v>0</v>
+      </c>
+      <c r="N378" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="E379" t="n">
+        <v>55</v>
+      </c>
+      <c r="F379" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="G379" t="n">
+        <v>118</v>
+      </c>
+      <c r="H379" t="n">
+        <v>93</v>
+      </c>
+      <c r="I379" t="n">
+        <v>0</v>
+      </c>
+      <c r="J379" t="n">
+        <v>0</v>
+      </c>
+      <c r="K379" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="L379" t="n">
+        <v>3</v>
+      </c>
+      <c r="M379" t="n">
+        <v>0</v>
+      </c>
+      <c r="N379" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="E380" t="n">
+        <v>59</v>
+      </c>
+      <c r="F380" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="G380" t="n">
+        <v>15</v>
+      </c>
+      <c r="H380" t="n">
+        <v>97</v>
+      </c>
+      <c r="I380" t="n">
+        <v>0</v>
+      </c>
+      <c r="J380" t="n">
+        <v>0</v>
+      </c>
+      <c r="K380" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="L380" t="n">
+        <v>3</v>
+      </c>
+      <c r="M380" t="n">
+        <v>0</v>
+      </c>
+      <c r="N380" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="E381" t="n">
+        <v>59</v>
+      </c>
+      <c r="F381" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0</v>
+      </c>
+      <c r="H381" t="n">
+        <v>77</v>
+      </c>
+      <c r="I381" t="n">
+        <v>0</v>
+      </c>
+      <c r="J381" t="n">
+        <v>0</v>
+      </c>
+      <c r="K381" t="n">
+        <v>0.234</v>
+      </c>
+      <c r="L381" t="n">
+        <v>3</v>
+      </c>
+      <c r="M381" t="n">
+        <v>0</v>
+      </c>
+      <c r="N381" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>19</v>
+      </c>
+      <c r="E382" t="n">
+        <v>61</v>
+      </c>
+      <c r="F382" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G382" t="n">
+        <v>0</v>
+      </c>
+      <c r="H382" t="n">
+        <v>100</v>
+      </c>
+      <c r="I382" t="n">
+        <v>0</v>
+      </c>
+      <c r="J382" t="n">
+        <v>0</v>
+      </c>
+      <c r="K382" t="n">
+        <v>0.234</v>
+      </c>
+      <c r="L382" t="n">
+        <v>3</v>
+      </c>
+      <c r="M382" t="n">
+        <v>0</v>
+      </c>
+      <c r="N382" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="E383" t="n">
+        <v>60</v>
+      </c>
+      <c r="F383" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="G383" t="n">
+        <v>0</v>
+      </c>
+      <c r="H383" t="n">
+        <v>100</v>
+      </c>
+      <c r="I383" t="n">
+        <v>0</v>
+      </c>
+      <c r="J383" t="n">
+        <v>0</v>
+      </c>
+      <c r="K383" t="n">
+        <v>0.233</v>
+      </c>
+      <c r="L383" t="n">
+        <v>3</v>
+      </c>
+      <c r="M383" t="n">
+        <v>0</v>
+      </c>
+      <c r="N383" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="E384" t="n">
+        <v>62</v>
+      </c>
+      <c r="F384" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="G384" t="n">
+        <v>0</v>
+      </c>
+      <c r="H384" t="n">
+        <v>97</v>
+      </c>
+      <c r="I384" t="n">
+        <v>0</v>
+      </c>
+      <c r="J384" t="n">
+        <v>0</v>
+      </c>
+      <c r="K384" t="n">
+        <v>0.233</v>
+      </c>
+      <c r="L384" t="n">
+        <v>3</v>
+      </c>
+      <c r="M384" t="n">
+        <v>0</v>
+      </c>
+      <c r="N384" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="E385" t="n">
+        <v>66</v>
+      </c>
+      <c r="F385" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0</v>
+      </c>
+      <c r="H385" t="n">
+        <v>84</v>
+      </c>
+      <c r="I385" t="n">
+        <v>0</v>
+      </c>
+      <c r="J385" t="n">
+        <v>0</v>
+      </c>
+      <c r="K385" t="n">
+        <v>0.232</v>
+      </c>
+      <c r="L385" t="n">
+        <v>3</v>
+      </c>
+      <c r="M385" t="n">
+        <v>0</v>
+      </c>
+      <c r="N385" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="E386" t="n">
+        <v>67</v>
+      </c>
+      <c r="F386" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G386" t="n">
+        <v>0</v>
+      </c>
+      <c r="H386" t="n">
+        <v>65</v>
+      </c>
+      <c r="I386" t="n">
+        <v>0</v>
+      </c>
+      <c r="J386" t="n">
+        <v>0</v>
+      </c>
+      <c r="K386" t="n">
+        <v>0.232</v>
+      </c>
+      <c r="L386" t="n">
+        <v>4</v>
+      </c>
+      <c r="M386" t="n">
+        <v>0</v>
+      </c>
+      <c r="N386" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>2026-10-19T05:03:39Z</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="E387" t="n">
+        <v>69</v>
+      </c>
+      <c r="F387" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="G387" t="n">
+        <v>0</v>
+      </c>
+      <c r="H387" t="n">
+        <v>75</v>
+      </c>
+      <c r="I387" t="n">
+        <v>0</v>
+      </c>
+      <c r="J387" t="n">
+        <v>0</v>
+      </c>
+      <c r="K387" t="n">
+        <v>0.232</v>
+      </c>
+      <c r="L387" t="n">
+        <v>4</v>
+      </c>
+      <c r="M387" t="n">
+        <v>0</v>
+      </c>
+      <c r="N387" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-19 13:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -16764,17 +16764,17 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>18.7</v>
+        <v>18.3</v>
       </c>
       <c r="E327" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F327" t="n">
-        <v>7.6</v>
+        <v>6.5</v>
       </c>
       <c r="G327" t="n">
         <v>557</v>
@@ -16789,7 +16789,7 @@
         <v>0</v>
       </c>
       <c r="K327" t="n">
-        <v>0.262</v>
+        <v>0.263</v>
       </c>
       <c r="L327" t="n">
         <v>1</v>
@@ -16814,20 +16814,20 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>19.6</v>
+        <v>19.2</v>
       </c>
       <c r="E328" t="n">
         <v>33</v>
       </c>
       <c r="F328" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="G328" t="n">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H328" t="n">
         <v>0</v>
@@ -16864,17 +16864,17 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>20.2</v>
+        <v>19.8</v>
       </c>
       <c r="E329" t="n">
         <v>33</v>
       </c>
       <c r="F329" t="n">
-        <v>5.8</v>
+        <v>4.7</v>
       </c>
       <c r="G329" t="n">
         <v>441</v>
@@ -16914,20 +16914,20 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>20.4</v>
+        <v>19.9</v>
       </c>
       <c r="E330" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F330" t="n">
-        <v>6.8</v>
+        <v>4.7</v>
       </c>
       <c r="G330" t="n">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="H330" t="n">
         <v>0</v>
@@ -16964,23 +16964,23 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>19.9</v>
+        <v>19.6</v>
       </c>
       <c r="E331" t="n">
         <v>34</v>
       </c>
       <c r="F331" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="G331" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H331" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="I331" t="n">
         <v>0</v>
@@ -17014,23 +17014,23 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D332" t="n">
         <v>17.6</v>
       </c>
       <c r="E332" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F332" t="n">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="G332" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H332" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I332" t="n">
         <v>0</v>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D333" t="n">
         <v>15.1</v>
       </c>
       <c r="E333" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F333" t="n">
-        <v>7.9</v>
+        <v>5.4</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>13.2</v>
+        <v>13</v>
       </c>
       <c r="E334" t="n">
         <v>54</v>
       </c>
       <c r="F334" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17164,17 +17164,17 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>12.1</v>
+        <v>11.7</v>
       </c>
       <c r="E335" t="n">
         <v>55</v>
       </c>
       <c r="F335" t="n">
-        <v>9.699999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
@@ -17214,23 +17214,23 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>11.5</v>
+        <v>10.9</v>
       </c>
       <c r="E336" t="n">
         <v>55</v>
       </c>
       <c r="F336" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
       </c>
       <c r="H336" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I336" t="n">
         <v>0</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="E337" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F337" t="n">
-        <v>6.8</v>
+        <v>6.5</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>34</v>
+        <v>87</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17289,7 +17289,7 @@
         <v>0</v>
       </c>
       <c r="K337" t="n">
-        <v>0.258</v>
+        <v>0.259</v>
       </c>
       <c r="L337" t="n">
         <v>1</v>
@@ -17314,23 +17314,23 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>9.4</v>
+        <v>9.6</v>
       </c>
       <c r="E338" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F338" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17339,7 +17339,7 @@
         <v>0</v>
       </c>
       <c r="K338" t="n">
-        <v>0.258</v>
+        <v>0.259</v>
       </c>
       <c r="L338" t="n">
         <v>2</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>8.699999999999999</v>
+        <v>9</v>
       </c>
       <c r="E339" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="F339" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>63</v>
+        <v>9</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.258</v>
+        <v>0.259</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>
@@ -17414,23 +17414,23 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D340" t="n">
         <v>7.8</v>
       </c>
       <c r="E340" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F340" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="I340" t="n">
         <v>0</v>
@@ -17439,7 +17439,7 @@
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>0.258</v>
+        <v>0.259</v>
       </c>
       <c r="L340" t="n">
         <v>2</v>
@@ -17464,23 +17464,23 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="E341" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F341" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="I341" t="n">
         <v>0</v>
@@ -17514,23 +17514,23 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="E342" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F342" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I342" t="n">
         <v>0</v>
@@ -17564,23 +17564,23 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="E343" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F343" t="n">
-        <v>5.4</v>
+        <v>4.7</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I343" t="n">
         <v>0</v>
@@ -17614,17 +17614,17 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="E344" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F344" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
@@ -17639,7 +17639,7 @@
         <v>0</v>
       </c>
       <c r="K344" t="n">
-        <v>0.259</v>
+        <v>0.26</v>
       </c>
       <c r="L344" t="n">
         <v>2</v>
@@ -17664,17 +17664,17 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="E345" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F345" t="n">
-        <v>6.5</v>
+        <v>7.2</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
@@ -17689,7 +17689,7 @@
         <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>0.259</v>
+        <v>0.26</v>
       </c>
       <c r="L345" t="n">
         <v>2</v>
@@ -17714,23 +17714,23 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D346" t="n">
         <v>5.8</v>
       </c>
       <c r="E346" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F346" t="n">
-        <v>7.2</v>
+        <v>9</v>
       </c>
       <c r="G346" t="n">
         <v>41</v>
       </c>
       <c r="H346" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I346" t="n">
         <v>0</v>
@@ -17739,7 +17739,7 @@
         <v>0</v>
       </c>
       <c r="K346" t="n">
-        <v>0.259</v>
+        <v>0.26</v>
       </c>
       <c r="L346" t="n">
         <v>2</v>
@@ -17764,23 +17764,23 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="E347" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F347" t="n">
-        <v>7.6</v>
+        <v>6.8</v>
       </c>
       <c r="G347" t="n">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="H347" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="I347" t="n">
         <v>0</v>
@@ -17789,7 +17789,7 @@
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>0.259</v>
+        <v>0.26</v>
       </c>
       <c r="L347" t="n">
         <v>2</v>
@@ -17814,23 +17814,23 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="E348" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F348" t="n">
-        <v>8.6</v>
+        <v>6.1</v>
       </c>
       <c r="G348" t="n">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="H348" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I348" t="n">
         <v>0</v>
@@ -17864,23 +17864,23 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>16.6</v>
+        <v>16.7</v>
       </c>
       <c r="E349" t="n">
         <v>42</v>
       </c>
       <c r="F349" t="n">
-        <v>9.699999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="G349" t="n">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="H349" t="n">
-        <v>1</v>
+        <v>94</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -17914,23 +17914,23 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>19</v>
+        <v>19.2</v>
       </c>
       <c r="E350" t="n">
         <v>36</v>
       </c>
       <c r="F350" t="n">
-        <v>10.8</v>
+        <v>10.1</v>
       </c>
       <c r="G350" t="n">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="H350" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="I350" t="n">
         <v>0</v>
@@ -17939,7 +17939,7 @@
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>0.256</v>
+        <v>0.257</v>
       </c>
       <c r="L350" t="n">
         <v>2</v>
@@ -17964,23 +17964,23 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="E351" t="n">
         <v>33</v>
       </c>
       <c r="F351" t="n">
-        <v>11.5</v>
+        <v>11.2</v>
       </c>
       <c r="G351" t="n">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="H351" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -17989,7 +17989,7 @@
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>0.254</v>
+        <v>0.255</v>
       </c>
       <c r="L351" t="n">
         <v>2</v>
@@ -18014,23 +18014,23 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>21.3</v>
+        <v>21</v>
       </c>
       <c r="E352" t="n">
         <v>30</v>
       </c>
       <c r="F352" t="n">
-        <v>11.5</v>
+        <v>10.1</v>
       </c>
       <c r="G352" t="n">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="H352" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -18064,23 +18064,23 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>21.9</v>
+        <v>21.5</v>
       </c>
       <c r="E353" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F353" t="n">
-        <v>10.4</v>
+        <v>10.8</v>
       </c>
       <c r="G353" t="n">
-        <v>432</v>
+        <v>418</v>
       </c>
       <c r="H353" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -18114,20 +18114,20 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>22.1</v>
+        <v>21.7</v>
       </c>
       <c r="E354" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F354" t="n">
-        <v>10.1</v>
+        <v>10.4</v>
       </c>
       <c r="G354" t="n">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="H354" t="n">
         <v>0</v>
@@ -18164,17 +18164,17 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>21.6</v>
+        <v>21.2</v>
       </c>
       <c r="E355" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F355" t="n">
-        <v>10.8</v>
+        <v>11.2</v>
       </c>
       <c r="G355" t="n">
         <v>157</v>
@@ -18214,17 +18214,17 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
       <c r="E356" t="n">
         <v>35</v>
       </c>
       <c r="F356" t="n">
-        <v>11.2</v>
+        <v>10.1</v>
       </c>
       <c r="G356" t="n">
         <v>27</v>
@@ -18264,17 +18264,17 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>16.5</v>
+        <v>16.2</v>
       </c>
       <c r="E357" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F357" t="n">
-        <v>11.5</v>
+        <v>10.4</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
@@ -18314,17 +18314,17 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>14.9</v>
+        <v>14.5</v>
       </c>
       <c r="E358" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F358" t="n">
-        <v>12.2</v>
+        <v>11.9</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
@@ -18364,17 +18364,17 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>13.3</v>
+        <v>13.1</v>
       </c>
       <c r="E359" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F359" t="n">
-        <v>9.699999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
@@ -18414,17 +18414,17 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>12.4</v>
+        <v>11.8</v>
       </c>
       <c r="E360" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F360" t="n">
-        <v>11.9</v>
+        <v>10.1</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
@@ -18464,23 +18464,23 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>12.3</v>
+        <v>11.3</v>
       </c>
       <c r="E361" t="n">
         <v>72</v>
       </c>
       <c r="F361" t="n">
-        <v>15.5</v>
+        <v>12.6</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
       </c>
       <c r="H361" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I361" t="n">
         <v>0</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>12.3</v>
+        <v>11</v>
       </c>
       <c r="E362" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="F362" t="n">
-        <v>16.2</v>
+        <v>14</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18564,17 +18564,17 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>12.4</v>
+        <v>11.3</v>
       </c>
       <c r="E363" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F363" t="n">
-        <v>16.9</v>
+        <v>16.6</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -18614,17 +18614,17 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>12.4</v>
+        <v>11.8</v>
       </c>
       <c r="E364" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F364" t="n">
-        <v>18.4</v>
+        <v>17.6</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
@@ -18664,14 +18664,14 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>12.3</v>
+        <v>11.8</v>
       </c>
       <c r="E365" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F365" t="n">
         <v>17.3</v>
@@ -18714,17 +18714,17 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="E366" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F366" t="n">
-        <v>16.9</v>
+        <v>14.8</v>
       </c>
       <c r="G366" t="n">
         <v>0</v>
@@ -18764,17 +18764,17 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>11.5</v>
+        <v>11.3</v>
       </c>
       <c r="E367" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F367" t="n">
-        <v>15.5</v>
+        <v>14.8</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
@@ -18814,23 +18814,23 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>11.1</v>
+        <v>10.9</v>
       </c>
       <c r="E368" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F368" t="n">
-        <v>15.8</v>
+        <v>13.7</v>
       </c>
       <c r="G368" t="n">
         <v>0</v>
       </c>
       <c r="H368" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="I368" t="n">
         <v>0</v>
@@ -18864,23 +18864,23 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>10.8</v>
+        <v>10.5</v>
       </c>
       <c r="E369" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F369" t="n">
-        <v>16.2</v>
+        <v>13.3</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>98</v>
+        <v>20</v>
       </c>
       <c r="I369" t="n">
         <v>0</v>
@@ -18914,23 +18914,23 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>11.1</v>
+        <v>10.9</v>
       </c>
       <c r="E370" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F370" t="n">
-        <v>16.6</v>
+        <v>15.8</v>
       </c>
       <c r="G370" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H370" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="I370" t="n">
         <v>0</v>
@@ -18964,20 +18964,20 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>13.3</v>
+        <v>13.4</v>
       </c>
       <c r="E371" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F371" t="n">
-        <v>17.6</v>
+        <v>19.4</v>
       </c>
       <c r="G371" t="n">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="H371" t="n">
         <v>0</v>
@@ -19014,20 +19014,20 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
       <c r="E372" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F372" t="n">
-        <v>18</v>
+        <v>18.7</v>
       </c>
       <c r="G372" t="n">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H372" t="n">
         <v>0</v>
@@ -19064,23 +19064,23 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>19.2</v>
+        <v>19.4</v>
       </c>
       <c r="E373" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F373" t="n">
-        <v>17.1</v>
+        <v>19.1</v>
       </c>
       <c r="G373" t="n">
-        <v>444</v>
+        <v>455</v>
       </c>
       <c r="H373" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I373" t="n">
         <v>0</v>
@@ -19114,23 +19114,23 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>21.3</v>
+        <v>21.8</v>
       </c>
       <c r="E374" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="F374" t="n">
-        <v>16.4</v>
+        <v>17.3</v>
       </c>
       <c r="G374" t="n">
-        <v>517</v>
+        <v>530</v>
       </c>
       <c r="H374" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="I374" t="n">
         <v>0</v>
@@ -19164,23 +19164,23 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>22.5</v>
+        <v>23.7</v>
       </c>
       <c r="E375" t="n">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="F375" t="n">
-        <v>15.7</v>
+        <v>16.9</v>
       </c>
       <c r="G375" t="n">
-        <v>533.8</v>
+        <v>551</v>
       </c>
       <c r="H375" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="I375" t="n">
         <v>0</v>
@@ -19214,23 +19214,23 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>22.8</v>
+        <v>25.1</v>
       </c>
       <c r="E376" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="F376" t="n">
-        <v>15.4</v>
+        <v>16.9</v>
       </c>
       <c r="G376" t="n">
-        <v>497</v>
+        <v>510</v>
       </c>
       <c r="H376" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I376" t="n">
         <v>0</v>
@@ -19264,23 +19264,23 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>23.1</v>
+        <v>25.9</v>
       </c>
       <c r="E377" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="F377" t="n">
-        <v>15.6</v>
+        <v>16.6</v>
       </c>
       <c r="G377" t="n">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="H377" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="I377" t="n">
         <v>0</v>
@@ -19314,23 +19314,23 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>22.8</v>
+        <v>25.9</v>
       </c>
       <c r="E378" t="n">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="F378" t="n">
-        <v>14.1</v>
+        <v>18</v>
       </c>
       <c r="G378" t="n">
-        <v>270</v>
+        <v>296</v>
       </c>
       <c r="H378" t="n">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="I378" t="n">
         <v>0</v>
@@ -19364,23 +19364,23 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>21.5</v>
+        <v>24</v>
       </c>
       <c r="E379" t="n">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="F379" t="n">
-        <v>14.3</v>
+        <v>20.2</v>
       </c>
       <c r="G379" t="n">
-        <v>118</v>
+        <v>145.5</v>
       </c>
       <c r="H379" t="n">
-        <v>93</v>
+        <v>21</v>
       </c>
       <c r="I379" t="n">
         <v>0</v>
@@ -19414,23 +19414,23 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>20.2</v>
+        <v>21.3</v>
       </c>
       <c r="E380" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="F380" t="n">
-        <v>15.7</v>
+        <v>18.4</v>
       </c>
       <c r="G380" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H380" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I380" t="n">
         <v>0</v>
@@ -19464,23 +19464,23 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="E381" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F381" t="n">
-        <v>16.2</v>
+        <v>17.2</v>
       </c>
       <c r="G381" t="n">
         <v>0</v>
       </c>
       <c r="H381" t="n">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="I381" t="n">
         <v>0</v>
@@ -19514,23 +19514,23 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>19</v>
+        <v>18.7</v>
       </c>
       <c r="E382" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F382" t="n">
-        <v>18.5</v>
+        <v>19.7</v>
       </c>
       <c r="G382" t="n">
         <v>0</v>
       </c>
       <c r="H382" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I382" t="n">
         <v>0</v>
@@ -19564,23 +19564,23 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>18.9</v>
+        <v>18.4</v>
       </c>
       <c r="E383" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F383" t="n">
-        <v>19.1</v>
+        <v>20.9</v>
       </c>
       <c r="G383" t="n">
         <v>0</v>
       </c>
       <c r="H383" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="I383" t="n">
         <v>0</v>
@@ -19614,23 +19614,23 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>18.6</v>
+        <v>17.8</v>
       </c>
       <c r="E384" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F384" t="n">
-        <v>18.7</v>
+        <v>21.4</v>
       </c>
       <c r="G384" t="n">
         <v>0</v>
       </c>
       <c r="H384" t="n">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="I384" t="n">
         <v>0</v>
@@ -19664,23 +19664,23 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>17.9</v>
+        <v>17.7</v>
       </c>
       <c r="E385" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F385" t="n">
-        <v>18.6</v>
+        <v>21.6</v>
       </c>
       <c r="G385" t="n">
         <v>0</v>
       </c>
       <c r="H385" t="n">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="I385" t="n">
         <v>0</v>
@@ -19689,7 +19689,7 @@
         <v>0</v>
       </c>
       <c r="K385" t="n">
-        <v>0.232</v>
+        <v>0.233</v>
       </c>
       <c r="L385" t="n">
         <v>3</v>
@@ -19714,23 +19714,23 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D386" t="n">
         <v>17.6</v>
       </c>
       <c r="E386" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F386" t="n">
-        <v>19.5</v>
+        <v>22.1</v>
       </c>
       <c r="G386" t="n">
         <v>0</v>
       </c>
       <c r="H386" t="n">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="I386" t="n">
         <v>0</v>
@@ -19764,32 +19764,32 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2026-10-19T05:03:39Z</t>
+          <t>2026-10-19T11:03:50Z</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>17.1</v>
+        <v>17</v>
       </c>
       <c r="E387" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F387" t="n">
-        <v>18.7</v>
+        <v>22.2</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
       </c>
       <c r="H387" t="n">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="I387" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J387" t="n">
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>0.232</v>
+        <v>0.233</v>
       </c>
       <c r="L387" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-19 19:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -17064,23 +17064,23 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>15.1</v>
+        <v>14.9</v>
       </c>
       <c r="E333" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F333" t="n">
-        <v>5.4</v>
+        <v>9.4</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="I333" t="n">
         <v>0</v>
@@ -17114,23 +17114,23 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>13</v>
+        <v>13.3</v>
       </c>
       <c r="E334" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F334" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
       </c>
       <c r="H334" t="n">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="I334" t="n">
         <v>0</v>
@@ -17164,17 +17164,17 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>11.7</v>
+        <v>12.5</v>
       </c>
       <c r="E335" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F335" t="n">
-        <v>7.6</v>
+        <v>10.1</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
@@ -17214,17 +17214,17 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>10.9</v>
+        <v>11.7</v>
       </c>
       <c r="E336" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F336" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G336" t="n">
         <v>0</v>
@@ -17264,23 +17264,23 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>10.3</v>
+        <v>10.8</v>
       </c>
       <c r="E337" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F337" t="n">
-        <v>6.5</v>
+        <v>4.7</v>
       </c>
       <c r="G337" t="n">
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="I337" t="n">
         <v>0</v>
@@ -17314,14 +17314,14 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="E338" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F338" t="n">
         <v>2.9</v>
@@ -17330,7 +17330,7 @@
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="I338" t="n">
         <v>0</v>
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D339" t="n">
         <v>9</v>
       </c>
       <c r="E339" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F339" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>9</v>
+        <v>100</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17414,23 +17414,23 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>7.8</v>
+        <v>8.4</v>
       </c>
       <c r="E340" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F340" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I340" t="n">
         <v>0</v>
@@ -17464,23 +17464,23 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="E341" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F341" t="n">
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I341" t="n">
         <v>0</v>
@@ -17514,23 +17514,23 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="E342" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F342" t="n">
-        <v>6.5</v>
+        <v>5.4</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I342" t="n">
         <v>0</v>
@@ -17564,14 +17564,14 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="E343" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F343" t="n">
         <v>4.7</v>
@@ -17580,7 +17580,7 @@
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I343" t="n">
         <v>0</v>
@@ -17614,23 +17614,23 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="E344" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F344" t="n">
-        <v>5</v>
+        <v>5.4</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I344" t="n">
         <v>0</v>
@@ -17664,23 +17664,23 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="E345" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="F345" t="n">
-        <v>7.2</v>
+        <v>6.1</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="I345" t="n">
         <v>0</v>
@@ -17714,23 +17714,23 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="E346" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F346" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="G346" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H346" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I346" t="n">
         <v>0</v>
@@ -17764,23 +17764,23 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D347" t="n">
         <v>9.1</v>
       </c>
       <c r="E347" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F347" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="G347" t="n">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H347" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="I347" t="n">
         <v>0</v>
@@ -17814,20 +17814,20 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>12.9</v>
+        <v>13</v>
       </c>
       <c r="E348" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F348" t="n">
         <v>6.1</v>
       </c>
       <c r="G348" t="n">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H348" t="n">
         <v>0</v>
@@ -17864,23 +17864,23 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D349" t="n">
         <v>16.7</v>
       </c>
       <c r="E349" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F349" t="n">
-        <v>6.8</v>
+        <v>5.4</v>
       </c>
       <c r="G349" t="n">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="H349" t="n">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -17914,23 +17914,23 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>19.2</v>
+        <v>19.1</v>
       </c>
       <c r="E350" t="n">
         <v>36</v>
       </c>
       <c r="F350" t="n">
-        <v>10.1</v>
+        <v>7.2</v>
       </c>
       <c r="G350" t="n">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="H350" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="I350" t="n">
         <v>0</v>
@@ -17964,7 +17964,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D351" t="n">
@@ -17974,13 +17974,13 @@
         <v>33</v>
       </c>
       <c r="F351" t="n">
-        <v>11.2</v>
+        <v>8.6</v>
       </c>
       <c r="G351" t="n">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="H351" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -18014,23 +18014,23 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>21</v>
+        <v>21.1</v>
       </c>
       <c r="E352" t="n">
         <v>30</v>
       </c>
       <c r="F352" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
       <c r="G352" t="n">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="H352" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -18064,23 +18064,23 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>21.5</v>
+        <v>21.7</v>
       </c>
       <c r="E353" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F353" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
       <c r="G353" t="n">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="H353" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -18114,23 +18114,23 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="E354" t="n">
         <v>28</v>
       </c>
       <c r="F354" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="G354" t="n">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="H354" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="I354" t="n">
         <v>0</v>
@@ -18164,23 +18164,23 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>21.2</v>
+        <v>21.4</v>
       </c>
       <c r="E355" t="n">
         <v>29</v>
       </c>
       <c r="F355" t="n">
-        <v>11.2</v>
+        <v>10.4</v>
       </c>
       <c r="G355" t="n">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H355" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I355" t="n">
         <v>0</v>
@@ -18214,23 +18214,23 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="E356" t="n">
         <v>35</v>
       </c>
       <c r="F356" t="n">
-        <v>10.1</v>
+        <v>9.4</v>
       </c>
       <c r="G356" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H356" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="I356" t="n">
         <v>0</v>
@@ -18264,11 +18264,11 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>16.2</v>
+        <v>16.4</v>
       </c>
       <c r="E357" t="n">
         <v>42</v>
@@ -18314,17 +18314,17 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D358" t="n">
         <v>14.5</v>
       </c>
       <c r="E358" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F358" t="n">
-        <v>11.9</v>
+        <v>10.1</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
@@ -18364,17 +18364,17 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>13.1</v>
+        <v>13.2</v>
       </c>
       <c r="E359" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F359" t="n">
-        <v>10.1</v>
+        <v>10.8</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
@@ -18414,17 +18414,17 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="E360" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F360" t="n">
-        <v>10.1</v>
+        <v>10.8</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
@@ -18464,23 +18464,23 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D361" t="n">
         <v>11.3</v>
       </c>
       <c r="E361" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F361" t="n">
-        <v>12.6</v>
+        <v>11.5</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
       </c>
       <c r="H361" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I361" t="n">
         <v>0</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="E362" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F362" t="n">
-        <v>14</v>
+        <v>13.3</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18564,17 +18564,17 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="E363" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F363" t="n">
-        <v>16.6</v>
+        <v>16.2</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -18614,17 +18614,17 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="E364" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F364" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
@@ -18664,17 +18664,17 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="E365" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F365" t="n">
-        <v>17.3</v>
+        <v>15.5</v>
       </c>
       <c r="G365" t="n">
         <v>0</v>
@@ -18714,17 +18714,17 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="E366" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F366" t="n">
-        <v>14.8</v>
+        <v>15.8</v>
       </c>
       <c r="G366" t="n">
         <v>0</v>
@@ -18764,17 +18764,17 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>11.3</v>
+        <v>11.1</v>
       </c>
       <c r="E367" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F367" t="n">
-        <v>14.8</v>
+        <v>15.5</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
@@ -18814,17 +18814,17 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="E368" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F368" t="n">
-        <v>13.7</v>
+        <v>15.5</v>
       </c>
       <c r="G368" t="n">
         <v>0</v>
@@ -18864,23 +18864,23 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="E369" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F369" t="n">
-        <v>13.3</v>
+        <v>15.5</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="I369" t="n">
         <v>0</v>
@@ -18889,7 +18889,7 @@
         <v>0</v>
       </c>
       <c r="K369" t="n">
-        <v>0.249</v>
+        <v>0.25</v>
       </c>
       <c r="L369" t="n">
         <v>3</v>
@@ -18914,7 +18914,7 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D370" t="n">
@@ -18924,13 +18924,13 @@
         <v>77</v>
       </c>
       <c r="F370" t="n">
-        <v>15.8</v>
+        <v>15.5</v>
       </c>
       <c r="G370" t="n">
         <v>40</v>
       </c>
       <c r="H370" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I370" t="n">
         <v>0</v>
@@ -18939,7 +18939,7 @@
         <v>0</v>
       </c>
       <c r="K370" t="n">
-        <v>0.249</v>
+        <v>0.25</v>
       </c>
       <c r="L370" t="n">
         <v>3</v>
@@ -18964,20 +18964,20 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>13.4</v>
+        <v>13</v>
       </c>
       <c r="E371" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F371" t="n">
-        <v>19.4</v>
+        <v>18</v>
       </c>
       <c r="G371" t="n">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="H371" t="n">
         <v>0</v>
@@ -19014,11 +19014,11 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>16.3</v>
+        <v>16.1</v>
       </c>
       <c r="E372" t="n">
         <v>54</v>
@@ -19027,7 +19027,7 @@
         <v>18.7</v>
       </c>
       <c r="G372" t="n">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="H372" t="n">
         <v>0</v>
@@ -19064,20 +19064,20 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>19.4</v>
+        <v>19.3</v>
       </c>
       <c r="E373" t="n">
         <v>42</v>
       </c>
       <c r="F373" t="n">
-        <v>19.1</v>
+        <v>18.7</v>
       </c>
       <c r="G373" t="n">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="H373" t="n">
         <v>0</v>
@@ -19089,7 +19089,7 @@
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>0.246</v>
+        <v>0.247</v>
       </c>
       <c r="L373" t="n">
         <v>3</v>
@@ -19114,20 +19114,20 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="E374" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F374" t="n">
-        <v>17.3</v>
+        <v>16.2</v>
       </c>
       <c r="G374" t="n">
-        <v>530</v>
+        <v>521</v>
       </c>
       <c r="H374" t="n">
         <v>0</v>
@@ -19139,7 +19139,7 @@
         <v>0</v>
       </c>
       <c r="K374" t="n">
-        <v>0.244</v>
+        <v>0.245</v>
       </c>
       <c r="L374" t="n">
         <v>3</v>
@@ -19164,23 +19164,23 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>23.7</v>
+        <v>24</v>
       </c>
       <c r="E375" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F375" t="n">
-        <v>16.9</v>
+        <v>17.6</v>
       </c>
       <c r="G375" t="n">
-        <v>551</v>
+        <v>540</v>
       </c>
       <c r="H375" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I375" t="n">
         <v>0</v>
@@ -19189,7 +19189,7 @@
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>0.242</v>
+        <v>0.243</v>
       </c>
       <c r="L375" t="n">
         <v>3</v>
@@ -19214,20 +19214,20 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>25.1</v>
+        <v>25.3</v>
       </c>
       <c r="E376" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F376" t="n">
-        <v>16.9</v>
+        <v>19.8</v>
       </c>
       <c r="G376" t="n">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="H376" t="n">
         <v>0</v>
@@ -19264,23 +19264,23 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="E377" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F377" t="n">
-        <v>16.6</v>
+        <v>20.2</v>
       </c>
       <c r="G377" t="n">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="H377" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="I377" t="n">
         <v>0</v>
@@ -19314,23 +19314,23 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D378" t="n">
         <v>25.9</v>
       </c>
       <c r="E378" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F378" t="n">
-        <v>18</v>
+        <v>18.7</v>
       </c>
       <c r="G378" t="n">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="H378" t="n">
-        <v>28</v>
+        <v>100</v>
       </c>
       <c r="I378" t="n">
         <v>0</v>
@@ -19339,7 +19339,7 @@
         <v>0</v>
       </c>
       <c r="K378" t="n">
-        <v>0.236</v>
+        <v>0.237</v>
       </c>
       <c r="L378" t="n">
         <v>3</v>
@@ -19364,23 +19364,23 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>24</v>
+        <v>24.7</v>
       </c>
       <c r="E379" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F379" t="n">
-        <v>20.2</v>
+        <v>21.6</v>
       </c>
       <c r="G379" t="n">
-        <v>145.5</v>
+        <v>90</v>
       </c>
       <c r="H379" t="n">
-        <v>21</v>
+        <v>100</v>
       </c>
       <c r="I379" t="n">
         <v>0</v>
@@ -19389,7 +19389,7 @@
         <v>0</v>
       </c>
       <c r="K379" t="n">
-        <v>0.235</v>
+        <v>0.236</v>
       </c>
       <c r="L379" t="n">
         <v>3</v>
@@ -19414,23 +19414,23 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>21.3</v>
+        <v>23.4</v>
       </c>
       <c r="E380" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F380" t="n">
-        <v>18.4</v>
+        <v>17.6</v>
       </c>
       <c r="G380" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="H380" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I380" t="n">
         <v>0</v>
@@ -19464,23 +19464,23 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>20</v>
+        <v>21.9</v>
       </c>
       <c r="E381" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="F381" t="n">
-        <v>17.2</v>
+        <v>14.4</v>
       </c>
       <c r="G381" t="n">
         <v>0</v>
       </c>
       <c r="H381" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I381" t="n">
         <v>0</v>
@@ -19489,7 +19489,7 @@
         <v>0</v>
       </c>
       <c r="K381" t="n">
-        <v>0.234</v>
+        <v>0.236</v>
       </c>
       <c r="L381" t="n">
         <v>3</v>
@@ -19514,23 +19514,23 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>18.7</v>
+        <v>21</v>
       </c>
       <c r="E382" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F382" t="n">
-        <v>19.7</v>
+        <v>18</v>
       </c>
       <c r="G382" t="n">
         <v>0</v>
       </c>
       <c r="H382" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I382" t="n">
         <v>0</v>
@@ -19539,7 +19539,7 @@
         <v>0</v>
       </c>
       <c r="K382" t="n">
-        <v>0.234</v>
+        <v>0.236</v>
       </c>
       <c r="L382" t="n">
         <v>3</v>
@@ -19564,23 +19564,23 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>18.4</v>
+        <v>19.9</v>
       </c>
       <c r="E383" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F383" t="n">
-        <v>20.9</v>
+        <v>25.2</v>
       </c>
       <c r="G383" t="n">
         <v>0</v>
       </c>
       <c r="H383" t="n">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="I383" t="n">
         <v>0</v>
@@ -19589,7 +19589,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>0.233</v>
+        <v>0.235</v>
       </c>
       <c r="L383" t="n">
         <v>3</v>
@@ -19614,23 +19614,23 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>17.8</v>
+        <v>19.3</v>
       </c>
       <c r="E384" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F384" t="n">
-        <v>21.4</v>
+        <v>24.1</v>
       </c>
       <c r="G384" t="n">
         <v>0</v>
       </c>
       <c r="H384" t="n">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="I384" t="n">
         <v>0</v>
@@ -19639,7 +19639,7 @@
         <v>0</v>
       </c>
       <c r="K384" t="n">
-        <v>0.233</v>
+        <v>0.235</v>
       </c>
       <c r="L384" t="n">
         <v>3</v>
@@ -19664,23 +19664,23 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>17.7</v>
+        <v>18.1</v>
       </c>
       <c r="E385" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="F385" t="n">
-        <v>21.6</v>
+        <v>22.7</v>
       </c>
       <c r="G385" t="n">
         <v>0</v>
       </c>
       <c r="H385" t="n">
-        <v>67</v>
+        <v>100</v>
       </c>
       <c r="I385" t="n">
         <v>0</v>
@@ -19689,7 +19689,7 @@
         <v>0</v>
       </c>
       <c r="K385" t="n">
-        <v>0.233</v>
+        <v>0.235</v>
       </c>
       <c r="L385" t="n">
         <v>3</v>
@@ -19714,23 +19714,23 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>17.6</v>
+        <v>17.4</v>
       </c>
       <c r="E386" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F386" t="n">
-        <v>22.1</v>
+        <v>19.1</v>
       </c>
       <c r="G386" t="n">
         <v>0</v>
       </c>
       <c r="H386" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I386" t="n">
         <v>0</v>
@@ -19739,7 +19739,7 @@
         <v>0</v>
       </c>
       <c r="K386" t="n">
-        <v>0.232</v>
+        <v>0.235</v>
       </c>
       <c r="L386" t="n">
         <v>4</v>
@@ -19764,32 +19764,32 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2026-10-19T11:03:50Z</t>
+          <t>2026-10-19T17:03:33Z</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>17</v>
+        <v>17.5</v>
       </c>
       <c r="E387" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="F387" t="n">
-        <v>22.2</v>
+        <v>13</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
       </c>
       <c r="H387" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I387" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J387" t="n">
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>0.233</v>
+        <v>0.235</v>
       </c>
       <c r="L387" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
prognoza biciklista (zvanicna): 2026-10-20 01:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -6614,7 +6614,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D134" t="n">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D135" t="n">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D136" t="n">
@@ -7264,7 +7264,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D137" t="n">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D142" t="n">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D146" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -17364,23 +17364,23 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E339" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F339" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="G339" t="n">
         <v>0</v>
       </c>
       <c r="H339" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I339" t="n">
         <v>0</v>
@@ -17389,7 +17389,7 @@
         <v>0</v>
       </c>
       <c r="K339" t="n">
-        <v>0.259</v>
+        <v>0.248</v>
       </c>
       <c r="L339" t="n">
         <v>2</v>
@@ -17414,23 +17414,23 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>8.4</v>
+        <v>8.1</v>
       </c>
       <c r="E340" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F340" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="G340" t="n">
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I340" t="n">
         <v>0</v>
@@ -17439,7 +17439,7 @@
         <v>0</v>
       </c>
       <c r="K340" t="n">
-        <v>0.259</v>
+        <v>0.248</v>
       </c>
       <c r="L340" t="n">
         <v>2</v>
@@ -17464,17 +17464,17 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D341" t="n">
         <v>7.8</v>
       </c>
       <c r="E341" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F341" t="n">
-        <v>1.1</v>
+        <v>3.2</v>
       </c>
       <c r="G341" t="n">
         <v>0</v>
@@ -17489,7 +17489,7 @@
         <v>0</v>
       </c>
       <c r="K341" t="n">
-        <v>0.259</v>
+        <v>0.248</v>
       </c>
       <c r="L341" t="n">
         <v>2</v>
@@ -17514,17 +17514,17 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="E342" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F342" t="n">
-        <v>5.4</v>
+        <v>4</v>
       </c>
       <c r="G342" t="n">
         <v>0</v>
@@ -17539,7 +17539,7 @@
         <v>0</v>
       </c>
       <c r="K342" t="n">
-        <v>0.259</v>
+        <v>0.249</v>
       </c>
       <c r="L342" t="n">
         <v>2</v>
@@ -17564,23 +17564,23 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="E343" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F343" t="n">
-        <v>4.7</v>
+        <v>4.3</v>
       </c>
       <c r="G343" t="n">
         <v>0</v>
       </c>
       <c r="H343" t="n">
-        <v>45</v>
+        <v>99</v>
       </c>
       <c r="I343" t="n">
         <v>0</v>
@@ -17589,7 +17589,7 @@
         <v>0</v>
       </c>
       <c r="K343" t="n">
-        <v>0.259</v>
+        <v>0.249</v>
       </c>
       <c r="L343" t="n">
         <v>2</v>
@@ -17614,23 +17614,23 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="E344" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F344" t="n">
-        <v>5.4</v>
+        <v>5.8</v>
       </c>
       <c r="G344" t="n">
         <v>0</v>
       </c>
       <c r="H344" t="n">
-        <v>1</v>
+        <v>67</v>
       </c>
       <c r="I344" t="n">
         <v>0</v>
@@ -17639,7 +17639,7 @@
         <v>0</v>
       </c>
       <c r="K344" t="n">
-        <v>0.26</v>
+        <v>0.249</v>
       </c>
       <c r="L344" t="n">
         <v>2</v>
@@ -17664,23 +17664,23 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>5.7</v>
+        <v>6.1</v>
       </c>
       <c r="E345" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F345" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="I345" t="n">
         <v>0</v>
@@ -17689,7 +17689,7 @@
         <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>0.26</v>
+        <v>0.249</v>
       </c>
       <c r="L345" t="n">
         <v>2</v>
@@ -17714,23 +17714,23 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="E346" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F346" t="n">
-        <v>7.6</v>
+        <v>8.6</v>
       </c>
       <c r="G346" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H346" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="I346" t="n">
         <v>0</v>
@@ -17739,7 +17739,7 @@
         <v>0</v>
       </c>
       <c r="K346" t="n">
-        <v>0.26</v>
+        <v>0.249</v>
       </c>
       <c r="L346" t="n">
         <v>2</v>
@@ -17764,23 +17764,23 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>9.1</v>
+        <v>9.5</v>
       </c>
       <c r="E347" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F347" t="n">
-        <v>6.1</v>
+        <v>7.6</v>
       </c>
       <c r="G347" t="n">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="H347" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="I347" t="n">
         <v>0</v>
@@ -17789,7 +17789,7 @@
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>0.26</v>
+        <v>0.249</v>
       </c>
       <c r="L347" t="n">
         <v>2</v>
@@ -17814,20 +17814,20 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>13</v>
+        <v>13.1</v>
       </c>
       <c r="E348" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F348" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="G348" t="n">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H348" t="n">
         <v>0</v>
@@ -17839,7 +17839,7 @@
         <v>0</v>
       </c>
       <c r="K348" t="n">
-        <v>0.259</v>
+        <v>0.249</v>
       </c>
       <c r="L348" t="n">
         <v>2</v>
@@ -17864,23 +17864,23 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>16.7</v>
+        <v>16.4</v>
       </c>
       <c r="E349" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F349" t="n">
-        <v>5.4</v>
+        <v>7.2</v>
       </c>
       <c r="G349" t="n">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="H349" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -17889,7 +17889,7 @@
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>0.258</v>
+        <v>0.248</v>
       </c>
       <c r="L349" t="n">
         <v>2</v>
@@ -17914,23 +17914,23 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>19.1</v>
+        <v>18.5</v>
       </c>
       <c r="E350" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F350" t="n">
-        <v>7.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G350" t="n">
-        <v>521</v>
+        <v>512</v>
       </c>
       <c r="H350" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I350" t="n">
         <v>0</v>
@@ -17939,7 +17939,7 @@
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>0.257</v>
+        <v>0.246</v>
       </c>
       <c r="L350" t="n">
         <v>2</v>
@@ -17964,23 +17964,23 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>20.3</v>
+        <v>19.8</v>
       </c>
       <c r="E351" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F351" t="n">
         <v>8.6</v>
       </c>
       <c r="G351" t="n">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="H351" t="n">
-        <v>2</v>
+        <v>98</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -17989,7 +17989,7 @@
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>0.255</v>
+        <v>0.245</v>
       </c>
       <c r="L351" t="n">
         <v>2</v>
@@ -18014,23 +18014,23 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>21.1</v>
+        <v>20.8</v>
       </c>
       <c r="E352" t="n">
         <v>30</v>
       </c>
       <c r="F352" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G352" t="n">
-        <v>511</v>
+        <v>497</v>
       </c>
       <c r="H352" t="n">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -18039,7 +18039,7 @@
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>0.253</v>
+        <v>0.243</v>
       </c>
       <c r="L352" t="n">
         <v>2</v>
@@ -18064,23 +18064,23 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="E353" t="n">
         <v>28</v>
       </c>
       <c r="F353" t="n">
-        <v>9</v>
+        <v>10.1</v>
       </c>
       <c r="G353" t="n">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="H353" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -18089,7 +18089,7 @@
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>0.251</v>
+        <v>0.241</v>
       </c>
       <c r="L353" t="n">
         <v>2</v>
@@ -18114,23 +18114,23 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>21.8</v>
+        <v>21.5</v>
       </c>
       <c r="E354" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F354" t="n">
-        <v>10.1</v>
+        <v>11.5</v>
       </c>
       <c r="G354" t="n">
-        <v>305</v>
+        <v>275</v>
       </c>
       <c r="H354" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I354" t="n">
         <v>0</v>
@@ -18139,7 +18139,7 @@
         <v>0</v>
       </c>
       <c r="K354" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="L354" t="n">
         <v>2</v>
@@ -18164,23 +18164,23 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>21.4</v>
+        <v>21.1</v>
       </c>
       <c r="E355" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F355" t="n">
         <v>10.4</v>
       </c>
       <c r="G355" t="n">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="H355" t="n">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="I355" t="n">
         <v>0</v>
@@ -18189,7 +18189,7 @@
         <v>0</v>
       </c>
       <c r="K355" t="n">
-        <v>0.249</v>
+        <v>0.239</v>
       </c>
       <c r="L355" t="n">
         <v>2</v>
@@ -18214,23 +18214,23 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>18.8</v>
+        <v>18.5</v>
       </c>
       <c r="E356" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F356" t="n">
-        <v>9.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G356" t="n">
         <v>26</v>
       </c>
       <c r="H356" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="I356" t="n">
         <v>0</v>
@@ -18239,7 +18239,7 @@
         <v>0</v>
       </c>
       <c r="K356" t="n">
-        <v>0.249</v>
+        <v>0.239</v>
       </c>
       <c r="L356" t="n">
         <v>2</v>
@@ -18264,23 +18264,23 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>16.4</v>
+        <v>16.1</v>
       </c>
       <c r="E357" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F357" t="n">
-        <v>10.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
       </c>
       <c r="H357" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="I357" t="n">
         <v>0</v>
@@ -18289,7 +18289,7 @@
         <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>0.249</v>
+        <v>0.239</v>
       </c>
       <c r="L357" t="n">
         <v>2</v>
@@ -18314,23 +18314,23 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="E358" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F358" t="n">
-        <v>10.1</v>
+        <v>11.9</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
       </c>
       <c r="H358" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="I358" t="n">
         <v>0</v>
@@ -18339,7 +18339,7 @@
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>0.249</v>
+        <v>0.239</v>
       </c>
       <c r="L358" t="n">
         <v>2</v>
@@ -18364,23 +18364,23 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="E359" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="F359" t="n">
-        <v>10.8</v>
+        <v>10.4</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
       </c>
       <c r="H359" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="I359" t="n">
         <v>0</v>
@@ -18389,7 +18389,7 @@
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>0.249</v>
+        <v>0.239</v>
       </c>
       <c r="L359" t="n">
         <v>2</v>
@@ -18414,14 +18414,14 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="E360" t="n">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F360" t="n">
         <v>10.8</v>
@@ -18430,7 +18430,7 @@
         <v>0</v>
       </c>
       <c r="H360" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="I360" t="n">
         <v>0</v>
@@ -18439,7 +18439,7 @@
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>0.249</v>
+        <v>0.239</v>
       </c>
       <c r="L360" t="n">
         <v>2</v>
@@ -18464,17 +18464,17 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>11.3</v>
+        <v>11.6</v>
       </c>
       <c r="E361" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F361" t="n">
-        <v>11.5</v>
+        <v>11.9</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
@@ -18489,7 +18489,7 @@
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L361" t="n">
         <v>2</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>11.1</v>
+        <v>11.7</v>
       </c>
       <c r="E362" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F362" t="n">
-        <v>13.3</v>
+        <v>15.1</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18539,7 +18539,7 @@
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L362" t="n">
         <v>3</v>
@@ -18564,17 +18564,17 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>11.4</v>
+        <v>12.1</v>
       </c>
       <c r="E363" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F363" t="n">
-        <v>16.2</v>
+        <v>17.6</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -18589,7 +18589,7 @@
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L363" t="n">
         <v>3</v>
@@ -18614,17 +18614,17 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>11.7</v>
+        <v>12.3</v>
       </c>
       <c r="E364" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F364" t="n">
-        <v>17.3</v>
+        <v>16.9</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
@@ -18639,7 +18639,7 @@
         <v>0</v>
       </c>
       <c r="K364" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L364" t="n">
         <v>3</v>
@@ -18664,17 +18664,17 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="E365" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F365" t="n">
-        <v>15.5</v>
+        <v>16.2</v>
       </c>
       <c r="G365" t="n">
         <v>0</v>
@@ -18689,7 +18689,7 @@
         <v>0</v>
       </c>
       <c r="K365" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L365" t="n">
         <v>3</v>
@@ -18714,17 +18714,17 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="E366" t="n">
         <v>75</v>
       </c>
       <c r="F366" t="n">
-        <v>15.8</v>
+        <v>15.5</v>
       </c>
       <c r="G366" t="n">
         <v>0</v>
@@ -18739,7 +18739,7 @@
         <v>0</v>
       </c>
       <c r="K366" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L366" t="n">
         <v>3</v>
@@ -18764,17 +18764,17 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>11.1</v>
+        <v>11.3</v>
       </c>
       <c r="E367" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F367" t="n">
-        <v>15.5</v>
+        <v>15.8</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
@@ -18789,7 +18789,7 @@
         <v>0</v>
       </c>
       <c r="K367" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L367" t="n">
         <v>3</v>
@@ -18814,23 +18814,23 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>10.8</v>
+        <v>11</v>
       </c>
       <c r="E368" t="n">
         <v>77</v>
       </c>
       <c r="F368" t="n">
-        <v>15.5</v>
+        <v>16.6</v>
       </c>
       <c r="G368" t="n">
         <v>0</v>
       </c>
       <c r="H368" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I368" t="n">
         <v>0</v>
@@ -18839,7 +18839,7 @@
         <v>0</v>
       </c>
       <c r="K368" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L368" t="n">
         <v>3</v>
@@ -18864,23 +18864,23 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="E369" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F369" t="n">
-        <v>15.5</v>
+        <v>15.8</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>46</v>
+        <v>84</v>
       </c>
       <c r="I369" t="n">
         <v>0</v>
@@ -18889,7 +18889,7 @@
         <v>0</v>
       </c>
       <c r="K369" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="L369" t="n">
         <v>3</v>
@@ -18914,23 +18914,23 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="E370" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F370" t="n">
-        <v>15.5</v>
+        <v>16.2</v>
       </c>
       <c r="G370" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H370" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I370" t="n">
         <v>0</v>
@@ -18939,7 +18939,7 @@
         <v>0</v>
       </c>
       <c r="K370" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="L370" t="n">
         <v>3</v>
@@ -18964,23 +18964,23 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D371" t="n">
         <v>13</v>
       </c>
       <c r="E371" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F371" t="n">
-        <v>18</v>
+        <v>18.7</v>
       </c>
       <c r="G371" t="n">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H371" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I371" t="n">
         <v>0</v>
@@ -18989,7 +18989,7 @@
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>0.249</v>
+        <v>0.24</v>
       </c>
       <c r="L371" t="n">
         <v>3</v>
@@ -19014,11 +19014,11 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
       <c r="E372" t="n">
         <v>54</v>
@@ -19027,10 +19027,10 @@
         <v>18.7</v>
       </c>
       <c r="G372" t="n">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H372" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I372" t="n">
         <v>0</v>
@@ -19039,7 +19039,7 @@
         <v>0</v>
       </c>
       <c r="K372" t="n">
-        <v>0.248</v>
+        <v>0.239</v>
       </c>
       <c r="L372" t="n">
         <v>3</v>
@@ -19064,20 +19064,20 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>19.3</v>
+        <v>19.4</v>
       </c>
       <c r="E373" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F373" t="n">
-        <v>18.7</v>
+        <v>20.2</v>
       </c>
       <c r="G373" t="n">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="H373" t="n">
         <v>0</v>
@@ -19089,7 +19089,7 @@
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>0.247</v>
+        <v>0.238</v>
       </c>
       <c r="L373" t="n">
         <v>3</v>
@@ -19114,20 +19114,20 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="E374" t="n">
         <v>37</v>
       </c>
       <c r="F374" t="n">
-        <v>16.2</v>
+        <v>19.8</v>
       </c>
       <c r="G374" t="n">
-        <v>521</v>
+        <v>515</v>
       </c>
       <c r="H374" t="n">
         <v>0</v>
@@ -19139,7 +19139,7 @@
         <v>0</v>
       </c>
       <c r="K374" t="n">
-        <v>0.245</v>
+        <v>0.236</v>
       </c>
       <c r="L374" t="n">
         <v>3</v>
@@ -19164,23 +19164,23 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
       <c r="E375" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F375" t="n">
-        <v>17.6</v>
+        <v>20.2</v>
       </c>
       <c r="G375" t="n">
-        <v>540</v>
+        <v>529</v>
       </c>
       <c r="H375" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="I375" t="n">
         <v>0</v>
@@ -19189,7 +19189,7 @@
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>0.243</v>
+        <v>0.234</v>
       </c>
       <c r="L375" t="n">
         <v>3</v>
@@ -19214,23 +19214,23 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>25.3</v>
+        <v>25.5</v>
       </c>
       <c r="E376" t="n">
         <v>31</v>
       </c>
       <c r="F376" t="n">
-        <v>19.8</v>
+        <v>20.2</v>
       </c>
       <c r="G376" t="n">
-        <v>502</v>
+        <v>475</v>
       </c>
       <c r="H376" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I376" t="n">
         <v>0</v>
@@ -19239,7 +19239,7 @@
         <v>0</v>
       </c>
       <c r="K376" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L376" t="n">
         <v>3</v>
@@ -19264,23 +19264,23 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>26</v>
+        <v>26.2</v>
       </c>
       <c r="E377" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F377" t="n">
-        <v>20.2</v>
+        <v>17.6</v>
       </c>
       <c r="G377" t="n">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="H377" t="n">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="I377" t="n">
         <v>0</v>
@@ -19289,7 +19289,7 @@
         <v>0</v>
       </c>
       <c r="K377" t="n">
-        <v>0.238</v>
+        <v>0.23</v>
       </c>
       <c r="L377" t="n">
         <v>3</v>
@@ -19314,23 +19314,23 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="E378" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F378" t="n">
-        <v>18.7</v>
+        <v>17.6</v>
       </c>
       <c r="G378" t="n">
-        <v>273</v>
+        <v>191</v>
       </c>
       <c r="H378" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="I378" t="n">
         <v>0</v>
@@ -19339,7 +19339,7 @@
         <v>0</v>
       </c>
       <c r="K378" t="n">
-        <v>0.237</v>
+        <v>0.229</v>
       </c>
       <c r="L378" t="n">
         <v>3</v>
@@ -19364,20 +19364,20 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
       <c r="E379" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F379" t="n">
-        <v>21.6</v>
+        <v>16.9</v>
       </c>
       <c r="G379" t="n">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="H379" t="n">
         <v>100</v>
@@ -19389,7 +19389,7 @@
         <v>0</v>
       </c>
       <c r="K379" t="n">
-        <v>0.236</v>
+        <v>0.229</v>
       </c>
       <c r="L379" t="n">
         <v>3</v>
@@ -19414,23 +19414,23 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>23.4</v>
+        <v>22.9</v>
       </c>
       <c r="E380" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F380" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="G380" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H380" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="I380" t="n">
         <v>0</v>
@@ -19439,7 +19439,7 @@
         <v>0</v>
       </c>
       <c r="K380" t="n">
-        <v>0.235</v>
+        <v>0.228</v>
       </c>
       <c r="L380" t="n">
         <v>3</v>
@@ -19464,23 +19464,23 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="E381" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F381" t="n">
-        <v>14.4</v>
+        <v>29.9</v>
       </c>
       <c r="G381" t="n">
         <v>0</v>
       </c>
       <c r="H381" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="I381" t="n">
         <v>0</v>
@@ -19489,7 +19489,7 @@
         <v>0</v>
       </c>
       <c r="K381" t="n">
-        <v>0.236</v>
+        <v>0.228</v>
       </c>
       <c r="L381" t="n">
         <v>3</v>
@@ -19514,17 +19514,17 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E382" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F382" t="n">
-        <v>18</v>
+        <v>22.7</v>
       </c>
       <c r="G382" t="n">
         <v>0</v>
@@ -19539,7 +19539,7 @@
         <v>0</v>
       </c>
       <c r="K382" t="n">
-        <v>0.236</v>
+        <v>0.228</v>
       </c>
       <c r="L382" t="n">
         <v>3</v>
@@ -19564,17 +19564,17 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>19.9</v>
+        <v>19.2</v>
       </c>
       <c r="E383" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F383" t="n">
-        <v>25.2</v>
+        <v>21.2</v>
       </c>
       <c r="G383" t="n">
         <v>0</v>
@@ -19589,7 +19589,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>0.235</v>
+        <v>0.227</v>
       </c>
       <c r="L383" t="n">
         <v>3</v>
@@ -19614,17 +19614,17 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>19.3</v>
+        <v>18.5</v>
       </c>
       <c r="E384" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F384" t="n">
-        <v>24.1</v>
+        <v>20.2</v>
       </c>
       <c r="G384" t="n">
         <v>0</v>
@@ -19639,7 +19639,7 @@
         <v>0</v>
       </c>
       <c r="K384" t="n">
-        <v>0.235</v>
+        <v>0.227</v>
       </c>
       <c r="L384" t="n">
         <v>3</v>
@@ -19664,17 +19664,17 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>18.1</v>
+        <v>18.3</v>
       </c>
       <c r="E385" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F385" t="n">
-        <v>22.7</v>
+        <v>23</v>
       </c>
       <c r="G385" t="n">
         <v>0</v>
@@ -19689,7 +19689,7 @@
         <v>0</v>
       </c>
       <c r="K385" t="n">
-        <v>0.235</v>
+        <v>0.229</v>
       </c>
       <c r="L385" t="n">
         <v>3</v>
@@ -19714,17 +19714,17 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>17.4</v>
+        <v>18.3</v>
       </c>
       <c r="E386" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F386" t="n">
-        <v>19.1</v>
+        <v>18</v>
       </c>
       <c r="G386" t="n">
         <v>0</v>
@@ -19739,7 +19739,7 @@
         <v>0</v>
       </c>
       <c r="K386" t="n">
-        <v>0.235</v>
+        <v>0.236</v>
       </c>
       <c r="L386" t="n">
         <v>4</v>
@@ -19764,23 +19764,23 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2026-10-19T17:03:33Z</t>
+          <t>2026-10-19T23:03:52Z</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>17.5</v>
+        <v>18</v>
       </c>
       <c r="E387" t="n">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="F387" t="n">
-        <v>13</v>
+        <v>19.8</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
       </c>
       <c r="H387" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="I387" t="n">
         <v>0</v>
@@ -19789,7 +19789,7 @@
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>0.235</v>
+        <v>0.236</v>
       </c>
       <c r="L387" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-20 07:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N387"/>
+  <dimension ref="A1:N411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -17664,23 +17664,23 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>6.1</v>
+        <v>4.7</v>
       </c>
       <c r="E345" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F345" t="n">
-        <v>6.5</v>
+        <v>7.2</v>
       </c>
       <c r="G345" t="n">
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="I345" t="n">
         <v>0</v>
@@ -17689,7 +17689,7 @@
         <v>0</v>
       </c>
       <c r="K345" t="n">
-        <v>0.249</v>
+        <v>0.241</v>
       </c>
       <c r="L345" t="n">
         <v>2</v>
@@ -17714,23 +17714,23 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>6.2</v>
+        <v>5.1</v>
       </c>
       <c r="E346" t="n">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F346" t="n">
-        <v>8.6</v>
+        <v>7.9</v>
       </c>
       <c r="G346" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H346" t="n">
-        <v>50</v>
+        <v>96</v>
       </c>
       <c r="I346" t="n">
         <v>0</v>
@@ -17739,7 +17739,7 @@
         <v>0</v>
       </c>
       <c r="K346" t="n">
-        <v>0.249</v>
+        <v>0.241</v>
       </c>
       <c r="L346" t="n">
         <v>2</v>
@@ -17764,23 +17764,23 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>9.5</v>
+        <v>8.4</v>
       </c>
       <c r="E347" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F347" t="n">
         <v>7.6</v>
       </c>
       <c r="G347" t="n">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="H347" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="I347" t="n">
         <v>0</v>
@@ -17789,7 +17789,7 @@
         <v>0</v>
       </c>
       <c r="K347" t="n">
-        <v>0.249</v>
+        <v>0.241</v>
       </c>
       <c r="L347" t="n">
         <v>2</v>
@@ -17814,23 +17814,23 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>13.1</v>
+        <v>12.3</v>
       </c>
       <c r="E348" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F348" t="n">
-        <v>6.5</v>
+        <v>7.6</v>
       </c>
       <c r="G348" t="n">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H348" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="I348" t="n">
         <v>0</v>
@@ -17839,7 +17839,7 @@
         <v>0</v>
       </c>
       <c r="K348" t="n">
-        <v>0.249</v>
+        <v>0.241</v>
       </c>
       <c r="L348" t="n">
         <v>2</v>
@@ -17864,23 +17864,23 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>16.4</v>
+        <v>16</v>
       </c>
       <c r="E349" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F349" t="n">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="G349" t="n">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="H349" t="n">
-        <v>70</v>
+        <v>97</v>
       </c>
       <c r="I349" t="n">
         <v>0</v>
@@ -17889,7 +17889,7 @@
         <v>0</v>
       </c>
       <c r="K349" t="n">
-        <v>0.248</v>
+        <v>0.24</v>
       </c>
       <c r="L349" t="n">
         <v>2</v>
@@ -17914,23 +17914,23 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>18.5</v>
+        <v>18.3</v>
       </c>
       <c r="E350" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F350" t="n">
-        <v>8.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="G350" t="n">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="H350" t="n">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="I350" t="n">
         <v>0</v>
@@ -17939,7 +17939,7 @@
         <v>0</v>
       </c>
       <c r="K350" t="n">
-        <v>0.246</v>
+        <v>0.239</v>
       </c>
       <c r="L350" t="n">
         <v>2</v>
@@ -17964,23 +17964,23 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>19.8</v>
+        <v>19.7</v>
       </c>
       <c r="E351" t="n">
         <v>34</v>
       </c>
       <c r="F351" t="n">
-        <v>8.6</v>
+        <v>10.1</v>
       </c>
       <c r="G351" t="n">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="H351" t="n">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="I351" t="n">
         <v>0</v>
@@ -17989,7 +17989,7 @@
         <v>0</v>
       </c>
       <c r="K351" t="n">
-        <v>0.245</v>
+        <v>0.237</v>
       </c>
       <c r="L351" t="n">
         <v>2</v>
@@ -18014,23 +18014,23 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="E352" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F352" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="G352" t="n">
-        <v>497</v>
+        <v>512</v>
       </c>
       <c r="H352" t="n">
-        <v>97</v>
+        <v>45</v>
       </c>
       <c r="I352" t="n">
         <v>0</v>
@@ -18039,7 +18039,7 @@
         <v>0</v>
       </c>
       <c r="K352" t="n">
-        <v>0.243</v>
+        <v>0.235</v>
       </c>
       <c r="L352" t="n">
         <v>2</v>
@@ -18064,23 +18064,23 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>21.5</v>
+        <v>21.3</v>
       </c>
       <c r="E353" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F353" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G353" t="n">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="H353" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I353" t="n">
         <v>0</v>
@@ -18089,7 +18089,7 @@
         <v>0</v>
       </c>
       <c r="K353" t="n">
-        <v>0.241</v>
+        <v>0.233</v>
       </c>
       <c r="L353" t="n">
         <v>2</v>
@@ -18114,23 +18114,23 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D354" t="n">
         <v>21.5</v>
       </c>
       <c r="E354" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F354" t="n">
-        <v>11.5</v>
+        <v>11.2</v>
       </c>
       <c r="G354" t="n">
-        <v>275</v>
+        <v>303</v>
       </c>
       <c r="H354" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="I354" t="n">
         <v>0</v>
@@ -18139,7 +18139,7 @@
         <v>0</v>
       </c>
       <c r="K354" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L354" t="n">
         <v>2</v>
@@ -18164,23 +18164,23 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>21.1</v>
+        <v>21</v>
       </c>
       <c r="E355" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F355" t="n">
-        <v>10.4</v>
+        <v>11.2</v>
       </c>
       <c r="G355" t="n">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="H355" t="n">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="I355" t="n">
         <v>0</v>
@@ -18189,7 +18189,7 @@
         <v>0</v>
       </c>
       <c r="K355" t="n">
-        <v>0.239</v>
+        <v>0.231</v>
       </c>
       <c r="L355" t="n">
         <v>2</v>
@@ -18214,14 +18214,14 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>18.5</v>
+        <v>18.3</v>
       </c>
       <c r="E356" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F356" t="n">
         <v>8.300000000000001</v>
@@ -18230,7 +18230,7 @@
         <v>26</v>
       </c>
       <c r="H356" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="I356" t="n">
         <v>0</v>
@@ -18239,7 +18239,7 @@
         <v>0</v>
       </c>
       <c r="K356" t="n">
-        <v>0.239</v>
+        <v>0.231</v>
       </c>
       <c r="L356" t="n">
         <v>2</v>
@@ -18264,23 +18264,23 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>16.1</v>
+        <v>15.6</v>
       </c>
       <c r="E357" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F357" t="n">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="G357" t="n">
         <v>0</v>
       </c>
       <c r="H357" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="I357" t="n">
         <v>0</v>
@@ -18289,7 +18289,7 @@
         <v>0</v>
       </c>
       <c r="K357" t="n">
-        <v>0.239</v>
+        <v>0.231</v>
       </c>
       <c r="L357" t="n">
         <v>2</v>
@@ -18314,23 +18314,23 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>14.6</v>
+        <v>14.2</v>
       </c>
       <c r="E358" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F358" t="n">
-        <v>11.9</v>
+        <v>11.5</v>
       </c>
       <c r="G358" t="n">
         <v>0</v>
       </c>
       <c r="H358" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="I358" t="n">
         <v>0</v>
@@ -18339,7 +18339,7 @@
         <v>0</v>
       </c>
       <c r="K358" t="n">
-        <v>0.239</v>
+        <v>0.231</v>
       </c>
       <c r="L358" t="n">
         <v>2</v>
@@ -18364,23 +18364,23 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="E359" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="F359" t="n">
-        <v>10.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
       </c>
       <c r="H359" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I359" t="n">
         <v>0</v>
@@ -18389,7 +18389,7 @@
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>0.239</v>
+        <v>0.231</v>
       </c>
       <c r="L359" t="n">
         <v>2</v>
@@ -18414,23 +18414,23 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>12.1</v>
+        <v>11.5</v>
       </c>
       <c r="E360" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F360" t="n">
-        <v>10.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
       </c>
       <c r="H360" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I360" t="n">
         <v>0</v>
@@ -18439,7 +18439,7 @@
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>0.239</v>
+        <v>0.231</v>
       </c>
       <c r="L360" t="n">
         <v>2</v>
@@ -18464,17 +18464,17 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>11.6</v>
+        <v>11.2</v>
       </c>
       <c r="E361" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F361" t="n">
-        <v>11.9</v>
+        <v>12.2</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
@@ -18489,7 +18489,7 @@
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L361" t="n">
         <v>2</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>11.7</v>
+        <v>11.4</v>
       </c>
       <c r="E362" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F362" t="n">
-        <v>15.1</v>
+        <v>15.5</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18539,7 +18539,7 @@
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L362" t="n">
         <v>3</v>
@@ -18564,17 +18564,17 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>12.1</v>
+        <v>11.8</v>
       </c>
       <c r="E363" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F363" t="n">
-        <v>17.6</v>
+        <v>16.9</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -18589,7 +18589,7 @@
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L363" t="n">
         <v>3</v>
@@ -18614,17 +18614,17 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>12.3</v>
+        <v>11.9</v>
       </c>
       <c r="E364" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F364" t="n">
-        <v>16.9</v>
+        <v>16.2</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
@@ -18639,7 +18639,7 @@
         <v>0</v>
       </c>
       <c r="K364" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L364" t="n">
         <v>3</v>
@@ -18664,17 +18664,17 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="E365" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F365" t="n">
-        <v>16.2</v>
+        <v>14.4</v>
       </c>
       <c r="G365" t="n">
         <v>0</v>
@@ -18689,7 +18689,7 @@
         <v>0</v>
       </c>
       <c r="K365" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L365" t="n">
         <v>3</v>
@@ -18714,17 +18714,17 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>11.6</v>
+        <v>11.2</v>
       </c>
       <c r="E366" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F366" t="n">
-        <v>15.5</v>
+        <v>15.8</v>
       </c>
       <c r="G366" t="n">
         <v>0</v>
@@ -18739,7 +18739,7 @@
         <v>0</v>
       </c>
       <c r="K366" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L366" t="n">
         <v>3</v>
@@ -18764,17 +18764,17 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>11.3</v>
+        <v>11</v>
       </c>
       <c r="E367" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F367" t="n">
-        <v>15.8</v>
+        <v>15.1</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
@@ -18789,7 +18789,7 @@
         <v>0</v>
       </c>
       <c r="K367" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L367" t="n">
         <v>3</v>
@@ -18814,14 +18814,14 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>11</v>
+        <v>10.7</v>
       </c>
       <c r="E368" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F368" t="n">
         <v>16.6</v>
@@ -18830,7 +18830,7 @@
         <v>0</v>
       </c>
       <c r="H368" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="I368" t="n">
         <v>0</v>
@@ -18839,7 +18839,7 @@
         <v>0</v>
       </c>
       <c r="K368" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L368" t="n">
         <v>3</v>
@@ -18864,23 +18864,23 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>10.6</v>
+        <v>10.3</v>
       </c>
       <c r="E369" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F369" t="n">
-        <v>15.8</v>
+        <v>16.9</v>
       </c>
       <c r="G369" t="n">
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="I369" t="n">
         <v>0</v>
@@ -18889,7 +18889,7 @@
         <v>0</v>
       </c>
       <c r="K369" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L369" t="n">
         <v>3</v>
@@ -18914,23 +18914,23 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D370" t="n">
         <v>10.8</v>
       </c>
       <c r="E370" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F370" t="n">
-        <v>16.2</v>
+        <v>16.9</v>
       </c>
       <c r="G370" t="n">
         <v>39</v>
       </c>
       <c r="H370" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="I370" t="n">
         <v>0</v>
@@ -18939,7 +18939,7 @@
         <v>0</v>
       </c>
       <c r="K370" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L370" t="n">
         <v>3</v>
@@ -18964,23 +18964,23 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D371" t="n">
         <v>13</v>
       </c>
       <c r="E371" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F371" t="n">
-        <v>18.7</v>
+        <v>17.6</v>
       </c>
       <c r="G371" t="n">
         <v>179</v>
       </c>
       <c r="H371" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I371" t="n">
         <v>0</v>
@@ -18989,7 +18989,7 @@
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>0.24</v>
+        <v>0.232</v>
       </c>
       <c r="L371" t="n">
         <v>3</v>
@@ -19014,23 +19014,23 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="E372" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F372" t="n">
-        <v>18.7</v>
+        <v>18.4</v>
       </c>
       <c r="G372" t="n">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="H372" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I372" t="n">
         <v>0</v>
@@ -19039,7 +19039,7 @@
         <v>0</v>
       </c>
       <c r="K372" t="n">
-        <v>0.239</v>
+        <v>0.231</v>
       </c>
       <c r="L372" t="n">
         <v>3</v>
@@ -19064,20 +19064,20 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>19.4</v>
+        <v>19.6</v>
       </c>
       <c r="E373" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F373" t="n">
-        <v>20.2</v>
+        <v>19.1</v>
       </c>
       <c r="G373" t="n">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="H373" t="n">
         <v>0</v>
@@ -19089,7 +19089,7 @@
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>0.238</v>
+        <v>0.23</v>
       </c>
       <c r="L373" t="n">
         <v>3</v>
@@ -19114,7 +19114,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D374" t="n">
@@ -19124,10 +19124,10 @@
         <v>37</v>
       </c>
       <c r="F374" t="n">
-        <v>19.8</v>
+        <v>18</v>
       </c>
       <c r="G374" t="n">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="H374" t="n">
         <v>0</v>
@@ -19139,7 +19139,7 @@
         <v>0</v>
       </c>
       <c r="K374" t="n">
-        <v>0.236</v>
+        <v>0.228</v>
       </c>
       <c r="L374" t="n">
         <v>3</v>
@@ -19164,7 +19164,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D375" t="n">
@@ -19177,10 +19177,10 @@
         <v>20.2</v>
       </c>
       <c r="G375" t="n">
-        <v>529</v>
+        <v>537</v>
       </c>
       <c r="H375" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="I375" t="n">
         <v>0</v>
@@ -19189,7 +19189,7 @@
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>0.234</v>
+        <v>0.226</v>
       </c>
       <c r="L375" t="n">
         <v>3</v>
@@ -19214,23 +19214,23 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D376" t="n">
         <v>25.5</v>
       </c>
       <c r="E376" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F376" t="n">
-        <v>20.2</v>
+        <v>18.4</v>
       </c>
       <c r="G376" t="n">
-        <v>475</v>
+        <v>498</v>
       </c>
       <c r="H376" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="I376" t="n">
         <v>0</v>
@@ -19239,7 +19239,7 @@
         <v>0</v>
       </c>
       <c r="K376" t="n">
-        <v>0.232</v>
+        <v>0.224</v>
       </c>
       <c r="L376" t="n">
         <v>3</v>
@@ -19264,23 +19264,23 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>26.2</v>
+        <v>26.1</v>
       </c>
       <c r="E377" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F377" t="n">
-        <v>17.6</v>
+        <v>16.2</v>
       </c>
       <c r="G377" t="n">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="H377" t="n">
-        <v>36</v>
+        <v>99</v>
       </c>
       <c r="I377" t="n">
         <v>0</v>
@@ -19289,7 +19289,7 @@
         <v>0</v>
       </c>
       <c r="K377" t="n">
-        <v>0.23</v>
+        <v>0.222</v>
       </c>
       <c r="L377" t="n">
         <v>3</v>
@@ -19314,23 +19314,23 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>26</v>
+        <v>25.4</v>
       </c>
       <c r="E378" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F378" t="n">
-        <v>17.6</v>
+        <v>13.7</v>
       </c>
       <c r="G378" t="n">
-        <v>191</v>
+        <v>96</v>
       </c>
       <c r="H378" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="I378" t="n">
         <v>0</v>
@@ -19339,7 +19339,7 @@
         <v>0</v>
       </c>
       <c r="K378" t="n">
-        <v>0.229</v>
+        <v>0.221</v>
       </c>
       <c r="L378" t="n">
         <v>3</v>
@@ -19364,20 +19364,20 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>24.6</v>
+        <v>24.1</v>
       </c>
       <c r="E379" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F379" t="n">
-        <v>16.9</v>
+        <v>15.1</v>
       </c>
       <c r="G379" t="n">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="H379" t="n">
         <v>100</v>
@@ -19389,7 +19389,7 @@
         <v>0</v>
       </c>
       <c r="K379" t="n">
-        <v>0.229</v>
+        <v>0.236</v>
       </c>
       <c r="L379" t="n">
         <v>3</v>
@@ -19414,23 +19414,23 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>22.9</v>
+        <v>23.1</v>
       </c>
       <c r="E380" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F380" t="n">
-        <v>18</v>
+        <v>18.4</v>
       </c>
       <c r="G380" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H380" t="n">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="I380" t="n">
         <v>0</v>
@@ -19439,7 +19439,7 @@
         <v>0</v>
       </c>
       <c r="K380" t="n">
-        <v>0.228</v>
+        <v>0.253</v>
       </c>
       <c r="L380" t="n">
         <v>3</v>
@@ -19464,23 +19464,23 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>21.8</v>
+        <v>21</v>
       </c>
       <c r="E381" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="F381" t="n">
-        <v>29.9</v>
+        <v>18</v>
       </c>
       <c r="G381" t="n">
         <v>0</v>
       </c>
       <c r="H381" t="n">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="I381" t="n">
         <v>0</v>
@@ -19489,7 +19489,7 @@
         <v>0</v>
       </c>
       <c r="K381" t="n">
-        <v>0.228</v>
+        <v>0.253</v>
       </c>
       <c r="L381" t="n">
         <v>3</v>
@@ -19514,23 +19514,23 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>20</v>
+        <v>19.1</v>
       </c>
       <c r="E382" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="F382" t="n">
-        <v>22.7</v>
+        <v>18</v>
       </c>
       <c r="G382" t="n">
         <v>0</v>
       </c>
       <c r="H382" t="n">
-        <v>100</v>
+        <v>34</v>
       </c>
       <c r="I382" t="n">
         <v>0</v>
@@ -19539,7 +19539,7 @@
         <v>0</v>
       </c>
       <c r="K382" t="n">
-        <v>0.228</v>
+        <v>0.253</v>
       </c>
       <c r="L382" t="n">
         <v>3</v>
@@ -19564,17 +19564,17 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>19.2</v>
+        <v>18</v>
       </c>
       <c r="E383" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F383" t="n">
-        <v>21.2</v>
+        <v>16.9</v>
       </c>
       <c r="G383" t="n">
         <v>0</v>
@@ -19589,7 +19589,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>0.227</v>
+        <v>0.253</v>
       </c>
       <c r="L383" t="n">
         <v>3</v>
@@ -19614,17 +19614,17 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>18.5</v>
+        <v>17.7</v>
       </c>
       <c r="E384" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F384" t="n">
-        <v>20.2</v>
+        <v>16.2</v>
       </c>
       <c r="G384" t="n">
         <v>0</v>
@@ -19639,7 +19639,7 @@
         <v>0</v>
       </c>
       <c r="K384" t="n">
-        <v>0.227</v>
+        <v>0.252</v>
       </c>
       <c r="L384" t="n">
         <v>3</v>
@@ -19664,23 +19664,23 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>18.3</v>
+        <v>17.6</v>
       </c>
       <c r="E385" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F385" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G385" t="n">
         <v>0</v>
       </c>
       <c r="H385" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="I385" t="n">
         <v>0</v>
@@ -19689,7 +19689,7 @@
         <v>0</v>
       </c>
       <c r="K385" t="n">
-        <v>0.229</v>
+        <v>0.252</v>
       </c>
       <c r="L385" t="n">
         <v>3</v>
@@ -19714,23 +19714,23 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>18.3</v>
+        <v>17.2</v>
       </c>
       <c r="E386" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F386" t="n">
-        <v>18</v>
+        <v>17.3</v>
       </c>
       <c r="G386" t="n">
         <v>0</v>
       </c>
       <c r="H386" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I386" t="n">
         <v>0</v>
@@ -19739,7 +19739,7 @@
         <v>0</v>
       </c>
       <c r="K386" t="n">
-        <v>0.236</v>
+        <v>0.252</v>
       </c>
       <c r="L386" t="n">
         <v>4</v>
@@ -19764,23 +19764,23 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2026-10-19T23:03:52Z</t>
+          <t>2026-10-20T05:03:22Z</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>18</v>
+        <v>16.1</v>
       </c>
       <c r="E387" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="F387" t="n">
-        <v>19.8</v>
+        <v>16.9</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
       </c>
       <c r="H387" t="n">
-        <v>84</v>
+        <v>7</v>
       </c>
       <c r="I387" t="n">
         <v>0</v>
@@ -19789,7 +19789,7 @@
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>0.236</v>
+        <v>0.253</v>
       </c>
       <c r="L387" t="n">
         <v>4</v>
@@ -19798,6 +19798,1206 @@
         <v>0</v>
       </c>
       <c r="N387" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="E388" t="n">
+        <v>85</v>
+      </c>
+      <c r="F388" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="G388" t="n">
+        <v>0</v>
+      </c>
+      <c r="H388" t="n">
+        <v>5</v>
+      </c>
+      <c r="I388" t="n">
+        <v>0</v>
+      </c>
+      <c r="J388" t="n">
+        <v>0</v>
+      </c>
+      <c r="K388" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="L388" t="n">
+        <v>4</v>
+      </c>
+      <c r="M388" t="n">
+        <v>0</v>
+      </c>
+      <c r="N388" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="E389" t="n">
+        <v>83</v>
+      </c>
+      <c r="F389" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="G389" t="n">
+        <v>0</v>
+      </c>
+      <c r="H389" t="n">
+        <v>100</v>
+      </c>
+      <c r="I389" t="n">
+        <v>0</v>
+      </c>
+      <c r="J389" t="n">
+        <v>0</v>
+      </c>
+      <c r="K389" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="L389" t="n">
+        <v>4</v>
+      </c>
+      <c r="M389" t="n">
+        <v>0</v>
+      </c>
+      <c r="N389" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="E390" t="n">
+        <v>83</v>
+      </c>
+      <c r="F390" t="n">
+        <v>13</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0</v>
+      </c>
+      <c r="H390" t="n">
+        <v>100</v>
+      </c>
+      <c r="I390" t="n">
+        <v>0</v>
+      </c>
+      <c r="J390" t="n">
+        <v>0</v>
+      </c>
+      <c r="K390" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="L390" t="n">
+        <v>4</v>
+      </c>
+      <c r="M390" t="n">
+        <v>0</v>
+      </c>
+      <c r="N390" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="E391" t="n">
+        <v>84</v>
+      </c>
+      <c r="F391" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G391" t="n">
+        <v>0</v>
+      </c>
+      <c r="H391" t="n">
+        <v>100</v>
+      </c>
+      <c r="I391" t="n">
+        <v>0</v>
+      </c>
+      <c r="J391" t="n">
+        <v>0</v>
+      </c>
+      <c r="K391" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="L391" t="n">
+        <v>4</v>
+      </c>
+      <c r="M391" t="n">
+        <v>0</v>
+      </c>
+      <c r="N391" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="E392" t="n">
+        <v>84</v>
+      </c>
+      <c r="F392" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G392" t="n">
+        <v>0</v>
+      </c>
+      <c r="H392" t="n">
+        <v>100</v>
+      </c>
+      <c r="I392" t="n">
+        <v>0</v>
+      </c>
+      <c r="J392" t="n">
+        <v>0</v>
+      </c>
+      <c r="K392" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="L392" t="n">
+        <v>4</v>
+      </c>
+      <c r="M392" t="n">
+        <v>0</v>
+      </c>
+      <c r="N392" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="E393" t="n">
+        <v>85</v>
+      </c>
+      <c r="F393" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G393" t="n">
+        <v>0</v>
+      </c>
+      <c r="H393" t="n">
+        <v>100</v>
+      </c>
+      <c r="I393" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J393" t="n">
+        <v>0</v>
+      </c>
+      <c r="K393" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="L393" t="n">
+        <v>4</v>
+      </c>
+      <c r="M393" t="n">
+        <v>0</v>
+      </c>
+      <c r="N393" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="E394" t="n">
+        <v>90</v>
+      </c>
+      <c r="F394" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G394" t="n">
+        <v>2</v>
+      </c>
+      <c r="H394" t="n">
+        <v>100</v>
+      </c>
+      <c r="I394" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J394" t="n">
+        <v>0</v>
+      </c>
+      <c r="K394" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="L394" t="n">
+        <v>4</v>
+      </c>
+      <c r="M394" t="n">
+        <v>0</v>
+      </c>
+      <c r="N394" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="E395" t="n">
+        <v>83</v>
+      </c>
+      <c r="F395" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G395" t="n">
+        <v>47</v>
+      </c>
+      <c r="H395" t="n">
+        <v>100</v>
+      </c>
+      <c r="I395" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J395" t="n">
+        <v>0</v>
+      </c>
+      <c r="K395" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="L395" t="n">
+        <v>4</v>
+      </c>
+      <c r="M395" t="n">
+        <v>0</v>
+      </c>
+      <c r="N395" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="E396" t="n">
+        <v>86</v>
+      </c>
+      <c r="F396" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="G396" t="n">
+        <v>58</v>
+      </c>
+      <c r="H396" t="n">
+        <v>100</v>
+      </c>
+      <c r="I396" t="n">
+        <v>0</v>
+      </c>
+      <c r="J396" t="n">
+        <v>0</v>
+      </c>
+      <c r="K396" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="L396" t="n">
+        <v>4</v>
+      </c>
+      <c r="M396" t="n">
+        <v>0</v>
+      </c>
+      <c r="N396" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E397" t="n">
+        <v>81</v>
+      </c>
+      <c r="F397" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="G397" t="n">
+        <v>235.5</v>
+      </c>
+      <c r="H397" t="n">
+        <v>80</v>
+      </c>
+      <c r="I397" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J397" t="n">
+        <v>0</v>
+      </c>
+      <c r="K397" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="L397" t="n">
+        <v>4</v>
+      </c>
+      <c r="M397" t="n">
+        <v>0</v>
+      </c>
+      <c r="N397" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="E398" t="n">
+        <v>75</v>
+      </c>
+      <c r="F398" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G398" t="n">
+        <v>334</v>
+      </c>
+      <c r="H398" t="n">
+        <v>92</v>
+      </c>
+      <c r="I398" t="n">
+        <v>0</v>
+      </c>
+      <c r="J398" t="n">
+        <v>0</v>
+      </c>
+      <c r="K398" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L398" t="n">
+        <v>4</v>
+      </c>
+      <c r="M398" t="n">
+        <v>0</v>
+      </c>
+      <c r="N398" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D399" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="E399" t="n">
+        <v>67</v>
+      </c>
+      <c r="F399" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G399" t="n">
+        <v>337</v>
+      </c>
+      <c r="H399" t="n">
+        <v>80</v>
+      </c>
+      <c r="I399" t="n">
+        <v>0</v>
+      </c>
+      <c r="J399" t="n">
+        <v>0</v>
+      </c>
+      <c r="K399" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="L399" t="n">
+        <v>4</v>
+      </c>
+      <c r="M399" t="n">
+        <v>0</v>
+      </c>
+      <c r="N399" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="E400" t="n">
+        <v>60</v>
+      </c>
+      <c r="F400" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G400" t="n">
+        <v>365</v>
+      </c>
+      <c r="H400" t="n">
+        <v>70</v>
+      </c>
+      <c r="I400" t="n">
+        <v>0</v>
+      </c>
+      <c r="J400" t="n">
+        <v>0</v>
+      </c>
+      <c r="K400" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="L400" t="n">
+        <v>4</v>
+      </c>
+      <c r="M400" t="n">
+        <v>0</v>
+      </c>
+      <c r="N400" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="E401" t="n">
+        <v>57</v>
+      </c>
+      <c r="F401" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G401" t="n">
+        <v>327</v>
+      </c>
+      <c r="H401" t="n">
+        <v>70</v>
+      </c>
+      <c r="I401" t="n">
+        <v>0</v>
+      </c>
+      <c r="J401" t="n">
+        <v>0</v>
+      </c>
+      <c r="K401" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="L401" t="n">
+        <v>4</v>
+      </c>
+      <c r="M401" t="n">
+        <v>0</v>
+      </c>
+      <c r="N401" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="E402" t="n">
+        <v>57</v>
+      </c>
+      <c r="F402" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="G402" t="n">
+        <v>242</v>
+      </c>
+      <c r="H402" t="n">
+        <v>72</v>
+      </c>
+      <c r="I402" t="n">
+        <v>0</v>
+      </c>
+      <c r="J402" t="n">
+        <v>0</v>
+      </c>
+      <c r="K402" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="L402" t="n">
+        <v>4</v>
+      </c>
+      <c r="M402" t="n">
+        <v>0</v>
+      </c>
+      <c r="N402" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="E403" t="n">
+        <v>61</v>
+      </c>
+      <c r="F403" t="n">
+        <v>12</v>
+      </c>
+      <c r="G403" t="n">
+        <v>114</v>
+      </c>
+      <c r="H403" t="n">
+        <v>94</v>
+      </c>
+      <c r="I403" t="n">
+        <v>0</v>
+      </c>
+      <c r="J403" t="n">
+        <v>0</v>
+      </c>
+      <c r="K403" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="L403" t="n">
+        <v>4</v>
+      </c>
+      <c r="M403" t="n">
+        <v>0</v>
+      </c>
+      <c r="N403" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="E404" t="n">
+        <v>65</v>
+      </c>
+      <c r="F404" t="n">
+        <v>10</v>
+      </c>
+      <c r="G404" t="n">
+        <v>14</v>
+      </c>
+      <c r="H404" t="n">
+        <v>96</v>
+      </c>
+      <c r="I404" t="n">
+        <v>0</v>
+      </c>
+      <c r="J404" t="n">
+        <v>0</v>
+      </c>
+      <c r="K404" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L404" t="n">
+        <v>4</v>
+      </c>
+      <c r="M404" t="n">
+        <v>0</v>
+      </c>
+      <c r="N404" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="E405" t="n">
+        <v>67</v>
+      </c>
+      <c r="F405" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G405" t="n">
+        <v>0</v>
+      </c>
+      <c r="H405" t="n">
+        <v>98</v>
+      </c>
+      <c r="I405" t="n">
+        <v>0</v>
+      </c>
+      <c r="J405" t="n">
+        <v>0</v>
+      </c>
+      <c r="K405" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L405" t="n">
+        <v>4</v>
+      </c>
+      <c r="M405" t="n">
+        <v>0</v>
+      </c>
+      <c r="N405" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="E406" t="n">
+        <v>72</v>
+      </c>
+      <c r="F406" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G406" t="n">
+        <v>0</v>
+      </c>
+      <c r="H406" t="n">
+        <v>100</v>
+      </c>
+      <c r="I406" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J406" t="n">
+        <v>0</v>
+      </c>
+      <c r="K406" t="n">
+        <v>0.261</v>
+      </c>
+      <c r="L406" t="n">
+        <v>4</v>
+      </c>
+      <c r="M406" t="n">
+        <v>0</v>
+      </c>
+      <c r="N406" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="E407" t="n">
+        <v>84</v>
+      </c>
+      <c r="F407" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="G407" t="n">
+        <v>0</v>
+      </c>
+      <c r="H407" t="n">
+        <v>100</v>
+      </c>
+      <c r="I407" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J407" t="n">
+        <v>0</v>
+      </c>
+      <c r="K407" t="n">
+        <v>0.268</v>
+      </c>
+      <c r="L407" t="n">
+        <v>4</v>
+      </c>
+      <c r="M407" t="n">
+        <v>0</v>
+      </c>
+      <c r="N407" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E408" t="n">
+        <v>87</v>
+      </c>
+      <c r="F408" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0</v>
+      </c>
+      <c r="H408" t="n">
+        <v>100</v>
+      </c>
+      <c r="I408" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J408" t="n">
+        <v>0</v>
+      </c>
+      <c r="K408" t="n">
+        <v>0.284</v>
+      </c>
+      <c r="L408" t="n">
+        <v>4</v>
+      </c>
+      <c r="M408" t="n">
+        <v>0</v>
+      </c>
+      <c r="N408" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="E409" t="n">
+        <v>88</v>
+      </c>
+      <c r="F409" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="G409" t="n">
+        <v>0</v>
+      </c>
+      <c r="H409" t="n">
+        <v>100</v>
+      </c>
+      <c r="I409" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J409" t="n">
+        <v>0</v>
+      </c>
+      <c r="K409" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="L409" t="n">
+        <v>4</v>
+      </c>
+      <c r="M409" t="n">
+        <v>0</v>
+      </c>
+      <c r="N409" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E410" t="n">
+        <v>89</v>
+      </c>
+      <c r="F410" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G410" t="n">
+        <v>0</v>
+      </c>
+      <c r="H410" t="n">
+        <v>100</v>
+      </c>
+      <c r="I410" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J410" t="n">
+        <v>0</v>
+      </c>
+      <c r="K410" t="n">
+        <v>0.306</v>
+      </c>
+      <c r="L410" t="n">
+        <v>5</v>
+      </c>
+      <c r="M410" t="n">
+        <v>0</v>
+      </c>
+      <c r="N410" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>2026-10-20T05:03:22Z</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>10</v>
+      </c>
+      <c r="E411" t="n">
+        <v>89</v>
+      </c>
+      <c r="F411" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G411" t="n">
+        <v>0</v>
+      </c>
+      <c r="H411" t="n">
+        <v>100</v>
+      </c>
+      <c r="I411" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J411" t="n">
+        <v>0</v>
+      </c>
+      <c r="K411" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="L411" t="n">
+        <v>5</v>
+      </c>
+      <c r="M411" t="n">
+        <v>0</v>
+      </c>
+      <c r="N411" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-20 19:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D150" t="n">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D158" t="n">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -8964,7 +8964,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -18364,17 +18364,17 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="E359" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F359" t="n">
-        <v>9.4</v>
+        <v>11.2</v>
       </c>
       <c r="G359" t="n">
         <v>0</v>
@@ -18389,7 +18389,7 @@
         <v>0</v>
       </c>
       <c r="K359" t="n">
-        <v>0.234</v>
+        <v>0.237</v>
       </c>
       <c r="L359" t="n">
         <v>2</v>
@@ -18414,17 +18414,17 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>10.4</v>
+        <v>10.9</v>
       </c>
       <c r="E360" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F360" t="n">
-        <v>9.699999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="G360" t="n">
         <v>0</v>
@@ -18439,7 +18439,7 @@
         <v>0</v>
       </c>
       <c r="K360" t="n">
-        <v>0.234</v>
+        <v>0.237</v>
       </c>
       <c r="L360" t="n">
         <v>2</v>
@@ -18464,17 +18464,17 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>10.1</v>
+        <v>10.7</v>
       </c>
       <c r="E361" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F361" t="n">
-        <v>12.2</v>
+        <v>12.6</v>
       </c>
       <c r="G361" t="n">
         <v>0</v>
@@ -18489,7 +18489,7 @@
         <v>0</v>
       </c>
       <c r="K361" t="n">
-        <v>0.234</v>
+        <v>0.237</v>
       </c>
       <c r="L361" t="n">
         <v>2</v>
@@ -18514,17 +18514,17 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="E362" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F362" t="n">
-        <v>16.6</v>
+        <v>15.1</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -18539,7 +18539,7 @@
         <v>0</v>
       </c>
       <c r="K362" t="n">
-        <v>0.234</v>
+        <v>0.237</v>
       </c>
       <c r="L362" t="n">
         <v>2</v>
@@ -18564,17 +18564,17 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="E363" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F363" t="n">
-        <v>16.9</v>
+        <v>15.1</v>
       </c>
       <c r="G363" t="n">
         <v>0</v>
@@ -18589,7 +18589,7 @@
         <v>0</v>
       </c>
       <c r="K363" t="n">
-        <v>0.234</v>
+        <v>0.238</v>
       </c>
       <c r="L363" t="n">
         <v>2</v>
@@ -18614,17 +18614,17 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>11.3</v>
+        <v>10.9</v>
       </c>
       <c r="E364" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F364" t="n">
-        <v>14.8</v>
+        <v>15.1</v>
       </c>
       <c r="G364" t="n">
         <v>0</v>
@@ -18639,7 +18639,7 @@
         <v>0</v>
       </c>
       <c r="K364" t="n">
-        <v>0.235</v>
+        <v>0.238</v>
       </c>
       <c r="L364" t="n">
         <v>3</v>
@@ -18664,17 +18664,17 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="E365" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F365" t="n">
-        <v>15.8</v>
+        <v>15.1</v>
       </c>
       <c r="G365" t="n">
         <v>0</v>
@@ -18689,7 +18689,7 @@
         <v>0</v>
       </c>
       <c r="K365" t="n">
-        <v>0.235</v>
+        <v>0.238</v>
       </c>
       <c r="L365" t="n">
         <v>3</v>
@@ -18714,17 +18714,17 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="E366" t="n">
         <v>82</v>
       </c>
       <c r="F366" t="n">
-        <v>14.4</v>
+        <v>15.1</v>
       </c>
       <c r="G366" t="n">
         <v>0</v>
@@ -18739,7 +18739,7 @@
         <v>0</v>
       </c>
       <c r="K366" t="n">
-        <v>0.235</v>
+        <v>0.238</v>
       </c>
       <c r="L366" t="n">
         <v>3</v>
@@ -18764,17 +18764,17 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="E367" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F367" t="n">
-        <v>15.1</v>
+        <v>14</v>
       </c>
       <c r="G367" t="n">
         <v>0</v>
@@ -18789,7 +18789,7 @@
         <v>0</v>
       </c>
       <c r="K367" t="n">
-        <v>0.235</v>
+        <v>0.238</v>
       </c>
       <c r="L367" t="n">
         <v>3</v>
@@ -18814,23 +18814,23 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>10</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E368" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F368" t="n">
-        <v>15.1</v>
+        <v>15.5</v>
       </c>
       <c r="G368" t="n">
         <v>0</v>
       </c>
       <c r="H368" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="I368" t="n">
         <v>0</v>
@@ -18839,7 +18839,7 @@
         <v>0</v>
       </c>
       <c r="K368" t="n">
-        <v>0.235</v>
+        <v>0.238</v>
       </c>
       <c r="L368" t="n">
         <v>3</v>
@@ -18864,14 +18864,14 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="E369" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F369" t="n">
         <v>15.8</v>
@@ -18880,7 +18880,7 @@
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="I369" t="n">
         <v>0</v>
@@ -18889,7 +18889,7 @@
         <v>0</v>
       </c>
       <c r="K369" t="n">
-        <v>0.236</v>
+        <v>0.238</v>
       </c>
       <c r="L369" t="n">
         <v>3</v>
@@ -18914,23 +18914,23 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="E370" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F370" t="n">
-        <v>15.8</v>
+        <v>17.6</v>
       </c>
       <c r="G370" t="n">
         <v>38</v>
       </c>
       <c r="H370" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I370" t="n">
         <v>0</v>
@@ -18939,7 +18939,7 @@
         <v>0</v>
       </c>
       <c r="K370" t="n">
-        <v>0.236</v>
+        <v>0.239</v>
       </c>
       <c r="L370" t="n">
         <v>3</v>
@@ -18964,23 +18964,23 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="E371" t="n">
         <v>68</v>
       </c>
       <c r="F371" t="n">
-        <v>16.9</v>
+        <v>18.7</v>
       </c>
       <c r="G371" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H371" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="I371" t="n">
         <v>0</v>
@@ -18989,7 +18989,7 @@
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>0.235</v>
+        <v>0.238</v>
       </c>
       <c r="L371" t="n">
         <v>3</v>
@@ -19014,23 +19014,23 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>15.8</v>
+        <v>16</v>
       </c>
       <c r="E372" t="n">
         <v>54</v>
       </c>
       <c r="F372" t="n">
-        <v>18.4</v>
+        <v>18.7</v>
       </c>
       <c r="G372" t="n">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="H372" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="I372" t="n">
         <v>0</v>
@@ -19039,7 +19039,7 @@
         <v>0</v>
       </c>
       <c r="K372" t="n">
-        <v>0.235</v>
+        <v>0.237</v>
       </c>
       <c r="L372" t="n">
         <v>3</v>
@@ -19064,23 +19064,23 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>19.1</v>
+        <v>19.4</v>
       </c>
       <c r="E373" t="n">
         <v>43</v>
       </c>
       <c r="F373" t="n">
-        <v>19.1</v>
+        <v>19.8</v>
       </c>
       <c r="G373" t="n">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="H373" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I373" t="n">
         <v>0</v>
@@ -19089,7 +19089,7 @@
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>0.233</v>
+        <v>0.236</v>
       </c>
       <c r="L373" t="n">
         <v>3</v>
@@ -19114,17 +19114,17 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>21.4</v>
+        <v>21.7</v>
       </c>
       <c r="E374" t="n">
         <v>38</v>
       </c>
       <c r="F374" t="n">
-        <v>18</v>
+        <v>18.7</v>
       </c>
       <c r="G374" t="n">
         <v>520</v>
@@ -19139,7 +19139,7 @@
         <v>0</v>
       </c>
       <c r="K374" t="n">
-        <v>0.231</v>
+        <v>0.234</v>
       </c>
       <c r="L374" t="n">
         <v>3</v>
@@ -19164,23 +19164,23 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>23.6</v>
+        <v>23.7</v>
       </c>
       <c r="E375" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F375" t="n">
-        <v>17.3</v>
+        <v>18</v>
       </c>
       <c r="G375" t="n">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="H375" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I375" t="n">
         <v>0</v>
@@ -19189,7 +19189,7 @@
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>0.229</v>
+        <v>0.232</v>
       </c>
       <c r="L375" t="n">
         <v>3</v>
@@ -19214,23 +19214,23 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D376" t="n">
         <v>25.1</v>
       </c>
       <c r="E376" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F376" t="n">
-        <v>16.9</v>
+        <v>16.6</v>
       </c>
       <c r="G376" t="n">
-        <v>504</v>
+        <v>477</v>
       </c>
       <c r="H376" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I376" t="n">
         <v>0</v>
@@ -19239,7 +19239,7 @@
         <v>0</v>
       </c>
       <c r="K376" t="n">
-        <v>0.227</v>
+        <v>0.23</v>
       </c>
       <c r="L376" t="n">
         <v>3</v>
@@ -19264,23 +19264,23 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D377" t="n">
         <v>25.9</v>
       </c>
       <c r="E377" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F377" t="n">
         <v>18.4</v>
       </c>
       <c r="G377" t="n">
-        <v>418</v>
+        <v>404</v>
       </c>
       <c r="H377" t="n">
-        <v>41</v>
+        <v>96</v>
       </c>
       <c r="I377" t="n">
         <v>0</v>
@@ -19289,7 +19289,7 @@
         <v>0</v>
       </c>
       <c r="K377" t="n">
-        <v>0.225</v>
+        <v>0.228</v>
       </c>
       <c r="L377" t="n">
         <v>3</v>
@@ -19314,23 +19314,23 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>25.9</v>
+        <v>25.4</v>
       </c>
       <c r="E378" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F378" t="n">
-        <v>18.4</v>
+        <v>15.8</v>
       </c>
       <c r="G378" t="n">
-        <v>279</v>
+        <v>142</v>
       </c>
       <c r="H378" t="n">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="I378" t="n">
         <v>0</v>
@@ -19339,7 +19339,7 @@
         <v>0</v>
       </c>
       <c r="K378" t="n">
-        <v>0.224</v>
+        <v>0.227</v>
       </c>
       <c r="L378" t="n">
         <v>3</v>
@@ -19364,20 +19364,20 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>24.8</v>
+        <v>22.6</v>
       </c>
       <c r="E379" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="F379" t="n">
-        <v>22.7</v>
+        <v>9.4</v>
       </c>
       <c r="G379" t="n">
-        <v>69</v>
+        <v>8</v>
       </c>
       <c r="H379" t="n">
         <v>100</v>
@@ -19389,7 +19389,7 @@
         <v>0</v>
       </c>
       <c r="K379" t="n">
-        <v>0.223</v>
+        <v>0.227</v>
       </c>
       <c r="L379" t="n">
         <v>3</v>
@@ -19414,32 +19414,32 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>21</v>
+        <v>21.2</v>
       </c>
       <c r="E380" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="F380" t="n">
-        <v>27.4</v>
+        <v>18.7</v>
       </c>
       <c r="G380" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H380" t="n">
         <v>100</v>
       </c>
       <c r="I380" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="J380" t="n">
         <v>0</v>
       </c>
       <c r="K380" t="n">
-        <v>0.223</v>
+        <v>0.227</v>
       </c>
       <c r="L380" t="n">
         <v>3</v>
@@ -19464,32 +19464,32 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>17.6</v>
+        <v>19.4</v>
       </c>
       <c r="E381" t="n">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="F381" t="n">
-        <v>18.4</v>
+        <v>21.6</v>
       </c>
       <c r="G381" t="n">
         <v>0</v>
       </c>
       <c r="H381" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I381" t="n">
-        <v>2.3</v>
+        <v>0</v>
       </c>
       <c r="J381" t="n">
         <v>0</v>
       </c>
       <c r="K381" t="n">
-        <v>0.224</v>
+        <v>0.228</v>
       </c>
       <c r="L381" t="n">
         <v>3</v>
@@ -19514,32 +19514,32 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>16.9</v>
+        <v>18.6</v>
       </c>
       <c r="E382" t="n">
+        <v>74</v>
+      </c>
+      <c r="F382" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="G382" t="n">
+        <v>0</v>
+      </c>
+      <c r="H382" t="n">
         <v>90</v>
       </c>
-      <c r="F382" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="G382" t="n">
-        <v>0</v>
-      </c>
-      <c r="H382" t="n">
-        <v>99</v>
-      </c>
       <c r="I382" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J382" t="n">
         <v>0</v>
       </c>
       <c r="K382" t="n">
-        <v>0.224</v>
+        <v>0.227</v>
       </c>
       <c r="L382" t="n">
         <v>3</v>
@@ -19564,23 +19564,23 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>16.1</v>
+        <v>17.8</v>
       </c>
       <c r="E383" t="n">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="F383" t="n">
-        <v>15.8</v>
+        <v>25.6</v>
       </c>
       <c r="G383" t="n">
         <v>0</v>
       </c>
       <c r="H383" t="n">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="I383" t="n">
         <v>0</v>
@@ -19589,7 +19589,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>0.223</v>
+        <v>0.227</v>
       </c>
       <c r="L383" t="n">
         <v>3</v>
@@ -19614,17 +19614,17 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>15.4</v>
+        <v>17.5</v>
       </c>
       <c r="E384" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="F384" t="n">
-        <v>22.7</v>
+        <v>24.8</v>
       </c>
       <c r="G384" t="n">
         <v>0</v>
@@ -19639,7 +19639,7 @@
         <v>0</v>
       </c>
       <c r="K384" t="n">
-        <v>0.223</v>
+        <v>0.227</v>
       </c>
       <c r="L384" t="n">
         <v>3</v>
@@ -19664,23 +19664,23 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>15</v>
+        <v>17.1</v>
       </c>
       <c r="E385" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="F385" t="n">
-        <v>20.5</v>
+        <v>21.6</v>
       </c>
       <c r="G385" t="n">
         <v>0</v>
       </c>
       <c r="H385" t="n">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="I385" t="n">
         <v>0</v>
@@ -19689,7 +19689,7 @@
         <v>0</v>
       </c>
       <c r="K385" t="n">
-        <v>0.223</v>
+        <v>0.227</v>
       </c>
       <c r="L385" t="n">
         <v>3</v>
@@ -19714,17 +19714,17 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>14.7</v>
+        <v>16.8</v>
       </c>
       <c r="E386" t="n">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="F386" t="n">
-        <v>19.1</v>
+        <v>17.3</v>
       </c>
       <c r="G386" t="n">
         <v>0</v>
@@ -19739,7 +19739,7 @@
         <v>0</v>
       </c>
       <c r="K386" t="n">
-        <v>0.223</v>
+        <v>0.227</v>
       </c>
       <c r="L386" t="n">
         <v>3</v>
@@ -19764,23 +19764,23 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>14.7</v>
+        <v>16.9</v>
       </c>
       <c r="E387" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="F387" t="n">
-        <v>18.4</v>
+        <v>18</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
       </c>
       <c r="H387" t="n">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="I387" t="n">
         <v>0</v>
@@ -19789,7 +19789,7 @@
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>0.222</v>
+        <v>0.227</v>
       </c>
       <c r="L387" t="n">
         <v>3</v>
@@ -19814,17 +19814,17 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>14.6</v>
+        <v>16.7</v>
       </c>
       <c r="E388" t="n">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="F388" t="n">
-        <v>17.6</v>
+        <v>15.1</v>
       </c>
       <c r="G388" t="n">
         <v>0</v>
@@ -19839,7 +19839,7 @@
         <v>0</v>
       </c>
       <c r="K388" t="n">
-        <v>0.222</v>
+        <v>0.229</v>
       </c>
       <c r="L388" t="n">
         <v>4</v>
@@ -19864,14 +19864,14 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>14.7</v>
+        <v>16.9</v>
       </c>
       <c r="E389" t="n">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="F389" t="n">
         <v>17.3</v>
@@ -19889,7 +19889,7 @@
         <v>0</v>
       </c>
       <c r="K389" t="n">
-        <v>0.223</v>
+        <v>0.231</v>
       </c>
       <c r="L389" t="n">
         <v>4</v>
@@ -19914,17 +19914,17 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>14.9</v>
+        <v>16.2</v>
       </c>
       <c r="E390" t="n">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="F390" t="n">
-        <v>17.6</v>
+        <v>13</v>
       </c>
       <c r="G390" t="n">
         <v>0</v>
@@ -19933,13 +19933,13 @@
         <v>100</v>
       </c>
       <c r="I390" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J390" t="n">
         <v>0</v>
       </c>
       <c r="K390" t="n">
-        <v>0.223</v>
+        <v>0.236</v>
       </c>
       <c r="L390" t="n">
         <v>4</v>
@@ -19964,17 +19964,17 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>14.9</v>
+        <v>15.4</v>
       </c>
       <c r="E391" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F391" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="G391" t="n">
         <v>0</v>
@@ -19983,13 +19983,13 @@
         <v>100</v>
       </c>
       <c r="I391" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J391" t="n">
         <v>0</v>
       </c>
       <c r="K391" t="n">
-        <v>0.225</v>
+        <v>0.237</v>
       </c>
       <c r="L391" t="n">
         <v>4</v>
@@ -20014,23 +20014,23 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>14.3</v>
+        <v>15.4</v>
       </c>
       <c r="E392" t="n">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F392" t="n">
-        <v>15.5</v>
+        <v>9.4</v>
       </c>
       <c r="G392" t="n">
         <v>0</v>
       </c>
       <c r="H392" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I392" t="n">
         <v>0</v>
@@ -20039,7 +20039,7 @@
         <v>0</v>
       </c>
       <c r="K392" t="n">
-        <v>0.225</v>
+        <v>0.238</v>
       </c>
       <c r="L392" t="n">
         <v>4</v>
@@ -20064,32 +20064,32 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>13.5</v>
+        <v>15</v>
       </c>
       <c r="E393" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="F393" t="n">
-        <v>13</v>
+        <v>2.2</v>
       </c>
       <c r="G393" t="n">
         <v>0</v>
       </c>
       <c r="H393" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="I393" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J393" t="n">
         <v>0</v>
       </c>
       <c r="K393" t="n">
-        <v>0.225</v>
+        <v>0.238</v>
       </c>
       <c r="L393" t="n">
         <v>4</v>
@@ -20114,32 +20114,32 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>14</v>
+        <v>14.8</v>
       </c>
       <c r="E394" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F394" t="n">
-        <v>11.2</v>
+        <v>3.2</v>
       </c>
       <c r="G394" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H394" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I394" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J394" t="n">
         <v>0</v>
       </c>
       <c r="K394" t="n">
-        <v>0.226</v>
+        <v>0.238</v>
       </c>
       <c r="L394" t="n">
         <v>4</v>
@@ -20164,32 +20164,32 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>15</v>
+        <v>15.3</v>
       </c>
       <c r="E395" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F395" t="n">
-        <v>6.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G395" t="n">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="H395" t="n">
         <v>100</v>
       </c>
       <c r="I395" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J395" t="n">
         <v>0</v>
       </c>
       <c r="K395" t="n">
-        <v>0.226</v>
+        <v>0.239</v>
       </c>
       <c r="L395" t="n">
         <v>4</v>
@@ -20214,20 +20214,20 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>16.8</v>
+        <v>16.1</v>
       </c>
       <c r="E396" t="n">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F396" t="n">
-        <v>23.4</v>
+        <v>27</v>
       </c>
       <c r="G396" t="n">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="H396" t="n">
         <v>100</v>
@@ -20239,7 +20239,7 @@
         <v>0</v>
       </c>
       <c r="K396" t="n">
-        <v>0.226</v>
+        <v>0.241</v>
       </c>
       <c r="L396" t="n">
         <v>4</v>
@@ -20264,20 +20264,20 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>13.4</v>
+        <v>13.1</v>
       </c>
       <c r="E397" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F397" t="n">
-        <v>23</v>
+        <v>21.2</v>
       </c>
       <c r="G397" t="n">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H397" t="n">
         <v>100</v>
@@ -20289,7 +20289,7 @@
         <v>0</v>
       </c>
       <c r="K397" t="n">
-        <v>0.229</v>
+        <v>0.24</v>
       </c>
       <c r="L397" t="n">
         <v>4</v>
@@ -20314,32 +20314,32 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>12.1</v>
+        <v>13.3</v>
       </c>
       <c r="E398" t="n">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="F398" t="n">
-        <v>20.5</v>
+        <v>14.4</v>
       </c>
       <c r="G398" t="n">
-        <v>90</v>
+        <v>219</v>
       </c>
       <c r="H398" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I398" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J398" t="n">
         <v>0</v>
       </c>
       <c r="K398" t="n">
-        <v>0.23</v>
+        <v>0.239</v>
       </c>
       <c r="L398" t="n">
         <v>4</v>
@@ -20364,32 +20364,32 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>12.4</v>
+        <v>14.4</v>
       </c>
       <c r="E399" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F399" t="n">
-        <v>15.8</v>
+        <v>14</v>
       </c>
       <c r="G399" t="n">
-        <v>201</v>
+        <v>426</v>
       </c>
       <c r="H399" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I399" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J399" t="n">
         <v>0</v>
       </c>
       <c r="K399" t="n">
-        <v>0.229</v>
+        <v>0.237</v>
       </c>
       <c r="L399" t="n">
         <v>4</v>
@@ -20414,20 +20414,20 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>12.8</v>
+        <v>14.6</v>
       </c>
       <c r="E400" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F400" t="n">
-        <v>15.1</v>
+        <v>16.6</v>
       </c>
       <c r="G400" t="n">
-        <v>218</v>
+        <v>305</v>
       </c>
       <c r="H400" t="n">
         <v>100</v>
@@ -20439,7 +20439,7 @@
         <v>0</v>
       </c>
       <c r="K400" t="n">
-        <v>0.228</v>
+        <v>0.236</v>
       </c>
       <c r="L400" t="n">
         <v>4</v>
@@ -20464,20 +20464,20 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>12.9</v>
+        <v>13.7</v>
       </c>
       <c r="E401" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="F401" t="n">
-        <v>17.6</v>
+        <v>18.7</v>
       </c>
       <c r="G401" t="n">
-        <v>125</v>
+        <v>76</v>
       </c>
       <c r="H401" t="n">
         <v>100</v>
@@ -20489,7 +20489,7 @@
         <v>0</v>
       </c>
       <c r="K401" t="n">
-        <v>0.226</v>
+        <v>0.234</v>
       </c>
       <c r="L401" t="n">
         <v>4</v>
@@ -20514,20 +20514,20 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D402" t="n">
-        <v>12.8</v>
+        <v>13.2</v>
       </c>
       <c r="E402" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="F402" t="n">
-        <v>15.1</v>
+        <v>16.6</v>
       </c>
       <c r="G402" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="H402" t="n">
         <v>100</v>
@@ -20539,7 +20539,7 @@
         <v>0</v>
       </c>
       <c r="K402" t="n">
-        <v>0.225</v>
+        <v>0.233</v>
       </c>
       <c r="L402" t="n">
         <v>4</v>
@@ -20564,23 +20564,23 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="E403" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F403" t="n">
-        <v>16.7</v>
+        <v>19.8</v>
       </c>
       <c r="G403" t="n">
-        <v>29.5</v>
+        <v>30</v>
       </c>
       <c r="H403" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I403" t="n">
         <v>0</v>
@@ -20589,7 +20589,7 @@
         <v>0</v>
       </c>
       <c r="K403" t="n">
-        <v>0.224</v>
+        <v>0.232</v>
       </c>
       <c r="L403" t="n">
         <v>4</v>
@@ -20614,23 +20614,23 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>13.1</v>
+        <v>12</v>
       </c>
       <c r="E404" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="F404" t="n">
-        <v>14.5</v>
+        <v>20.5</v>
       </c>
       <c r="G404" t="n">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H404" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I404" t="n">
         <v>0</v>
@@ -20639,7 +20639,7 @@
         <v>0</v>
       </c>
       <c r="K404" t="n">
-        <v>0.224</v>
+        <v>0.233</v>
       </c>
       <c r="L404" t="n">
         <v>4</v>
@@ -20664,23 +20664,23 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D405" t="n">
-        <v>12.9</v>
+        <v>11.5</v>
       </c>
       <c r="E405" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F405" t="n">
-        <v>12.2</v>
+        <v>18.7</v>
       </c>
       <c r="G405" t="n">
         <v>0</v>
       </c>
       <c r="H405" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I405" t="n">
         <v>0</v>
@@ -20689,7 +20689,7 @@
         <v>0</v>
       </c>
       <c r="K405" t="n">
-        <v>0.224</v>
+        <v>0.234</v>
       </c>
       <c r="L405" t="n">
         <v>4</v>
@@ -20714,17 +20714,17 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D406" t="n">
-        <v>12.8</v>
+        <v>11.3</v>
       </c>
       <c r="E406" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="F406" t="n">
-        <v>13.9</v>
+        <v>14.4</v>
       </c>
       <c r="G406" t="n">
         <v>0</v>
@@ -20739,7 +20739,7 @@
         <v>0</v>
       </c>
       <c r="K406" t="n">
-        <v>0.223</v>
+        <v>0.234</v>
       </c>
       <c r="L406" t="n">
         <v>4</v>
@@ -20764,17 +20764,17 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>11.6</v>
+        <v>11.3</v>
       </c>
       <c r="E407" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F407" t="n">
-        <v>11.2</v>
+        <v>14.4</v>
       </c>
       <c r="G407" t="n">
         <v>0</v>
@@ -20783,13 +20783,13 @@
         <v>100</v>
       </c>
       <c r="I407" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J407" t="n">
         <v>0</v>
       </c>
       <c r="K407" t="n">
-        <v>0.225</v>
+        <v>0.234</v>
       </c>
       <c r="L407" t="n">
         <v>4</v>
@@ -20814,32 +20814,32 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="E408" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F408" t="n">
-        <v>11.5</v>
+        <v>13.3</v>
       </c>
       <c r="G408" t="n">
         <v>0</v>
       </c>
       <c r="H408" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I408" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J408" t="n">
         <v>0</v>
       </c>
       <c r="K408" t="n">
-        <v>0.227</v>
+        <v>0.234</v>
       </c>
       <c r="L408" t="n">
         <v>4</v>
@@ -20864,23 +20864,23 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D409" t="n">
-        <v>10.9</v>
+        <v>10.5</v>
       </c>
       <c r="E409" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F409" t="n">
-        <v>12.5</v>
+        <v>11.2</v>
       </c>
       <c r="G409" t="n">
         <v>0</v>
       </c>
       <c r="H409" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="I409" t="n">
         <v>0</v>
@@ -20889,7 +20889,7 @@
         <v>0</v>
       </c>
       <c r="K409" t="n">
-        <v>0.227</v>
+        <v>0.234</v>
       </c>
       <c r="L409" t="n">
         <v>4</v>
@@ -20914,23 +20914,23 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D410" t="n">
-        <v>10.5</v>
+        <v>10.2</v>
       </c>
       <c r="E410" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F410" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="G410" t="n">
         <v>0</v>
       </c>
       <c r="H410" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="I410" t="n">
         <v>0</v>
@@ -20939,7 +20939,7 @@
         <v>0</v>
       </c>
       <c r="K410" t="n">
-        <v>0.227</v>
+        <v>0.234</v>
       </c>
       <c r="L410" t="n">
         <v>4</v>
@@ -20964,23 +20964,23 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>2026-10-20T11:03:36Z</t>
+          <t>2026-10-20T17:03:47Z</t>
         </is>
       </c>
       <c r="D411" t="n">
         <v>10.1</v>
       </c>
       <c r="E411" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F411" t="n">
-        <v>11.9</v>
+        <v>10.1</v>
       </c>
       <c r="G411" t="n">
         <v>0</v>
       </c>
       <c r="H411" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="I411" t="n">
         <v>0</v>
@@ -20989,7 +20989,7 @@
         <v>0</v>
       </c>
       <c r="K411" t="n">
-        <v>0.226</v>
+        <v>0.234</v>
       </c>
       <c r="L411" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-21 07:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N411"/>
+  <dimension ref="A1:N435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -18964,23 +18964,23 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>12.7</v>
+        <v>13</v>
       </c>
       <c r="E371" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F371" t="n">
-        <v>18.7</v>
+        <v>18.4</v>
       </c>
       <c r="G371" t="n">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H371" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="I371" t="n">
         <v>0</v>
@@ -18989,7 +18989,7 @@
         <v>0</v>
       </c>
       <c r="K371" t="n">
-        <v>0.238</v>
+        <v>0.218</v>
       </c>
       <c r="L371" t="n">
         <v>3</v>
@@ -19014,23 +19014,23 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>16</v>
+        <v>16.4</v>
       </c>
       <c r="E372" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F372" t="n">
-        <v>18.7</v>
+        <v>20.2</v>
       </c>
       <c r="G372" t="n">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H372" t="n">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="I372" t="n">
         <v>0</v>
@@ -19039,7 +19039,7 @@
         <v>0</v>
       </c>
       <c r="K372" t="n">
-        <v>0.237</v>
+        <v>0.217</v>
       </c>
       <c r="L372" t="n">
         <v>3</v>
@@ -19064,23 +19064,23 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>19.4</v>
+        <v>19.8</v>
       </c>
       <c r="E373" t="n">
         <v>43</v>
       </c>
       <c r="F373" t="n">
-        <v>19.8</v>
+        <v>20.2</v>
       </c>
       <c r="G373" t="n">
         <v>443</v>
       </c>
       <c r="H373" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I373" t="n">
         <v>0</v>
@@ -19089,7 +19089,7 @@
         <v>0</v>
       </c>
       <c r="K373" t="n">
-        <v>0.236</v>
+        <v>0.215</v>
       </c>
       <c r="L373" t="n">
         <v>3</v>
@@ -19114,20 +19114,20 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>21.7</v>
+        <v>22.4</v>
       </c>
       <c r="E374" t="n">
         <v>38</v>
       </c>
       <c r="F374" t="n">
-        <v>18.7</v>
+        <v>19.8</v>
       </c>
       <c r="G374" t="n">
-        <v>520</v>
+        <v>514</v>
       </c>
       <c r="H374" t="n">
         <v>0</v>
@@ -19139,7 +19139,7 @@
         <v>0</v>
       </c>
       <c r="K374" t="n">
-        <v>0.234</v>
+        <v>0.213</v>
       </c>
       <c r="L374" t="n">
         <v>3</v>
@@ -19164,23 +19164,23 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>23.7</v>
+        <v>24.6</v>
       </c>
       <c r="E375" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F375" t="n">
-        <v>18</v>
+        <v>19.4</v>
       </c>
       <c r="G375" t="n">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="H375" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I375" t="n">
         <v>0</v>
@@ -19189,7 +19189,7 @@
         <v>0</v>
       </c>
       <c r="K375" t="n">
-        <v>0.232</v>
+        <v>0.211</v>
       </c>
       <c r="L375" t="n">
         <v>3</v>
@@ -19214,23 +19214,23 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>25.1</v>
+        <v>25.9</v>
       </c>
       <c r="E376" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F376" t="n">
-        <v>16.6</v>
+        <v>16.9</v>
       </c>
       <c r="G376" t="n">
-        <v>477</v>
+        <v>501</v>
       </c>
       <c r="H376" t="n">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="I376" t="n">
         <v>0</v>
@@ -19239,7 +19239,7 @@
         <v>0</v>
       </c>
       <c r="K376" t="n">
-        <v>0.23</v>
+        <v>0.209</v>
       </c>
       <c r="L376" t="n">
         <v>3</v>
@@ -19264,23 +19264,23 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>25.9</v>
+        <v>26.4</v>
       </c>
       <c r="E377" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F377" t="n">
-        <v>18.4</v>
+        <v>15.8</v>
       </c>
       <c r="G377" t="n">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="H377" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="I377" t="n">
         <v>0</v>
@@ -19289,7 +19289,7 @@
         <v>0</v>
       </c>
       <c r="K377" t="n">
-        <v>0.228</v>
+        <v>0.207</v>
       </c>
       <c r="L377" t="n">
         <v>3</v>
@@ -19314,20 +19314,20 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>25.4</v>
+        <v>25.2</v>
       </c>
       <c r="E378" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F378" t="n">
-        <v>15.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G378" t="n">
-        <v>142</v>
+        <v>48</v>
       </c>
       <c r="H378" t="n">
         <v>100</v>
@@ -19339,7 +19339,7 @@
         <v>0</v>
       </c>
       <c r="K378" t="n">
-        <v>0.227</v>
+        <v>0.206</v>
       </c>
       <c r="L378" t="n">
         <v>3</v>
@@ -19364,20 +19364,20 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>22.6</v>
+        <v>23.1</v>
       </c>
       <c r="E379" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F379" t="n">
-        <v>9.4</v>
+        <v>25.9</v>
       </c>
       <c r="G379" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="H379" t="n">
         <v>100</v>
@@ -19389,7 +19389,7 @@
         <v>0</v>
       </c>
       <c r="K379" t="n">
-        <v>0.227</v>
+        <v>0.206</v>
       </c>
       <c r="L379" t="n">
         <v>3</v>
@@ -19414,32 +19414,32 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>21.2</v>
+        <v>20.1</v>
       </c>
       <c r="E380" t="n">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="F380" t="n">
-        <v>18.7</v>
+        <v>17.3</v>
       </c>
       <c r="G380" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H380" t="n">
         <v>100</v>
       </c>
       <c r="I380" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="J380" t="n">
         <v>0</v>
       </c>
       <c r="K380" t="n">
-        <v>0.227</v>
+        <v>0.207</v>
       </c>
       <c r="L380" t="n">
         <v>3</v>
@@ -19464,32 +19464,32 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>19.4</v>
+        <v>17.7</v>
       </c>
       <c r="E381" t="n">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="F381" t="n">
-        <v>21.6</v>
+        <v>12.2</v>
       </c>
       <c r="G381" t="n">
         <v>0</v>
       </c>
       <c r="H381" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I381" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="J381" t="n">
         <v>0</v>
       </c>
       <c r="K381" t="n">
-        <v>0.228</v>
+        <v>0.208</v>
       </c>
       <c r="L381" t="n">
         <v>3</v>
@@ -19514,23 +19514,23 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>18.6</v>
+        <v>17.3</v>
       </c>
       <c r="E382" t="n">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="F382" t="n">
-        <v>24.8</v>
+        <v>21.2</v>
       </c>
       <c r="G382" t="n">
         <v>0</v>
       </c>
       <c r="H382" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="I382" t="n">
         <v>0</v>
@@ -19539,7 +19539,7 @@
         <v>0</v>
       </c>
       <c r="K382" t="n">
-        <v>0.227</v>
+        <v>0.211</v>
       </c>
       <c r="L382" t="n">
         <v>3</v>
@@ -19564,23 +19564,23 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>17.8</v>
+        <v>16.6</v>
       </c>
       <c r="E383" t="n">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="F383" t="n">
-        <v>25.6</v>
+        <v>24.1</v>
       </c>
       <c r="G383" t="n">
         <v>0</v>
       </c>
       <c r="H383" t="n">
-        <v>98</v>
+        <v>47</v>
       </c>
       <c r="I383" t="n">
         <v>0</v>
@@ -19589,7 +19589,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>0.227</v>
+        <v>0.211</v>
       </c>
       <c r="L383" t="n">
         <v>3</v>
@@ -19614,23 +19614,23 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>17.5</v>
+        <v>15.5</v>
       </c>
       <c r="E384" t="n">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="F384" t="n">
-        <v>24.8</v>
+        <v>19.8</v>
       </c>
       <c r="G384" t="n">
         <v>0</v>
       </c>
       <c r="H384" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="I384" t="n">
         <v>0</v>
@@ -19639,7 +19639,7 @@
         <v>0</v>
       </c>
       <c r="K384" t="n">
-        <v>0.227</v>
+        <v>0.212</v>
       </c>
       <c r="L384" t="n">
         <v>3</v>
@@ -19664,23 +19664,23 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>17.1</v>
+        <v>15.2</v>
       </c>
       <c r="E385" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="F385" t="n">
-        <v>21.6</v>
+        <v>20.9</v>
       </c>
       <c r="G385" t="n">
         <v>0</v>
       </c>
       <c r="H385" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="I385" t="n">
         <v>0</v>
@@ -19689,7 +19689,7 @@
         <v>0</v>
       </c>
       <c r="K385" t="n">
-        <v>0.227</v>
+        <v>0.214</v>
       </c>
       <c r="L385" t="n">
         <v>3</v>
@@ -19714,23 +19714,23 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>16.8</v>
+        <v>15.3</v>
       </c>
       <c r="E386" t="n">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="F386" t="n">
-        <v>17.3</v>
+        <v>19.1</v>
       </c>
       <c r="G386" t="n">
         <v>0</v>
       </c>
       <c r="H386" t="n">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="I386" t="n">
         <v>0</v>
@@ -19739,7 +19739,7 @@
         <v>0</v>
       </c>
       <c r="K386" t="n">
-        <v>0.227</v>
+        <v>0.215</v>
       </c>
       <c r="L386" t="n">
         <v>3</v>
@@ -19764,23 +19764,23 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>16.9</v>
+        <v>15</v>
       </c>
       <c r="E387" t="n">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="F387" t="n">
-        <v>18</v>
+        <v>15.8</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
       </c>
       <c r="H387" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="I387" t="n">
         <v>0</v>
@@ -19789,7 +19789,7 @@
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>0.227</v>
+        <v>0.216</v>
       </c>
       <c r="L387" t="n">
         <v>3</v>
@@ -19814,14 +19814,14 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>16.7</v>
+        <v>15.1</v>
       </c>
       <c r="E388" t="n">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="F388" t="n">
         <v>15.1</v>
@@ -19839,7 +19839,7 @@
         <v>0</v>
       </c>
       <c r="K388" t="n">
-        <v>0.229</v>
+        <v>0.218</v>
       </c>
       <c r="L388" t="n">
         <v>4</v>
@@ -19864,17 +19864,17 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>16.9</v>
+        <v>14.4</v>
       </c>
       <c r="E389" t="n">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F389" t="n">
-        <v>17.3</v>
+        <v>10.8</v>
       </c>
       <c r="G389" t="n">
         <v>0</v>
@@ -19889,7 +19889,7 @@
         <v>0</v>
       </c>
       <c r="K389" t="n">
-        <v>0.231</v>
+        <v>0.219</v>
       </c>
       <c r="L389" t="n">
         <v>4</v>
@@ -19914,17 +19914,17 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>16.2</v>
+        <v>14.6</v>
       </c>
       <c r="E390" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="F390" t="n">
-        <v>13</v>
+        <v>10.4</v>
       </c>
       <c r="G390" t="n">
         <v>0</v>
@@ -19933,13 +19933,13 @@
         <v>100</v>
       </c>
       <c r="I390" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J390" t="n">
         <v>0</v>
       </c>
       <c r="K390" t="n">
-        <v>0.236</v>
+        <v>0.22</v>
       </c>
       <c r="L390" t="n">
         <v>4</v>
@@ -19964,17 +19964,17 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>15.4</v>
+        <v>14.7</v>
       </c>
       <c r="E391" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F391" t="n">
-        <v>13.3</v>
+        <v>6.5</v>
       </c>
       <c r="G391" t="n">
         <v>0</v>
@@ -19983,13 +19983,13 @@
         <v>100</v>
       </c>
       <c r="I391" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J391" t="n">
         <v>0</v>
       </c>
       <c r="K391" t="n">
-        <v>0.237</v>
+        <v>0.22</v>
       </c>
       <c r="L391" t="n">
         <v>4</v>
@@ -20014,17 +20014,17 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>15.4</v>
+        <v>14.6</v>
       </c>
       <c r="E392" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F392" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="G392" t="n">
         <v>0</v>
@@ -20033,13 +20033,13 @@
         <v>100</v>
       </c>
       <c r="I392" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="J392" t="n">
         <v>0</v>
       </c>
       <c r="K392" t="n">
-        <v>0.238</v>
+        <v>0.221</v>
       </c>
       <c r="L392" t="n">
         <v>4</v>
@@ -20064,17 +20064,17 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="E393" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F393" t="n">
-        <v>2.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G393" t="n">
         <v>0</v>
@@ -20083,13 +20083,13 @@
         <v>100</v>
       </c>
       <c r="I393" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J393" t="n">
         <v>0</v>
       </c>
       <c r="K393" t="n">
-        <v>0.238</v>
+        <v>0.221</v>
       </c>
       <c r="L393" t="n">
         <v>4</v>
@@ -20114,32 +20114,32 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>14.8</v>
+        <v>14.6</v>
       </c>
       <c r="E394" t="n">
         <v>94</v>
       </c>
       <c r="F394" t="n">
-        <v>3.2</v>
+        <v>6.1</v>
       </c>
       <c r="G394" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H394" t="n">
         <v>100</v>
       </c>
       <c r="I394" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J394" t="n">
         <v>0</v>
       </c>
       <c r="K394" t="n">
-        <v>0.238</v>
+        <v>0.221</v>
       </c>
       <c r="L394" t="n">
         <v>4</v>
@@ -20164,32 +20164,32 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>15.3</v>
+        <v>14.9</v>
       </c>
       <c r="E395" t="n">
         <v>91</v>
       </c>
       <c r="F395" t="n">
-        <v>8.300000000000001</v>
+        <v>19.8</v>
       </c>
       <c r="G395" t="n">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="H395" t="n">
         <v>100</v>
       </c>
       <c r="I395" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J395" t="n">
         <v>0</v>
       </c>
       <c r="K395" t="n">
-        <v>0.239</v>
+        <v>0.222</v>
       </c>
       <c r="L395" t="n">
         <v>4</v>
@@ -20214,32 +20214,32 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>16.1</v>
+        <v>12.9</v>
       </c>
       <c r="E396" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F396" t="n">
-        <v>27</v>
+        <v>22.7</v>
       </c>
       <c r="G396" t="n">
-        <v>165</v>
+        <v>18</v>
       </c>
       <c r="H396" t="n">
         <v>100</v>
       </c>
       <c r="I396" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J396" t="n">
         <v>0</v>
       </c>
       <c r="K396" t="n">
-        <v>0.241</v>
+        <v>0.224</v>
       </c>
       <c r="L396" t="n">
         <v>4</v>
@@ -20264,20 +20264,20 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>13.1</v>
+        <v>12.1</v>
       </c>
       <c r="E397" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F397" t="n">
-        <v>21.2</v>
+        <v>11.2</v>
       </c>
       <c r="G397" t="n">
-        <v>127</v>
+        <v>44</v>
       </c>
       <c r="H397" t="n">
         <v>100</v>
@@ -20289,7 +20289,7 @@
         <v>0</v>
       </c>
       <c r="K397" t="n">
-        <v>0.24</v>
+        <v>0.224</v>
       </c>
       <c r="L397" t="n">
         <v>4</v>
@@ -20314,23 +20314,23 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="E398" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F398" t="n">
-        <v>14.4</v>
+        <v>14.8</v>
       </c>
       <c r="G398" t="n">
-        <v>219</v>
+        <v>125</v>
       </c>
       <c r="H398" t="n">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="I398" t="n">
         <v>0</v>
@@ -20339,7 +20339,7 @@
         <v>0</v>
       </c>
       <c r="K398" t="n">
-        <v>0.239</v>
+        <v>0.223</v>
       </c>
       <c r="L398" t="n">
         <v>4</v>
@@ -20364,23 +20364,23 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D399" t="n">
         <v>14.4</v>
       </c>
       <c r="E399" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F399" t="n">
-        <v>14</v>
+        <v>16.2</v>
       </c>
       <c r="G399" t="n">
-        <v>426</v>
+        <v>471</v>
       </c>
       <c r="H399" t="n">
-        <v>99</v>
+        <v>58</v>
       </c>
       <c r="I399" t="n">
         <v>0</v>
@@ -20389,7 +20389,7 @@
         <v>0</v>
       </c>
       <c r="K399" t="n">
-        <v>0.237</v>
+        <v>0.222</v>
       </c>
       <c r="L399" t="n">
         <v>4</v>
@@ -20414,20 +20414,20 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D400" t="n">
         <v>14.6</v>
       </c>
       <c r="E400" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F400" t="n">
-        <v>16.6</v>
+        <v>18.7</v>
       </c>
       <c r="G400" t="n">
-        <v>305</v>
+        <v>418</v>
       </c>
       <c r="H400" t="n">
         <v>100</v>
@@ -20439,7 +20439,7 @@
         <v>0</v>
       </c>
       <c r="K400" t="n">
-        <v>0.236</v>
+        <v>0.22</v>
       </c>
       <c r="L400" t="n">
         <v>4</v>
@@ -20464,20 +20464,20 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="E401" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F401" t="n">
-        <v>18.7</v>
+        <v>17.6</v>
       </c>
       <c r="G401" t="n">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="H401" t="n">
         <v>100</v>
@@ -20489,7 +20489,7 @@
         <v>0</v>
       </c>
       <c r="K401" t="n">
-        <v>0.234</v>
+        <v>0.219</v>
       </c>
       <c r="L401" t="n">
         <v>4</v>
@@ -20514,20 +20514,20 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D402" t="n">
-        <v>13.2</v>
+        <v>13.9</v>
       </c>
       <c r="E402" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F402" t="n">
         <v>16.6</v>
       </c>
       <c r="G402" t="n">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="H402" t="n">
         <v>100</v>
@@ -20539,7 +20539,7 @@
         <v>0</v>
       </c>
       <c r="K402" t="n">
-        <v>0.233</v>
+        <v>0.217</v>
       </c>
       <c r="L402" t="n">
         <v>4</v>
@@ -20564,20 +20564,20 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>12.6</v>
+        <v>13.7</v>
       </c>
       <c r="E403" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F403" t="n">
-        <v>19.8</v>
+        <v>16.6</v>
       </c>
       <c r="G403" t="n">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="H403" t="n">
         <v>100</v>
@@ -20589,7 +20589,7 @@
         <v>0</v>
       </c>
       <c r="K403" t="n">
-        <v>0.232</v>
+        <v>0.217</v>
       </c>
       <c r="L403" t="n">
         <v>4</v>
@@ -20614,20 +20614,20 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E404" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="F404" t="n">
-        <v>20.5</v>
+        <v>15.5</v>
       </c>
       <c r="G404" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="H404" t="n">
         <v>100</v>
@@ -20639,7 +20639,7 @@
         <v>0</v>
       </c>
       <c r="K404" t="n">
-        <v>0.233</v>
+        <v>0.216</v>
       </c>
       <c r="L404" t="n">
         <v>4</v>
@@ -20664,17 +20664,17 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D405" t="n">
-        <v>11.5</v>
+        <v>12.8</v>
       </c>
       <c r="E405" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F405" t="n">
-        <v>18.7</v>
+        <v>17.3</v>
       </c>
       <c r="G405" t="n">
         <v>0</v>
@@ -20689,7 +20689,7 @@
         <v>0</v>
       </c>
       <c r="K405" t="n">
-        <v>0.234</v>
+        <v>0.232</v>
       </c>
       <c r="L405" t="n">
         <v>4</v>
@@ -20714,17 +20714,17 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D406" t="n">
-        <v>11.3</v>
+        <v>12.3</v>
       </c>
       <c r="E406" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="F406" t="n">
-        <v>14.4</v>
+        <v>16.2</v>
       </c>
       <c r="G406" t="n">
         <v>0</v>
@@ -20739,7 +20739,7 @@
         <v>0</v>
       </c>
       <c r="K406" t="n">
-        <v>0.234</v>
+        <v>0.26</v>
       </c>
       <c r="L406" t="n">
         <v>4</v>
@@ -20764,17 +20764,17 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>11.3</v>
+        <v>11.7</v>
       </c>
       <c r="E407" t="n">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="F407" t="n">
-        <v>14.4</v>
+        <v>16.9</v>
       </c>
       <c r="G407" t="n">
         <v>0</v>
@@ -20783,13 +20783,13 @@
         <v>100</v>
       </c>
       <c r="I407" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="J407" t="n">
         <v>0</v>
       </c>
       <c r="K407" t="n">
-        <v>0.234</v>
+        <v>0.26</v>
       </c>
       <c r="L407" t="n">
         <v>4</v>
@@ -20814,32 +20814,32 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>10.9</v>
+        <v>11.6</v>
       </c>
       <c r="E408" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="F408" t="n">
-        <v>13.3</v>
+        <v>15.8</v>
       </c>
       <c r="G408" t="n">
         <v>0</v>
       </c>
       <c r="H408" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I408" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J408" t="n">
         <v>0</v>
       </c>
       <c r="K408" t="n">
-        <v>0.234</v>
+        <v>0.26</v>
       </c>
       <c r="L408" t="n">
         <v>4</v>
@@ -20864,14 +20864,14 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D409" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="E409" t="n">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="F409" t="n">
         <v>11.2</v>
@@ -20880,7 +20880,7 @@
         <v>0</v>
       </c>
       <c r="H409" t="n">
-        <v>93</v>
+        <v>56</v>
       </c>
       <c r="I409" t="n">
         <v>0</v>
@@ -20889,7 +20889,7 @@
         <v>0</v>
       </c>
       <c r="K409" t="n">
-        <v>0.234</v>
+        <v>0.26</v>
       </c>
       <c r="L409" t="n">
         <v>4</v>
@@ -20914,23 +20914,23 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D410" t="n">
         <v>10.2</v>
       </c>
       <c r="E410" t="n">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="F410" t="n">
-        <v>11.9</v>
+        <v>11.5</v>
       </c>
       <c r="G410" t="n">
         <v>0</v>
       </c>
       <c r="H410" t="n">
-        <v>93</v>
+        <v>2</v>
       </c>
       <c r="I410" t="n">
         <v>0</v>
@@ -20939,7 +20939,7 @@
         <v>0</v>
       </c>
       <c r="K410" t="n">
-        <v>0.234</v>
+        <v>0.26</v>
       </c>
       <c r="L410" t="n">
         <v>4</v>
@@ -20964,23 +20964,23 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>2026-10-20T17:03:47Z</t>
+          <t>2026-10-21T05:03:45Z</t>
         </is>
       </c>
       <c r="D411" t="n">
-        <v>10.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E411" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="F411" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G411" t="n">
         <v>0</v>
       </c>
       <c r="H411" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I411" t="n">
         <v>0</v>
@@ -20989,7 +20989,7 @@
         <v>0</v>
       </c>
       <c r="K411" t="n">
-        <v>0.234</v>
+        <v>0.26</v>
       </c>
       <c r="L411" t="n">
         <v>4</v>
@@ -20998,6 +20998,1206 @@
         <v>0</v>
       </c>
       <c r="N411" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E412" t="n">
+        <v>93</v>
+      </c>
+      <c r="F412" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G412" t="n">
+        <v>0</v>
+      </c>
+      <c r="H412" t="n">
+        <v>0</v>
+      </c>
+      <c r="I412" t="n">
+        <v>0</v>
+      </c>
+      <c r="J412" t="n">
+        <v>0</v>
+      </c>
+      <c r="K412" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="L412" t="n">
+        <v>5</v>
+      </c>
+      <c r="M412" t="n">
+        <v>0</v>
+      </c>
+      <c r="N412" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E413" t="n">
+        <v>96</v>
+      </c>
+      <c r="F413" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="G413" t="n">
+        <v>0</v>
+      </c>
+      <c r="H413" t="n">
+        <v>0</v>
+      </c>
+      <c r="I413" t="n">
+        <v>0</v>
+      </c>
+      <c r="J413" t="n">
+        <v>0</v>
+      </c>
+      <c r="K413" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="L413" t="n">
+        <v>5</v>
+      </c>
+      <c r="M413" t="n">
+        <v>0</v>
+      </c>
+      <c r="N413" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E414" t="n">
+        <v>98</v>
+      </c>
+      <c r="F414" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G414" t="n">
+        <v>0</v>
+      </c>
+      <c r="H414" t="n">
+        <v>0</v>
+      </c>
+      <c r="I414" t="n">
+        <v>0</v>
+      </c>
+      <c r="J414" t="n">
+        <v>0</v>
+      </c>
+      <c r="K414" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="L414" t="n">
+        <v>5</v>
+      </c>
+      <c r="M414" t="n">
+        <v>0</v>
+      </c>
+      <c r="N414" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E415" t="n">
+        <v>98</v>
+      </c>
+      <c r="F415" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="G415" t="n">
+        <v>0</v>
+      </c>
+      <c r="H415" t="n">
+        <v>0</v>
+      </c>
+      <c r="I415" t="n">
+        <v>0</v>
+      </c>
+      <c r="J415" t="n">
+        <v>0</v>
+      </c>
+      <c r="K415" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="L415" t="n">
+        <v>5</v>
+      </c>
+      <c r="M415" t="n">
+        <v>0</v>
+      </c>
+      <c r="N415" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E416" t="n">
+        <v>99</v>
+      </c>
+      <c r="F416" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G416" t="n">
+        <v>0</v>
+      </c>
+      <c r="H416" t="n">
+        <v>0</v>
+      </c>
+      <c r="I416" t="n">
+        <v>0</v>
+      </c>
+      <c r="J416" t="n">
+        <v>0</v>
+      </c>
+      <c r="K416" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="L416" t="n">
+        <v>5</v>
+      </c>
+      <c r="M416" t="n">
+        <v>0</v>
+      </c>
+      <c r="N416" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E417" t="n">
+        <v>99</v>
+      </c>
+      <c r="F417" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G417" t="n">
+        <v>0</v>
+      </c>
+      <c r="H417" t="n">
+        <v>0</v>
+      </c>
+      <c r="I417" t="n">
+        <v>0</v>
+      </c>
+      <c r="J417" t="n">
+        <v>0</v>
+      </c>
+      <c r="K417" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="L417" t="n">
+        <v>5</v>
+      </c>
+      <c r="M417" t="n">
+        <v>0</v>
+      </c>
+      <c r="N417" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E418" t="n">
+        <v>100</v>
+      </c>
+      <c r="F418" t="n">
+        <v>9</v>
+      </c>
+      <c r="G418" t="n">
+        <v>35</v>
+      </c>
+      <c r="H418" t="n">
+        <v>85</v>
+      </c>
+      <c r="I418" t="n">
+        <v>0</v>
+      </c>
+      <c r="J418" t="n">
+        <v>0</v>
+      </c>
+      <c r="K418" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="L418" t="n">
+        <v>5</v>
+      </c>
+      <c r="M418" t="n">
+        <v>0</v>
+      </c>
+      <c r="N418" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E419" t="n">
+        <v>92</v>
+      </c>
+      <c r="F419" t="n">
+        <v>9</v>
+      </c>
+      <c r="G419" t="n">
+        <v>165</v>
+      </c>
+      <c r="H419" t="n">
+        <v>0</v>
+      </c>
+      <c r="I419" t="n">
+        <v>0</v>
+      </c>
+      <c r="J419" t="n">
+        <v>0</v>
+      </c>
+      <c r="K419" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="L419" t="n">
+        <v>5</v>
+      </c>
+      <c r="M419" t="n">
+        <v>0</v>
+      </c>
+      <c r="N419" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E420" t="n">
+        <v>78</v>
+      </c>
+      <c r="F420" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="G420" t="n">
+        <v>328</v>
+      </c>
+      <c r="H420" t="n">
+        <v>0</v>
+      </c>
+      <c r="I420" t="n">
+        <v>0</v>
+      </c>
+      <c r="J420" t="n">
+        <v>0</v>
+      </c>
+      <c r="K420" t="n">
+        <v>0.257</v>
+      </c>
+      <c r="L420" t="n">
+        <v>5</v>
+      </c>
+      <c r="M420" t="n">
+        <v>0</v>
+      </c>
+      <c r="N420" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="E421" t="n">
+        <v>66</v>
+      </c>
+      <c r="F421" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G421" t="n">
+        <v>447.8</v>
+      </c>
+      <c r="H421" t="n">
+        <v>1</v>
+      </c>
+      <c r="I421" t="n">
+        <v>0</v>
+      </c>
+      <c r="J421" t="n">
+        <v>0</v>
+      </c>
+      <c r="K421" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="L421" t="n">
+        <v>5</v>
+      </c>
+      <c r="M421" t="n">
+        <v>0</v>
+      </c>
+      <c r="N421" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="E422" t="n">
+        <v>56</v>
+      </c>
+      <c r="F422" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G422" t="n">
+        <v>521.5</v>
+      </c>
+      <c r="H422" t="n">
+        <v>0</v>
+      </c>
+      <c r="I422" t="n">
+        <v>0</v>
+      </c>
+      <c r="J422" t="n">
+        <v>0</v>
+      </c>
+      <c r="K422" t="n">
+        <v>0.254</v>
+      </c>
+      <c r="L422" t="n">
+        <v>5</v>
+      </c>
+      <c r="M422" t="n">
+        <v>0</v>
+      </c>
+      <c r="N422" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="E423" t="n">
+        <v>49</v>
+      </c>
+      <c r="F423" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G423" t="n">
+        <v>543.3</v>
+      </c>
+      <c r="H423" t="n">
+        <v>0</v>
+      </c>
+      <c r="I423" t="n">
+        <v>0</v>
+      </c>
+      <c r="J423" t="n">
+        <v>0</v>
+      </c>
+      <c r="K423" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="L423" t="n">
+        <v>5</v>
+      </c>
+      <c r="M423" t="n">
+        <v>0</v>
+      </c>
+      <c r="N423" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="E424" t="n">
+        <v>47</v>
+      </c>
+      <c r="F424" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G424" t="n">
+        <v>510</v>
+      </c>
+      <c r="H424" t="n">
+        <v>0</v>
+      </c>
+      <c r="I424" t="n">
+        <v>0</v>
+      </c>
+      <c r="J424" t="n">
+        <v>0</v>
+      </c>
+      <c r="K424" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L424" t="n">
+        <v>5</v>
+      </c>
+      <c r="M424" t="n">
+        <v>0</v>
+      </c>
+      <c r="N424" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="E425" t="n">
+        <v>47</v>
+      </c>
+      <c r="F425" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G425" t="n">
+        <v>426</v>
+      </c>
+      <c r="H425" t="n">
+        <v>0</v>
+      </c>
+      <c r="I425" t="n">
+        <v>0</v>
+      </c>
+      <c r="J425" t="n">
+        <v>0</v>
+      </c>
+      <c r="K425" t="n">
+        <v>0.249</v>
+      </c>
+      <c r="L425" t="n">
+        <v>5</v>
+      </c>
+      <c r="M425" t="n">
+        <v>0</v>
+      </c>
+      <c r="N425" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="E426" t="n">
+        <v>47</v>
+      </c>
+      <c r="F426" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G426" t="n">
+        <v>297</v>
+      </c>
+      <c r="H426" t="n">
+        <v>0</v>
+      </c>
+      <c r="I426" t="n">
+        <v>0</v>
+      </c>
+      <c r="J426" t="n">
+        <v>0</v>
+      </c>
+      <c r="K426" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="L426" t="n">
+        <v>5</v>
+      </c>
+      <c r="M426" t="n">
+        <v>0</v>
+      </c>
+      <c r="N426" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="E427" t="n">
+        <v>59</v>
+      </c>
+      <c r="F427" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G427" t="n">
+        <v>144</v>
+      </c>
+      <c r="H427" t="n">
+        <v>10</v>
+      </c>
+      <c r="I427" t="n">
+        <v>0</v>
+      </c>
+      <c r="J427" t="n">
+        <v>0</v>
+      </c>
+      <c r="K427" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="L427" t="n">
+        <v>5</v>
+      </c>
+      <c r="M427" t="n">
+        <v>0</v>
+      </c>
+      <c r="N427" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="E428" t="n">
+        <v>67</v>
+      </c>
+      <c r="F428" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G428" t="n">
+        <v>19</v>
+      </c>
+      <c r="H428" t="n">
+        <v>13</v>
+      </c>
+      <c r="I428" t="n">
+        <v>0</v>
+      </c>
+      <c r="J428" t="n">
+        <v>0</v>
+      </c>
+      <c r="K428" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L428" t="n">
+        <v>5</v>
+      </c>
+      <c r="M428" t="n">
+        <v>0</v>
+      </c>
+      <c r="N428" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E429" t="n">
+        <v>72</v>
+      </c>
+      <c r="F429" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="G429" t="n">
+        <v>0</v>
+      </c>
+      <c r="H429" t="n">
+        <v>2</v>
+      </c>
+      <c r="I429" t="n">
+        <v>0</v>
+      </c>
+      <c r="J429" t="n">
+        <v>0</v>
+      </c>
+      <c r="K429" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L429" t="n">
+        <v>5</v>
+      </c>
+      <c r="M429" t="n">
+        <v>0</v>
+      </c>
+      <c r="N429" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="E430" t="n">
+        <v>73</v>
+      </c>
+      <c r="F430" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G430" t="n">
+        <v>0</v>
+      </c>
+      <c r="H430" t="n">
+        <v>2</v>
+      </c>
+      <c r="I430" t="n">
+        <v>0</v>
+      </c>
+      <c r="J430" t="n">
+        <v>0</v>
+      </c>
+      <c r="K430" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L430" t="n">
+        <v>5</v>
+      </c>
+      <c r="M430" t="n">
+        <v>0</v>
+      </c>
+      <c r="N430" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="E431" t="n">
+        <v>74</v>
+      </c>
+      <c r="F431" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="G431" t="n">
+        <v>0</v>
+      </c>
+      <c r="H431" t="n">
+        <v>0</v>
+      </c>
+      <c r="I431" t="n">
+        <v>0</v>
+      </c>
+      <c r="J431" t="n">
+        <v>0</v>
+      </c>
+      <c r="K431" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L431" t="n">
+        <v>5</v>
+      </c>
+      <c r="M431" t="n">
+        <v>0</v>
+      </c>
+      <c r="N431" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>9</v>
+      </c>
+      <c r="E432" t="n">
+        <v>76</v>
+      </c>
+      <c r="F432" t="n">
+        <v>7</v>
+      </c>
+      <c r="G432" t="n">
+        <v>0</v>
+      </c>
+      <c r="H432" t="n">
+        <v>10</v>
+      </c>
+      <c r="I432" t="n">
+        <v>0</v>
+      </c>
+      <c r="J432" t="n">
+        <v>0</v>
+      </c>
+      <c r="K432" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L432" t="n">
+        <v>5</v>
+      </c>
+      <c r="M432" t="n">
+        <v>0</v>
+      </c>
+      <c r="N432" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="E433" t="n">
+        <v>75</v>
+      </c>
+      <c r="F433" t="n">
+        <v>8</v>
+      </c>
+      <c r="G433" t="n">
+        <v>0</v>
+      </c>
+      <c r="H433" t="n">
+        <v>11</v>
+      </c>
+      <c r="I433" t="n">
+        <v>0</v>
+      </c>
+      <c r="J433" t="n">
+        <v>0</v>
+      </c>
+      <c r="K433" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L433" t="n">
+        <v>5</v>
+      </c>
+      <c r="M433" t="n">
+        <v>0</v>
+      </c>
+      <c r="N433" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E434" t="n">
+        <v>77</v>
+      </c>
+      <c r="F434" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G434" t="n">
+        <v>0</v>
+      </c>
+      <c r="H434" t="n">
+        <v>45</v>
+      </c>
+      <c r="I434" t="n">
+        <v>0</v>
+      </c>
+      <c r="J434" t="n">
+        <v>0</v>
+      </c>
+      <c r="K434" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L434" t="n">
+        <v>5</v>
+      </c>
+      <c r="M434" t="n">
+        <v>0</v>
+      </c>
+      <c r="N434" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>24:00</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>2026-10-21T05:03:45Z</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E435" t="n">
+        <v>77</v>
+      </c>
+      <c r="F435" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G435" t="n">
+        <v>0</v>
+      </c>
+      <c r="H435" t="n">
+        <v>69</v>
+      </c>
+      <c r="I435" t="n">
+        <v>0</v>
+      </c>
+      <c r="J435" t="n">
+        <v>0</v>
+      </c>
+      <c r="K435" t="n">
+        <v>0.246</v>
+      </c>
+      <c r="L435" t="n">
+        <v>5</v>
+      </c>
+      <c r="M435" t="n">
+        <v>0</v>
+      </c>
+      <c r="N435" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-21 13:05
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -19264,20 +19264,20 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="E377" t="n">
         <v>34</v>
       </c>
       <c r="F377" t="n">
-        <v>15.8</v>
+        <v>18</v>
       </c>
       <c r="G377" t="n">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="H377" t="n">
         <v>100</v>
@@ -19289,7 +19289,7 @@
         <v>0</v>
       </c>
       <c r="K377" t="n">
-        <v>0.207</v>
+        <v>0.208</v>
       </c>
       <c r="L377" t="n">
         <v>3</v>
@@ -19314,20 +19314,20 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>25.2</v>
+        <v>24.2</v>
       </c>
       <c r="E378" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F378" t="n">
-        <v>9.699999999999999</v>
+        <v>30.2</v>
       </c>
       <c r="G378" t="n">
-        <v>48</v>
+        <v>110</v>
       </c>
       <c r="H378" t="n">
         <v>100</v>
@@ -19339,7 +19339,7 @@
         <v>0</v>
       </c>
       <c r="K378" t="n">
-        <v>0.206</v>
+        <v>0.207</v>
       </c>
       <c r="L378" t="n">
         <v>3</v>
@@ -19364,26 +19364,26 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>23.1</v>
+        <v>20.9</v>
       </c>
       <c r="E379" t="n">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="F379" t="n">
-        <v>25.9</v>
+        <v>10.4</v>
       </c>
       <c r="G379" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="H379" t="n">
         <v>100</v>
       </c>
       <c r="I379" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="J379" t="n">
         <v>0</v>
@@ -19414,32 +19414,32 @@
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>20.1</v>
+        <v>18.7</v>
       </c>
       <c r="E380" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F380" t="n">
-        <v>17.3</v>
+        <v>15.5</v>
       </c>
       <c r="G380" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H380" t="n">
         <v>100</v>
       </c>
       <c r="I380" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="J380" t="n">
         <v>0</v>
       </c>
       <c r="K380" t="n">
-        <v>0.207</v>
+        <v>0.206</v>
       </c>
       <c r="L380" t="n">
         <v>3</v>
@@ -19464,17 +19464,17 @@
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>17.7</v>
+        <v>18.6</v>
       </c>
       <c r="E381" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="F381" t="n">
-        <v>12.2</v>
+        <v>17.3</v>
       </c>
       <c r="G381" t="n">
         <v>0</v>
@@ -19483,13 +19483,13 @@
         <v>100</v>
       </c>
       <c r="I381" t="n">
-        <v>1.1</v>
+        <v>0.1</v>
       </c>
       <c r="J381" t="n">
         <v>0</v>
       </c>
       <c r="K381" t="n">
-        <v>0.208</v>
+        <v>0.205</v>
       </c>
       <c r="L381" t="n">
         <v>3</v>
@@ -19514,23 +19514,23 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>17.3</v>
+        <v>18</v>
       </c>
       <c r="E382" t="n">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="F382" t="n">
-        <v>21.2</v>
+        <v>23.4</v>
       </c>
       <c r="G382" t="n">
         <v>0</v>
       </c>
       <c r="H382" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I382" t="n">
         <v>0</v>
@@ -19539,7 +19539,7 @@
         <v>0</v>
       </c>
       <c r="K382" t="n">
-        <v>0.211</v>
+        <v>0.205</v>
       </c>
       <c r="L382" t="n">
         <v>3</v>
@@ -19564,23 +19564,23 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>16.6</v>
+        <v>17.3</v>
       </c>
       <c r="E383" t="n">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="F383" t="n">
-        <v>24.1</v>
+        <v>27.4</v>
       </c>
       <c r="G383" t="n">
         <v>0</v>
       </c>
       <c r="H383" t="n">
-        <v>47</v>
+        <v>95</v>
       </c>
       <c r="I383" t="n">
         <v>0</v>
@@ -19589,7 +19589,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>0.211</v>
+        <v>0.205</v>
       </c>
       <c r="L383" t="n">
         <v>3</v>
@@ -19614,23 +19614,23 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>15.5</v>
+        <v>17.1</v>
       </c>
       <c r="E384" t="n">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="F384" t="n">
-        <v>19.8</v>
+        <v>23.4</v>
       </c>
       <c r="G384" t="n">
         <v>0</v>
       </c>
       <c r="H384" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="I384" t="n">
         <v>0</v>
@@ -19639,7 +19639,7 @@
         <v>0</v>
       </c>
       <c r="K384" t="n">
-        <v>0.212</v>
+        <v>0.207</v>
       </c>
       <c r="L384" t="n">
         <v>3</v>
@@ -19664,14 +19664,14 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>15.2</v>
+        <v>16.8</v>
       </c>
       <c r="E385" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F385" t="n">
         <v>20.9</v>
@@ -19680,7 +19680,7 @@
         <v>0</v>
       </c>
       <c r="H385" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I385" t="n">
         <v>0</v>
@@ -19689,7 +19689,7 @@
         <v>0</v>
       </c>
       <c r="K385" t="n">
-        <v>0.214</v>
+        <v>0.209</v>
       </c>
       <c r="L385" t="n">
         <v>3</v>
@@ -19714,23 +19714,23 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>15.3</v>
+        <v>16.4</v>
       </c>
       <c r="E386" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="F386" t="n">
-        <v>19.1</v>
+        <v>22</v>
       </c>
       <c r="G386" t="n">
         <v>0</v>
       </c>
       <c r="H386" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="I386" t="n">
         <v>0</v>
@@ -19739,7 +19739,7 @@
         <v>0</v>
       </c>
       <c r="K386" t="n">
-        <v>0.215</v>
+        <v>0.211</v>
       </c>
       <c r="L386" t="n">
         <v>3</v>
@@ -19764,17 +19764,17 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>15</v>
+        <v>16.3</v>
       </c>
       <c r="E387" t="n">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="F387" t="n">
-        <v>15.8</v>
+        <v>18.7</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
@@ -19789,7 +19789,7 @@
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>0.216</v>
+        <v>0.214</v>
       </c>
       <c r="L387" t="n">
         <v>3</v>
@@ -19814,17 +19814,17 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>15.1</v>
+        <v>16.4</v>
       </c>
       <c r="E388" t="n">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="F388" t="n">
-        <v>15.1</v>
+        <v>18</v>
       </c>
       <c r="G388" t="n">
         <v>0</v>
@@ -19833,13 +19833,13 @@
         <v>100</v>
       </c>
       <c r="I388" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J388" t="n">
         <v>0</v>
       </c>
       <c r="K388" t="n">
-        <v>0.218</v>
+        <v>0.216</v>
       </c>
       <c r="L388" t="n">
         <v>4</v>
@@ -19864,17 +19864,17 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>14.4</v>
+        <v>16.1</v>
       </c>
       <c r="E389" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="F389" t="n">
-        <v>10.8</v>
+        <v>17.3</v>
       </c>
       <c r="G389" t="n">
         <v>0</v>
@@ -19914,17 +19914,17 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>14.6</v>
+        <v>15.6</v>
       </c>
       <c r="E390" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F390" t="n">
-        <v>10.4</v>
+        <v>14.4</v>
       </c>
       <c r="G390" t="n">
         <v>0</v>
@@ -19933,13 +19933,13 @@
         <v>100</v>
       </c>
       <c r="I390" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="J390" t="n">
         <v>0</v>
       </c>
       <c r="K390" t="n">
-        <v>0.22</v>
+        <v>0.223</v>
       </c>
       <c r="L390" t="n">
         <v>4</v>
@@ -19964,17 +19964,17 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>14.7</v>
+        <v>15.3</v>
       </c>
       <c r="E391" t="n">
         <v>90</v>
       </c>
       <c r="F391" t="n">
-        <v>6.5</v>
+        <v>12.6</v>
       </c>
       <c r="G391" t="n">
         <v>0</v>
@@ -19989,7 +19989,7 @@
         <v>0</v>
       </c>
       <c r="K391" t="n">
-        <v>0.22</v>
+        <v>0.225</v>
       </c>
       <c r="L391" t="n">
         <v>4</v>
@@ -20014,17 +20014,17 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>14.6</v>
+        <v>15.4</v>
       </c>
       <c r="E392" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F392" t="n">
-        <v>10.4</v>
+        <v>7.6</v>
       </c>
       <c r="G392" t="n">
         <v>0</v>
@@ -20033,13 +20033,13 @@
         <v>100</v>
       </c>
       <c r="I392" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="J392" t="n">
         <v>0</v>
       </c>
       <c r="K392" t="n">
-        <v>0.221</v>
+        <v>0.226</v>
       </c>
       <c r="L392" t="n">
         <v>4</v>
@@ -20064,14 +20064,14 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>14.5</v>
+        <v>15.8</v>
       </c>
       <c r="E393" t="n">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="F393" t="n">
         <v>8.300000000000001</v>
@@ -20089,7 +20089,7 @@
         <v>0</v>
       </c>
       <c r="K393" t="n">
-        <v>0.221</v>
+        <v>0.226</v>
       </c>
       <c r="L393" t="n">
         <v>4</v>
@@ -20114,20 +20114,20 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>14.6</v>
+        <v>16</v>
       </c>
       <c r="E394" t="n">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="F394" t="n">
-        <v>6.1</v>
+        <v>18.7</v>
       </c>
       <c r="G394" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H394" t="n">
         <v>100</v>
@@ -20139,7 +20139,7 @@
         <v>0</v>
       </c>
       <c r="K394" t="n">
-        <v>0.221</v>
+        <v>0.226</v>
       </c>
       <c r="L394" t="n">
         <v>4</v>
@@ -20164,32 +20164,32 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>14.9</v>
+        <v>12.9</v>
       </c>
       <c r="E395" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F395" t="n">
-        <v>19.8</v>
+        <v>22</v>
       </c>
       <c r="G395" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="H395" t="n">
         <v>100</v>
       </c>
       <c r="I395" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J395" t="n">
         <v>0</v>
       </c>
       <c r="K395" t="n">
-        <v>0.222</v>
+        <v>0.235</v>
       </c>
       <c r="L395" t="n">
         <v>4</v>
@@ -20214,32 +20214,32 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>12.9</v>
+        <v>12.2</v>
       </c>
       <c r="E396" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F396" t="n">
-        <v>22.7</v>
+        <v>15.8</v>
       </c>
       <c r="G396" t="n">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="H396" t="n">
         <v>100</v>
       </c>
       <c r="I396" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="J396" t="n">
         <v>0</v>
       </c>
       <c r="K396" t="n">
-        <v>0.224</v>
+        <v>0.24</v>
       </c>
       <c r="L396" t="n">
         <v>4</v>
@@ -20264,23 +20264,23 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>12.1</v>
+        <v>12.9</v>
       </c>
       <c r="E397" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="F397" t="n">
-        <v>11.2</v>
+        <v>16.2</v>
       </c>
       <c r="G397" t="n">
-        <v>44</v>
+        <v>142</v>
       </c>
       <c r="H397" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="I397" t="n">
         <v>0</v>
@@ -20289,7 +20289,7 @@
         <v>0</v>
       </c>
       <c r="K397" t="n">
-        <v>0.224</v>
+        <v>0.24</v>
       </c>
       <c r="L397" t="n">
         <v>4</v>
@@ -20314,23 +20314,23 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>12.8</v>
+        <v>14</v>
       </c>
       <c r="E398" t="n">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="F398" t="n">
-        <v>14.8</v>
+        <v>18</v>
       </c>
       <c r="G398" t="n">
-        <v>125</v>
+        <v>410</v>
       </c>
       <c r="H398" t="n">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="I398" t="n">
         <v>0</v>
@@ -20339,7 +20339,7 @@
         <v>0</v>
       </c>
       <c r="K398" t="n">
-        <v>0.223</v>
+        <v>0.239</v>
       </c>
       <c r="L398" t="n">
         <v>4</v>
@@ -20364,23 +20364,23 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>14.4</v>
+        <v>14.1</v>
       </c>
       <c r="E399" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F399" t="n">
-        <v>16.2</v>
+        <v>19.4</v>
       </c>
       <c r="G399" t="n">
-        <v>471</v>
+        <v>293</v>
       </c>
       <c r="H399" t="n">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="I399" t="n">
         <v>0</v>
@@ -20389,7 +20389,7 @@
         <v>0</v>
       </c>
       <c r="K399" t="n">
-        <v>0.222</v>
+        <v>0.237</v>
       </c>
       <c r="L399" t="n">
         <v>4</v>
@@ -20414,20 +20414,20 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D400" t="n">
         <v>14.6</v>
       </c>
       <c r="E400" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="F400" t="n">
-        <v>18.7</v>
+        <v>20.5</v>
       </c>
       <c r="G400" t="n">
-        <v>418</v>
+        <v>344</v>
       </c>
       <c r="H400" t="n">
         <v>100</v>
@@ -20439,7 +20439,7 @@
         <v>0</v>
       </c>
       <c r="K400" t="n">
-        <v>0.22</v>
+        <v>0.235</v>
       </c>
       <c r="L400" t="n">
         <v>4</v>
@@ -20464,23 +20464,23 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>13.9</v>
+        <v>14.7</v>
       </c>
       <c r="E401" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="F401" t="n">
-        <v>17.6</v>
+        <v>21.6</v>
       </c>
       <c r="G401" t="n">
-        <v>126</v>
+        <v>207</v>
       </c>
       <c r="H401" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I401" t="n">
         <v>0</v>
@@ -20489,7 +20489,7 @@
         <v>0</v>
       </c>
       <c r="K401" t="n">
-        <v>0.219</v>
+        <v>0.233</v>
       </c>
       <c r="L401" t="n">
         <v>4</v>
@@ -20514,23 +20514,23 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D402" t="n">
-        <v>13.9</v>
+        <v>14.5</v>
       </c>
       <c r="E402" t="n">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="F402" t="n">
-        <v>16.6</v>
+        <v>18.7</v>
       </c>
       <c r="G402" t="n">
-        <v>89</v>
+        <v>163</v>
       </c>
       <c r="H402" t="n">
-        <v>100</v>
+        <v>28</v>
       </c>
       <c r="I402" t="n">
         <v>0</v>
@@ -20539,7 +20539,7 @@
         <v>0</v>
       </c>
       <c r="K402" t="n">
-        <v>0.217</v>
+        <v>0.232</v>
       </c>
       <c r="L402" t="n">
         <v>4</v>
@@ -20564,20 +20564,20 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>13.7</v>
+        <v>14.5</v>
       </c>
       <c r="E403" t="n">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="F403" t="n">
-        <v>16.6</v>
+        <v>15.8</v>
       </c>
       <c r="G403" t="n">
-        <v>74</v>
+        <v>119</v>
       </c>
       <c r="H403" t="n">
         <v>100</v>
@@ -20589,7 +20589,7 @@
         <v>0</v>
       </c>
       <c r="K403" t="n">
-        <v>0.217</v>
+        <v>0.231</v>
       </c>
       <c r="L403" t="n">
         <v>4</v>
@@ -20614,20 +20614,20 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>13</v>
+        <v>14.4</v>
       </c>
       <c r="E404" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="F404" t="n">
-        <v>15.5</v>
+        <v>14.4</v>
       </c>
       <c r="G404" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H404" t="n">
         <v>100</v>
@@ -20639,7 +20639,7 @@
         <v>0</v>
       </c>
       <c r="K404" t="n">
-        <v>0.216</v>
+        <v>0.231</v>
       </c>
       <c r="L404" t="n">
         <v>4</v>
@@ -20664,17 +20664,17 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D405" t="n">
-        <v>12.8</v>
+        <v>14</v>
       </c>
       <c r="E405" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="F405" t="n">
-        <v>17.3</v>
+        <v>12.2</v>
       </c>
       <c r="G405" t="n">
         <v>0</v>
@@ -20714,17 +20714,17 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D406" t="n">
-        <v>12.3</v>
+        <v>13.2</v>
       </c>
       <c r="E406" t="n">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="F406" t="n">
-        <v>16.2</v>
+        <v>15.5</v>
       </c>
       <c r="G406" t="n">
         <v>0</v>
@@ -20739,7 +20739,7 @@
         <v>0</v>
       </c>
       <c r="K406" t="n">
-        <v>0.26</v>
+        <v>0.235</v>
       </c>
       <c r="L406" t="n">
         <v>4</v>
@@ -20764,17 +20764,17 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>11.7</v>
+        <v>12.2</v>
       </c>
       <c r="E407" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F407" t="n">
-        <v>16.9</v>
+        <v>17.3</v>
       </c>
       <c r="G407" t="n">
         <v>0</v>
@@ -20783,13 +20783,13 @@
         <v>100</v>
       </c>
       <c r="I407" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J407" t="n">
         <v>0</v>
       </c>
       <c r="K407" t="n">
-        <v>0.26</v>
+        <v>0.241</v>
       </c>
       <c r="L407" t="n">
         <v>4</v>
@@ -20814,17 +20814,17 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="E408" t="n">
         <v>87</v>
       </c>
       <c r="F408" t="n">
-        <v>15.8</v>
+        <v>14</v>
       </c>
       <c r="G408" t="n">
         <v>0</v>
@@ -20833,13 +20833,13 @@
         <v>97</v>
       </c>
       <c r="I408" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J408" t="n">
         <v>0</v>
       </c>
       <c r="K408" t="n">
-        <v>0.26</v>
+        <v>0.246</v>
       </c>
       <c r="L408" t="n">
         <v>4</v>
@@ -20864,23 +20864,23 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D409" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="E409" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F409" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="G409" t="n">
         <v>0</v>
       </c>
       <c r="H409" t="n">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="I409" t="n">
         <v>0</v>
@@ -20889,7 +20889,7 @@
         <v>0</v>
       </c>
       <c r="K409" t="n">
-        <v>0.26</v>
+        <v>0.246</v>
       </c>
       <c r="L409" t="n">
         <v>4</v>
@@ -20914,23 +20914,23 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D410" t="n">
-        <v>10.2</v>
+        <v>9.9</v>
       </c>
       <c r="E410" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="F410" t="n">
-        <v>11.5</v>
+        <v>9</v>
       </c>
       <c r="G410" t="n">
         <v>0</v>
       </c>
       <c r="H410" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I410" t="n">
         <v>0</v>
@@ -20939,7 +20939,7 @@
         <v>0</v>
       </c>
       <c r="K410" t="n">
-        <v>0.26</v>
+        <v>0.246</v>
       </c>
       <c r="L410" t="n">
         <v>4</v>
@@ -20964,14 +20964,14 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D411" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="E411" t="n">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F411" t="n">
         <v>9.699999999999999</v>
@@ -20989,7 +20989,7 @@
         <v>0</v>
       </c>
       <c r="K411" t="n">
-        <v>0.26</v>
+        <v>0.246</v>
       </c>
       <c r="L411" t="n">
         <v>4</v>
@@ -21014,17 +21014,17 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E412" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F412" t="n">
-        <v>9.4</v>
+        <v>10.1</v>
       </c>
       <c r="G412" t="n">
         <v>0</v>
@@ -21039,7 +21039,7 @@
         <v>0</v>
       </c>
       <c r="K412" t="n">
-        <v>0.26</v>
+        <v>0.246</v>
       </c>
       <c r="L412" t="n">
         <v>5</v>
@@ -21064,17 +21064,17 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D413" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
       <c r="E413" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F413" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="G413" t="n">
         <v>0</v>
@@ -21089,7 +21089,7 @@
         <v>0</v>
       </c>
       <c r="K413" t="n">
-        <v>0.259</v>
+        <v>0.246</v>
       </c>
       <c r="L413" t="n">
         <v>5</v>
@@ -21114,17 +21114,17 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D414" t="n">
         <v>6.9</v>
       </c>
       <c r="E414" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F414" t="n">
-        <v>10.1</v>
+        <v>7.9</v>
       </c>
       <c r="G414" t="n">
         <v>0</v>
@@ -21139,7 +21139,7 @@
         <v>0</v>
       </c>
       <c r="K414" t="n">
-        <v>0.259</v>
+        <v>0.246</v>
       </c>
       <c r="L414" t="n">
         <v>5</v>
@@ -21164,7 +21164,7 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D415" t="n">
@@ -21189,7 +21189,7 @@
         <v>0</v>
       </c>
       <c r="K415" t="n">
-        <v>0.259</v>
+        <v>0.246</v>
       </c>
       <c r="L415" t="n">
         <v>5</v>
@@ -21214,23 +21214,23 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D416" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
       <c r="E416" t="n">
         <v>99</v>
       </c>
       <c r="F416" t="n">
-        <v>8.6</v>
+        <v>9.4</v>
       </c>
       <c r="G416" t="n">
         <v>0</v>
       </c>
       <c r="H416" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I416" t="n">
         <v>0</v>
@@ -21239,7 +21239,7 @@
         <v>0</v>
       </c>
       <c r="K416" t="n">
-        <v>0.259</v>
+        <v>0.246</v>
       </c>
       <c r="L416" t="n">
         <v>5</v>
@@ -21264,23 +21264,23 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="E417" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F417" t="n">
-        <v>8.300000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="G417" t="n">
         <v>0</v>
       </c>
       <c r="H417" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I417" t="n">
         <v>0</v>
@@ -21289,7 +21289,7 @@
         <v>0</v>
       </c>
       <c r="K417" t="n">
-        <v>0.259</v>
+        <v>0.246</v>
       </c>
       <c r="L417" t="n">
         <v>5</v>
@@ -21314,23 +21314,23 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="E418" t="n">
         <v>100</v>
       </c>
       <c r="F418" t="n">
-        <v>9</v>
+        <v>7.9</v>
       </c>
       <c r="G418" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H418" t="n">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="I418" t="n">
         <v>0</v>
@@ -21339,7 +21339,7 @@
         <v>0</v>
       </c>
       <c r="K418" t="n">
-        <v>0.258</v>
+        <v>0.246</v>
       </c>
       <c r="L418" t="n">
         <v>5</v>
@@ -21364,23 +21364,23 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="E419" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F419" t="n">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="G419" t="n">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="H419" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I419" t="n">
         <v>0</v>
@@ -21389,7 +21389,7 @@
         <v>0</v>
       </c>
       <c r="K419" t="n">
-        <v>0.258</v>
+        <v>0.245</v>
       </c>
       <c r="L419" t="n">
         <v>5</v>
@@ -21414,17 +21414,17 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D420" t="n">
         <v>10.5</v>
       </c>
       <c r="E420" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F420" t="n">
-        <v>11.2</v>
+        <v>6.1</v>
       </c>
       <c r="G420" t="n">
         <v>328</v>
@@ -21439,7 +21439,7 @@
         <v>0</v>
       </c>
       <c r="K420" t="n">
-        <v>0.257</v>
+        <v>0.245</v>
       </c>
       <c r="L420" t="n">
         <v>5</v>
@@ -21464,23 +21464,23 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D421" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
       <c r="E421" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F421" t="n">
-        <v>10.5</v>
+        <v>7.2</v>
       </c>
       <c r="G421" t="n">
-        <v>447.8</v>
+        <v>450</v>
       </c>
       <c r="H421" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I421" t="n">
         <v>0</v>
@@ -21489,7 +21489,7 @@
         <v>0</v>
       </c>
       <c r="K421" t="n">
-        <v>0.256</v>
+        <v>0.243</v>
       </c>
       <c r="L421" t="n">
         <v>5</v>
@@ -21514,20 +21514,20 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D422" t="n">
-        <v>14.1</v>
+        <v>14.4</v>
       </c>
       <c r="E422" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F422" t="n">
-        <v>8.800000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="G422" t="n">
-        <v>521.5</v>
+        <v>527</v>
       </c>
       <c r="H422" t="n">
         <v>0</v>
@@ -21539,7 +21539,7 @@
         <v>0</v>
       </c>
       <c r="K422" t="n">
-        <v>0.254</v>
+        <v>0.242</v>
       </c>
       <c r="L422" t="n">
         <v>5</v>
@@ -21564,20 +21564,20 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D423" t="n">
-        <v>14.9</v>
+        <v>15.2</v>
       </c>
       <c r="E423" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F423" t="n">
-        <v>6.4</v>
+        <v>5</v>
       </c>
       <c r="G423" t="n">
-        <v>543.3</v>
+        <v>551</v>
       </c>
       <c r="H423" t="n">
         <v>0</v>
@@ -21589,7 +21589,7 @@
         <v>0</v>
       </c>
       <c r="K423" t="n">
-        <v>0.252</v>
+        <v>0.24</v>
       </c>
       <c r="L423" t="n">
         <v>5</v>
@@ -21614,20 +21614,20 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D424" t="n">
-        <v>15.3</v>
+        <v>15.7</v>
       </c>
       <c r="E424" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="F424" t="n">
-        <v>4.7</v>
+        <v>2.5</v>
       </c>
       <c r="G424" t="n">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="H424" t="n">
         <v>0</v>
@@ -21639,7 +21639,7 @@
         <v>0</v>
       </c>
       <c r="K424" t="n">
-        <v>0.25</v>
+        <v>0.239</v>
       </c>
       <c r="L424" t="n">
         <v>5</v>
@@ -21664,20 +21664,20 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D425" t="n">
-        <v>15.4</v>
+        <v>16.1</v>
       </c>
       <c r="E425" t="n">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="F425" t="n">
-        <v>4.5</v>
+        <v>1.4</v>
       </c>
       <c r="G425" t="n">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="H425" t="n">
         <v>0</v>
@@ -21689,7 +21689,7 @@
         <v>0</v>
       </c>
       <c r="K425" t="n">
-        <v>0.249</v>
+        <v>0.237</v>
       </c>
       <c r="L425" t="n">
         <v>5</v>
@@ -21714,20 +21714,20 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D426" t="n">
-        <v>15.1</v>
+        <v>16.4</v>
       </c>
       <c r="E426" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="F426" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="G426" t="n">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="H426" t="n">
         <v>0</v>
@@ -21739,7 +21739,7 @@
         <v>0</v>
       </c>
       <c r="K426" t="n">
-        <v>0.247</v>
+        <v>0.236</v>
       </c>
       <c r="L426" t="n">
         <v>5</v>
@@ -21764,23 +21764,23 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D427" t="n">
-        <v>13.8</v>
+        <v>15.7</v>
       </c>
       <c r="E427" t="n">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="F427" t="n">
-        <v>3.2</v>
+        <v>5.2</v>
       </c>
       <c r="G427" t="n">
-        <v>144</v>
+        <v>148.5</v>
       </c>
       <c r="H427" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I427" t="n">
         <v>0</v>
@@ -21789,7 +21789,7 @@
         <v>0</v>
       </c>
       <c r="K427" t="n">
-        <v>0.247</v>
+        <v>0.235</v>
       </c>
       <c r="L427" t="n">
         <v>5</v>
@@ -21814,23 +21814,23 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D428" t="n">
-        <v>11.4</v>
+        <v>13.2</v>
       </c>
       <c r="E428" t="n">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="F428" t="n">
-        <v>5.2</v>
+        <v>5.8</v>
       </c>
       <c r="G428" t="n">
         <v>19</v>
       </c>
       <c r="H428" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="I428" t="n">
         <v>0</v>
@@ -21839,7 +21839,7 @@
         <v>0</v>
       </c>
       <c r="K428" t="n">
-        <v>0.246</v>
+        <v>0.235</v>
       </c>
       <c r="L428" t="n">
         <v>5</v>
@@ -21864,23 +21864,23 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>10.4</v>
+        <v>11.7</v>
       </c>
       <c r="E429" t="n">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="F429" t="n">
-        <v>4.3</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G429" t="n">
         <v>0</v>
       </c>
       <c r="H429" t="n">
-        <v>2</v>
+        <v>85</v>
       </c>
       <c r="I429" t="n">
         <v>0</v>
@@ -21889,7 +21889,7 @@
         <v>0</v>
       </c>
       <c r="K429" t="n">
-        <v>0.246</v>
+        <v>0.235</v>
       </c>
       <c r="L429" t="n">
         <v>5</v>
@@ -21914,23 +21914,23 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>10.1</v>
+        <v>11.1</v>
       </c>
       <c r="E430" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F430" t="n">
-        <v>5.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G430" t="n">
         <v>0</v>
       </c>
       <c r="H430" t="n">
-        <v>2</v>
+        <v>84</v>
       </c>
       <c r="I430" t="n">
         <v>0</v>
@@ -21939,7 +21939,7 @@
         <v>0</v>
       </c>
       <c r="K430" t="n">
-        <v>0.246</v>
+        <v>0.235</v>
       </c>
       <c r="L430" t="n">
         <v>5</v>
@@ -21964,23 +21964,23 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>9.6</v>
+        <v>10.9</v>
       </c>
       <c r="E431" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="F431" t="n">
-        <v>6.3</v>
+        <v>10.2</v>
       </c>
       <c r="G431" t="n">
         <v>0</v>
       </c>
       <c r="H431" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I431" t="n">
         <v>0</v>
@@ -21989,7 +21989,7 @@
         <v>0</v>
       </c>
       <c r="K431" t="n">
-        <v>0.246</v>
+        <v>0.235</v>
       </c>
       <c r="L431" t="n">
         <v>5</v>
@@ -22014,23 +22014,23 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E432" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F432" t="n">
-        <v>7</v>
+        <v>10.3</v>
       </c>
       <c r="G432" t="n">
         <v>0</v>
       </c>
       <c r="H432" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I432" t="n">
         <v>0</v>
@@ -22039,7 +22039,7 @@
         <v>0</v>
       </c>
       <c r="K432" t="n">
-        <v>0.246</v>
+        <v>0.235</v>
       </c>
       <c r="L432" t="n">
         <v>5</v>
@@ -22064,23 +22064,23 @@
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D433" t="n">
-        <v>8.9</v>
+        <v>9.4</v>
       </c>
       <c r="E433" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F433" t="n">
-        <v>8</v>
+        <v>11.1</v>
       </c>
       <c r="G433" t="n">
         <v>0</v>
       </c>
       <c r="H433" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I433" t="n">
         <v>0</v>
@@ -22089,7 +22089,7 @@
         <v>0</v>
       </c>
       <c r="K433" t="n">
-        <v>0.246</v>
+        <v>0.234</v>
       </c>
       <c r="L433" t="n">
         <v>5</v>
@@ -22114,23 +22114,23 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D434" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="E434" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F434" t="n">
-        <v>8.699999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="G434" t="n">
         <v>0</v>
       </c>
       <c r="H434" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="I434" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>0</v>
       </c>
       <c r="K434" t="n">
-        <v>0.246</v>
+        <v>0.234</v>
       </c>
       <c r="L434" t="n">
         <v>5</v>
@@ -22164,23 +22164,23 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>2026-10-21T05:03:45Z</t>
+          <t>2026-10-21T11:03:31Z</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="E435" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F435" t="n">
-        <v>9.5</v>
+        <v>9.9</v>
       </c>
       <c r="G435" t="n">
         <v>0</v>
       </c>
       <c r="H435" t="n">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="I435" t="n">
         <v>0</v>
@@ -22189,7 +22189,7 @@
         <v>0</v>
       </c>
       <c r="K435" t="n">
-        <v>0.246</v>
+        <v>0.234</v>
       </c>
       <c r="L435" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
prognoza biciklista (osvezavanje): 2026-10-21 19:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -19564,23 +19564,23 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>17.3</v>
+        <v>18</v>
       </c>
       <c r="E383" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F383" t="n">
-        <v>27.4</v>
+        <v>20.9</v>
       </c>
       <c r="G383" t="n">
         <v>0</v>
       </c>
       <c r="H383" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="I383" t="n">
         <v>0</v>
@@ -19589,7 +19589,7 @@
         <v>0</v>
       </c>
       <c r="K383" t="n">
-        <v>0.205</v>
+        <v>0.212</v>
       </c>
       <c r="L383" t="n">
         <v>3</v>
@@ -19614,23 +19614,23 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>17.1</v>
+        <v>16.8</v>
       </c>
       <c r="E384" t="n">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F384" t="n">
-        <v>23.4</v>
+        <v>15.1</v>
       </c>
       <c r="G384" t="n">
         <v>0</v>
       </c>
       <c r="H384" t="n">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="I384" t="n">
         <v>0</v>
@@ -19639,7 +19639,7 @@
         <v>0</v>
       </c>
       <c r="K384" t="n">
-        <v>0.207</v>
+        <v>0.211</v>
       </c>
       <c r="L384" t="n">
         <v>3</v>
@@ -19664,23 +19664,23 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="E385" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F385" t="n">
-        <v>20.9</v>
+        <v>17.3</v>
       </c>
       <c r="G385" t="n">
         <v>0</v>
       </c>
       <c r="H385" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I385" t="n">
         <v>0</v>
@@ -19689,7 +19689,7 @@
         <v>0</v>
       </c>
       <c r="K385" t="n">
-        <v>0.209</v>
+        <v>0.211</v>
       </c>
       <c r="L385" t="n">
         <v>3</v>
@@ -19714,23 +19714,23 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D386" t="n">
         <v>16.4</v>
       </c>
       <c r="E386" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F386" t="n">
-        <v>22</v>
+        <v>15.1</v>
       </c>
       <c r="G386" t="n">
         <v>0</v>
       </c>
       <c r="H386" t="n">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="I386" t="n">
         <v>0</v>
@@ -19739,7 +19739,7 @@
         <v>0</v>
       </c>
       <c r="K386" t="n">
-        <v>0.211</v>
+        <v>0.212</v>
       </c>
       <c r="L386" t="n">
         <v>3</v>
@@ -19764,23 +19764,23 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>16.3</v>
+        <v>15.9</v>
       </c>
       <c r="E387" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F387" t="n">
-        <v>18.7</v>
+        <v>16.6</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
       </c>
       <c r="H387" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I387" t="n">
         <v>0</v>
@@ -19789,7 +19789,7 @@
         <v>0</v>
       </c>
       <c r="K387" t="n">
-        <v>0.214</v>
+        <v>0.222</v>
       </c>
       <c r="L387" t="n">
         <v>3</v>
@@ -19814,32 +19814,32 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>16.4</v>
+        <v>15.4</v>
       </c>
       <c r="E388" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F388" t="n">
-        <v>18</v>
+        <v>16.9</v>
       </c>
       <c r="G388" t="n">
         <v>0</v>
       </c>
       <c r="H388" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="I388" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J388" t="n">
         <v>0</v>
       </c>
       <c r="K388" t="n">
-        <v>0.216</v>
+        <v>0.223</v>
       </c>
       <c r="L388" t="n">
         <v>4</v>
@@ -19864,17 +19864,17 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>16.1</v>
+        <v>15</v>
       </c>
       <c r="E389" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F389" t="n">
-        <v>17.3</v>
+        <v>15.5</v>
       </c>
       <c r="G389" t="n">
         <v>0</v>
@@ -19889,7 +19889,7 @@
         <v>0</v>
       </c>
       <c r="K389" t="n">
-        <v>0.219</v>
+        <v>0.223</v>
       </c>
       <c r="L389" t="n">
         <v>4</v>
@@ -19914,17 +19914,17 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>15.6</v>
+        <v>15.3</v>
       </c>
       <c r="E390" t="n">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="F390" t="n">
-        <v>14.4</v>
+        <v>12.6</v>
       </c>
       <c r="G390" t="n">
         <v>0</v>
@@ -19933,13 +19933,13 @@
         <v>100</v>
       </c>
       <c r="I390" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="J390" t="n">
         <v>0</v>
       </c>
       <c r="K390" t="n">
-        <v>0.223</v>
+        <v>0.224</v>
       </c>
       <c r="L390" t="n">
         <v>4</v>
@@ -19964,17 +19964,17 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>15.3</v>
+        <v>15.6</v>
       </c>
       <c r="E391" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="F391" t="n">
-        <v>12.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G391" t="n">
         <v>0</v>
@@ -20014,17 +20014,17 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>15.4</v>
+        <v>16</v>
       </c>
       <c r="E392" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="F392" t="n">
-        <v>7.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G392" t="n">
         <v>0</v>
@@ -20039,7 +20039,7 @@
         <v>0</v>
       </c>
       <c r="K392" t="n">
-        <v>0.226</v>
+        <v>0.23</v>
       </c>
       <c r="L392" t="n">
         <v>4</v>
@@ -20064,17 +20064,17 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>15.8</v>
+        <v>16.5</v>
       </c>
       <c r="E393" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F393" t="n">
-        <v>8.300000000000001</v>
+        <v>11.5</v>
       </c>
       <c r="G393" t="n">
         <v>0</v>
@@ -20089,7 +20089,7 @@
         <v>0</v>
       </c>
       <c r="K393" t="n">
-        <v>0.226</v>
+        <v>0.233</v>
       </c>
       <c r="L393" t="n">
         <v>4</v>
@@ -20114,20 +20114,20 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>16</v>
+        <v>16.7</v>
       </c>
       <c r="E394" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F394" t="n">
-        <v>18.7</v>
+        <v>13.7</v>
       </c>
       <c r="G394" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H394" t="n">
         <v>100</v>
@@ -20139,7 +20139,7 @@
         <v>0</v>
       </c>
       <c r="K394" t="n">
-        <v>0.226</v>
+        <v>0.259</v>
       </c>
       <c r="L394" t="n">
         <v>4</v>
@@ -20164,32 +20164,32 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>12.9</v>
+        <v>13.7</v>
       </c>
       <c r="E395" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F395" t="n">
-        <v>22</v>
+        <v>23.8</v>
       </c>
       <c r="G395" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H395" t="n">
         <v>100</v>
       </c>
       <c r="I395" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="J395" t="n">
         <v>0</v>
       </c>
       <c r="K395" t="n">
-        <v>0.235</v>
+        <v>0.259</v>
       </c>
       <c r="L395" t="n">
         <v>4</v>
@@ -20214,32 +20214,32 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>12.2</v>
+        <v>12.8</v>
       </c>
       <c r="E396" t="n">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="F396" t="n">
-        <v>15.8</v>
+        <v>19.1</v>
       </c>
       <c r="G396" t="n">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="H396" t="n">
         <v>100</v>
       </c>
       <c r="I396" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J396" t="n">
         <v>0</v>
       </c>
       <c r="K396" t="n">
-        <v>0.24</v>
+        <v>0.259</v>
       </c>
       <c r="L396" t="n">
         <v>4</v>
@@ -20264,23 +20264,23 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>12.9</v>
+        <v>13.3</v>
       </c>
       <c r="E397" t="n">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="F397" t="n">
-        <v>16.2</v>
+        <v>16.6</v>
       </c>
       <c r="G397" t="n">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="H397" t="n">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="I397" t="n">
         <v>0</v>
@@ -20289,7 +20289,7 @@
         <v>0</v>
       </c>
       <c r="K397" t="n">
-        <v>0.24</v>
+        <v>0.258</v>
       </c>
       <c r="L397" t="n">
         <v>4</v>
@@ -20314,23 +20314,23 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>14</v>
+        <v>14.5</v>
       </c>
       <c r="E398" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F398" t="n">
-        <v>18</v>
+        <v>17.3</v>
       </c>
       <c r="G398" t="n">
-        <v>410</v>
+        <v>290</v>
       </c>
       <c r="H398" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="I398" t="n">
         <v>0</v>
@@ -20339,7 +20339,7 @@
         <v>0</v>
       </c>
       <c r="K398" t="n">
-        <v>0.239</v>
+        <v>0.256</v>
       </c>
       <c r="L398" t="n">
         <v>4</v>
@@ -20364,23 +20364,23 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>14.1</v>
+        <v>15.6</v>
       </c>
       <c r="E399" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="F399" t="n">
-        <v>19.4</v>
+        <v>19.1</v>
       </c>
       <c r="G399" t="n">
-        <v>293</v>
+        <v>400</v>
       </c>
       <c r="H399" t="n">
-        <v>31</v>
+        <v>100</v>
       </c>
       <c r="I399" t="n">
         <v>0</v>
@@ -20389,7 +20389,7 @@
         <v>0</v>
       </c>
       <c r="K399" t="n">
-        <v>0.237</v>
+        <v>0.254</v>
       </c>
       <c r="L399" t="n">
         <v>4</v>
@@ -20414,20 +20414,20 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>14.6</v>
+        <v>15.3</v>
       </c>
       <c r="E400" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F400" t="n">
-        <v>20.5</v>
+        <v>20.2</v>
       </c>
       <c r="G400" t="n">
-        <v>344</v>
+        <v>141</v>
       </c>
       <c r="H400" t="n">
         <v>100</v>
@@ -20439,7 +20439,7 @@
         <v>0</v>
       </c>
       <c r="K400" t="n">
-        <v>0.235</v>
+        <v>0.252</v>
       </c>
       <c r="L400" t="n">
         <v>4</v>
@@ -20464,23 +20464,23 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="E401" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F401" t="n">
-        <v>21.6</v>
+        <v>21.2</v>
       </c>
       <c r="G401" t="n">
-        <v>207</v>
+        <v>91</v>
       </c>
       <c r="H401" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I401" t="n">
         <v>0</v>
@@ -20489,7 +20489,7 @@
         <v>0</v>
       </c>
       <c r="K401" t="n">
-        <v>0.233</v>
+        <v>0.25</v>
       </c>
       <c r="L401" t="n">
         <v>4</v>
@@ -20514,23 +20514,23 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D402" t="n">
         <v>14.5</v>
       </c>
       <c r="E402" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F402" t="n">
-        <v>18.7</v>
+        <v>19.4</v>
       </c>
       <c r="G402" t="n">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="H402" t="n">
-        <v>28</v>
+        <v>100</v>
       </c>
       <c r="I402" t="n">
         <v>0</v>
@@ -20539,7 +20539,7 @@
         <v>0</v>
       </c>
       <c r="K402" t="n">
-        <v>0.232</v>
+        <v>0.249</v>
       </c>
       <c r="L402" t="n">
         <v>4</v>
@@ -20564,20 +20564,20 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>14.5</v>
+        <v>14.1</v>
       </c>
       <c r="E403" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F403" t="n">
-        <v>15.8</v>
+        <v>16.6</v>
       </c>
       <c r="G403" t="n">
-        <v>119</v>
+        <v>48</v>
       </c>
       <c r="H403" t="n">
         <v>100</v>
@@ -20589,7 +20589,7 @@
         <v>0</v>
       </c>
       <c r="K403" t="n">
-        <v>0.231</v>
+        <v>0.248</v>
       </c>
       <c r="L403" t="n">
         <v>4</v>
@@ -20614,20 +20614,20 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>14.4</v>
+        <v>13.5</v>
       </c>
       <c r="E404" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="F404" t="n">
-        <v>14.4</v>
+        <v>15.5</v>
       </c>
       <c r="G404" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H404" t="n">
         <v>100</v>
@@ -20639,7 +20639,7 @@
         <v>0</v>
       </c>
       <c r="K404" t="n">
-        <v>0.231</v>
+        <v>0.249</v>
       </c>
       <c r="L404" t="n">
         <v>4</v>
@@ -20664,17 +20664,17 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D405" t="n">
-        <v>14</v>
+        <v>12.6</v>
       </c>
       <c r="E405" t="n">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="F405" t="n">
-        <v>12.2</v>
+        <v>16.9</v>
       </c>
       <c r="G405" t="n">
         <v>0</v>
@@ -20689,7 +20689,7 @@
         <v>0</v>
       </c>
       <c r="K405" t="n">
-        <v>0.232</v>
+        <v>0.248</v>
       </c>
       <c r="L405" t="n">
         <v>4</v>
@@ -20714,17 +20714,17 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D406" t="n">
-        <v>13.2</v>
+        <v>12</v>
       </c>
       <c r="E406" t="n">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="F406" t="n">
-        <v>15.5</v>
+        <v>16.2</v>
       </c>
       <c r="G406" t="n">
         <v>0</v>
@@ -20733,13 +20733,13 @@
         <v>100</v>
       </c>
       <c r="I406" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J406" t="n">
         <v>0</v>
       </c>
       <c r="K406" t="n">
-        <v>0.235</v>
+        <v>0.249</v>
       </c>
       <c r="L406" t="n">
         <v>4</v>
@@ -20764,17 +20764,17 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>12.2</v>
+        <v>11.8</v>
       </c>
       <c r="E407" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F407" t="n">
-        <v>17.3</v>
+        <v>15.8</v>
       </c>
       <c r="G407" t="n">
         <v>0</v>
@@ -20789,7 +20789,7 @@
         <v>0</v>
       </c>
       <c r="K407" t="n">
-        <v>0.241</v>
+        <v>0.256</v>
       </c>
       <c r="L407" t="n">
         <v>4</v>
@@ -20814,23 +20814,23 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D408" t="n">
         <v>11.5</v>
       </c>
       <c r="E408" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F408" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G408" t="n">
         <v>0</v>
       </c>
       <c r="H408" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I408" t="n">
         <v>0</v>
@@ -20839,7 +20839,7 @@
         <v>0</v>
       </c>
       <c r="K408" t="n">
-        <v>0.246</v>
+        <v>0.257</v>
       </c>
       <c r="L408" t="n">
         <v>4</v>
@@ -20864,23 +20864,23 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D409" t="n">
         <v>10.9</v>
       </c>
       <c r="E409" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F409" t="n">
-        <v>11.5</v>
+        <v>10.8</v>
       </c>
       <c r="G409" t="n">
         <v>0</v>
       </c>
       <c r="H409" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="I409" t="n">
         <v>0</v>
@@ -20889,7 +20889,7 @@
         <v>0</v>
       </c>
       <c r="K409" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L409" t="n">
         <v>4</v>
@@ -20914,17 +20914,17 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D410" t="n">
-        <v>9.9</v>
+        <v>10</v>
       </c>
       <c r="E410" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F410" t="n">
-        <v>9</v>
+        <v>10.1</v>
       </c>
       <c r="G410" t="n">
         <v>0</v>
@@ -20939,7 +20939,7 @@
         <v>0</v>
       </c>
       <c r="K410" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L410" t="n">
         <v>4</v>
@@ -20964,17 +20964,17 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D411" t="n">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="E411" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F411" t="n">
-        <v>9.699999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="G411" t="n">
         <v>0</v>
@@ -20989,7 +20989,7 @@
         <v>0</v>
       </c>
       <c r="K411" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L411" t="n">
         <v>4</v>
@@ -21014,17 +21014,17 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="E412" t="n">
         <v>97</v>
       </c>
       <c r="F412" t="n">
-        <v>10.1</v>
+        <v>9.4</v>
       </c>
       <c r="G412" t="n">
         <v>0</v>
@@ -21039,7 +21039,7 @@
         <v>0</v>
       </c>
       <c r="K412" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L412" t="n">
         <v>5</v>
@@ -21064,17 +21064,17 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D413" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="E413" t="n">
         <v>98</v>
       </c>
       <c r="F413" t="n">
-        <v>9.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G413" t="n">
         <v>0</v>
@@ -21089,7 +21089,7 @@
         <v>0</v>
       </c>
       <c r="K413" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L413" t="n">
         <v>5</v>
@@ -21114,17 +21114,17 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="E414" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F414" t="n">
-        <v>7.9</v>
+        <v>6.8</v>
       </c>
       <c r="G414" t="n">
         <v>0</v>
@@ -21139,7 +21139,7 @@
         <v>0</v>
       </c>
       <c r="K414" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L414" t="n">
         <v>5</v>
@@ -21164,17 +21164,17 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D415" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="E415" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F415" t="n">
-        <v>7.9</v>
+        <v>7.2</v>
       </c>
       <c r="G415" t="n">
         <v>0</v>
@@ -21189,7 +21189,7 @@
         <v>0</v>
       </c>
       <c r="K415" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L415" t="n">
         <v>5</v>
@@ -21214,7 +21214,7 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D416" t="n">
@@ -21224,13 +21224,13 @@
         <v>99</v>
       </c>
       <c r="F416" t="n">
-        <v>9.4</v>
+        <v>7.6</v>
       </c>
       <c r="G416" t="n">
         <v>0</v>
       </c>
       <c r="H416" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I416" t="n">
         <v>0</v>
@@ -21239,7 +21239,7 @@
         <v>0</v>
       </c>
       <c r="K416" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L416" t="n">
         <v>5</v>
@@ -21264,23 +21264,23 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="E417" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F417" t="n">
-        <v>7.6</v>
+        <v>6.5</v>
       </c>
       <c r="G417" t="n">
         <v>0</v>
       </c>
       <c r="H417" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I417" t="n">
         <v>0</v>
@@ -21289,7 +21289,7 @@
         <v>0</v>
       </c>
       <c r="K417" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L417" t="n">
         <v>5</v>
@@ -21314,23 +21314,23 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="E418" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F418" t="n">
-        <v>7.9</v>
+        <v>6.1</v>
       </c>
       <c r="G418" t="n">
         <v>37</v>
       </c>
       <c r="H418" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I418" t="n">
         <v>0</v>
@@ -21339,7 +21339,7 @@
         <v>0</v>
       </c>
       <c r="K418" t="n">
-        <v>0.246</v>
+        <v>0.256</v>
       </c>
       <c r="L418" t="n">
         <v>5</v>
@@ -21364,23 +21364,23 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>7.3</v>
+        <v>8.1</v>
       </c>
       <c r="E419" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="F419" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="G419" t="n">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="H419" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I419" t="n">
         <v>0</v>
@@ -21389,7 +21389,7 @@
         <v>0</v>
       </c>
       <c r="K419" t="n">
-        <v>0.245</v>
+        <v>0.256</v>
       </c>
       <c r="L419" t="n">
         <v>5</v>
@@ -21414,20 +21414,20 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>10.5</v>
+        <v>10.6</v>
       </c>
       <c r="E420" t="n">
         <v>76</v>
       </c>
       <c r="F420" t="n">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
       <c r="G420" t="n">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H420" t="n">
         <v>0</v>
@@ -21439,7 +21439,7 @@
         <v>0</v>
       </c>
       <c r="K420" t="n">
-        <v>0.245</v>
+        <v>0.255</v>
       </c>
       <c r="L420" t="n">
         <v>5</v>
@@ -21464,20 +21464,20 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D421" t="n">
-        <v>12.9</v>
+        <v>12.3</v>
       </c>
       <c r="E421" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="F421" t="n">
-        <v>7.2</v>
+        <v>4.3</v>
       </c>
       <c r="G421" t="n">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H421" t="n">
         <v>0</v>
@@ -21489,7 +21489,7 @@
         <v>0</v>
       </c>
       <c r="K421" t="n">
-        <v>0.243</v>
+        <v>0.254</v>
       </c>
       <c r="L421" t="n">
         <v>5</v>
@@ -21514,20 +21514,20 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D422" t="n">
-        <v>14.4</v>
+        <v>13.3</v>
       </c>
       <c r="E422" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F422" t="n">
-        <v>7.9</v>
+        <v>2.2</v>
       </c>
       <c r="G422" t="n">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="H422" t="n">
         <v>0</v>
@@ -21539,7 +21539,7 @@
         <v>0</v>
       </c>
       <c r="K422" t="n">
-        <v>0.242</v>
+        <v>0.252</v>
       </c>
       <c r="L422" t="n">
         <v>5</v>
@@ -21564,20 +21564,20 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D423" t="n">
-        <v>15.2</v>
+        <v>14.1</v>
       </c>
       <c r="E423" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F423" t="n">
-        <v>5</v>
+        <v>1.4</v>
       </c>
       <c r="G423" t="n">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="H423" t="n">
         <v>0</v>
@@ -21589,7 +21589,7 @@
         <v>0</v>
       </c>
       <c r="K423" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="L423" t="n">
         <v>5</v>
@@ -21614,20 +21614,20 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D424" t="n">
-        <v>15.7</v>
+        <v>15.2</v>
       </c>
       <c r="E424" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="F424" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
       <c r="G424" t="n">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="H424" t="n">
         <v>0</v>
@@ -21639,7 +21639,7 @@
         <v>0</v>
       </c>
       <c r="K424" t="n">
-        <v>0.239</v>
+        <v>0.248</v>
       </c>
       <c r="L424" t="n">
         <v>5</v>
@@ -21664,20 +21664,20 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D425" t="n">
-        <v>16.1</v>
+        <v>16.2</v>
       </c>
       <c r="E425" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F425" t="n">
-        <v>1.4</v>
+        <v>5.8</v>
       </c>
       <c r="G425" t="n">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="H425" t="n">
         <v>0</v>
@@ -21689,7 +21689,7 @@
         <v>0</v>
       </c>
       <c r="K425" t="n">
-        <v>0.237</v>
+        <v>0.246</v>
       </c>
       <c r="L425" t="n">
         <v>5</v>
@@ -21714,23 +21714,23 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D426" t="n">
         <v>16.4</v>
       </c>
       <c r="E426" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F426" t="n">
-        <v>2.5</v>
+        <v>9</v>
       </c>
       <c r="G426" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H426" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I426" t="n">
         <v>0</v>
@@ -21739,7 +21739,7 @@
         <v>0</v>
       </c>
       <c r="K426" t="n">
-        <v>0.236</v>
+        <v>0.245</v>
       </c>
       <c r="L426" t="n">
         <v>5</v>
@@ -21764,23 +21764,23 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D427" t="n">
-        <v>15.7</v>
+        <v>15.9</v>
       </c>
       <c r="E427" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F427" t="n">
-        <v>5.2</v>
+        <v>9</v>
       </c>
       <c r="G427" t="n">
-        <v>148.5</v>
+        <v>137</v>
       </c>
       <c r="H427" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="I427" t="n">
         <v>0</v>
@@ -21789,7 +21789,7 @@
         <v>0</v>
       </c>
       <c r="K427" t="n">
-        <v>0.235</v>
+        <v>0.244</v>
       </c>
       <c r="L427" t="n">
         <v>5</v>
@@ -21814,23 +21814,23 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D428" t="n">
-        <v>13.2</v>
+        <v>14.7</v>
       </c>
       <c r="E428" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F428" t="n">
-        <v>5.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G428" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H428" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="I428" t="n">
         <v>0</v>
@@ -21839,7 +21839,7 @@
         <v>0</v>
       </c>
       <c r="K428" t="n">
-        <v>0.235</v>
+        <v>0.244</v>
       </c>
       <c r="L428" t="n">
         <v>5</v>
@@ -21864,23 +21864,23 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>11.7</v>
+        <v>12.9</v>
       </c>
       <c r="E429" t="n">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="F429" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="G429" t="n">
         <v>0</v>
       </c>
       <c r="H429" t="n">
-        <v>85</v>
+        <v>8</v>
       </c>
       <c r="I429" t="n">
         <v>0</v>
@@ -21889,7 +21889,7 @@
         <v>0</v>
       </c>
       <c r="K429" t="n">
-        <v>0.235</v>
+        <v>0.244</v>
       </c>
       <c r="L429" t="n">
         <v>5</v>
@@ -21914,23 +21914,23 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="E430" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="F430" t="n">
-        <v>9.300000000000001</v>
+        <v>10.8</v>
       </c>
       <c r="G430" t="n">
         <v>0</v>
       </c>
       <c r="H430" t="n">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="I430" t="n">
         <v>0</v>
@@ -21939,7 +21939,7 @@
         <v>0</v>
       </c>
       <c r="K430" t="n">
-        <v>0.235</v>
+        <v>0.244</v>
       </c>
       <c r="L430" t="n">
         <v>5</v>
@@ -21964,23 +21964,23 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>10.9</v>
+        <v>10</v>
       </c>
       <c r="E431" t="n">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="F431" t="n">
-        <v>10.2</v>
+        <v>11.9</v>
       </c>
       <c r="G431" t="n">
         <v>0</v>
       </c>
       <c r="H431" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I431" t="n">
         <v>0</v>
@@ -21989,7 +21989,7 @@
         <v>0</v>
       </c>
       <c r="K431" t="n">
-        <v>0.235</v>
+        <v>0.244</v>
       </c>
       <c r="L431" t="n">
         <v>5</v>
@@ -22014,17 +22014,17 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>9.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E432" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F432" t="n">
-        <v>10.3</v>
+        <v>13</v>
       </c>
       <c r="G432" t="n">
         <v>0</v>
@@ -22039,7 +22039,7 @@
         <v>0</v>
       </c>
       <c r="K432" t="n">
-        <v>0.235</v>
+        <v>0.243</v>
       </c>
       <c r="L432" t="n">
         <v>5</v>
@@ -22064,23 +22064,23 @@
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D433" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="E433" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="F433" t="n">
-        <v>11.1</v>
+        <v>12.6</v>
       </c>
       <c r="G433" t="n">
         <v>0</v>
       </c>
       <c r="H433" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="I433" t="n">
         <v>0</v>
@@ -22089,7 +22089,7 @@
         <v>0</v>
       </c>
       <c r="K433" t="n">
-        <v>0.234</v>
+        <v>0.243</v>
       </c>
       <c r="L433" t="n">
         <v>5</v>
@@ -22114,23 +22114,23 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D434" t="n">
-        <v>9</v>
+        <v>7.8</v>
       </c>
       <c r="E434" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="F434" t="n">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="G434" t="n">
         <v>0</v>
       </c>
       <c r="H434" t="n">
-        <v>7</v>
+        <v>72</v>
       </c>
       <c r="I434" t="n">
         <v>0</v>
@@ -22139,7 +22139,7 @@
         <v>0</v>
       </c>
       <c r="K434" t="n">
-        <v>0.234</v>
+        <v>0.243</v>
       </c>
       <c r="L434" t="n">
         <v>5</v>
@@ -22164,23 +22164,23 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>2026-10-21T11:03:31Z</t>
+          <t>2026-10-21T17:03:41Z</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>8.5</v>
+        <v>7.1</v>
       </c>
       <c r="E435" t="n">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F435" t="n">
-        <v>9.9</v>
+        <v>11.2</v>
       </c>
       <c r="G435" t="n">
         <v>0</v>
       </c>
       <c r="H435" t="n">
-        <v>37</v>
+        <v>94</v>
       </c>
       <c r="I435" t="n">
         <v>0</v>
@@ -22189,7 +22189,7 @@
         <v>0</v>
       </c>
       <c r="K435" t="n">
-        <v>0.234</v>
+        <v>0.243</v>
       </c>
       <c r="L435" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
prognoza biciklista (zvanicna): 2026-10-22 01:06
</commit_message>
<xml_diff>
--- a/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
+++ b/podaci/vremenska_prognoza/excel/vremenska_prognoza_2026-10.xlsx
@@ -9014,7 +9014,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D178" t="n">
@@ -9364,7 +9364,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D179" t="n">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D180" t="n">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D183" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -9764,7 +9764,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D190" t="n">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D191" t="n">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -10114,7 +10114,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D194" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D196" t="n">
@@ -10264,7 +10264,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D197" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -10364,7 +10364,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -10514,7 +10514,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -10564,7 +10564,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -19864,23 +19864,23 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>15</v>
+        <v>14.7</v>
       </c>
       <c r="E389" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="F389" t="n">
-        <v>15.5</v>
+        <v>14.8</v>
       </c>
       <c r="G389" t="n">
         <v>0</v>
       </c>
       <c r="H389" t="n">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="I389" t="n">
         <v>0</v>
@@ -19889,7 +19889,7 @@
         <v>0</v>
       </c>
       <c r="K389" t="n">
-        <v>0.223</v>
+        <v>0.2</v>
       </c>
       <c r="L389" t="n">
         <v>4</v>
@@ -19914,17 +19914,17 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>15.3</v>
+        <v>14.6</v>
       </c>
       <c r="E390" t="n">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="F390" t="n">
-        <v>12.6</v>
+        <v>13</v>
       </c>
       <c r="G390" t="n">
         <v>0</v>
@@ -19939,7 +19939,7 @@
         <v>0</v>
       </c>
       <c r="K390" t="n">
-        <v>0.224</v>
+        <v>0.2</v>
       </c>
       <c r="L390" t="n">
         <v>4</v>
@@ -19964,23 +19964,23 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>15.6</v>
+        <v>15.1</v>
       </c>
       <c r="E391" t="n">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="F391" t="n">
-        <v>8.300000000000001</v>
+        <v>10.8</v>
       </c>
       <c r="G391" t="n">
         <v>0</v>
       </c>
       <c r="H391" t="n">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="I391" t="n">
         <v>0</v>
@@ -19989,7 +19989,7 @@
         <v>0</v>
       </c>
       <c r="K391" t="n">
-        <v>0.225</v>
+        <v>0.203</v>
       </c>
       <c r="L391" t="n">
         <v>4</v>
@@ -20014,17 +20014,17 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>16</v>
+        <v>14.8</v>
       </c>
       <c r="E392" t="n">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="F392" t="n">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="G392" t="n">
         <v>0</v>
@@ -20033,13 +20033,13 @@
         <v>100</v>
       </c>
       <c r="I392" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J392" t="n">
         <v>0</v>
       </c>
       <c r="K392" t="n">
-        <v>0.23</v>
+        <v>0.205</v>
       </c>
       <c r="L392" t="n">
         <v>4</v>
@@ -20064,17 +20064,17 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>16.5</v>
+        <v>15.5</v>
       </c>
       <c r="E393" t="n">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="F393" t="n">
-        <v>11.5</v>
+        <v>12.2</v>
       </c>
       <c r="G393" t="n">
         <v>0</v>
@@ -20089,7 +20089,7 @@
         <v>0</v>
       </c>
       <c r="K393" t="n">
-        <v>0.233</v>
+        <v>0.215</v>
       </c>
       <c r="L393" t="n">
         <v>4</v>
@@ -20114,32 +20114,32 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>16.7</v>
+        <v>15.3</v>
       </c>
       <c r="E394" t="n">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="F394" t="n">
-        <v>13.7</v>
+        <v>18.4</v>
       </c>
       <c r="G394" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H394" t="n">
         <v>100</v>
       </c>
       <c r="I394" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="J394" t="n">
         <v>0</v>
       </c>
       <c r="K394" t="n">
-        <v>0.259</v>
+        <v>0.242</v>
       </c>
       <c r="L394" t="n">
         <v>4</v>
@@ -20164,32 +20164,32 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>13.7</v>
+        <v>12.4</v>
       </c>
       <c r="E395" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="F395" t="n">
-        <v>23.8</v>
+        <v>25.2</v>
       </c>
       <c r="G395" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="H395" t="n">
         <v>100</v>
       </c>
       <c r="I395" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J395" t="n">
         <v>0</v>
       </c>
       <c r="K395" t="n">
-        <v>0.259</v>
+        <v>0.26</v>
       </c>
       <c r="L395" t="n">
         <v>4</v>
@@ -20214,32 +20214,32 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>12.8</v>
+        <v>11.9</v>
       </c>
       <c r="E396" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="F396" t="n">
-        <v>19.1</v>
+        <v>18</v>
       </c>
       <c r="G396" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H396" t="n">
         <v>100</v>
       </c>
       <c r="I396" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J396" t="n">
         <v>0</v>
       </c>
       <c r="K396" t="n">
-        <v>0.259</v>
+        <v>0.266</v>
       </c>
       <c r="L396" t="n">
         <v>4</v>
@@ -20264,20 +20264,20 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>13.3</v>
+        <v>12.1</v>
       </c>
       <c r="E397" t="n">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F397" t="n">
-        <v>16.6</v>
+        <v>18.4</v>
       </c>
       <c r="G397" t="n">
-        <v>131</v>
+        <v>94</v>
       </c>
       <c r="H397" t="n">
         <v>100</v>
@@ -20289,7 +20289,7 @@
         <v>0</v>
       </c>
       <c r="K397" t="n">
-        <v>0.258</v>
+        <v>0.265</v>
       </c>
       <c r="L397" t="n">
         <v>4</v>
@@ -20314,23 +20314,23 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>14.5</v>
+        <v>13.5</v>
       </c>
       <c r="E398" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="F398" t="n">
-        <v>17.3</v>
+        <v>20.5</v>
       </c>
       <c r="G398" t="n">
-        <v>290</v>
+        <v>336</v>
       </c>
       <c r="H398" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="I398" t="n">
         <v>0</v>
@@ -20339,7 +20339,7 @@
         <v>0</v>
       </c>
       <c r="K398" t="n">
-        <v>0.256</v>
+        <v>0.264</v>
       </c>
       <c r="L398" t="n">
         <v>4</v>
@@ -20364,23 +20364,23 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>15.6</v>
+        <v>13.9</v>
       </c>
       <c r="E399" t="n">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="F399" t="n">
-        <v>19.1</v>
+        <v>18.4</v>
       </c>
       <c r="G399" t="n">
-        <v>400</v>
+        <v>257</v>
       </c>
       <c r="H399" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I399" t="n">
         <v>0</v>
@@ -20389,7 +20389,7 @@
         <v>0</v>
       </c>
       <c r="K399" t="n">
-        <v>0.254</v>
+        <v>0.261</v>
       </c>
       <c r="L399" t="n">
         <v>4</v>
@@ -20414,20 +20414,20 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>15.3</v>
+        <v>14</v>
       </c>
       <c r="E400" t="n">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="F400" t="n">
-        <v>20.2</v>
+        <v>19.4</v>
       </c>
       <c r="G400" t="n">
-        <v>141</v>
+        <v>289</v>
       </c>
       <c r="H400" t="n">
         <v>100</v>
@@ -20439,7 +20439,7 @@
         <v>0</v>
       </c>
       <c r="K400" t="n">
-        <v>0.252</v>
+        <v>0.26</v>
       </c>
       <c r="L400" t="n">
         <v>4</v>
@@ -20464,20 +20464,20 @@
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>14.8</v>
+        <v>13.5</v>
       </c>
       <c r="E401" t="n">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="F401" t="n">
-        <v>21.2</v>
+        <v>19.1</v>
       </c>
       <c r="G401" t="n">
-        <v>91</v>
+        <v>169</v>
       </c>
       <c r="H401" t="n">
         <v>100</v>
@@ -20489,7 +20489,7 @@
         <v>0</v>
       </c>
       <c r="K401" t="n">
-        <v>0.25</v>
+        <v>0.258</v>
       </c>
       <c r="L401" t="n">
         <v>4</v>
@@ -20514,23 +20514,23 @@
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D402" t="n">
-        <v>14.5</v>
+        <v>13.1</v>
       </c>
       <c r="E402" t="n">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="F402" t="n">
-        <v>19.4</v>
+        <v>17.3</v>
       </c>
       <c r="G402" t="n">
-        <v>73</v>
+        <v>230</v>
       </c>
       <c r="H402" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="I402" t="n">
         <v>0</v>
@@ -20539,7 +20539,7 @@
         <v>0</v>
       </c>
       <c r="K402" t="n">
-        <v>0.249</v>
+        <v>0.257</v>
       </c>
       <c r="L402" t="n">
         <v>4</v>
@@ -20564,23 +20564,23 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>14.1</v>
+        <v>12.4</v>
       </c>
       <c r="E403" t="n">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="F403" t="n">
-        <v>16.6</v>
+        <v>16.2</v>
       </c>
       <c r="G403" t="n">
-        <v>48</v>
+        <v>114</v>
       </c>
       <c r="H403" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I403" t="n">
         <v>0</v>
@@ -20589,7 +20589,7 @@
         <v>0</v>
       </c>
       <c r="K403" t="n">
-        <v>0.248</v>
+        <v>0.255</v>
       </c>
       <c r="L403" t="n">
         <v>4</v>
@@ -20614,20 +20614,20 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>13.5</v>
+        <v>11.8</v>
       </c>
       <c r="E404" t="n">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="F404" t="n">
-        <v>15.5</v>
+        <v>14</v>
       </c>
       <c r="G404" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H404" t="n">
         <v>100</v>
@@ -20639,7 +20639,7 @@
         <v>0</v>
       </c>
       <c r="K404" t="n">
-        <v>0.249</v>
+        <v>0.256</v>
       </c>
       <c r="L404" t="n">
         <v>4</v>
@@ -20664,17 +20664,17 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D405" t="n">
-        <v>12.6</v>
+        <v>11.4</v>
       </c>
       <c r="E405" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="F405" t="n">
-        <v>16.9</v>
+        <v>14.4</v>
       </c>
       <c r="G405" t="n">
         <v>0</v>
@@ -20689,7 +20689,7 @@
         <v>0</v>
       </c>
       <c r="K405" t="n">
-        <v>0.248</v>
+        <v>0.258</v>
       </c>
       <c r="L405" t="n">
         <v>4</v>
@@ -20714,17 +20714,17 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D406" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="E406" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F406" t="n">
-        <v>16.2</v>
+        <v>14.4</v>
       </c>
       <c r="G406" t="n">
         <v>0</v>
@@ -20733,13 +20733,13 @@
         <v>100</v>
       </c>
       <c r="I406" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="J406" t="n">
         <v>0</v>
       </c>
       <c r="K406" t="n">
-        <v>0.249</v>
+        <v>0.259</v>
       </c>
       <c r="L406" t="n">
         <v>4</v>
@@ -20764,17 +20764,17 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>11.8</v>
+        <v>11.2</v>
       </c>
       <c r="E407" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F407" t="n">
-        <v>15.8</v>
+        <v>11.9</v>
       </c>
       <c r="G407" t="n">
         <v>0</v>
@@ -20789,7 +20789,7 @@
         <v>0</v>
       </c>
       <c r="K407" t="n">
-        <v>0.256</v>
+        <v>0.261</v>
       </c>
       <c r="L407" t="n">
         <v>4</v>
@@ -20814,23 +20814,23 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>11.5</v>
+        <v>11</v>
       </c>
       <c r="E408" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="F408" t="n">
-        <v>13</v>
+        <v>11.2</v>
       </c>
       <c r="G408" t="n">
         <v>0</v>
       </c>
       <c r="H408" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I408" t="n">
         <v>0</v>
@@ -20839,7 +20839,7 @@
         <v>0</v>
       </c>
       <c r="K408" t="n">
-        <v>0.257</v>
+        <v>0.262</v>
       </c>
       <c r="L408" t="n">
         <v>4</v>
@@ -20864,23 +20864,23 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D409" t="n">
-        <v>10.9</v>
+        <v>10.7</v>
       </c>
       <c r="E409" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="F409" t="n">
-        <v>10.8</v>
+        <v>10.4</v>
       </c>
       <c r="G409" t="n">
         <v>0</v>
       </c>
       <c r="H409" t="n">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="I409" t="n">
         <v>0</v>
@@ -20889,7 +20889,7 @@
         <v>0</v>
       </c>
       <c r="K409" t="n">
-        <v>0.256</v>
+        <v>0.262</v>
       </c>
       <c r="L409" t="n">
         <v>4</v>
@@ -20914,23 +20914,23 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D410" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="E410" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F410" t="n">
-        <v>10.1</v>
+        <v>12.6</v>
       </c>
       <c r="G410" t="n">
         <v>0</v>
       </c>
       <c r="H410" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="I410" t="n">
         <v>0</v>
@@ -20939,7 +20939,7 @@
         <v>0</v>
       </c>
       <c r="K410" t="n">
-        <v>0.256</v>
+        <v>0.262</v>
       </c>
       <c r="L410" t="n">
         <v>4</v>
@@ -20964,23 +20964,23 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D411" t="n">
-        <v>9.4</v>
+        <v>10.2</v>
       </c>
       <c r="E411" t="n">
         <v>96</v>
       </c>
       <c r="F411" t="n">
-        <v>9.4</v>
+        <v>12.2</v>
       </c>
       <c r="G411" t="n">
         <v>0</v>
       </c>
       <c r="H411" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="I411" t="n">
         <v>0</v>
@@ -20989,7 +20989,7 @@
         <v>0</v>
       </c>
       <c r="K411" t="n">
-        <v>0.256</v>
+        <v>0.262</v>
       </c>
       <c r="L411" t="n">
         <v>4</v>
@@ -21014,17 +21014,17 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>8.6</v>
+        <v>9.6</v>
       </c>
       <c r="E412" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F412" t="n">
-        <v>9.4</v>
+        <v>10.1</v>
       </c>
       <c r="G412" t="n">
         <v>0</v>
@@ -21039,7 +21039,7 @@
         <v>0</v>
       </c>
       <c r="K412" t="n">
-        <v>0.256</v>
+        <v>0.262</v>
       </c>
       <c r="L412" t="n">
         <v>5</v>
@@ -21064,17 +21064,17 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D413" t="n">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E413" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F413" t="n">
-        <v>9.699999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="G413" t="n">
         <v>0</v>
@@ -21089,7 +21089,7 @@
         <v>0</v>
       </c>
       <c r="K413" t="n">
-        <v>0.256</v>
+        <v>0.261</v>
       </c>
       <c r="L413" t="n">
         <v>5</v>
@@ -21114,14 +21114,14 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="E414" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F414" t="n">
         <v>6.8</v>
@@ -21139,7 +21139,7 @@
         <v>0</v>
       </c>
       <c r="K414" t="n">
-        <v>0.256</v>
+        <v>0.261</v>
       </c>
       <c r="L414" t="n">
         <v>5</v>
@@ -21164,17 +21164,17 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D415" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="E415" t="n">
         <v>99</v>
       </c>
       <c r="F415" t="n">
-        <v>7.2</v>
+        <v>8.6</v>
       </c>
       <c r="G415" t="n">
         <v>0</v>
@@ -21189,7 +21189,7 @@
         <v>0</v>
       </c>
       <c r="K415" t="n">
-        <v>0.256</v>
+        <v>0.261</v>
       </c>
       <c r="L415" t="n">
         <v>5</v>
@@ -21214,23 +21214,23 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D416" t="n">
         <v>5.8</v>
       </c>
       <c r="E416" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F416" t="n">
-        <v>7.6</v>
+        <v>6.5</v>
       </c>
       <c r="G416" t="n">
         <v>0</v>
       </c>
       <c r="H416" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I416" t="n">
         <v>0</v>
@@ -21239,7 +21239,7 @@
         <v>0</v>
       </c>
       <c r="K416" t="n">
-        <v>0.256</v>
+        <v>0.261</v>
       </c>
       <c r="L416" t="n">
         <v>5</v>
@@ -21264,23 +21264,23 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D417" t="n">
         <v>5.3</v>
       </c>
       <c r="E417" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F417" t="n">
-        <v>6.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G417" t="n">
         <v>0</v>
       </c>
       <c r="H417" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="I417" t="n">
         <v>0</v>
@@ -21289,7 +21289,7 @@
         <v>0</v>
       </c>
       <c r="K417" t="n">
-        <v>0.256</v>
+        <v>0.261</v>
       </c>
       <c r="L417" t="n">
         <v>5</v>
@@ -21314,23 +21314,23 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>5.6</v>
+        <v>5.1</v>
       </c>
       <c r="E418" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F418" t="n">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
       <c r="G418" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="H418" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I418" t="n">
         <v>0</v>
@@ -21339,7 +21339,7 @@
         <v>0</v>
       </c>
       <c r="K418" t="n">
-        <v>0.256</v>
+        <v>0.261</v>
       </c>
       <c r="L418" t="n">
         <v>5</v>
@@ -21364,23 +21364,23 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>8.1</v>
+        <v>7.3</v>
       </c>
       <c r="E419" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="F419" t="n">
-        <v>6.1</v>
+        <v>5.4</v>
       </c>
       <c r="G419" t="n">
-        <v>179</v>
+        <v>160</v>
       </c>
       <c r="H419" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I419" t="n">
         <v>0</v>
@@ -21389,7 +21389,7 @@
         <v>0</v>
       </c>
       <c r="K419" t="n">
-        <v>0.256</v>
+        <v>0.261</v>
       </c>
       <c r="L419" t="n">
         <v>5</v>
@@ -21414,17 +21414,17 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>10.6</v>
+        <v>10</v>
       </c>
       <c r="E420" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F420" t="n">
-        <v>7.2</v>
+        <v>4.7</v>
       </c>
       <c r="G420" t="n">
         <v>329</v>
@@ -21439,7 +21439,7 @@
         <v>0</v>
       </c>
       <c r="K420" t="n">
-        <v>0.255</v>
+        <v>0.26</v>
       </c>
       <c r="L420" t="n">
         <v>5</v>
@@ -21464,20 +21464,20 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D421" t="n">
-        <v>12.3</v>
+        <v>11.6</v>
       </c>
       <c r="E421" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="F421" t="n">
-        <v>4.3</v>
+        <v>1.4</v>
       </c>
       <c r="G421" t="n">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="H421" t="n">
         <v>0</v>
@@ -21489,7 +21489,7 @@
         <v>0</v>
       </c>
       <c r="K421" t="n">
-        <v>0.254</v>
+        <v>0.259</v>
       </c>
       <c r="L421" t="n">
         <v>5</v>
@@ -21514,20 +21514,20 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D422" t="n">
-        <v>13.3</v>
+        <v>13</v>
       </c>
       <c r="E422" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="F422" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="G422" t="n">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="H422" t="n">
         <v>0</v>
@@ -21539,7 +21539,7 @@
         <v>0</v>
       </c>
       <c r="K422" t="n">
-        <v>0.252</v>
+        <v>0.257</v>
       </c>
       <c r="L422" t="n">
         <v>5</v>
@@ -21564,20 +21564,20 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D423" t="n">
-        <v>14.1</v>
+        <v>13.9</v>
       </c>
       <c r="E423" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="F423" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
       <c r="G423" t="n">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="H423" t="n">
         <v>0</v>
@@ -21589,7 +21589,7 @@
         <v>0</v>
       </c>
       <c r="K423" t="n">
-        <v>0.25</v>
+        <v>0.255</v>
       </c>
       <c r="L423" t="n">
         <v>5</v>
@@ -21614,20 +21614,20 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D424" t="n">
-        <v>15.2</v>
+        <v>14.6</v>
       </c>
       <c r="E424" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="F424" t="n">
-        <v>2.9</v>
+        <v>5.4</v>
       </c>
       <c r="G424" t="n">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="H424" t="n">
         <v>0</v>
@@ -21639,7 +21639,7 @@
         <v>0</v>
       </c>
       <c r="K424" t="n">
-        <v>0.248</v>
+        <v>0.253</v>
       </c>
       <c r="L424" t="n">
         <v>5</v>
@@ -21664,20 +21664,20 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D425" t="n">
-        <v>16.2</v>
+        <v>14.7</v>
       </c>
       <c r="E425" t="n">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="F425" t="n">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="G425" t="n">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="H425" t="n">
         <v>0</v>
@@ -21689,7 +21689,7 @@
         <v>0</v>
       </c>
       <c r="K425" t="n">
-        <v>0.246</v>
+        <v>0.251</v>
       </c>
       <c r="L425" t="n">
         <v>5</v>
@@ -21714,23 +21714,23 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>2026-10-21T17:03:41Z</t>
+          <t>2026-10-21T23:03:44Z</t>
         </is>
       </c>
       <c r="D426" t="n">
-        <v>16.4</v>
+        <v>14.6</v>
       </c>
       <c r="E426" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="F426" t="n">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G426" t="n">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="H426" t="n">
-        <v>10</v>
+       